<commit_message>
auto: 2026-06-14 07:20 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-06-13 06:55</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-06-14 06:55</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-06-13) 상위: 반도체  점수 69.0점</t>
+          <t>⚡ 최신(2026-06-14) 상위: 반도체  점수 74.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-06-13) 상위: 로봇  점수 27.0점</t>
+          <t>⚡ 최신(2026-06-14) 상위: 바이오  점수 23.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-06-13) 상위: 인공지능  점수 23.0점</t>
+          <t>⚡ 최신(2026-06-14) 상위: 로봇  점수 22.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -967,14 +967,14 @@
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -990,17 +990,19 @@
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K15" s="17" t="n">
-        <v/>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K15" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1008,14 +1010,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1031,7 +1033,7 @@
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
@@ -1043,7 +1045,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1051,14 +1053,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1074,7 +1076,7 @@
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
@@ -1086,7 +1088,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1094,14 +1096,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1110,14 +1112,14 @@
         <v>0</v>
       </c>
       <c r="H18" s="18" t="n">
-        <v>7.86</v>
+        <v>1.68</v>
       </c>
       <c r="I18" s="19" t="n">
-        <v>-1.98</v>
+        <v>-13.29</v>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K18" s="17" t="inlineStr">
@@ -1129,7 +1131,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1137,14 +1139,14 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1153,14 +1155,14 @@
         <v>0</v>
       </c>
       <c r="H19" s="18" t="n">
-        <v>1.68</v>
+        <v>7.86</v>
       </c>
       <c r="I19" s="19" t="n">
-        <v>-13.29</v>
+        <v>-1.98</v>
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K19" s="17" t="n">
@@ -1170,7 +1172,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1178,7 +1180,7 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
@@ -1193,15 +1195,15 @@
       <c r="G20" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I20" s="15" t="n">
-        <v/>
+      <c r="H20" s="19" t="n">
+        <v>-0.93</v>
+      </c>
+      <c r="I20" s="19" t="n">
+        <v>-13.34</v>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K20" s="17" t="inlineStr">
@@ -1213,7 +1215,7 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1221,14 +1223,14 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>KB금융</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
@@ -1236,27 +1238,27 @@
       <c r="G21" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="18" t="n">
-        <v>6.4</v>
+      <c r="H21" s="19" t="n">
+        <v>-5.04</v>
       </c>
       <c r="I21" s="19" t="n">
-        <v>-6.06</v>
+        <v>-2.45</v>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR) / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1264,14 +1266,14 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -1279,15 +1281,15 @@
       <c r="G22" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="19" t="n">
-        <v>-0.93</v>
-      </c>
-      <c r="I22" s="19" t="n">
-        <v>-13.34</v>
+      <c r="H22" s="18" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="I22" s="18" t="n">
+        <v>3.86</v>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="n">
@@ -1297,7 +1299,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1309,13 +1311,13 @@
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E23" s="15" t="n">
         <v>10</v>
       </c>
       <c r="F23" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G23" s="15" t="n">
         <v>0</v>
@@ -1328,7 +1330,7 @@
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K23" s="17" t="inlineStr">
@@ -1340,7 +1342,7 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1348,14 +1350,14 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>CSA 코스믹</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>0</v>
@@ -1363,27 +1365,27 @@
       <c r="G24" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H24" s="18" t="n">
-        <v>29.93</v>
-      </c>
-      <c r="I24" s="18" t="n">
-        <v>69.53</v>
+      <c r="H24" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I24" s="15" t="n">
+        <v/>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +158% / 중요공시 5건 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K24" s="17" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1391,42 +1393,42 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>CSA 코스믹</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E25" s="15" t="n">
         <v>9</v>
       </c>
       <c r="F25" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G25" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H25" s="18" t="n">
-        <v>2.33</v>
+        <v>29.93</v>
       </c>
       <c r="I25" s="18" t="n">
-        <v>3.86</v>
+        <v>69.53</v>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +244% / 중요공시 5건 / 중요공시 3일 +150% / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K25" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1467,7 +1469,7 @@
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -1508,7 +1510,7 @@
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B28" s="15" t="n">
@@ -1516,169 +1518,169 @@
       </c>
       <c r="C28" s="16" t="inlineStr">
         <is>
-          <t>NH투자증권</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="D28" s="15" t="n">
         <v>8</v>
       </c>
       <c r="E28" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="F28" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G28" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="18" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="I28" s="19" t="n">
+        <v>-4.41</v>
+      </c>
+      <c r="J28" s="17" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 3일 +200% / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K28" s="17" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>모바일어플라이언스</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="F28" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="18" t="n">
+      <c r="E29" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F29" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G29" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="H29" s="19" t="n">
+        <v>-2.09</v>
+      </c>
+      <c r="I29" s="19" t="n">
+        <v>-27.06</v>
+      </c>
+      <c r="J29" s="17" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +50%</t>
+        </is>
+      </c>
+      <c r="K29" s="17" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>NH투자증권</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="F30" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="18" t="n">
         <v>1.76</v>
       </c>
-      <c r="I28" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" s="17" t="inlineStr">
+      <c r="I30" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="17" t="inlineStr">
         <is>
           <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
-      <c r="K28" s="17" t="n">
+      <c r="K30" s="17" t="n">
         <v/>
       </c>
     </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="20" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="B29" s="20" t="n">
-        <v>16</v>
-      </c>
-      <c r="C29" s="21" t="inlineStr">
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
         <is>
           <t>에이팩트</t>
         </is>
       </c>
-      <c r="D29" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E29" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="F29" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H29" s="22" t="n">
+      <c r="D31" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="E31" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F31" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="H31" s="18" t="n">
         <v>13.08</v>
       </c>
-      <c r="I29" s="22" t="n">
+      <c r="I31" s="18" t="n">
         <v>45.57</v>
       </c>
-      <c r="J29" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +81% / 중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K29" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="20" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="B30" s="20" t="n">
-        <v>17</v>
-      </c>
-      <c r="C30" s="21" t="inlineStr">
-        <is>
-          <t>우리금융지주</t>
-        </is>
-      </c>
-      <c r="D30" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E30" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="F30" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="22" t="n">
-        <v>3.32</v>
-      </c>
-      <c r="I30" s="24" t="n">
-        <v>-0.16</v>
-      </c>
-      <c r="J30" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / Google 급상승 검색어 등장 (KR)</t>
-        </is>
-      </c>
-      <c r="K30" s="23" t="inlineStr">
-        <is>
-          <t>공시, Google</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="20" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="B31" s="20" t="n">
-        <v>18</v>
-      </c>
-      <c r="C31" s="21" t="inlineStr">
-        <is>
-          <t>성호전자</t>
-        </is>
-      </c>
-      <c r="D31" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E31" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="F31" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" s="22" t="n">
-        <v>2.41</v>
-      </c>
-      <c r="I31" s="24" t="n">
-        <v>-4.41</v>
-      </c>
-      <c r="J31" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 3건 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K31" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="J31" s="17" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +137% / 중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K31" s="17" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1686,7 +1688,7 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>엑시온그룹</t>
+          <t>후성</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
@@ -1702,26 +1704,26 @@
         <v>0</v>
       </c>
       <c r="H32" s="22" t="n">
-        <v>5.63</v>
+        <v>20.55</v>
       </c>
       <c r="I32" s="22" t="n">
-        <v>4.85</v>
+        <v>63.46</v>
       </c>
       <c r="J32" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 매일경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +322% / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K32" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1729,30 +1731,30 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>모바일어플라이언스</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F33" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G33" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H33" s="24" t="n">
-        <v>-2.09</v>
-      </c>
-      <c r="I33" s="24" t="n">
-        <v>-27.06</v>
+        <v>-4.68</v>
+      </c>
+      <c r="I33" s="22" t="n">
+        <v>19.54</v>
       </c>
       <c r="J33" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 7일 +50%</t>
+          <t>중요공시 4건 / 중요공시 3일 +100%</t>
         </is>
       </c>
       <c r="K33" s="23" t="inlineStr">
@@ -1764,7 +1766,7 @@
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1772,7 +1774,7 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>대양금속</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
@@ -1788,26 +1790,24 @@
         <v>0</v>
       </c>
       <c r="H34" s="22" t="n">
-        <v>1.55</v>
+        <v>2.35</v>
       </c>
       <c r="I34" s="24" t="n">
-        <v>-13.65</v>
+        <v>-7.27</v>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / Google 급상승 검색어 등장 (KR)</t>
-        </is>
-      </c>
-      <c r="K34" s="23" t="inlineStr">
-        <is>
-          <t>공시, Google</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K34" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1815,40 +1815,42 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F35" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G35" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" s="24" t="n">
-        <v>-5.04</v>
+        <v>3</v>
+      </c>
+      <c r="H35" s="22" t="n">
+        <v>6.32</v>
       </c>
       <c r="I35" s="24" t="n">
-        <v>-2.45</v>
+        <v>-3.06</v>
       </c>
       <c r="J35" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K35" s="23" t="n">
-        <v/>
+          <t>중요공시 3건 / 중요공시 7일 +200%</t>
+        </is>
+      </c>
+      <c r="K35" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1856,42 +1858,42 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>에스아이리소스</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F36" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G36" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H36" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I36" s="20" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H36" s="24" t="n">
+        <v>-6.32</v>
+      </c>
+      <c r="I36" s="24" t="n">
+        <v>-9.18</v>
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K36" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1899,7 +1901,7 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>엑시온그룹</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
@@ -1914,25 +1916,27 @@
       <c r="G37" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H37" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I37" s="20" t="n">
-        <v/>
+      <c r="H37" s="22" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="I37" s="22" t="n">
+        <v>4.85</v>
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K37" s="23" t="n">
-        <v/>
+          <t>중요공시 3건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K37" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1973,7 +1977,7 @@
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1981,7 +1985,7 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>태양금속</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
@@ -1997,26 +2001,26 @@
         <v>0</v>
       </c>
       <c r="H39" s="22" t="n">
-        <v>3.3</v>
+        <v>7.85</v>
       </c>
       <c r="I39" s="22" t="n">
-        <v>29.88</v>
+        <v>0.45</v>
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K39" s="23" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2024,42 +2028,42 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>BNK금융지주</t>
+          <t>알엔티엑스</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F40" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G40" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H40" s="22" t="n">
-        <v>5.05</v>
-      </c>
-      <c r="I40" s="22" t="n">
-        <v>2.49</v>
+      <c r="H40" s="24" t="n">
+        <v>-0.44</v>
+      </c>
+      <c r="I40" s="24" t="n">
+        <v>-17.65</v>
       </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
+          <t>중요공시 5건 / 중요공시 3일 +150%</t>
         </is>
       </c>
       <c r="K40" s="23" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2067,14 +2071,14 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>라이콤</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E41" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F41" s="20" t="n">
         <v>0</v>
@@ -2082,27 +2086,27 @@
       <c r="G41" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="22" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="I41" s="24" t="n">
-        <v>-2.1</v>
+      <c r="H41" s="24" t="n">
+        <v>-12.4</v>
+      </c>
+      <c r="I41" s="22" t="n">
+        <v>30.29</v>
       </c>
       <c r="J41" s="23" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
+          <t>네이버 검색 당일 +214% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K41" s="23" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2110,14 +2114,14 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>JB금융지주</t>
+          <t>원익IPS</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E42" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F42" s="20" t="n">
         <v>0</v>
@@ -2126,26 +2130,26 @@
         <v>0</v>
       </c>
       <c r="H42" s="22" t="n">
-        <v>2.69</v>
+        <v>30</v>
       </c>
       <c r="I42" s="22" t="n">
-        <v>3.69</v>
+        <v>38.13</v>
       </c>
       <c r="J42" s="23" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
+          <t>네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K42" s="23" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2153,14 +2157,14 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>iM금융지주</t>
+          <t>하림</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E43" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F43" s="20" t="n">
         <v>0</v>
@@ -2169,26 +2173,24 @@
         <v>0</v>
       </c>
       <c r="H43" s="24" t="n">
-        <v>-3.38</v>
-      </c>
-      <c r="I43" s="20" t="n">
-        <v>0</v>
+        <v>-0.87</v>
+      </c>
+      <c r="I43" s="22" t="n">
+        <v>0.71</v>
       </c>
       <c r="J43" s="23" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
-        </is>
-      </c>
-      <c r="K43" s="23" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
+          <t>한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K43" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2196,14 +2198,14 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>금호타이어</t>
+          <t>대한광통신</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E44" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F44" s="20" t="n">
         <v>0</v>
@@ -2212,26 +2214,26 @@
         <v>0</v>
       </c>
       <c r="H44" s="22" t="n">
-        <v>5.97</v>
+        <v>11.54</v>
       </c>
       <c r="I44" s="22" t="n">
-        <v>3.01</v>
+        <v>5.31</v>
       </c>
       <c r="J44" s="23" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
+          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K44" s="23" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2239,42 +2241,42 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>금호전기</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E45" s="20" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F45" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G45" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H45" s="22" t="n">
-        <v>1.83</v>
-      </c>
-      <c r="I45" s="24" t="n">
-        <v>-6.17</v>
+        <v>28.36</v>
+      </c>
+      <c r="I45" s="22" t="n">
+        <v>19.41</v>
       </c>
       <c r="J45" s="23" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K45" s="23" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
@@ -2282,14 +2284,14 @@
       </c>
       <c r="C46" s="21" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>삼성바이오로직스</t>
         </is>
       </c>
       <c r="D46" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E46" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F46" s="20" t="n">
         <v>0</v>
@@ -2298,26 +2300,26 @@
         <v>0</v>
       </c>
       <c r="H46" s="22" t="n">
-        <v>4.57</v>
+        <v>0.7</v>
       </c>
       <c r="I46" s="24" t="n">
-        <v>-2.43</v>
+        <v>-3.36</v>
       </c>
       <c r="J46" s="23" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
+          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K46" s="23" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B47" s="20" t="n">
@@ -2325,14 +2327,14 @@
       </c>
       <c r="C47" s="21" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="D47" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E47" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F47" s="20" t="n">
         <v>0</v>
@@ -2348,19 +2350,17 @@
       </c>
       <c r="J47" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K47" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K47" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="20" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B48" s="20" t="n">
@@ -2368,7 +2368,7 @@
       </c>
       <c r="C48" s="21" t="inlineStr">
         <is>
-          <t>라이콤</t>
+          <t>KB금융</t>
         </is>
       </c>
       <c r="D48" s="20" t="n">
@@ -2383,27 +2383,25 @@
       <c r="G48" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H48" s="24" t="n">
-        <v>-12.4</v>
-      </c>
-      <c r="I48" s="22" t="n">
-        <v>30.29</v>
+      <c r="H48" s="22" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="I48" s="24" t="n">
+        <v>-6.06</v>
       </c>
       <c r="J48" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +160% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K48" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K48" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="20" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B49" s="20" t="n">
@@ -2411,7 +2409,7 @@
       </c>
       <c r="C49" s="21" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="D49" s="20" t="n">
@@ -2426,197 +2424,199 @@
       <c r="G49" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="22" t="n">
-        <v>7.85</v>
-      </c>
-      <c r="I49" s="22" t="n">
-        <v>0.45</v>
+      <c r="H49" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I49" s="20" t="n">
+        <v/>
       </c>
       <c r="J49" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K49" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="20" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="B50" s="20" t="n">
+      <c r="A50" s="25" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B50" s="25" t="n">
         <v>37</v>
       </c>
-      <c r="C50" s="21" t="inlineStr">
-        <is>
-          <t>대한광통신</t>
-        </is>
-      </c>
-      <c r="D50" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E50" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F50" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G50" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H50" s="22" t="n">
-        <v>11.54</v>
-      </c>
-      <c r="I50" s="22" t="n">
-        <v>5.31</v>
-      </c>
-      <c r="J50" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K50" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
+      <c r="C50" s="26" t="inlineStr">
+        <is>
+          <t>세미티에스</t>
+        </is>
+      </c>
+      <c r="D50" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E50" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F50" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="27" t="n">
+        <v>29.97</v>
+      </c>
+      <c r="I50" s="28" t="n">
+        <v>-7.54</v>
+      </c>
+      <c r="J50" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +4221%</t>
+        </is>
+      </c>
+      <c r="K50" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="20" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="B51" s="20" t="n">
+      <c r="A51" s="25" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B51" s="25" t="n">
         <v>38</v>
       </c>
-      <c r="C51" s="21" t="inlineStr">
-        <is>
-          <t>에스아이리소스</t>
-        </is>
-      </c>
-      <c r="D51" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E51" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F51" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G51" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H51" s="24" t="n">
-        <v>-6.32</v>
-      </c>
-      <c r="I51" s="24" t="n">
-        <v>-9.18</v>
-      </c>
-      <c r="J51" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K51" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C51" s="26" t="inlineStr">
+        <is>
+          <t>화신정공</t>
+        </is>
+      </c>
+      <c r="D51" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E51" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F51" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="27" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="I51" s="27" t="n">
+        <v>142.33</v>
+      </c>
+      <c r="J51" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +2072%</t>
+        </is>
+      </c>
+      <c r="K51" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="20" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="B52" s="20" t="n">
+      <c r="A52" s="25" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B52" s="25" t="n">
         <v>39</v>
       </c>
-      <c r="C52" s="21" t="inlineStr">
-        <is>
-          <t>현대건설</t>
-        </is>
-      </c>
-      <c r="D52" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E52" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F52" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G52" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H52" s="22" t="n">
-        <v>28.36</v>
-      </c>
-      <c r="I52" s="22" t="n">
-        <v>19.41</v>
-      </c>
-      <c r="J52" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K52" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C52" s="26" t="inlineStr">
+        <is>
+          <t>마니커</t>
+        </is>
+      </c>
+      <c r="D52" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E52" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F52" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" s="28" t="n">
+        <v>-5.97</v>
+      </c>
+      <c r="I52" s="27" t="n">
+        <v>24.75</v>
+      </c>
+      <c r="J52" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +495%</t>
+        </is>
+      </c>
+      <c r="K52" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="20" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="B53" s="20" t="n">
+      <c r="A53" s="25" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B53" s="25" t="n">
         <v>40</v>
       </c>
-      <c r="C53" s="21" t="inlineStr">
-        <is>
-          <t>DB</t>
-        </is>
-      </c>
-      <c r="D53" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E53" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F53" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G53" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H53" s="22" t="n">
-        <v>3.09</v>
-      </c>
-      <c r="I53" s="22" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="J53" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K53" s="23" t="n">
-        <v/>
+      <c r="C53" s="26" t="inlineStr">
+        <is>
+          <t>SK이터닉스</t>
+        </is>
+      </c>
+      <c r="D53" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E53" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F53" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" s="27" t="n">
+        <v>6.04</v>
+      </c>
+      <c r="I53" s="27" t="n">
+        <v>21.64</v>
+      </c>
+      <c r="J53" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +264%</t>
+        </is>
+      </c>
+      <c r="K53" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2624,7 +2624,7 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>세미티에스</t>
+          <t>마니커에프앤지</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -2639,15 +2639,15 @@
       <c r="G54" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H54" s="27" t="n">
-        <v>29.97</v>
-      </c>
-      <c r="I54" s="28" t="n">
-        <v>-7.54</v>
+      <c r="H54" s="28" t="n">
+        <v>-15.17</v>
+      </c>
+      <c r="I54" s="27" t="n">
+        <v>3.85</v>
       </c>
       <c r="J54" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +3403%</t>
+          <t>네이버 검색 당일 +190%</t>
         </is>
       </c>
       <c r="K54" s="29" t="inlineStr">
@@ -2659,7 +2659,7 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>화신정공</t>
+          <t>랩지노믹스</t>
         </is>
       </c>
       <c r="D55" s="25" t="n">
@@ -2682,15 +2682,15 @@
       <c r="G55" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H55" s="27" t="n">
-        <v>6.18</v>
+      <c r="H55" s="28" t="n">
+        <v>-3.41</v>
       </c>
       <c r="I55" s="27" t="n">
-        <v>142.33</v>
+        <v>24.65</v>
       </c>
       <c r="J55" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1692%</t>
+          <t>네이버 검색 당일 +138%</t>
         </is>
       </c>
       <c r="K55" s="29" t="inlineStr">
@@ -2702,7 +2702,7 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2710,7 +2710,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>마니커</t>
+          <t>아이로보틱스</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2725,15 +2725,15 @@
       <c r="G56" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H56" s="28" t="n">
-        <v>-5.97</v>
+      <c r="H56" s="27" t="n">
+        <v>22.3</v>
       </c>
       <c r="I56" s="27" t="n">
-        <v>24.75</v>
+        <v>27.7</v>
       </c>
       <c r="J56" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +267%</t>
+          <t>네이버 검색 당일 +137%</t>
         </is>
       </c>
       <c r="K56" s="29" t="inlineStr">
@@ -2745,7 +2745,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2753,7 +2753,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>후성</t>
+          <t>테크윙</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2769,14 +2769,14 @@
         <v>0</v>
       </c>
       <c r="H57" s="27" t="n">
-        <v>20.55</v>
+        <v>6.87</v>
       </c>
       <c r="I57" s="27" t="n">
-        <v>63.46</v>
+        <v>19.38</v>
       </c>
       <c r="J57" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +216%</t>
+          <t>네이버 검색 당일 +128%</t>
         </is>
       </c>
       <c r="K57" s="29" t="inlineStr">
@@ -2788,7 +2788,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>SK이터닉스</t>
+          <t>제주은행</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2812,14 +2812,14 @@
         <v>0</v>
       </c>
       <c r="H58" s="27" t="n">
-        <v>6.04</v>
+        <v>0.16</v>
       </c>
       <c r="I58" s="27" t="n">
-        <v>21.64</v>
+        <v>15.07</v>
       </c>
       <c r="J58" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +211%</t>
+          <t>네이버 검색 당일 +100%</t>
         </is>
       </c>
       <c r="K58" s="29" t="inlineStr">
@@ -2831,7 +2831,7 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2839,7 +2839,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>랩지노믹스</t>
+          <t>SK네트웍스</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2854,15 +2854,15 @@
       <c r="G59" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H59" s="28" t="n">
-        <v>-3.41</v>
+      <c r="H59" s="27" t="n">
+        <v>11.4</v>
       </c>
       <c r="I59" s="27" t="n">
-        <v>24.65</v>
+        <v>19.27</v>
       </c>
       <c r="J59" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +115%</t>
+          <t>네이버 검색 당일 +73% / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K59" s="29" t="inlineStr">
@@ -2874,7 +2874,7 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2882,7 +2882,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>하나마이크론</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2897,27 +2897,27 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="28" t="n">
-        <v>-4.68</v>
+      <c r="H60" s="27" t="n">
+        <v>2.09</v>
       </c>
       <c r="I60" s="27" t="n">
-        <v>19.54</v>
+        <v>16.97</v>
       </c>
       <c r="J60" s="29" t="inlineStr">
         <is>
-          <t>중요공시 4건</t>
+          <t>네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K60" s="29" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2925,7 +2925,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>하림</t>
+          <t>저스템</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2940,15 +2940,15 @@
       <c r="G61" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H61" s="28" t="n">
-        <v>-0.87</v>
+      <c r="H61" s="27" t="n">
+        <v>15.21</v>
       </c>
       <c r="I61" s="27" t="n">
-        <v>0.71</v>
+        <v>19.29</v>
       </c>
       <c r="J61" s="29" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K61" s="29" t="n">
@@ -2958,7 +2958,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2966,7 +2966,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>NAVER</t>
+          <t>리노공업</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2982,26 +2982,24 @@
         <v>0</v>
       </c>
       <c r="H62" s="27" t="n">
-        <v>10.27</v>
-      </c>
-      <c r="I62" s="28" t="n">
-        <v>-3.33</v>
+        <v>4.71</v>
+      </c>
+      <c r="I62" s="27" t="n">
+        <v>11.05</v>
       </c>
       <c r="J62" s="29" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K62" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K62" s="29" t="n">
+        <v/>
       </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3009,7 +3007,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>저스템</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3025,14 +3023,14 @@
         <v>0</v>
       </c>
       <c r="H63" s="27" t="n">
-        <v>15.21</v>
-      </c>
-      <c r="I63" s="27" t="n">
-        <v>19.29</v>
+        <v>5.08</v>
+      </c>
+      <c r="I63" s="28" t="n">
+        <v>-2.62</v>
       </c>
       <c r="J63" s="29" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K63" s="29" t="n">
@@ -3132,22 +3130,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3156,29 +3154,29 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B4" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H4" s="25" t="n"/>
@@ -3187,29 +3185,29 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H5" s="25" t="n"/>
@@ -3218,29 +3216,29 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H6" s="25" t="n"/>
@@ -3249,77 +3247,77 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H7" s="27" t="n">
-        <v>7.86</v>
+        <v>1.68</v>
       </c>
       <c r="I7" s="28" t="n">
-        <v>-1.98</v>
+        <v>-13.29</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="H8" s="27" t="n">
-        <v>1.68</v>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="H8" s="28" t="n">
+        <v>-0.93</v>
       </c>
       <c r="I8" s="28" t="n">
-        <v>-13.29</v>
+        <v>-13.34</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
@@ -3336,190 +3334,190 @@
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="H9" s="25" t="n"/>
-      <c r="I9" s="25" t="n"/>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="H9" s="28" t="n">
+        <v>-5.04</v>
+      </c>
+      <c r="I9" s="28" t="n">
+        <v>-2.45</v>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>KB금융</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H10" s="27" t="n">
-        <v>6.4</v>
+        <v>7.86</v>
       </c>
       <c r="I10" s="28" t="n">
-        <v>-6.06</v>
+        <v>-1.98</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="H11" s="28" t="n">
-        <v>-0.93</v>
-      </c>
-      <c r="I11" s="28" t="n">
-        <v>-13.34</v>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="H11" s="27" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="I11" s="27" t="n">
+        <v>3.86</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>한미반도체</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="H12" s="27" t="n">
-        <v>24.05</v>
-      </c>
-      <c r="I12" s="27" t="n">
-        <v>27.56</v>
-      </c>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="H12" s="25" t="n"/>
+      <c r="I12" s="25" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>CSA 코스믹</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H13" s="27" t="n">
-        <v>29.93</v>
+        <v>24.05</v>
       </c>
       <c r="I13" s="27" t="n">
-        <v>69.53</v>
+        <v>27.56</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>CSA 코스믹</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H14" s="27" t="n">
-        <v>2.33</v>
+        <v>29.93</v>
       </c>
       <c r="I14" s="27" t="n">
-        <v>3.86</v>
+        <v>69.53</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
@@ -3542,12 +3540,12 @@
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H15" s="25" t="n"/>
@@ -3573,12 +3571,12 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H16" s="27" t="n">
@@ -3608,12 +3606,12 @@
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H17" s="27" t="n">
@@ -3626,108 +3624,112 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>모바일어플라이언스</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E18" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="H18" s="25" t="n"/>
-      <c r="I18" s="25" t="n"/>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="H18" s="28" t="n">
+        <v>-2.09</v>
+      </c>
+      <c r="I18" s="28" t="n">
+        <v>-27.06</v>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>대양금속</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H19" s="27" t="n">
-        <v>1.55</v>
+        <v>2.41</v>
       </c>
       <c r="I19" s="28" t="n">
-        <v>-13.65</v>
+        <v>-4.41</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>모바일어플라이언스</t>
+          <t>에이팩트</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D20" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="H20" s="28" t="n">
-        <v>-2.09</v>
-      </c>
-      <c r="I20" s="28" t="n">
-        <v>-27.06</v>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="H20" s="27" t="n">
+        <v>13.08</v>
+      </c>
+      <c r="I20" s="27" t="n">
+        <v>45.57</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -3744,25 +3746,25 @@
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="H21" s="28" t="n">
-        <v>-5.04</v>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="H21" s="27" t="n">
+        <v>2.35</v>
       </c>
       <c r="I21" s="28" t="n">
-        <v>-2.45</v>
+        <v>-7.27</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -3779,25 +3781,25 @@
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H22" s="27" t="n">
-        <v>2.41</v>
+        <v>6.32</v>
       </c>
       <c r="I22" s="28" t="n">
-        <v>-4.41</v>
+        <v>-3.06</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3814,21 +3816,25 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="H23" s="25" t="n"/>
-      <c r="I23" s="25" t="n"/>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="H23" s="28" t="n">
+        <v>-4.68</v>
+      </c>
+      <c r="I23" s="27" t="n">
+        <v>19.54</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>에이팩트</t>
+          <t>에스아이리소스</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3845,19 +3851,19 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="H24" s="27" t="n">
-        <v>13.08</v>
-      </c>
-      <c r="I24" s="27" t="n">
-        <v>45.57</v>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="H24" s="28" t="n">
+        <v>-6.32</v>
+      </c>
+      <c r="I24" s="28" t="n">
+        <v>-9.18</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
@@ -3880,12 +3886,12 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H25" s="27" t="n">
@@ -3898,7 +3904,7 @@
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>우리금융지주</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
@@ -3915,25 +3921,25 @@
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H26" s="27" t="n">
-        <v>3.32</v>
-      </c>
-      <c r="I26" s="28" t="n">
-        <v>-0.16</v>
+        <v>10.67</v>
+      </c>
+      <c r="I26" s="27" t="n">
+        <v>8.93</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>후성</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
@@ -3950,25 +3956,25 @@
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H27" s="27" t="n">
-        <v>10.67</v>
+        <v>20.55</v>
       </c>
       <c r="I27" s="27" t="n">
-        <v>8.93</v>
+        <v>63.46</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>알엔티엑스</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
@@ -3985,21 +3991,25 @@
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="H28" s="25" t="n"/>
-      <c r="I28" s="25" t="n"/>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="H28" s="28" t="n">
+        <v>-0.44</v>
+      </c>
+      <c r="I28" s="28" t="n">
+        <v>-17.65</v>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>BNK금융지주</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
@@ -4016,270 +4026,262 @@
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H29" s="27" t="n">
-        <v>5.05</v>
+        <v>7.85</v>
       </c>
       <c r="I29" s="27" t="n">
-        <v>2.49</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>JB금융지주</t>
+          <t>KB금융</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C30" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D30" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E30" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H30" s="27" t="n">
-        <v>2.69</v>
-      </c>
-      <c r="I30" s="27" t="n">
-        <v>3.69</v>
+        <v>6.4</v>
+      </c>
+      <c r="I30" s="28" t="n">
+        <v>-6.06</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>iM금융지주</t>
+          <t>대한광통신</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C31" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D31" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E31" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="H31" s="28" t="n">
-        <v>-3.38</v>
-      </c>
-      <c r="I31" s="25" t="n">
-        <v>0</v>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="H31" s="27" t="n">
+        <v>11.54</v>
+      </c>
+      <c r="I31" s="27" t="n">
+        <v>5.31</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>금호전기</t>
+          <t>라이콤</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C32" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D32" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E32" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="H32" s="27" t="n">
-        <v>1.83</v>
-      </c>
-      <c r="I32" s="28" t="n">
-        <v>-6.17</v>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="H32" s="28" t="n">
+        <v>-12.4</v>
+      </c>
+      <c r="I32" s="27" t="n">
+        <v>30.29</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>금호타이어</t>
+          <t>삼성바이오로직스</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C33" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D33" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E33" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H33" s="27" t="n">
-        <v>5.97</v>
-      </c>
-      <c r="I33" s="27" t="n">
-        <v>3.01</v>
+        <v>0.7</v>
+      </c>
+      <c r="I33" s="28" t="n">
+        <v>-3.36</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>태양금속</t>
+          <t>원익IPS</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C34" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D34" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E34" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H34" s="27" t="n">
-        <v>3.3</v>
+        <v>30</v>
       </c>
       <c r="I34" s="27" t="n">
-        <v>29.88</v>
+        <v>38.13</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D35" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E35" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="H35" s="27" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="I35" s="28" t="n">
-        <v>-2.1</v>
-      </c>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="H35" s="25" t="n"/>
+      <c r="I35" s="25" t="n"/>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C36" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D36" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E36" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="H36" s="27" t="n">
-        <v>4.57</v>
-      </c>
-      <c r="I36" s="28" t="n">
-        <v>-2.43</v>
-      </c>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="H36" s="25" t="n"/>
+      <c r="I36" s="25" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>하림</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
@@ -4296,25 +4298,25 @@
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="H37" s="27" t="n">
-        <v>3.09</v>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="H37" s="28" t="n">
+        <v>-0.87</v>
       </c>
       <c r="I37" s="27" t="n">
-        <v>4.4</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>대한광통신</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4331,165 +4333,165 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H38" s="27" t="n">
-        <v>11.54</v>
+        <v>28.36</v>
       </c>
       <c r="I38" s="27" t="n">
-        <v>5.31</v>
+        <v>19.41</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>라이콤</t>
+          <t>SK네트웍스</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C39" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D39" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E39" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="H39" s="28" t="n">
-        <v>-12.4</v>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="H39" s="27" t="n">
+        <v>11.4</v>
       </c>
       <c r="I39" s="27" t="n">
-        <v>30.29</v>
+        <v>19.27</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>에스아이리소스</t>
+          <t>SK이터닉스</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C40" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D40" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E40" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="H40" s="28" t="n">
-        <v>-6.32</v>
-      </c>
-      <c r="I40" s="28" t="n">
-        <v>-9.18</v>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="H40" s="27" t="n">
+        <v>6.04</v>
+      </c>
+      <c r="I40" s="27" t="n">
+        <v>21.64</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C41" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D41" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E41" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H41" s="27" t="n">
-        <v>7.85</v>
-      </c>
-      <c r="I41" s="27" t="n">
-        <v>0.45</v>
+        <v>5.08</v>
+      </c>
+      <c r="I41" s="28" t="n">
+        <v>-2.62</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>현대건설</t>
+          <t>랩지노믹스</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C42" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D42" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E42" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="H42" s="27" t="n">
-        <v>28.36</v>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="H42" s="28" t="n">
+        <v>-3.41</v>
       </c>
       <c r="I42" s="27" t="n">
-        <v>19.41</v>
+        <v>24.65</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>NAVER</t>
+          <t>리노공업</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4506,25 +4508,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H43" s="27" t="n">
-        <v>10.27</v>
-      </c>
-      <c r="I43" s="28" t="n">
-        <v>-3.33</v>
+        <v>4.71</v>
+      </c>
+      <c r="I43" s="27" t="n">
+        <v>11.05</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>SK이터닉스</t>
+          <t>마니커</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4541,25 +4543,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="H44" s="27" t="n">
-        <v>6.04</v>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="H44" s="28" t="n">
+        <v>-5.97</v>
       </c>
       <c r="I44" s="27" t="n">
-        <v>21.64</v>
+        <v>24.75</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>랩지노믹스</t>
+          <t>마니커에프앤지</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4576,25 +4578,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H45" s="28" t="n">
-        <v>-3.41</v>
+        <v>-15.17</v>
       </c>
       <c r="I45" s="27" t="n">
-        <v>24.65</v>
+        <v>3.85</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>마니커</t>
+          <t>세미티에스</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4611,25 +4613,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="H46" s="28" t="n">
-        <v>-5.97</v>
-      </c>
-      <c r="I46" s="27" t="n">
-        <v>24.75</v>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="H46" s="27" t="n">
+        <v>29.97</v>
+      </c>
+      <c r="I46" s="28" t="n">
+        <v>-7.54</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>세미티에스</t>
+          <t>아이로보틱스</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4646,25 +4648,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H47" s="27" t="n">
-        <v>29.97</v>
-      </c>
-      <c r="I47" s="28" t="n">
-        <v>-7.54</v>
+        <v>22.3</v>
+      </c>
+      <c r="I47" s="27" t="n">
+        <v>27.7</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>저스템</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4681,25 +4683,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="H48" s="28" t="n">
-        <v>-4.68</v>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="H48" s="27" t="n">
+        <v>15.21</v>
       </c>
       <c r="I48" s="27" t="n">
-        <v>19.54</v>
+        <v>19.29</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>저스템</t>
+          <t>제주은행</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4716,25 +4718,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H49" s="27" t="n">
-        <v>15.21</v>
+        <v>0.16</v>
       </c>
       <c r="I49" s="27" t="n">
-        <v>19.29</v>
+        <v>15.07</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>하림</t>
+          <t>테크윙</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4751,25 +4753,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="H50" s="28" t="n">
-        <v>-0.87</v>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="H50" s="27" t="n">
+        <v>6.87</v>
       </c>
       <c r="I50" s="27" t="n">
-        <v>0.71</v>
+        <v>19.38</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>화신정공</t>
+          <t>하나마이크론</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4786,25 +4788,25 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H51" s="27" t="n">
-        <v>6.18</v>
+        <v>2.09</v>
       </c>
       <c r="I51" s="27" t="n">
-        <v>142.33</v>
+        <v>16.97</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="26" t="inlineStr">
         <is>
-          <t>후성</t>
+          <t>화신정공</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -4821,19 +4823,19 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="H52" s="27" t="n">
-        <v>20.55</v>
+        <v>6.18</v>
       </c>
       <c r="I52" s="27" t="n">
-        <v>63.46</v>
+        <v>142.33</v>
       </c>
     </row>
   </sheetData>
@@ -4917,19 +4919,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4948,19 +4950,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4972,26 +4974,26 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="35" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B5" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5003,26 +5005,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5034,26 +5036,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5065,26 +5067,26 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5096,26 +5098,26 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B9" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5127,26 +5129,26 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="35" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B10" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="36" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="D10" s="36" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="E10" s="36" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="F10" s="37" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G10" s="37" t="inlineStr">
@@ -5212,7 +5214,7 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -5239,7 +5241,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5428,7 +5430,7 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -5455,7 +5457,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -5482,7 +5484,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>Tesla</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -5509,7 +5511,7 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>Tesla</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-06-15 07:21 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-06-14 06:55</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-06-15 06:54</t>
         </is>
       </c>
     </row>
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-06-14) 상위: 반도체  점수 74.0점</t>
+          <t>⚡ 최신(2026-06-15) 상위: 반도체  점수 68.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-06-14) 상위: 바이오  점수 23.0점</t>
+          <t>⚡ 최신(2026-06-15) 상위: 인공지능  점수 17.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-06-14) 상위: 로봇  점수 22.0점</t>
+          <t>⚡ 최신(2026-06-15) 상위: 삼성전자  점수 15.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -967,14 +967,14 @@
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -990,7 +990,7 @@
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1010,14 +1010,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1025,15 +1025,15 @@
       <c r="G16" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I16" s="15" t="n">
-        <v/>
+      <c r="H16" s="18" t="n">
+        <v>7.86</v>
+      </c>
+      <c r="I16" s="19" t="n">
+        <v>-1.98</v>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
@@ -1045,7 +1045,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1053,14 +1053,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1068,27 +1068,25 @@
       <c r="G17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="15" t="n">
+      <c r="H17" s="19" t="n">
+        <v>-5.04</v>
+      </c>
+      <c r="I17" s="19" t="n">
+        <v>-2.45</v>
+      </c>
+      <c r="J17" s="17" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K17" s="17" t="n">
         <v/>
-      </c>
-      <c r="I17" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J17" s="17" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K17" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1096,14 +1094,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1111,15 +1109,15 @@
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="18" t="n">
-        <v>1.68</v>
-      </c>
-      <c r="I18" s="19" t="n">
-        <v>-13.29</v>
+      <c r="H18" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I18" s="15" t="n">
+        <v/>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K18" s="17" t="inlineStr">
@@ -1131,7 +1129,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1139,7 +1137,7 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
@@ -1154,25 +1152,27 @@
       <c r="G19" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="18" t="n">
-        <v>7.86</v>
-      </c>
-      <c r="I19" s="19" t="n">
-        <v>-1.98</v>
+      <c r="H19" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I19" s="15" t="n">
+        <v/>
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K19" s="17" t="n">
-        <v/>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K19" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K20" s="17" t="inlineStr">
@@ -1215,7 +1215,7 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1223,14 +1223,14 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
@@ -1238,15 +1238,15 @@
       <c r="G21" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="19" t="n">
-        <v>-5.04</v>
+      <c r="H21" s="18" t="n">
+        <v>2.35</v>
       </c>
       <c r="I21" s="19" t="n">
-        <v>-2.45</v>
+        <v>-7.27</v>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
@@ -1258,7 +1258,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1270,10 +1270,10 @@
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="n">
@@ -1299,7 +1299,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1307,42 +1307,42 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>한미반도체</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F23" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G23" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="18" t="n">
-        <v>24.05</v>
-      </c>
-      <c r="I23" s="18" t="n">
-        <v>27.56</v>
+      <c r="H23" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I23" s="15" t="n">
+        <v/>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K23" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1350,42 +1350,42 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>CSA 코스믹</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G24" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H24" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I24" s="15" t="n">
-        <v/>
+      <c r="H24" s="18" t="n">
+        <v>29.93</v>
+      </c>
+      <c r="I24" s="18" t="n">
+        <v>69.53</v>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +262% / 중요공시 5건 / 중요공시 3일 +67%</t>
         </is>
       </c>
       <c r="K24" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1393,14 +1393,14 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>CSA 코스믹</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F25" s="15" t="n">
         <v>2</v>
@@ -1409,26 +1409,26 @@
         <v>0</v>
       </c>
       <c r="H25" s="18" t="n">
-        <v>29.93</v>
-      </c>
-      <c r="I25" s="18" t="n">
-        <v>69.53</v>
+        <v>2.41</v>
+      </c>
+      <c r="I25" s="19" t="n">
+        <v>-4.41</v>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +244% / 중요공시 5건 / 중요공시 3일 +150% / 매일경제 헤드라인 언급</t>
+          <t>중요공시 3건 / 중요공시 3일 +200% / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K25" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1436,40 +1436,42 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>알엔티엑스</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="F26" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G26" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I26" s="15" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H26" s="19" t="n">
+        <v>-0.44</v>
+      </c>
+      <c r="I26" s="19" t="n">
+        <v>-17.65</v>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K26" s="17" t="n">
-        <v/>
+          <t>중요공시 5건 / 중요공시 3일 +150% / 중요공시 7일 +67%</t>
+        </is>
+      </c>
+      <c r="K26" s="17" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -1477,40 +1479,42 @@
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>모바일어플라이언스</t>
         </is>
       </c>
       <c r="D27" s="15" t="n">
         <v>8</v>
       </c>
       <c r="E27" s="15" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F27" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G27" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="18" t="n">
-        <v>7.26</v>
-      </c>
-      <c r="I27" s="18" t="n">
-        <v>6.83</v>
+        <v>3</v>
+      </c>
+      <c r="H27" s="19" t="n">
+        <v>-2.09</v>
+      </c>
+      <c r="I27" s="19" t="n">
+        <v>-27.06</v>
       </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K27" s="17" t="n">
-        <v/>
+          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +200%</t>
+        </is>
+      </c>
+      <c r="K27" s="17" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B28" s="15" t="n">
@@ -1518,42 +1522,42 @@
       </c>
       <c r="C28" s="16" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>에이팩트</t>
         </is>
       </c>
       <c r="D28" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E28" s="15" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F28" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G28" s="15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H28" s="18" t="n">
-        <v>2.41</v>
-      </c>
-      <c r="I28" s="19" t="n">
-        <v>-4.41</v>
+        <v>13.08</v>
+      </c>
+      <c r="I28" s="18" t="n">
+        <v>45.57</v>
       </c>
       <c r="J28" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200% / 한국경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +148% / 중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K28" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B29" s="15" t="n">
@@ -1561,30 +1565,30 @@
       </c>
       <c r="C29" s="16" t="inlineStr">
         <is>
-          <t>모바일어플라이언스</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="D29" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E29" s="15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F29" s="15" t="n">
         <v>2</v>
       </c>
       <c r="G29" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H29" s="19" t="n">
-        <v>-2.09</v>
-      </c>
-      <c r="I29" s="19" t="n">
-        <v>-27.06</v>
+        <v>0</v>
+      </c>
+      <c r="H29" s="18" t="n">
+        <v>24.05</v>
+      </c>
+      <c r="I29" s="18" t="n">
+        <v>27.56</v>
       </c>
       <c r="J29" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +50%</t>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K29" s="17" t="inlineStr">
@@ -1596,7 +1600,7 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="15" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B30" s="15" t="n">
@@ -1604,14 +1608,14 @@
       </c>
       <c r="C30" s="16" t="inlineStr">
         <is>
-          <t>NH투자증권</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="D30" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E30" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F30" s="15" t="n">
         <v>0</v>
@@ -1619,15 +1623,15 @@
       <c r="G30" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H30" s="18" t="n">
-        <v>1.76</v>
+      <c r="H30" s="15" t="n">
+        <v/>
       </c>
       <c r="I30" s="15" t="n">
-        <v>0</v>
+        <v/>
       </c>
       <c r="J30" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K30" s="17" t="n">
@@ -1637,7 +1641,7 @@
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="15" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B31" s="15" t="n">
@@ -1645,42 +1649,42 @@
       </c>
       <c r="C31" s="16" t="inlineStr">
         <is>
-          <t>에이팩트</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D31" s="15" t="n">
         <v>7</v>
       </c>
       <c r="E31" s="15" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F31" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G31" s="15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H31" s="18" t="n">
-        <v>13.08</v>
-      </c>
-      <c r="I31" s="18" t="n">
-        <v>45.57</v>
+        <v>1.68</v>
+      </c>
+      <c r="I31" s="19" t="n">
+        <v>-13.29</v>
       </c>
       <c r="J31" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +137% / 중요공시 2건 / 중요공시 7일 +100%</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K31" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1711,7 +1715,7 @@
       </c>
       <c r="J32" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +322% / 매일경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +343% / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K32" s="23" t="inlineStr">
@@ -1723,7 +1727,7 @@
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1731,30 +1735,30 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F33" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G33" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H33" s="24" t="n">
-        <v>-4.68</v>
-      </c>
-      <c r="I33" s="22" t="n">
-        <v>19.54</v>
+        <v>3</v>
+      </c>
+      <c r="H33" s="22" t="n">
+        <v>6.32</v>
+      </c>
+      <c r="I33" s="24" t="n">
+        <v>-3.06</v>
       </c>
       <c r="J33" s="23" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 중요공시 3일 +100%</t>
+          <t>중요공시 3건 / 중요공시 7일 +50%</t>
         </is>
       </c>
       <c r="K33" s="23" t="inlineStr">
@@ -1766,7 +1770,7 @@
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1774,7 +1778,7 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
@@ -1789,15 +1793,15 @@
       <c r="G34" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="22" t="n">
-        <v>2.35</v>
-      </c>
-      <c r="I34" s="24" t="n">
-        <v>-7.27</v>
+      <c r="H34" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I34" s="20" t="n">
+        <v/>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K34" s="23" t="n">
@@ -1807,7 +1811,7 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1815,42 +1819,42 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>삼성중공업</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F35" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G35" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H35" s="22" t="n">
-        <v>6.32</v>
-      </c>
-      <c r="I35" s="24" t="n">
-        <v>-3.06</v>
+        <v>0</v>
+      </c>
+      <c r="H35" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I35" s="20" t="n">
+        <v/>
       </c>
       <c r="J35" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 7일 +200%</t>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K35" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1858,42 +1862,40 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>에스아이리소스</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F36" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G36" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H36" s="24" t="n">
-        <v>-6.32</v>
-      </c>
-      <c r="I36" s="24" t="n">
-        <v>-9.18</v>
+        <v>0</v>
+      </c>
+      <c r="H36" s="22" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="I36" s="22" t="n">
+        <v>8.93</v>
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K36" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K36" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1901,30 +1903,30 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>엑시온그룹</t>
+          <t>피노</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E37" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F37" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G37" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H37" s="22" t="n">
-        <v>5.63</v>
-      </c>
-      <c r="I37" s="22" t="n">
-        <v>4.85</v>
+      <c r="H37" s="24" t="n">
+        <v>-3.76</v>
+      </c>
+      <c r="I37" s="24" t="n">
+        <v>-13.44</v>
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 3건 / 중요공시 3일 +200%</t>
         </is>
       </c>
       <c r="K37" s="23" t="inlineStr">
@@ -1936,7 +1938,7 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1944,14 +1946,14 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F38" s="20" t="n">
         <v>0</v>
@@ -1959,15 +1961,15 @@
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H38" s="22" t="n">
-        <v>10.67</v>
-      </c>
-      <c r="I38" s="22" t="n">
-        <v>8.93</v>
+      <c r="H38" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I38" s="20" t="n">
+        <v/>
       </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K38" s="23" t="n">
@@ -1977,7 +1979,7 @@
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1985,7 +1987,7 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>NH투자증권</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
@@ -2001,26 +2003,24 @@
         <v>0</v>
       </c>
       <c r="H39" s="22" t="n">
-        <v>7.85</v>
-      </c>
-      <c r="I39" s="22" t="n">
-        <v>0.45</v>
+        <v>1.76</v>
+      </c>
+      <c r="I39" s="20" t="n">
+        <v>0</v>
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K39" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K39" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2028,42 +2028,42 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>알엔티엑스</t>
+          <t>라이콤</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F40" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G40" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H40" s="24" t="n">
-        <v>-0.44</v>
-      </c>
-      <c r="I40" s="24" t="n">
-        <v>-17.65</v>
+        <v>-12.4</v>
+      </c>
+      <c r="I40" s="22" t="n">
+        <v>30.29</v>
       </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
-          <t>중요공시 5건 / 중요공시 3일 +150%</t>
+          <t>네이버 검색 당일 +229% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K40" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2071,7 +2071,7 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>라이콤</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
@@ -2087,26 +2087,26 @@
         <v>0</v>
       </c>
       <c r="H41" s="24" t="n">
-        <v>-12.4</v>
+        <v>-4.68</v>
       </c>
       <c r="I41" s="22" t="n">
-        <v>30.29</v>
+        <v>19.54</v>
       </c>
       <c r="J41" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +214% / 중요공시 1건</t>
+          <t>중요공시 4건</t>
         </is>
       </c>
       <c r="K41" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2114,42 +2114,42 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>원익IPS</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E42" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F42" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G42" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H42" s="22" t="n">
-        <v>30</v>
+        <v>28.36</v>
       </c>
       <c r="I42" s="22" t="n">
-        <v>38.13</v>
+        <v>19.41</v>
       </c>
       <c r="J42" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K42" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2157,7 +2157,7 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>하림</t>
+          <t>삼성바이오로직스</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
@@ -2172,25 +2172,27 @@
       <c r="G43" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H43" s="24" t="n">
-        <v>-0.87</v>
-      </c>
-      <c r="I43" s="22" t="n">
-        <v>0.71</v>
+      <c r="H43" s="22" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I43" s="24" t="n">
+        <v>-3.36</v>
       </c>
       <c r="J43" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K43" s="23" t="n">
-        <v/>
+          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K43" s="23" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2198,7 +2200,7 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>대한광통신</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
@@ -2213,27 +2215,27 @@
       <c r="G44" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="22" t="n">
-        <v>11.54</v>
-      </c>
-      <c r="I44" s="22" t="n">
-        <v>5.31</v>
+      <c r="H44" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I44" s="20" t="n">
+        <v/>
       </c>
       <c r="J44" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K44" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2241,42 +2243,42 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>현대건설</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E45" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F45" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G45" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H45" s="22" t="n">
-        <v>28.36</v>
-      </c>
-      <c r="I45" s="22" t="n">
-        <v>19.41</v>
+        <v>8.710000000000001</v>
+      </c>
+      <c r="I45" s="24" t="n">
+        <v>-2.65</v>
       </c>
       <c r="J45" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K45" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
@@ -2284,7 +2286,7 @@
       </c>
       <c r="C46" s="21" t="inlineStr">
         <is>
-          <t>삼성바이오로직스</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="D46" s="20" t="n">
@@ -2299,143 +2301,147 @@
       <c r="G46" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H46" s="22" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="I46" s="24" t="n">
-        <v>-3.36</v>
+      <c r="H46" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I46" s="20" t="n">
+        <v/>
       </c>
       <c r="J46" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K46" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="20" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B47" s="20" t="n">
+      <c r="A47" s="25" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B47" s="25" t="n">
         <v>34</v>
       </c>
-      <c r="C47" s="21" t="inlineStr">
-        <is>
-          <t>전기차</t>
-        </is>
-      </c>
-      <c r="D47" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E47" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F47" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I47" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J47" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K47" s="23" t="n">
-        <v/>
+      <c r="C47" s="26" t="inlineStr">
+        <is>
+          <t>세미티에스</t>
+        </is>
+      </c>
+      <c r="D47" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E47" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F47" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="27" t="n">
+        <v>29.97</v>
+      </c>
+      <c r="I47" s="28" t="n">
+        <v>-7.54</v>
+      </c>
+      <c r="J47" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +4464%</t>
+        </is>
+      </c>
+      <c r="K47" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="20" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B48" s="20" t="n">
+      <c r="A48" s="25" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B48" s="25" t="n">
         <v>35</v>
       </c>
-      <c r="C48" s="21" t="inlineStr">
-        <is>
-          <t>KB금융</t>
-        </is>
-      </c>
-      <c r="D48" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E48" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F48" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="22" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="I48" s="24" t="n">
-        <v>-6.06</v>
-      </c>
-      <c r="J48" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K48" s="23" t="n">
-        <v/>
+      <c r="C48" s="26" t="inlineStr">
+        <is>
+          <t>화신정공</t>
+        </is>
+      </c>
+      <c r="D48" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F48" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="27" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="I48" s="27" t="n">
+        <v>142.33</v>
+      </c>
+      <c r="J48" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +2148%</t>
+        </is>
+      </c>
+      <c r="K48" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="20" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B49" s="20" t="n">
+      <c r="A49" s="25" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B49" s="25" t="n">
         <v>36</v>
       </c>
-      <c r="C49" s="21" t="inlineStr">
-        <is>
-          <t>철강</t>
-        </is>
-      </c>
-      <c r="D49" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E49" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F49" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G49" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H49" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I49" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J49" s="23" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K49" s="23" t="inlineStr">
+      <c r="C49" s="26" t="inlineStr">
+        <is>
+          <t>마니커</t>
+        </is>
+      </c>
+      <c r="D49" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E49" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F49" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="28" t="n">
+        <v>-5.97</v>
+      </c>
+      <c r="I49" s="27" t="n">
+        <v>24.75</v>
+      </c>
+      <c r="J49" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +519%</t>
+        </is>
+      </c>
+      <c r="K49" s="29" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -2444,7 +2450,7 @@
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -2452,7 +2458,7 @@
       </c>
       <c r="C50" s="26" t="inlineStr">
         <is>
-          <t>세미티에스</t>
+          <t>SK이터닉스</t>
         </is>
       </c>
       <c r="D50" s="25" t="n">
@@ -2468,14 +2474,14 @@
         <v>0</v>
       </c>
       <c r="H50" s="27" t="n">
-        <v>29.97</v>
-      </c>
-      <c r="I50" s="28" t="n">
-        <v>-7.54</v>
+        <v>6.04</v>
+      </c>
+      <c r="I50" s="27" t="n">
+        <v>21.64</v>
       </c>
       <c r="J50" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +4221%</t>
+          <t>네이버 검색 당일 +274%</t>
         </is>
       </c>
       <c r="K50" s="29" t="inlineStr">
@@ -2487,7 +2493,7 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -2495,7 +2501,7 @@
       </c>
       <c r="C51" s="26" t="inlineStr">
         <is>
-          <t>화신정공</t>
+          <t>마니커에프앤지</t>
         </is>
       </c>
       <c r="D51" s="25" t="n">
@@ -2510,15 +2516,15 @@
       <c r="G51" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H51" s="27" t="n">
-        <v>6.18</v>
+      <c r="H51" s="28" t="n">
+        <v>-15.17</v>
       </c>
       <c r="I51" s="27" t="n">
-        <v>142.33</v>
+        <v>3.85</v>
       </c>
       <c r="J51" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +2072%</t>
+          <t>네이버 검색 당일 +203%</t>
         </is>
       </c>
       <c r="K51" s="29" t="inlineStr">
@@ -2530,7 +2536,7 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -2538,7 +2544,7 @@
       </c>
       <c r="C52" s="26" t="inlineStr">
         <is>
-          <t>마니커</t>
+          <t>아이로보틱스</t>
         </is>
       </c>
       <c r="D52" s="25" t="n">
@@ -2553,15 +2559,15 @@
       <c r="G52" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H52" s="28" t="n">
-        <v>-5.97</v>
+      <c r="H52" s="27" t="n">
+        <v>22.3</v>
       </c>
       <c r="I52" s="27" t="n">
-        <v>24.75</v>
+        <v>27.7</v>
       </c>
       <c r="J52" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +495%</t>
+          <t>네이버 검색 당일 +146%</t>
         </is>
       </c>
       <c r="K52" s="29" t="inlineStr">
@@ -2573,7 +2579,7 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2581,7 +2587,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>SK이터닉스</t>
+          <t>랩지노믹스</t>
         </is>
       </c>
       <c r="D53" s="25" t="n">
@@ -2596,15 +2602,15 @@
       <c r="G53" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="27" t="n">
-        <v>6.04</v>
+      <c r="H53" s="28" t="n">
+        <v>-3.41</v>
       </c>
       <c r="I53" s="27" t="n">
-        <v>21.64</v>
+        <v>24.65</v>
       </c>
       <c r="J53" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +264%</t>
+          <t>네이버 검색 당일 +144%</t>
         </is>
       </c>
       <c r="K53" s="29" t="inlineStr">
@@ -2616,7 +2622,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2624,7 +2630,7 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>마니커에프앤지</t>
+          <t>테크윙</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -2639,15 +2645,15 @@
       <c r="G54" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H54" s="28" t="n">
-        <v>-15.17</v>
+      <c r="H54" s="27" t="n">
+        <v>6.87</v>
       </c>
       <c r="I54" s="27" t="n">
-        <v>3.85</v>
+        <v>19.38</v>
       </c>
       <c r="J54" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +190%</t>
+          <t>네이버 검색 당일 +141%</t>
         </is>
       </c>
       <c r="K54" s="29" t="inlineStr">
@@ -2659,7 +2665,7 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2667,7 +2673,7 @@
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>랩지노믹스</t>
+          <t>제주은행</t>
         </is>
       </c>
       <c r="D55" s="25" t="n">
@@ -2682,15 +2688,15 @@
       <c r="G55" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H55" s="28" t="n">
-        <v>-3.41</v>
+      <c r="H55" s="27" t="n">
+        <v>0.16</v>
       </c>
       <c r="I55" s="27" t="n">
-        <v>24.65</v>
+        <v>15.07</v>
       </c>
       <c r="J55" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +138%</t>
+          <t>네이버 검색 당일 +106%</t>
         </is>
       </c>
       <c r="K55" s="29" t="inlineStr">
@@ -2702,7 +2708,7 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2710,7 +2716,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>아이로보틱스</t>
+          <t>윈팩</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2725,15 +2731,15 @@
       <c r="G56" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H56" s="27" t="n">
-        <v>22.3</v>
+      <c r="H56" s="28" t="n">
+        <v>-4.93</v>
       </c>
       <c r="I56" s="27" t="n">
-        <v>27.7</v>
+        <v>20.38</v>
       </c>
       <c r="J56" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +137%</t>
+          <t>네이버 검색 당일 +102%</t>
         </is>
       </c>
       <c r="K56" s="29" t="inlineStr">
@@ -2745,7 +2751,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2753,7 +2759,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>테크윙</t>
+          <t>SK네트웍스</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2769,14 +2775,14 @@
         <v>0</v>
       </c>
       <c r="H57" s="27" t="n">
-        <v>6.87</v>
+        <v>11.4</v>
       </c>
       <c r="I57" s="27" t="n">
-        <v>19.38</v>
+        <v>19.27</v>
       </c>
       <c r="J57" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +128%</t>
+          <t>네이버 검색 당일 +78% / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K57" s="29" t="inlineStr">
@@ -2788,7 +2794,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2796,7 +2802,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>제주은행</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2812,26 +2818,24 @@
         <v>0</v>
       </c>
       <c r="H58" s="27" t="n">
-        <v>0.16</v>
+        <v>6.92</v>
       </c>
       <c r="I58" s="27" t="n">
-        <v>15.07</v>
+        <v>3.54</v>
       </c>
       <c r="J58" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +100%</t>
-        </is>
-      </c>
-      <c r="K58" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K58" s="29" t="n">
+        <v/>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2839,7 +2843,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>SK네트웍스</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2854,27 +2858,25 @@
       <c r="G59" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H59" s="27" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="I59" s="27" t="n">
-        <v>19.27</v>
+      <c r="H59" s="28" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="I59" s="28" t="n">
+        <v>-25.58</v>
       </c>
       <c r="J59" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +73% / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K59" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K59" s="29" t="n">
+        <v/>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2882,7 +2884,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>하나마이크론</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2898,26 +2900,26 @@
         <v>0</v>
       </c>
       <c r="H60" s="27" t="n">
-        <v>2.09</v>
-      </c>
-      <c r="I60" s="27" t="n">
-        <v>16.97</v>
+        <v>0.14</v>
+      </c>
+      <c r="I60" s="28" t="n">
+        <v>-3.65</v>
       </c>
       <c r="J60" s="29" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 3건</t>
         </is>
       </c>
       <c r="K60" s="29" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2925,7 +2927,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>저스템</t>
+          <t>엑시온그룹</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2941,24 +2943,26 @@
         <v>0</v>
       </c>
       <c r="H61" s="27" t="n">
-        <v>15.21</v>
+        <v>5.63</v>
       </c>
       <c r="I61" s="27" t="n">
-        <v>19.29</v>
+        <v>4.85</v>
       </c>
       <c r="J61" s="29" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K61" s="29" t="n">
-        <v/>
+          <t>중요공시 3건</t>
+        </is>
+      </c>
+      <c r="K61" s="29" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2966,40 +2970,42 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>리노공업</t>
+          <t>한성크린텍</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E62" s="25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F62" s="25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G62" s="25" t="n">
         <v>0</v>
       </c>
       <c r="H62" s="27" t="n">
-        <v>4.71</v>
+        <v>2.75</v>
       </c>
       <c r="I62" s="27" t="n">
-        <v>11.05</v>
+        <v>0.79</v>
       </c>
       <c r="J62" s="29" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K62" s="29" t="n">
-        <v/>
+          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+        </is>
+      </c>
+      <c r="K62" s="29" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3007,7 +3013,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3023,18 +3029,20 @@
         <v>0</v>
       </c>
       <c r="H63" s="27" t="n">
-        <v>5.08</v>
-      </c>
-      <c r="I63" s="28" t="n">
-        <v>-2.62</v>
+        <v>4.09</v>
+      </c>
+      <c r="I63" s="27" t="n">
+        <v>0.93</v>
       </c>
       <c r="J63" s="29" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K63" s="29" t="n">
-        <v/>
+          <t>네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K63" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3130,22 +3138,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3154,29 +3162,29 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B4" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H4" s="25" t="n"/>
@@ -3185,99 +3193,103 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H5" s="25" t="n"/>
-      <c r="I5" s="25" t="n"/>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H5" s="28" t="n">
+        <v>-5.04</v>
+      </c>
+      <c r="I5" s="28" t="n">
+        <v>-2.45</v>
+      </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H6" s="25" t="n"/>
-      <c r="I6" s="25" t="n"/>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H6" s="27" t="n">
+        <v>7.86</v>
+      </c>
+      <c r="I6" s="28" t="n">
+        <v>-1.98</v>
+      </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H7" s="27" t="n">
-        <v>1.68</v>
-      </c>
-      <c r="I7" s="28" t="n">
-        <v>-13.29</v>
-      </c>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H7" s="25" t="n"/>
+      <c r="I7" s="25" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
@@ -3299,12 +3311,12 @@
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H8" s="28" t="n">
@@ -3317,7 +3329,7 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
@@ -3334,54 +3346,50 @@
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H9" s="28" t="n">
-        <v>-5.04</v>
-      </c>
-      <c r="I9" s="28" t="n">
-        <v>-2.45</v>
-      </c>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H9" s="25" t="n"/>
+      <c r="I9" s="25" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H10" s="27" t="n">
-        <v>7.86</v>
+        <v>2.35</v>
       </c>
       <c r="I10" s="28" t="n">
-        <v>-1.98</v>
+        <v>-7.27</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
@@ -3394,22 +3402,22 @@
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H11" s="27" t="n">
@@ -3429,22 +3437,22 @@
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H12" s="25" t="n"/>
@@ -3453,108 +3461,112 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>한미반도체</t>
+          <t>CSA 코스믹</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H13" s="27" t="n">
-        <v>24.05</v>
+        <v>29.93</v>
       </c>
       <c r="I13" s="27" t="n">
-        <v>27.56</v>
+        <v>69.53</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>CSA 코스믹</t>
+          <t>모바일어플라이언스</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H14" s="27" t="n">
-        <v>29.93</v>
-      </c>
-      <c r="I14" s="27" t="n">
-        <v>69.53</v>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H14" s="28" t="n">
+        <v>-2.09</v>
+      </c>
+      <c r="I14" s="28" t="n">
+        <v>-27.06</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E15" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H15" s="25" t="n"/>
-      <c r="I15" s="25" t="n"/>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H15" s="27" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="I15" s="28" t="n">
+        <v>-4.41</v>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>NH투자증권</t>
+          <t>알엔티엑스</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -3571,130 +3583,126 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H16" s="27" t="n">
-        <v>1.76</v>
-      </c>
-      <c r="I16" s="25" t="n">
-        <v>0</v>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H16" s="28" t="n">
+        <v>-0.44</v>
+      </c>
+      <c r="I16" s="28" t="n">
+        <v>-17.65</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>에이팩트</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E17" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H17" s="27" t="n">
-        <v>7.26</v>
+        <v>13.08</v>
       </c>
       <c r="I17" s="27" t="n">
-        <v>6.83</v>
+        <v>45.57</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>모바일어플라이언스</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E18" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H18" s="28" t="n">
-        <v>-2.09</v>
-      </c>
-      <c r="I18" s="28" t="n">
-        <v>-27.06</v>
-      </c>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H18" s="25" t="n"/>
+      <c r="I18" s="25" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H19" s="27" t="n">
-        <v>2.41</v>
-      </c>
-      <c r="I19" s="28" t="n">
-        <v>-4.41</v>
+        <v>24.05</v>
+      </c>
+      <c r="I19" s="27" t="n">
+        <v>27.56</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>에이팩트</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
@@ -3711,25 +3719,25 @@
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H20" s="27" t="n">
-        <v>13.08</v>
-      </c>
-      <c r="I20" s="27" t="n">
-        <v>45.57</v>
+        <v>1.68</v>
+      </c>
+      <c r="I20" s="28" t="n">
+        <v>-13.29</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -3746,20 +3754,16 @@
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H21" s="27" t="n">
-        <v>2.35</v>
-      </c>
-      <c r="I21" s="28" t="n">
-        <v>-7.27</v>
-      </c>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H21" s="25" t="n"/>
+      <c r="I21" s="25" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
@@ -3781,12 +3785,12 @@
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H22" s="27" t="n">
@@ -3799,7 +3803,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3816,25 +3820,21 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H23" s="28" t="n">
-        <v>-4.68</v>
-      </c>
-      <c r="I23" s="27" t="n">
-        <v>19.54</v>
-      </c>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H23" s="25" t="n"/>
+      <c r="I23" s="25" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>에스아이리소스</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3851,25 +3851,25 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H24" s="28" t="n">
-        <v>-6.32</v>
-      </c>
-      <c r="I24" s="28" t="n">
-        <v>-9.18</v>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H24" s="27" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="I24" s="27" t="n">
+        <v>8.93</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>엑시온그룹</t>
+          <t>후성</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3886,95 +3886,91 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H25" s="27" t="n">
-        <v>5.63</v>
+        <v>20.55</v>
       </c>
       <c r="I25" s="27" t="n">
-        <v>4.85</v>
+        <v>63.46</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>NH투자증권</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C26" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D26" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E26" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H26" s="27" t="n">
-        <v>10.67</v>
-      </c>
-      <c r="I26" s="27" t="n">
-        <v>8.93</v>
+        <v>1.76</v>
+      </c>
+      <c r="I26" s="25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>후성</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C27" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D27" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E27" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H27" s="27" t="n">
-        <v>20.55</v>
-      </c>
-      <c r="I27" s="27" t="n">
-        <v>63.46</v>
-      </c>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H27" s="25" t="n"/>
+      <c r="I27" s="25" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>알엔티엑스</t>
+          <t>피노</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
@@ -3991,60 +3987,60 @@
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H28" s="28" t="n">
-        <v>-0.44</v>
+        <v>-3.76</v>
       </c>
       <c r="I28" s="28" t="n">
-        <v>-17.65</v>
+        <v>-13.44</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>라이콤</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C29" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D29" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E29" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H29" s="27" t="n">
-        <v>7.85</v>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H29" s="28" t="n">
+        <v>-12.4</v>
       </c>
       <c r="I29" s="27" t="n">
-        <v>0.45</v>
+        <v>30.29</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>KB금융</t>
+          <t>삼성바이오로직스</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -4061,25 +4057,25 @@
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H30" s="27" t="n">
-        <v>6.4</v>
+        <v>0.7</v>
       </c>
       <c r="I30" s="28" t="n">
-        <v>-6.06</v>
+        <v>-3.36</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>대한광통신</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
@@ -4096,25 +4092,25 @@
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H31" s="27" t="n">
-        <v>11.54</v>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H31" s="28" t="n">
+        <v>-4.68</v>
       </c>
       <c r="I31" s="27" t="n">
-        <v>5.31</v>
+        <v>19.54</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>라이콤</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -4131,25 +4127,21 @@
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H32" s="28" t="n">
-        <v>-12.4</v>
-      </c>
-      <c r="I32" s="27" t="n">
-        <v>30.29</v>
-      </c>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H32" s="25" t="n"/>
+      <c r="I32" s="25" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>삼성바이오로직스</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4166,25 +4158,21 @@
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H33" s="27" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="I33" s="28" t="n">
-        <v>-3.36</v>
-      </c>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H33" s="25" t="n"/>
+      <c r="I33" s="25" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>원익IPS</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4201,25 +4189,25 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H34" s="27" t="n">
-        <v>30</v>
+        <v>28.36</v>
       </c>
       <c r="I34" s="27" t="n">
-        <v>38.13</v>
+        <v>19.41</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -4236,122 +4224,130 @@
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H35" s="25" t="n"/>
-      <c r="I35" s="25" t="n"/>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H35" s="27" t="n">
+        <v>8.710000000000001</v>
+      </c>
+      <c r="I35" s="28" t="n">
+        <v>-2.65</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C36" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D36" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E36" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H36" s="25" t="n"/>
-      <c r="I36" s="25" t="n"/>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H36" s="28" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="I36" s="28" t="n">
+        <v>-25.58</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>하림</t>
+          <t>SK네트웍스</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C37" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D37" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E37" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H37" s="28" t="n">
-        <v>-0.87</v>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H37" s="27" t="n">
+        <v>11.4</v>
       </c>
       <c r="I37" s="27" t="n">
-        <v>0.71</v>
+        <v>19.27</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>현대건설</t>
+          <t>SK이터닉스</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C38" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D38" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E38" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H38" s="27" t="n">
-        <v>28.36</v>
+        <v>6.04</v>
       </c>
       <c r="I38" s="27" t="n">
-        <v>19.41</v>
+        <v>21.64</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>SK네트웍스</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4368,25 +4364,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H39" s="27" t="n">
-        <v>11.4</v>
+        <v>6.92</v>
       </c>
       <c r="I39" s="27" t="n">
-        <v>19.27</v>
+        <v>3.54</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>SK이터닉스</t>
+          <t>랩지노믹스</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4403,25 +4399,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H40" s="27" t="n">
-        <v>6.04</v>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H40" s="28" t="n">
+        <v>-3.41</v>
       </c>
       <c r="I40" s="27" t="n">
-        <v>21.64</v>
+        <v>24.65</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>마니커</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4438,25 +4434,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H41" s="27" t="n">
-        <v>5.08</v>
-      </c>
-      <c r="I41" s="28" t="n">
-        <v>-2.62</v>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H41" s="28" t="n">
+        <v>-5.97</v>
+      </c>
+      <c r="I41" s="27" t="n">
+        <v>24.75</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>랩지노믹스</t>
+          <t>마니커에프앤지</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4473,25 +4469,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H42" s="28" t="n">
-        <v>-3.41</v>
+        <v>-15.17</v>
       </c>
       <c r="I42" s="27" t="n">
-        <v>24.65</v>
+        <v>3.85</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>리노공업</t>
+          <t>세미티에스</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4508,25 +4504,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H43" s="27" t="n">
-        <v>4.71</v>
-      </c>
-      <c r="I43" s="27" t="n">
-        <v>11.05</v>
+        <v>29.97</v>
+      </c>
+      <c r="I43" s="28" t="n">
+        <v>-7.54</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>마니커</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4543,25 +4539,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H44" s="28" t="n">
-        <v>-5.97</v>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H44" s="27" t="n">
+        <v>4.09</v>
       </c>
       <c r="I44" s="27" t="n">
-        <v>24.75</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>마니커에프앤지</t>
+          <t>아이로보틱스</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4578,25 +4574,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H45" s="28" t="n">
-        <v>-15.17</v>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H45" s="27" t="n">
+        <v>22.3</v>
       </c>
       <c r="I45" s="27" t="n">
-        <v>3.85</v>
+        <v>27.7</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>세미티에스</t>
+          <t>엑시온그룹</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4613,25 +4609,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H46" s="27" t="n">
-        <v>29.97</v>
-      </c>
-      <c r="I46" s="28" t="n">
-        <v>-7.54</v>
+        <v>5.63</v>
+      </c>
+      <c r="I46" s="27" t="n">
+        <v>4.85</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>아이로보틱스</t>
+          <t>윈팩</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4648,25 +4644,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="H47" s="27" t="n">
-        <v>22.3</v>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H47" s="28" t="n">
+        <v>-4.93</v>
       </c>
       <c r="I47" s="27" t="n">
-        <v>27.7</v>
+        <v>20.38</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>저스템</t>
+          <t>제주은행</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4683,25 +4679,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H48" s="27" t="n">
-        <v>15.21</v>
+        <v>0.16</v>
       </c>
       <c r="I48" s="27" t="n">
-        <v>19.29</v>
+        <v>15.07</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>제주은행</t>
+          <t>테크윙</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4718,25 +4714,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H49" s="27" t="n">
-        <v>0.16</v>
+        <v>6.87</v>
       </c>
       <c r="I49" s="27" t="n">
-        <v>15.07</v>
+        <v>19.38</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>테크윙</t>
+          <t>한성크린텍</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4753,25 +4749,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H50" s="27" t="n">
-        <v>6.87</v>
+        <v>2.75</v>
       </c>
       <c r="I50" s="27" t="n">
-        <v>19.38</v>
+        <v>0.79</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>하나마이크론</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4788,19 +4784,19 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H51" s="27" t="n">
-        <v>2.09</v>
-      </c>
-      <c r="I51" s="27" t="n">
-        <v>16.97</v>
+        <v>0.14</v>
+      </c>
+      <c r="I51" s="28" t="n">
+        <v>-3.65</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
@@ -4823,12 +4819,12 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H52" s="27" t="n">
@@ -4919,19 +4915,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4950,19 +4946,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4981,19 +4977,19 @@
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5005,26 +5001,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5036,26 +5032,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5067,26 +5063,26 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5098,26 +5094,26 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B9" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5129,92 +5125,100 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="35" t="inlineStr">
         <is>
+          <t>철강</t>
+        </is>
+      </c>
+      <c r="B10" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="D10" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" s="36" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="F10" s="37" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="G10" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>제약</t>
+        </is>
+      </c>
+      <c r="B11" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="36" t="n">
+        <v>9</v>
+      </c>
+      <c r="D11" s="36" t="n">
+        <v>9</v>
+      </c>
+      <c r="E11" s="36" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="F11" s="37" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="G11" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="35" t="inlineStr">
+        <is>
           <t>인공지능</t>
         </is>
       </c>
-      <c r="B10" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" s="36" t="n">
-        <v>21</v>
-      </c>
-      <c r="D10" s="36" t="n">
-        <v>21</v>
-      </c>
-      <c r="E10" s="36" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="F10" s="37" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="G10" s="37" t="inlineStr">
+      <c r="B12" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="36" t="n">
+        <v>17</v>
+      </c>
+      <c r="D12" s="36" t="n">
+        <v>17</v>
+      </c>
+      <c r="E12" s="36" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="F12" s="37" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="G12" s="37" t="inlineStr">
         <is>
           <t>⚡ 관심</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="26" t="inlineStr">
-        <is>
-          <t>이차전지</t>
-        </is>
-      </c>
-      <c r="B11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F11" s="29" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G11" s="29" t="inlineStr"/>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="26" t="inlineStr">
-        <is>
-          <t>AI반도체</t>
-        </is>
-      </c>
-      <c r="B12" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F12" s="29" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G12" s="29" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>이차전지</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -5241,7 +5245,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5268,7 +5272,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5295,7 +5299,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -5322,7 +5326,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -5349,7 +5353,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>핀테크</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -5376,7 +5380,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>핀테크</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-06-21 06:58 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -258,13 +258,13 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-06-20 06:55</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-06-21 06:55</t>
         </is>
       </c>
     </row>
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-06-20) 상위: 반도체  점수 60.0점</t>
+          <t>⚡ 최신(2026-06-21) 상위: 반도체  점수 60.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-06-20) 상위: SK  점수 47.0점</t>
+          <t>⚡ 최신(2026-06-21) 상위: SK  점수 56.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-06-20) 상위: SK하이닉스  점수 31.0점</t>
+          <t>⚡ 최신(2026-06-21) 상위: SK하이닉스  점수 41.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -971,10 +971,10 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -990,7 +990,7 @@
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1014,10 +1014,10 @@
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1033,17 +1033,19 @@
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K16" s="17" t="n">
-        <v/>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K16" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1051,14 +1053,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1066,27 +1068,27 @@
       <c r="G17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="18" t="n">
-        <v>3.18</v>
+      <c r="H17" s="19" t="n">
+        <v>-2.34</v>
       </c>
       <c r="I17" s="18" t="n">
-        <v>32.44</v>
+        <v>9.77</v>
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR) / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1094,7 +1096,7 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
@@ -1109,25 +1111,27 @@
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="19" t="n">
-        <v>-2.34</v>
+      <c r="H18" s="18" t="n">
+        <v>2</v>
       </c>
       <c r="I18" s="18" t="n">
-        <v>9.77</v>
+        <v>0.99</v>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K18" s="17" t="n">
-        <v/>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K18" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1135,14 +1139,14 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1150,15 +1154,15 @@
       <c r="G19" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="18" t="n">
-        <v>2</v>
+      <c r="H19" s="19" t="n">
+        <v>-3.12</v>
       </c>
       <c r="I19" s="18" t="n">
-        <v>0.99</v>
+        <v>5.08</v>
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K19" s="17" t="n">
@@ -1168,7 +1172,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1176,14 +1180,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1191,15 +1195,15 @@
       <c r="G20" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="19" t="n">
-        <v>-3.12</v>
+      <c r="H20" s="18" t="n">
+        <v>3.18</v>
       </c>
       <c r="I20" s="18" t="n">
-        <v>5.08</v>
+        <v>32.44</v>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K20" s="17" t="n">
@@ -1209,7 +1213,7 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1221,10 +1225,10 @@
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
@@ -1252,7 +1256,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1260,14 +1264,14 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -1283,7 +1287,7 @@
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="inlineStr">
@@ -1295,7 +1299,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1303,14 +1307,14 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F23" s="15" t="n">
         <v>0</v>
@@ -1318,15 +1322,15 @@
       <c r="G23" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I23" s="15" t="n">
-        <v/>
+      <c r="H23" s="19" t="n">
+        <v>-0.91</v>
+      </c>
+      <c r="I23" s="18" t="n">
+        <v>2.25</v>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K23" s="17" t="inlineStr">
@@ -1338,7 +1342,7 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1346,7 +1350,7 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>넥써쓰</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
@@ -1361,27 +1365,27 @@
       <c r="G24" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H24" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I24" s="15" t="n">
-        <v/>
+      <c r="H24" s="19" t="n">
+        <v>-27.47</v>
+      </c>
+      <c r="I24" s="19" t="n">
+        <v>-4.83</v>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+          <t>네이버 검색 당일 +102% / 중요공시 3건 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K24" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1389,14 +1393,14 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>넥써쓰</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F25" s="15" t="n">
         <v>0</v>
@@ -1404,27 +1408,27 @@
       <c r="G25" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H25" s="19" t="n">
-        <v>-27.47</v>
-      </c>
-      <c r="I25" s="19" t="n">
-        <v>-4.83</v>
+      <c r="H25" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I25" s="15" t="n">
+        <v/>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K25" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1432,7 +1436,7 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
@@ -1448,26 +1452,26 @@
         <v>0</v>
       </c>
       <c r="H26" s="19" t="n">
-        <v>-2.13</v>
+        <v>-1.9</v>
       </c>
       <c r="I26" s="19" t="n">
-        <v>-0.72</v>
+        <v>-1.56</v>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 2건 / Google 급상승 검색어 등장 (KR) / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K26" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시, Google</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -1475,7 +1479,7 @@
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="D27" s="15" t="n">
@@ -1491,24 +1495,26 @@
         <v>0</v>
       </c>
       <c r="H27" s="19" t="n">
-        <v>-0.91</v>
-      </c>
-      <c r="I27" s="18" t="n">
-        <v>2.25</v>
+        <v>-2.13</v>
+      </c>
+      <c r="I27" s="19" t="n">
+        <v>-0.72</v>
       </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K27" s="17" t="n">
-        <v/>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K27" s="17" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B28" s="20" t="n">
@@ -1516,7 +1522,7 @@
       </c>
       <c r="C28" s="21" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>보해양조</t>
         </is>
       </c>
       <c r="D28" s="20" t="n">
@@ -1532,26 +1538,26 @@
         <v>0</v>
       </c>
       <c r="H28" s="22" t="n">
-        <v>-3.85</v>
+        <v>29.88</v>
       </c>
       <c r="I28" s="22" t="n">
-        <v>-6.79</v>
+        <v>58.36</v>
       </c>
       <c r="J28" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
+          <t>네이버 검색 당일 +186% / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K28" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B29" s="20" t="n">
@@ -1559,7 +1565,7 @@
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>SK스퀘어</t>
+          <t>한화</t>
         </is>
       </c>
       <c r="D29" s="20" t="n">
@@ -1575,24 +1581,26 @@
         <v>0</v>
       </c>
       <c r="H29" s="24" t="n">
-        <v>4.71</v>
+        <v>-4.71</v>
       </c>
       <c r="I29" s="24" t="n">
-        <v>31.08</v>
+        <v>-0.95</v>
       </c>
       <c r="J29" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K29" s="23" t="n">
-        <v/>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K29" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
@@ -1600,14 +1608,14 @@
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="D30" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E30" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F30" s="20" t="n">
         <v>0</v>
@@ -1616,24 +1624,26 @@
         <v>0</v>
       </c>
       <c r="H30" s="24" t="n">
-        <v>1.24</v>
+        <v>-26.16</v>
       </c>
       <c r="I30" s="24" t="n">
-        <v>13.77</v>
+        <v>-19.9</v>
       </c>
       <c r="J30" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K30" s="23" t="n">
-        <v/>
+          <t>네이버 검색 당일 +100% / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K30" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1641,14 +1651,14 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F31" s="20" t="n">
         <v>0</v>
@@ -1656,27 +1666,27 @@
       <c r="G31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I31" s="20" t="n">
-        <v/>
+      <c r="H31" s="22" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="I31" s="22" t="n">
+        <v>13.93</v>
       </c>
       <c r="J31" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K31" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1684,7 +1694,7 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>씨피시스템</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
@@ -1700,26 +1710,26 @@
         <v>0</v>
       </c>
       <c r="H32" s="24" t="n">
-        <v>29.88</v>
+        <v>-3.85</v>
       </c>
       <c r="I32" s="24" t="n">
-        <v>20.79</v>
+        <v>-6.79</v>
       </c>
       <c r="J32" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K32" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1742,10 +1752,10 @@
       <c r="G33" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H33" s="22" t="n">
+      <c r="H33" s="24" t="n">
         <v>-17.67</v>
       </c>
-      <c r="I33" s="22" t="n">
+      <c r="I33" s="24" t="n">
         <v>-24.4</v>
       </c>
       <c r="J33" s="23" t="inlineStr">
@@ -1762,7 +1772,7 @@
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1770,7 +1780,7 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
@@ -1785,25 +1795,27 @@
       <c r="G34" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="22" t="n">
-        <v>-0.37</v>
-      </c>
-      <c r="I34" s="22" t="n">
-        <v>-2.74</v>
+      <c r="H34" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I34" s="20" t="n">
+        <v/>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K34" s="23" t="n">
-        <v/>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K34" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1811,14 +1823,14 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>남화토건</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F35" s="20" t="n">
         <v>0</v>
@@ -1827,26 +1839,24 @@
         <v>0</v>
       </c>
       <c r="H35" s="24" t="n">
-        <v>12.73</v>
+        <v>-0.37</v>
       </c>
       <c r="I35" s="24" t="n">
-        <v>45.92</v>
+        <v>-2.74</v>
       </c>
       <c r="J35" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +314% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K35" s="23" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K35" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1854,42 +1864,42 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>한솔테크닉스</t>
+          <t>남화토건</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F36" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G36" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H36" s="22" t="n">
-        <v>-4.87</v>
-      </c>
-      <c r="I36" s="24" t="n">
-        <v>7.83</v>
+        <v>12.73</v>
+      </c>
+      <c r="I36" s="22" t="n">
+        <v>45.92</v>
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>네이버 검색 당일 +819% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K36" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1897,7 +1907,7 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>씨피시스템</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
@@ -1913,24 +1923,26 @@
         <v>0</v>
       </c>
       <c r="H37" s="22" t="n">
-        <v>-26.16</v>
+        <v>29.88</v>
       </c>
       <c r="I37" s="22" t="n">
-        <v>-19.9</v>
+        <v>20.79</v>
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K37" s="23" t="n">
-        <v/>
+          <t>네이버 검색 당일 +73% / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K37" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1938,7 +1950,7 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>보해양조</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
@@ -1954,14 +1966,14 @@
         <v>0</v>
       </c>
       <c r="H38" s="24" t="n">
-        <v>29.88</v>
+        <v>-7.44</v>
       </c>
       <c r="I38" s="24" t="n">
-        <v>58.36</v>
+        <v>-6.21</v>
       </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K38" s="23" t="n">
@@ -1971,7 +1983,7 @@
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1979,40 +1991,42 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>HJ중공업</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F39" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G39" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H39" s="22" t="n">
-        <v>-7.44</v>
+        <v>3</v>
+      </c>
+      <c r="H39" s="24" t="n">
+        <v>-3.67</v>
       </c>
       <c r="I39" s="22" t="n">
-        <v>-6.21</v>
+        <v>3.24</v>
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K39" s="23" t="n">
-        <v/>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K39" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2020,30 +2034,30 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>HJ중공업</t>
+          <t>HD현대중공업</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F40" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G40" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H40" s="22" t="n">
-        <v>-3.67</v>
-      </c>
-      <c r="I40" s="24" t="n">
-        <v>3.24</v>
+        <v>0</v>
+      </c>
+      <c r="H40" s="24" t="n">
+        <v>-2.49</v>
+      </c>
+      <c r="I40" s="22" t="n">
+        <v>2.62</v>
       </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K40" s="23" t="inlineStr">
@@ -2055,7 +2069,7 @@
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2063,7 +2077,7 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
@@ -2078,27 +2092,27 @@
       <c r="G41" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="22" t="n">
-        <v>-2.49</v>
-      </c>
-      <c r="I41" s="24" t="n">
-        <v>2.62</v>
+      <c r="H41" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I41" s="20" t="n">
+        <v/>
       </c>
       <c r="J41" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K41" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2141,7 +2155,7 @@
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2149,7 +2163,7 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>HD현대</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
@@ -2164,15 +2178,15 @@
       <c r="G43" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H43" s="22" t="n">
-        <v>-3.35</v>
-      </c>
-      <c r="I43" s="22" t="n">
-        <v>-5.53</v>
+      <c r="H43" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I43" s="20" t="n">
+        <v/>
       </c>
       <c r="J43" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K43" s="23" t="n">
@@ -2180,52 +2194,50 @@
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="25" t="inlineStr">
-        <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="B44" s="25" t="n">
+      <c r="A44" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B44" s="20" t="n">
         <v>31</v>
       </c>
-      <c r="C44" s="26" t="inlineStr">
-        <is>
-          <t>JW신약</t>
-        </is>
-      </c>
-      <c r="D44" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E44" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F44" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G44" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H44" s="27" t="n">
-        <v>13.08</v>
-      </c>
-      <c r="I44" s="27" t="n">
-        <v>70.94</v>
-      </c>
-      <c r="J44" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +953%</t>
-        </is>
-      </c>
-      <c r="K44" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+      <c r="C44" s="21" t="inlineStr">
+        <is>
+          <t>HD현대</t>
+        </is>
+      </c>
+      <c r="D44" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E44" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F44" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="24" t="n">
+        <v>-3.35</v>
+      </c>
+      <c r="I44" s="24" t="n">
+        <v>-5.53</v>
+      </c>
+      <c r="J44" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K44" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -2233,7 +2245,7 @@
       </c>
       <c r="C45" s="26" t="inlineStr">
         <is>
-          <t>강동씨앤엘</t>
+          <t>JW신약</t>
         </is>
       </c>
       <c r="D45" s="25" t="n">
@@ -2249,14 +2261,14 @@
         <v>0</v>
       </c>
       <c r="H45" s="27" t="n">
-        <v>29.91</v>
+        <v>13.08</v>
       </c>
       <c r="I45" s="27" t="n">
-        <v>121.56</v>
+        <v>70.94</v>
       </c>
       <c r="J45" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +830%</t>
+          <t>네이버 검색 당일 +1348%</t>
         </is>
       </c>
       <c r="K45" s="28" t="inlineStr">
@@ -2268,7 +2280,7 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -2276,7 +2288,7 @@
       </c>
       <c r="C46" s="26" t="inlineStr">
         <is>
-          <t>삼익제약</t>
+          <t>강동씨앤엘</t>
         </is>
       </c>
       <c r="D46" s="25" t="n">
@@ -2292,14 +2304,14 @@
         <v>0</v>
       </c>
       <c r="H46" s="27" t="n">
-        <v>29.98</v>
+        <v>29.91</v>
       </c>
       <c r="I46" s="27" t="n">
-        <v>41.82</v>
+        <v>121.56</v>
       </c>
       <c r="J46" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +439%</t>
+          <t>네이버 검색 당일 +1305%</t>
         </is>
       </c>
       <c r="K46" s="28" t="inlineStr">
@@ -2311,7 +2323,7 @@
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -2319,7 +2331,7 @@
       </c>
       <c r="C47" s="26" t="inlineStr">
         <is>
-          <t>현대약품</t>
+          <t>삼익제약</t>
         </is>
       </c>
       <c r="D47" s="25" t="n">
@@ -2334,15 +2346,15 @@
       <c r="G47" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H47" s="29" t="n">
-        <v>-4.12</v>
+      <c r="H47" s="27" t="n">
+        <v>29.98</v>
       </c>
       <c r="I47" s="27" t="n">
-        <v>42.23</v>
+        <v>41.82</v>
       </c>
       <c r="J47" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +339%</t>
+          <t>네이버 검색 당일 +720%</t>
         </is>
       </c>
       <c r="K47" s="28" t="inlineStr">
@@ -2354,7 +2366,7 @@
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -2362,7 +2374,7 @@
       </c>
       <c r="C48" s="26" t="inlineStr">
         <is>
-          <t>위더스제약</t>
+          <t>현대약품</t>
         </is>
       </c>
       <c r="D48" s="25" t="n">
@@ -2377,15 +2389,15 @@
       <c r="G48" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H48" s="27" t="n">
-        <v>13.59</v>
+      <c r="H48" s="29" t="n">
+        <v>-4.12</v>
       </c>
       <c r="I48" s="27" t="n">
-        <v>33.03</v>
+        <v>42.23</v>
       </c>
       <c r="J48" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +269%</t>
+          <t>네이버 검색 당일 +416%</t>
         </is>
       </c>
       <c r="K48" s="28" t="inlineStr">
@@ -2397,7 +2409,7 @@
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -2405,7 +2417,7 @@
       </c>
       <c r="C49" s="26" t="inlineStr">
         <is>
-          <t>삼화전자</t>
+          <t>위더스제약</t>
         </is>
       </c>
       <c r="D49" s="25" t="n">
@@ -2421,14 +2433,14 @@
         <v>0</v>
       </c>
       <c r="H49" s="27" t="n">
-        <v>2.81</v>
+        <v>13.59</v>
       </c>
       <c r="I49" s="27" t="n">
-        <v>73.59</v>
+        <v>33.03</v>
       </c>
       <c r="J49" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +230%</t>
+          <t>네이버 검색 당일 +394%</t>
         </is>
       </c>
       <c r="K49" s="28" t="inlineStr">
@@ -2440,7 +2452,7 @@
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -2448,7 +2460,7 @@
       </c>
       <c r="C50" s="26" t="inlineStr">
         <is>
-          <t>율촌</t>
+          <t>삼화전자</t>
         </is>
       </c>
       <c r="D50" s="25" t="n">
@@ -2463,15 +2475,15 @@
       <c r="G50" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H50" s="29" t="n">
-        <v>-13.55</v>
+      <c r="H50" s="27" t="n">
+        <v>2.81</v>
       </c>
       <c r="I50" s="27" t="n">
-        <v>30.73</v>
+        <v>73.59</v>
       </c>
       <c r="J50" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +153%</t>
+          <t>네이버 검색 당일 +391%</t>
         </is>
       </c>
       <c r="K50" s="28" t="inlineStr">
@@ -2483,7 +2495,7 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -2491,7 +2503,7 @@
       </c>
       <c r="C51" s="26" t="inlineStr">
         <is>
-          <t>티웨이홀딩스</t>
+          <t>율촌</t>
         </is>
       </c>
       <c r="D51" s="25" t="n">
@@ -2507,14 +2519,14 @@
         <v>0</v>
       </c>
       <c r="H51" s="29" t="n">
-        <v>-7.09</v>
+        <v>-13.55</v>
       </c>
       <c r="I51" s="27" t="n">
-        <v>26.88</v>
+        <v>30.73</v>
       </c>
       <c r="J51" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +141%</t>
+          <t>네이버 검색 당일 +196%</t>
         </is>
       </c>
       <c r="K51" s="28" t="inlineStr">
@@ -2526,7 +2538,7 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -2557,7 +2569,7 @@
       </c>
       <c r="J52" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +111%</t>
+          <t>네이버 검색 당일 +175%</t>
         </is>
       </c>
       <c r="K52" s="28" t="inlineStr">
@@ -2569,7 +2581,7 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2577,7 +2589,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>동일스틸럭스</t>
+          <t>티웨이홀딩스</t>
         </is>
       </c>
       <c r="D53" s="25" t="n">
@@ -2593,14 +2605,14 @@
         <v>0</v>
       </c>
       <c r="H53" s="29" t="n">
-        <v>-11.15</v>
+        <v>-7.09</v>
       </c>
       <c r="I53" s="27" t="n">
-        <v>29.05</v>
+        <v>26.88</v>
       </c>
       <c r="J53" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +105%</t>
+          <t>네이버 검색 당일 +174%</t>
         </is>
       </c>
       <c r="K53" s="28" t="inlineStr">
@@ -2612,7 +2624,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2620,7 +2632,7 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>부국철강</t>
+          <t>메리츠제2호스팩</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -2635,15 +2647,15 @@
       <c r="G54" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H54" s="29" t="n">
-        <v>-13.76</v>
-      </c>
-      <c r="I54" s="27" t="n">
-        <v>3.49</v>
+      <c r="H54" s="25" t="n">
+        <v/>
+      </c>
+      <c r="I54" s="25" t="n">
+        <v/>
       </c>
       <c r="J54" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +104%</t>
+          <t>네이버 검색 당일 +172%</t>
         </is>
       </c>
       <c r="K54" s="28" t="inlineStr">
@@ -2655,7 +2667,7 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2663,7 +2675,7 @@
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>대원전선</t>
+          <t>부국철강</t>
         </is>
       </c>
       <c r="D55" s="25" t="n">
@@ -2679,26 +2691,26 @@
         <v>0</v>
       </c>
       <c r="H55" s="29" t="n">
-        <v>-3.73</v>
+        <v>-13.76</v>
       </c>
       <c r="I55" s="27" t="n">
-        <v>6.02</v>
+        <v>3.49</v>
       </c>
       <c r="J55" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +60% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +160%</t>
         </is>
       </c>
       <c r="K55" s="28" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2706,7 +2718,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>HMM</t>
+          <t>피앤에스로보틱스</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2721,25 +2733,27 @@
       <c r="G56" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H56" s="29" t="n">
-        <v>-1.47</v>
+      <c r="H56" s="27" t="n">
+        <v>22.04</v>
       </c>
       <c r="I56" s="27" t="n">
-        <v>0.5</v>
+        <v>20.74</v>
       </c>
       <c r="J56" s="28" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K56" s="28" t="n">
-        <v/>
+          <t>네이버 검색 당일 +151%</t>
+        </is>
+      </c>
+      <c r="K56" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2747,7 +2761,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>우리기술</t>
+          <t>동일스틸럭스</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2763,14 +2777,14 @@
         <v>0</v>
       </c>
       <c r="H57" s="29" t="n">
-        <v>-1.89</v>
-      </c>
-      <c r="I57" s="29" t="n">
-        <v>-17.47</v>
+        <v>-11.15</v>
+      </c>
+      <c r="I57" s="27" t="n">
+        <v>29.05</v>
       </c>
       <c r="J57" s="28" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
+          <t>네이버 검색 당일 +147%</t>
         </is>
       </c>
       <c r="K57" s="28" t="inlineStr">
@@ -2782,7 +2796,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2790,7 +2804,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>휴림로봇</t>
+          <t>대원전선</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2806,26 +2820,26 @@
         <v>0</v>
       </c>
       <c r="H58" s="29" t="n">
-        <v>-3.34</v>
-      </c>
-      <c r="I58" s="29" t="n">
-        <v>-13.73</v>
+        <v>-3.73</v>
+      </c>
+      <c r="I58" s="27" t="n">
+        <v>6.02</v>
       </c>
       <c r="J58" s="28" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
+          <t>네이버 검색 당일 +95% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K58" s="28" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2833,7 +2847,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>LB세미콘</t>
+          <t>비엘팜텍</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2849,26 +2863,26 @@
         <v>0</v>
       </c>
       <c r="H59" s="29" t="n">
-        <v>-3.58</v>
+        <v>-20.26</v>
       </c>
       <c r="I59" s="27" t="n">
-        <v>0.97</v>
+        <v>4.23</v>
       </c>
       <c r="J59" s="28" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>네이버 검색 당일 +78% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K59" s="28" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2876,7 +2890,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>모아데이타</t>
+          <t>한솔테크닉스</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2891,27 +2905,27 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="27" t="n">
-        <v>2.44</v>
+      <c r="H60" s="29" t="n">
+        <v>-4.87</v>
       </c>
       <c r="I60" s="27" t="n">
-        <v>13.39</v>
+        <v>7.83</v>
       </c>
       <c r="J60" s="28" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>네이버 검색 당일 +76% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K60" s="28" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2919,42 +2933,42 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>오르비텍</t>
+          <t>삼보산업</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E61" s="25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F61" s="25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G61" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H61" s="29" t="n">
-        <v>-8.24</v>
-      </c>
-      <c r="I61" s="29" t="n">
-        <v>-10.69</v>
+      <c r="H61" s="27" t="n">
+        <v>11.54</v>
+      </c>
+      <c r="I61" s="27" t="n">
+        <v>45.97</v>
       </c>
       <c r="J61" s="28" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>네이버 검색 당일 +61% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K61" s="28" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2962,7 +2976,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>한전기술</t>
+          <t>다스코</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2977,25 +2991,27 @@
       <c r="G62" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H62" s="29" t="n">
-        <v>-9.51</v>
-      </c>
-      <c r="I62" s="29" t="n">
-        <v>-18.24</v>
+      <c r="H62" s="27" t="n">
+        <v>29.96</v>
+      </c>
+      <c r="I62" s="27" t="n">
+        <v>31.44</v>
       </c>
       <c r="J62" s="28" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K62" s="28" t="n">
-        <v/>
+          <t>네이버 검색 당일 +59% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K62" s="28" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
       </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3003,7 +3019,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>한화</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3019,18 +3035,20 @@
         <v>0</v>
       </c>
       <c r="H63" s="29" t="n">
-        <v>-4.71</v>
+        <v>-7.41</v>
       </c>
       <c r="I63" s="29" t="n">
-        <v>-0.95</v>
+        <v>-2.75</v>
       </c>
       <c r="J63" s="28" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K63" s="28" t="n">
-        <v/>
+          <t>네이버 검색 당일 +58% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K63" s="28" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3136,12 +3154,12 @@
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3157,22 +3175,22 @@
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H4" s="27" t="n">
@@ -3192,22 +3210,22 @@
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H5" s="27" t="n">
@@ -3220,42 +3238,42 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H6" s="27" t="n">
-        <v>3.18</v>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H6" s="29" t="n">
+        <v>-2.34</v>
       </c>
       <c r="I6" s="27" t="n">
-        <v>32.44</v>
+        <v>9.77</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
@@ -3272,117 +3290,117 @@
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H7" s="29" t="n">
-        <v>-2.34</v>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H7" s="27" t="n">
+        <v>2</v>
       </c>
       <c r="I7" s="27" t="n">
-        <v>9.77</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H8" s="27" t="n">
-        <v>2</v>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H8" s="29" t="n">
+        <v>-3.12</v>
       </c>
       <c r="I8" s="27" t="n">
-        <v>0.99</v>
+        <v>5.08</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H9" s="29" t="n">
-        <v>-3.12</v>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H9" s="27" t="n">
+        <v>3.18</v>
       </c>
       <c r="I9" s="27" t="n">
-        <v>5.08</v>
+        <v>32.44</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H10" s="25" t="n"/>
@@ -3391,60 +3409,64 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H11" s="25" t="n"/>
-      <c r="I11" s="25" t="n"/>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H11" s="29" t="n">
+        <v>-0.91</v>
+      </c>
+      <c r="I11" s="27" t="n">
+        <v>2.25</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H12" s="25" t="n"/>
@@ -3453,7 +3475,7 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>넥써쓰</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -3470,56 +3492,56 @@
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H13" s="25" t="n"/>
-      <c r="I13" s="25" t="n"/>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H13" s="29" t="n">
+        <v>-27.47</v>
+      </c>
+      <c r="I13" s="29" t="n">
+        <v>-4.83</v>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H14" s="29" t="n">
-        <v>-0.91</v>
-      </c>
-      <c r="I14" s="27" t="n">
-        <v>2.25</v>
-      </c>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H14" s="25" t="n"/>
+      <c r="I14" s="25" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>넥써쓰</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -3536,19 +3558,19 @@
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H15" s="29" t="n">
-        <v>-27.47</v>
+        <v>-1.9</v>
       </c>
       <c r="I15" s="29" t="n">
-        <v>-4.83</v>
+        <v>-1.56</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
@@ -3571,12 +3593,12 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H16" s="29" t="n">
@@ -3589,7 +3611,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>SK스퀘어</t>
+          <t>보해양조</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -3606,25 +3628,25 @@
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H17" s="27" t="n">
-        <v>4.71</v>
+        <v>29.88</v>
       </c>
       <c r="I17" s="27" t="n">
-        <v>31.08</v>
+        <v>58.36</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>한화</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -3641,91 +3663,95 @@
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H18" s="29" t="n">
-        <v>-3.85</v>
+        <v>-4.71</v>
       </c>
       <c r="I18" s="29" t="n">
-        <v>-6.79</v>
+        <v>-0.95</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H19" s="27" t="n">
-        <v>1.24</v>
-      </c>
-      <c r="I19" s="27" t="n">
-        <v>13.77</v>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H19" s="29" t="n">
+        <v>-0.37</v>
+      </c>
+      <c r="I19" s="29" t="n">
+        <v>-2.74</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D20" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H20" s="25" t="n"/>
-      <c r="I20" s="25" t="n"/>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H20" s="29" t="n">
+        <v>-26.16</v>
+      </c>
+      <c r="I20" s="29" t="n">
+        <v>-19.9</v>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -3742,25 +3768,25 @@
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H21" s="29" t="n">
-        <v>-0.37</v>
+        <v>-3.85</v>
       </c>
       <c r="I21" s="29" t="n">
-        <v>-2.74</v>
+        <v>-6.79</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>씨피시스템</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -3777,20 +3803,16 @@
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H22" s="27" t="n">
-        <v>29.88</v>
-      </c>
-      <c r="I22" s="27" t="n">
-        <v>20.79</v>
-      </c>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H22" s="25" t="n"/>
+      <c r="I22" s="25" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
@@ -3812,12 +3834,12 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H23" s="29" t="n">
@@ -3830,42 +3852,42 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>HD현대</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C24" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D24" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E24" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H24" s="29" t="n">
-        <v>-3.35</v>
-      </c>
-      <c r="I24" s="29" t="n">
-        <v>-5.53</v>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H24" s="27" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="I24" s="27" t="n">
+        <v>13.93</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>HD현대</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3882,25 +3904,25 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H25" s="29" t="n">
-        <v>-2.49</v>
-      </c>
-      <c r="I25" s="27" t="n">
-        <v>2.62</v>
+        <v>-3.35</v>
+      </c>
+      <c r="I25" s="29" t="n">
+        <v>-5.53</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>HJ중공업</t>
+          <t>HD현대중공업</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
@@ -3917,25 +3939,25 @@
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H26" s="29" t="n">
-        <v>-3.67</v>
+        <v>-2.49</v>
       </c>
       <c r="I26" s="27" t="n">
-        <v>3.24</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>HJ중공업</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
@@ -3952,25 +3974,25 @@
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H27" s="29" t="n">
-        <v>-7.44</v>
-      </c>
-      <c r="I27" s="29" t="n">
-        <v>-6.21</v>
+        <v>-3.67</v>
+      </c>
+      <c r="I27" s="27" t="n">
+        <v>3.24</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
@@ -3987,19 +4009,19 @@
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H28" s="29" t="n">
-        <v>-26.16</v>
+        <v>-7.44</v>
       </c>
       <c r="I28" s="29" t="n">
-        <v>-19.9</v>
+        <v>-6.21</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
@@ -4022,12 +4044,12 @@
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H29" s="27" t="n">
@@ -4040,7 +4062,7 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>보해양조</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -4057,25 +4079,21 @@
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H30" s="27" t="n">
-        <v>29.88</v>
-      </c>
-      <c r="I30" s="27" t="n">
-        <v>58.36</v>
-      </c>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H30" s="25" t="n"/>
+      <c r="I30" s="25" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>씨피시스템</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
@@ -4092,21 +4110,25 @@
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H31" s="25" t="n"/>
-      <c r="I31" s="25" t="n"/>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H31" s="27" t="n">
+        <v>29.88</v>
+      </c>
+      <c r="I31" s="27" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>한솔테크닉스</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -4123,55 +4145,47 @@
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H32" s="29" t="n">
-        <v>-4.87</v>
-      </c>
-      <c r="I32" s="27" t="n">
-        <v>7.83</v>
-      </c>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H32" s="25" t="n"/>
+      <c r="I32" s="25" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>HMM</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C33" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D33" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E33" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H33" s="29" t="n">
-        <v>-1.47</v>
-      </c>
-      <c r="I33" s="27" t="n">
-        <v>0.5</v>
-      </c>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H33" s="25" t="n"/>
+      <c r="I33" s="25" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
@@ -4193,12 +4207,12 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H34" s="27" t="n">
@@ -4211,7 +4225,7 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>LB세미콘</t>
+          <t>강동씨앤엘</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -4228,25 +4242,25 @@
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H35" s="29" t="n">
-        <v>-3.58</v>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H35" s="27" t="n">
+        <v>29.91</v>
       </c>
       <c r="I35" s="27" t="n">
-        <v>0.97</v>
+        <v>121.56</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>강동씨앤엘</t>
+          <t>다스코</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
@@ -4263,25 +4277,25 @@
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H36" s="27" t="n">
-        <v>29.91</v>
+        <v>29.96</v>
       </c>
       <c r="I36" s="27" t="n">
-        <v>121.56</v>
+        <v>31.44</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>대원전선</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
@@ -4298,25 +4312,25 @@
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H37" s="29" t="n">
-        <v>-3.73</v>
-      </c>
-      <c r="I37" s="27" t="n">
-        <v>6.02</v>
+        <v>-7.41</v>
+      </c>
+      <c r="I37" s="29" t="n">
+        <v>-2.75</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>동일스틸럭스</t>
+          <t>대원전선</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4333,25 +4347,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H38" s="29" t="n">
-        <v>-11.15</v>
+        <v>-3.73</v>
       </c>
       <c r="I38" s="27" t="n">
-        <v>29.05</v>
+        <v>6.02</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>모아데이타</t>
+          <t>동일스틸럭스</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4368,25 +4382,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H39" s="27" t="n">
-        <v>2.44</v>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H39" s="29" t="n">
+        <v>-11.15</v>
       </c>
       <c r="I39" s="27" t="n">
-        <v>13.39</v>
+        <v>29.05</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>부국철강</t>
+          <t>메리츠제2호스팩</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4403,25 +4417,21 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H40" s="29" t="n">
-        <v>-13.76</v>
-      </c>
-      <c r="I40" s="27" t="n">
-        <v>3.49</v>
-      </c>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H40" s="25" t="n"/>
+      <c r="I40" s="25" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>삼익제약</t>
+          <t>부국철강</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4438,25 +4448,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H41" s="27" t="n">
-        <v>29.98</v>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H41" s="29" t="n">
+        <v>-13.76</v>
       </c>
       <c r="I41" s="27" t="n">
-        <v>41.82</v>
+        <v>3.49</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>삼화전자</t>
+          <t>비엘팜텍</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4473,25 +4483,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H42" s="27" t="n">
-        <v>2.81</v>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H42" s="29" t="n">
+        <v>-20.26</v>
       </c>
       <c r="I42" s="27" t="n">
-        <v>73.59</v>
+        <v>4.23</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>성문전자</t>
+          <t>삼보산업</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4508,25 +4518,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H43" s="27" t="n">
-        <v>4.43</v>
+        <v>11.54</v>
       </c>
       <c r="I43" s="27" t="n">
-        <v>40.24</v>
+        <v>45.97</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>오르비텍</t>
+          <t>삼익제약</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4543,25 +4553,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H44" s="29" t="n">
-        <v>-8.24</v>
-      </c>
-      <c r="I44" s="29" t="n">
-        <v>-10.69</v>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H44" s="27" t="n">
+        <v>29.98</v>
+      </c>
+      <c r="I44" s="27" t="n">
+        <v>41.82</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>우리기술</t>
+          <t>삼화전자</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4578,25 +4588,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H45" s="29" t="n">
-        <v>-1.89</v>
-      </c>
-      <c r="I45" s="29" t="n">
-        <v>-17.47</v>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H45" s="27" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="I45" s="27" t="n">
+        <v>73.59</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>위더스제약</t>
+          <t>성문전자</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4613,25 +4623,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H46" s="27" t="n">
-        <v>13.59</v>
+        <v>4.43</v>
       </c>
       <c r="I46" s="27" t="n">
-        <v>33.03</v>
+        <v>40.24</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>율촌</t>
+          <t>위더스제약</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4648,25 +4658,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H47" s="29" t="n">
-        <v>-13.55</v>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H47" s="27" t="n">
+        <v>13.59</v>
       </c>
       <c r="I47" s="27" t="n">
-        <v>30.73</v>
+        <v>33.03</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>티웨이홀딩스</t>
+          <t>율촌</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4683,25 +4693,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H48" s="29" t="n">
-        <v>-7.09</v>
+        <v>-13.55</v>
       </c>
       <c r="I48" s="27" t="n">
-        <v>26.88</v>
+        <v>30.73</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>한전기술</t>
+          <t>티웨이홀딩스</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4718,25 +4728,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H49" s="29" t="n">
-        <v>-9.51</v>
-      </c>
-      <c r="I49" s="29" t="n">
-        <v>-18.24</v>
+        <v>-7.09</v>
+      </c>
+      <c r="I49" s="27" t="n">
+        <v>26.88</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>한화</t>
+          <t>피앤에스로보틱스</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4753,25 +4763,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="H50" s="29" t="n">
-        <v>-4.71</v>
-      </c>
-      <c r="I50" s="29" t="n">
-        <v>-0.95</v>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="H50" s="27" t="n">
+        <v>22.04</v>
+      </c>
+      <c r="I50" s="27" t="n">
+        <v>20.74</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>현대약품</t>
+          <t>한솔테크닉스</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4788,25 +4798,25 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H51" s="29" t="n">
-        <v>-4.12</v>
+        <v>-4.87</v>
       </c>
       <c r="I51" s="27" t="n">
-        <v>42.23</v>
+        <v>7.83</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="26" t="inlineStr">
         <is>
-          <t>휴림로봇</t>
+          <t>현대약품</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -4823,19 +4833,19 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="H52" s="29" t="n">
-        <v>-3.34</v>
-      </c>
-      <c r="I52" s="29" t="n">
-        <v>-13.73</v>
+        <v>-4.12</v>
+      </c>
+      <c r="I52" s="27" t="n">
+        <v>42.23</v>
       </c>
     </row>
   </sheetData>
@@ -4926,12 +4936,12 @@
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4950,19 +4960,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4988,12 +4998,12 @@
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5005,26 +5015,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5036,26 +5046,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5067,26 +5077,26 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5098,65 +5108,69 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
+          <t>제약</t>
+        </is>
+      </c>
+      <c r="B9" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" s="36" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="F9" s="37" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="G9" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
           <t>인공지능</t>
         </is>
       </c>
-      <c r="B9" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" s="36" t="n">
-        <v>9</v>
-      </c>
-      <c r="D9" s="36" t="n">
-        <v>9</v>
-      </c>
-      <c r="E9" s="36" t="inlineStr">
-        <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="F9" s="37" t="inlineStr">
-        <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="G9" s="37" t="inlineStr">
+      <c r="B10" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="36" t="n">
+        <v>12</v>
+      </c>
+      <c r="D10" s="36" t="n">
+        <v>12</v>
+      </c>
+      <c r="E10" s="36" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="F10" s="37" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="G10" s="37" t="inlineStr">
         <is>
           <t>⚡ 관심</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="26" t="inlineStr">
-        <is>
-          <t>이차전지</t>
-        </is>
-      </c>
-      <c r="B10" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" s="28" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>이차전지</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
@@ -5183,7 +5197,7 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
@@ -5264,7 +5278,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5291,7 +5305,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -5318,7 +5332,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>핀테크</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -5345,7 +5359,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>핀테크</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -5372,7 +5386,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-06-22 07:00 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -258,13 +258,13 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-06-21 06:55</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-06-22 06:55</t>
         </is>
       </c>
     </row>
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-06-21) 상위: 반도체  점수 60.0점</t>
+          <t>⚡ 최신(2026-06-22) 상위: 반도체  점수 82.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-06-21) 상위: SK  점수 56.0점</t>
+          <t>⚡ 최신(2026-06-22) 상위: SK  점수 46.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-06-21) 상위: SK하이닉스  점수 41.0점</t>
+          <t>⚡ 최신(2026-06-22) 상위: SK하이닉스  점수 44.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>60</v>
+        <v>82</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>60</v>
+        <v>82</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -971,10 +971,10 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -990,7 +990,7 @@
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1014,10 +1014,10 @@
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
@@ -1045,7 +1045,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1053,14 +1053,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1069,26 +1069,26 @@
         <v>0</v>
       </c>
       <c r="H17" s="19" t="n">
-        <v>-2.34</v>
+        <v>-0.91</v>
       </c>
       <c r="I17" s="18" t="n">
-        <v>9.77</v>
+        <v>2.25</v>
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>Google 급상승 검색어 등장 (KR) / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1096,14 +1096,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1111,27 +1111,27 @@
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="18" t="n">
-        <v>2</v>
+      <c r="H18" s="19" t="n">
+        <v>-2.34</v>
       </c>
       <c r="I18" s="18" t="n">
-        <v>0.99</v>
+        <v>9.77</v>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>Google 급상승 검색어 등장 (KR) / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K18" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>Google, 네이버</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1139,14 +1139,14 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1154,25 +1154,27 @@
       <c r="G19" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="19" t="n">
-        <v>-3.12</v>
+      <c r="H19" s="18" t="n">
+        <v>2</v>
       </c>
       <c r="I19" s="18" t="n">
-        <v>5.08</v>
+        <v>0.99</v>
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K19" s="17" t="n">
-        <v/>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K19" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1180,14 +1182,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1195,25 +1197,27 @@
       <c r="G20" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="18" t="n">
-        <v>3.18</v>
-      </c>
-      <c r="I20" s="18" t="n">
-        <v>32.44</v>
+      <c r="H20" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I20" s="15" t="n">
+        <v/>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K20" s="17" t="n">
-        <v/>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K20" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1225,10 +1229,10 @@
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
@@ -1244,7 +1248,7 @@
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
@@ -1256,7 +1260,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1264,14 +1268,14 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -1287,19 +1291,17 @@
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K22" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K22" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1307,14 +1309,14 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F23" s="15" t="n">
         <v>0</v>
@@ -1322,15 +1324,15 @@
       <c r="G23" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="19" t="n">
-        <v>-0.91</v>
-      </c>
-      <c r="I23" s="18" t="n">
-        <v>2.25</v>
+      <c r="H23" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I23" s="15" t="n">
+        <v/>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K23" s="17" t="inlineStr">
@@ -1342,7 +1344,7 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1350,14 +1352,14 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>넥써쓰</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>0</v>
@@ -1366,26 +1368,24 @@
         <v>0</v>
       </c>
       <c r="H24" s="19" t="n">
-        <v>-27.47</v>
-      </c>
-      <c r="I24" s="19" t="n">
-        <v>-4.83</v>
+        <v>-3.12</v>
+      </c>
+      <c r="I24" s="18" t="n">
+        <v>5.08</v>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +102% / 중요공시 3건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K24" s="17" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K24" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1393,14 +1393,14 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>삼성E&amp;A</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F25" s="15" t="n">
         <v>0</v>
@@ -1408,27 +1408,27 @@
       <c r="G25" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H25" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I25" s="15" t="n">
-        <v/>
+      <c r="H25" s="19" t="n">
+        <v>-2.11</v>
+      </c>
+      <c r="I25" s="18" t="n">
+        <v>2.21</v>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +91% / Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K25" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>Google, 네이버</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
@@ -1452,26 +1452,24 @@
         <v>0</v>
       </c>
       <c r="H26" s="19" t="n">
-        <v>-1.9</v>
+        <v>-7.44</v>
       </c>
       <c r="I26" s="19" t="n">
-        <v>-1.56</v>
+        <v>-6.21</v>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>중요공시 2건 / Google 급상승 검색어 등장 (KR) / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K26" s="17" t="inlineStr">
-        <is>
-          <t>네이버, 공시, Google</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K26" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -1479,7 +1477,7 @@
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D27" s="15" t="n">
@@ -1494,27 +1492,27 @@
       <c r="G27" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H27" s="19" t="n">
-        <v>-2.13</v>
-      </c>
-      <c r="I27" s="19" t="n">
-        <v>-0.72</v>
+      <c r="H27" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I27" s="15" t="n">
+        <v/>
       </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K27" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B28" s="20" t="n">
@@ -1522,7 +1520,7 @@
       </c>
       <c r="C28" s="21" t="inlineStr">
         <is>
-          <t>보해양조</t>
+          <t>넥써쓰</t>
         </is>
       </c>
       <c r="D28" s="20" t="n">
@@ -1538,26 +1536,26 @@
         <v>0</v>
       </c>
       <c r="H28" s="22" t="n">
-        <v>29.88</v>
+        <v>-27.47</v>
       </c>
       <c r="I28" s="22" t="n">
-        <v>58.36</v>
+        <v>-4.83</v>
       </c>
       <c r="J28" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +186% / 매일경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +113% / 중요공시 3건</t>
         </is>
       </c>
       <c r="K28" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B29" s="20" t="n">
@@ -1565,7 +1563,7 @@
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>한화</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="D29" s="20" t="n">
@@ -1580,15 +1578,15 @@
       <c r="G29" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H29" s="24" t="n">
-        <v>-4.71</v>
-      </c>
-      <c r="I29" s="24" t="n">
-        <v>-0.95</v>
+      <c r="H29" s="22" t="n">
+        <v>-26.16</v>
+      </c>
+      <c r="I29" s="22" t="n">
+        <v>-19.9</v>
       </c>
       <c r="J29" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +112% / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K29" s="23" t="inlineStr">
@@ -1600,7 +1598,7 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
@@ -1608,42 +1606,42 @@
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>한솔테크닉스</t>
         </is>
       </c>
       <c r="D30" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E30" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F30" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G30" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="24" t="n">
-        <v>-26.16</v>
+        <v>3</v>
+      </c>
+      <c r="H30" s="22" t="n">
+        <v>-4.87</v>
       </c>
       <c r="I30" s="24" t="n">
-        <v>-19.9</v>
+        <v>7.83</v>
       </c>
       <c r="J30" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +100% / 매일경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +81% / 중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K30" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1651,42 +1649,42 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>HJ중공업</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F31" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G31" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H31" s="22" t="n">
-        <v>2.64</v>
-      </c>
-      <c r="I31" s="22" t="n">
-        <v>13.93</v>
+        <v>-3.67</v>
+      </c>
+      <c r="I31" s="24" t="n">
+        <v>3.24</v>
       </c>
       <c r="J31" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K31" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1694,14 +1692,14 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>삼성바이오로직스</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F32" s="20" t="n">
         <v>0</v>
@@ -1709,27 +1707,27 @@
       <c r="G32" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H32" s="24" t="n">
-        <v>-3.85</v>
+      <c r="H32" s="22" t="n">
+        <v>-3.92</v>
       </c>
       <c r="I32" s="24" t="n">
-        <v>-6.79</v>
+        <v>6.1</v>
       </c>
       <c r="J32" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 1건 / Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K32" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>Google, 공시</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1737,42 +1735,42 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>진원생명과학</t>
+          <t>삼성전자우</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F33" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G33" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H33" s="24" t="n">
-        <v>-17.67</v>
+      <c r="H33" s="22" t="n">
+        <v>-2.84</v>
       </c>
       <c r="I33" s="24" t="n">
-        <v>-24.4</v>
+        <v>7.25</v>
       </c>
       <c r="J33" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +50%</t>
+          <t>Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K33" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1780,7 +1778,7 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
@@ -1795,27 +1793,27 @@
       <c r="G34" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I34" s="20" t="n">
-        <v/>
+      <c r="H34" s="22" t="n">
+        <v>-0.54</v>
+      </c>
+      <c r="I34" s="24" t="n">
+        <v>2.42</v>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K34" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1823,40 +1821,42 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>진원생명과학</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F35" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G35" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H35" s="24" t="n">
-        <v>-0.37</v>
-      </c>
-      <c r="I35" s="24" t="n">
-        <v>-2.74</v>
+      <c r="H35" s="22" t="n">
+        <v>-17.67</v>
+      </c>
+      <c r="I35" s="22" t="n">
+        <v>-24.4</v>
       </c>
       <c r="J35" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K35" s="23" t="n">
-        <v/>
+          <t>중요공시 3건 / 중요공시 3일 +50%</t>
+        </is>
+      </c>
+      <c r="K35" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1864,14 +1864,14 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>남화토건</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F36" s="20" t="n">
         <v>0</v>
@@ -1879,27 +1879,27 @@
       <c r="G36" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H36" s="22" t="n">
-        <v>12.73</v>
-      </c>
-      <c r="I36" s="22" t="n">
-        <v>45.92</v>
+      <c r="H36" s="24" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="I36" s="24" t="n">
+        <v>32.44</v>
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +819% / 중요공시 1건</t>
+          <t>Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K36" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1907,14 +1907,14 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>씨피시스템</t>
+          <t>삼성물산</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E37" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F37" s="20" t="n">
         <v>0</v>
@@ -1922,27 +1922,27 @@
       <c r="G37" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H37" s="22" t="n">
-        <v>29.88</v>
-      </c>
-      <c r="I37" s="22" t="n">
-        <v>20.79</v>
+      <c r="H37" s="24" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="I37" s="24" t="n">
+        <v>13.77</v>
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +73% / 한국경제 헤드라인 언급</t>
+          <t>Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K37" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1950,14 +1950,14 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>삼성SDI</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F38" s="20" t="n">
         <v>0</v>
@@ -1966,24 +1966,26 @@
         <v>0</v>
       </c>
       <c r="H38" s="24" t="n">
-        <v>-7.44</v>
+        <v>6.32</v>
       </c>
       <c r="I38" s="24" t="n">
-        <v>-6.21</v>
+        <v>2.97</v>
       </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K38" s="23" t="n">
-        <v/>
+          <t>Google 급상승 검색어 등장 (KR)</t>
+        </is>
+      </c>
+      <c r="K38" s="23" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1991,42 +1993,42 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>HJ중공업</t>
+          <t>삼성제약</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F39" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G39" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H39" s="24" t="n">
-        <v>-3.67</v>
-      </c>
-      <c r="I39" s="22" t="n">
-        <v>3.24</v>
+        <v>0</v>
+      </c>
+      <c r="H39" s="22" t="n">
+        <v>-3.9</v>
+      </c>
+      <c r="I39" s="24" t="n">
+        <v>3.92</v>
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+          <t>Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K39" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2034,14 +2036,14 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F40" s="20" t="n">
         <v>0</v>
@@ -2050,26 +2052,26 @@
         <v>0</v>
       </c>
       <c r="H40" s="24" t="n">
-        <v>-2.49</v>
-      </c>
-      <c r="I40" s="22" t="n">
-        <v>2.62</v>
+        <v>5.97</v>
+      </c>
+      <c r="I40" s="24" t="n">
+        <v>28.92</v>
       </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+          <t>Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K40" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2077,14 +2079,14 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E41" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F41" s="20" t="n">
         <v>0</v>
@@ -2092,27 +2094,27 @@
       <c r="G41" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I41" s="20" t="n">
-        <v/>
+      <c r="H41" s="22" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="I41" s="24" t="n">
+        <v>0.08</v>
       </c>
       <c r="J41" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K41" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2120,14 +2122,14 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>삼성에스디에스</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E42" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F42" s="20" t="n">
         <v>0</v>
@@ -2135,27 +2137,27 @@
       <c r="G42" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H42" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I42" s="20" t="n">
-        <v/>
+      <c r="H42" s="22" t="n">
+        <v>-4.07</v>
+      </c>
+      <c r="I42" s="22" t="n">
+        <v>-10.55</v>
       </c>
       <c r="J42" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K42" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2163,14 +2165,14 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>한화</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E43" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F43" s="20" t="n">
         <v>0</v>
@@ -2178,15 +2180,15 @@
       <c r="G43" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H43" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I43" s="20" t="n">
-        <v/>
+      <c r="H43" s="22" t="n">
+        <v>-4.71</v>
+      </c>
+      <c r="I43" s="22" t="n">
+        <v>-0.95</v>
       </c>
       <c r="J43" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K43" s="23" t="n">
@@ -2196,7 +2198,7 @@
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2204,7 +2206,7 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>HD현대</t>
+          <t>남화토건</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
@@ -2220,282 +2222,278 @@
         <v>0</v>
       </c>
       <c r="H44" s="24" t="n">
-        <v>-3.35</v>
+        <v>12.73</v>
       </c>
       <c r="I44" s="24" t="n">
-        <v>-5.53</v>
+        <v>45.92</v>
       </c>
       <c r="J44" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K44" s="23" t="n">
+          <t>네이버 검색 당일 +921% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K44" s="23" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B45" s="20" t="n">
+        <v>32</v>
+      </c>
+      <c r="C45" s="21" t="inlineStr">
+        <is>
+          <t>HMM</t>
+        </is>
+      </c>
+      <c r="D45" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E45" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F45" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="22" t="n">
+        <v>-1.47</v>
+      </c>
+      <c r="I45" s="24" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J45" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K45" s="23" t="n">
         <v/>
       </c>
     </row>
-    <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="25" t="inlineStr">
-        <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="B45" s="25" t="n">
-        <v>32</v>
-      </c>
-      <c r="C45" s="26" t="inlineStr">
-        <is>
-          <t>JW신약</t>
-        </is>
-      </c>
-      <c r="D45" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E45" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F45" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G45" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H45" s="27" t="n">
-        <v>13.08</v>
-      </c>
-      <c r="I45" s="27" t="n">
-        <v>70.94</v>
-      </c>
-      <c r="J45" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +1348%</t>
-        </is>
-      </c>
-      <c r="K45" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="25" t="inlineStr">
-        <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="B46" s="25" t="n">
+      <c r="A46" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B46" s="20" t="n">
         <v>33</v>
       </c>
-      <c r="C46" s="26" t="inlineStr">
-        <is>
-          <t>강동씨앤엘</t>
-        </is>
-      </c>
-      <c r="D46" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E46" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F46" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G46" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" s="27" t="n">
-        <v>29.91</v>
-      </c>
-      <c r="I46" s="27" t="n">
-        <v>121.56</v>
-      </c>
-      <c r="J46" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +1305%</t>
-        </is>
-      </c>
-      <c r="K46" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
+      <c r="C46" s="21" t="inlineStr">
+        <is>
+          <t>센서뷰</t>
+        </is>
+      </c>
+      <c r="D46" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E46" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H46" s="22" t="n">
+        <v>-5.11</v>
+      </c>
+      <c r="I46" s="22" t="n">
+        <v>-12.29</v>
+      </c>
+      <c r="J46" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K46" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="25" t="inlineStr">
-        <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="B47" s="25" t="n">
+      <c r="A47" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B47" s="20" t="n">
         <v>34</v>
       </c>
-      <c r="C47" s="26" t="inlineStr">
-        <is>
-          <t>삼익제약</t>
-        </is>
-      </c>
-      <c r="D47" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E47" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F47" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" s="27" t="n">
-        <v>29.98</v>
-      </c>
-      <c r="I47" s="27" t="n">
-        <v>41.82</v>
-      </c>
-      <c r="J47" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +720%</t>
-        </is>
-      </c>
-      <c r="K47" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
+      <c r="C47" s="21" t="inlineStr">
+        <is>
+          <t>파두</t>
+        </is>
+      </c>
+      <c r="D47" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E47" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H47" s="22" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="I47" s="24" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J47" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K47" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="25" t="inlineStr">
-        <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="B48" s="25" t="n">
+      <c r="A48" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B48" s="20" t="n">
         <v>35</v>
       </c>
-      <c r="C48" s="26" t="inlineStr">
-        <is>
-          <t>현대약품</t>
-        </is>
-      </c>
-      <c r="D48" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E48" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F48" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="29" t="n">
-        <v>-4.12</v>
-      </c>
-      <c r="I48" s="27" t="n">
-        <v>42.23</v>
-      </c>
-      <c r="J48" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +416%</t>
-        </is>
-      </c>
-      <c r="K48" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
+      <c r="C48" s="21" t="inlineStr">
+        <is>
+          <t>현대로템</t>
+        </is>
+      </c>
+      <c r="D48" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E48" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F48" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="22" t="n">
+        <v>-2.13</v>
+      </c>
+      <c r="I48" s="22" t="n">
+        <v>-0.72</v>
+      </c>
+      <c r="J48" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K48" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="25" t="inlineStr">
-        <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="B49" s="25" t="n">
+      <c r="A49" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B49" s="20" t="n">
         <v>36</v>
       </c>
-      <c r="C49" s="26" t="inlineStr">
-        <is>
-          <t>위더스제약</t>
-        </is>
-      </c>
-      <c r="D49" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E49" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F49" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G49" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H49" s="27" t="n">
-        <v>13.59</v>
-      </c>
-      <c r="I49" s="27" t="n">
-        <v>33.03</v>
-      </c>
-      <c r="J49" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +394%</t>
-        </is>
-      </c>
-      <c r="K49" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+      <c r="C49" s="21" t="inlineStr">
+        <is>
+          <t>태양광</t>
+        </is>
+      </c>
+      <c r="D49" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E49" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F49" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I49" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J49" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K49" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="25" t="inlineStr">
-        <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="B50" s="25" t="n">
+      <c r="A50" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B50" s="20" t="n">
         <v>37</v>
       </c>
-      <c r="C50" s="26" t="inlineStr">
-        <is>
-          <t>삼화전자</t>
-        </is>
-      </c>
-      <c r="D50" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E50" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F50" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G50" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H50" s="27" t="n">
-        <v>2.81</v>
-      </c>
-      <c r="I50" s="27" t="n">
-        <v>73.59</v>
-      </c>
-      <c r="J50" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +391%</t>
-        </is>
-      </c>
-      <c r="K50" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+      <c r="C50" s="21" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="D50" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E50" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F50" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="22" t="n">
+        <v>-2.39</v>
+      </c>
+      <c r="I50" s="22" t="n">
+        <v>-6.55</v>
+      </c>
+      <c r="J50" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K50" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -2503,7 +2501,7 @@
       </c>
       <c r="C51" s="26" t="inlineStr">
         <is>
-          <t>율촌</t>
+          <t>강동씨앤엘</t>
         </is>
       </c>
       <c r="D51" s="25" t="n">
@@ -2518,15 +2516,15 @@
       <c r="G51" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H51" s="29" t="n">
-        <v>-13.55</v>
+      <c r="H51" s="27" t="n">
+        <v>29.91</v>
       </c>
       <c r="I51" s="27" t="n">
-        <v>30.73</v>
+        <v>121.56</v>
       </c>
       <c r="J51" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +196%</t>
+          <t>네이버 검색 당일 +1463%</t>
         </is>
       </c>
       <c r="K51" s="28" t="inlineStr">
@@ -2538,7 +2536,7 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -2546,7 +2544,7 @@
       </c>
       <c r="C52" s="26" t="inlineStr">
         <is>
-          <t>성문전자</t>
+          <t>JW신약</t>
         </is>
       </c>
       <c r="D52" s="25" t="n">
@@ -2562,14 +2560,14 @@
         <v>0</v>
       </c>
       <c r="H52" s="27" t="n">
-        <v>4.43</v>
+        <v>13.08</v>
       </c>
       <c r="I52" s="27" t="n">
-        <v>40.24</v>
+        <v>70.94</v>
       </c>
       <c r="J52" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +175%</t>
+          <t>네이버 검색 당일 +1428%</t>
         </is>
       </c>
       <c r="K52" s="28" t="inlineStr">
@@ -2581,7 +2579,7 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2589,7 +2587,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>티웨이홀딩스</t>
+          <t>삼익제약</t>
         </is>
       </c>
       <c r="D53" s="25" t="n">
@@ -2604,15 +2602,15 @@
       <c r="G53" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="29" t="n">
-        <v>-7.09</v>
+      <c r="H53" s="27" t="n">
+        <v>29.98</v>
       </c>
       <c r="I53" s="27" t="n">
-        <v>26.88</v>
+        <v>41.82</v>
       </c>
       <c r="J53" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +174%</t>
+          <t>네이버 검색 당일 +800%</t>
         </is>
       </c>
       <c r="K53" s="28" t="inlineStr">
@@ -2624,7 +2622,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2632,7 +2630,7 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>메리츠제2호스팩</t>
+          <t>현대약품</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -2647,15 +2645,15 @@
       <c r="G54" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H54" s="25" t="n">
-        <v/>
-      </c>
-      <c r="I54" s="25" t="n">
-        <v/>
+      <c r="H54" s="29" t="n">
+        <v>-4.12</v>
+      </c>
+      <c r="I54" s="27" t="n">
+        <v>42.23</v>
       </c>
       <c r="J54" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +172%</t>
+          <t>네이버 검색 당일 +429%</t>
         </is>
       </c>
       <c r="K54" s="28" t="inlineStr">
@@ -2667,7 +2665,7 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2675,7 +2673,7 @@
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>부국철강</t>
+          <t>위더스제약</t>
         </is>
       </c>
       <c r="D55" s="25" t="n">
@@ -2690,15 +2688,15 @@
       <c r="G55" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H55" s="29" t="n">
-        <v>-13.76</v>
+      <c r="H55" s="27" t="n">
+        <v>13.59</v>
       </c>
       <c r="I55" s="27" t="n">
-        <v>3.49</v>
+        <v>33.03</v>
       </c>
       <c r="J55" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +160%</t>
+          <t>네이버 검색 당일 +422%</t>
         </is>
       </c>
       <c r="K55" s="28" t="inlineStr">
@@ -2710,7 +2708,7 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2718,7 +2716,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>피앤에스로보틱스</t>
+          <t>삼화전자</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2734,14 +2732,14 @@
         <v>0</v>
       </c>
       <c r="H56" s="27" t="n">
-        <v>22.04</v>
+        <v>2.81</v>
       </c>
       <c r="I56" s="27" t="n">
-        <v>20.74</v>
+        <v>73.59</v>
       </c>
       <c r="J56" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +151%</t>
+          <t>네이버 검색 당일 +412%</t>
         </is>
       </c>
       <c r="K56" s="28" t="inlineStr">
@@ -2753,7 +2751,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2761,7 +2759,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>동일스틸럭스</t>
+          <t>보해양조</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2776,15 +2774,15 @@
       <c r="G57" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H57" s="29" t="n">
-        <v>-11.15</v>
+      <c r="H57" s="27" t="n">
+        <v>29.88</v>
       </c>
       <c r="I57" s="27" t="n">
-        <v>29.05</v>
+        <v>58.36</v>
       </c>
       <c r="J57" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +147%</t>
+          <t>네이버 검색 당일 +237%</t>
         </is>
       </c>
       <c r="K57" s="28" t="inlineStr">
@@ -2796,7 +2794,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2804,7 +2802,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>대원전선</t>
+          <t>율촌</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2820,26 +2818,26 @@
         <v>0</v>
       </c>
       <c r="H58" s="29" t="n">
-        <v>-3.73</v>
+        <v>-13.55</v>
       </c>
       <c r="I58" s="27" t="n">
-        <v>6.02</v>
+        <v>30.73</v>
       </c>
       <c r="J58" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +95% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +208%</t>
         </is>
       </c>
       <c r="K58" s="28" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2847,7 +2845,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>비엘팜텍</t>
+          <t>성문전자</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2862,27 +2860,27 @@
       <c r="G59" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H59" s="29" t="n">
-        <v>-20.26</v>
+      <c r="H59" s="27" t="n">
+        <v>4.43</v>
       </c>
       <c r="I59" s="27" t="n">
-        <v>4.23</v>
+        <v>40.24</v>
       </c>
       <c r="J59" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +78% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +187%</t>
         </is>
       </c>
       <c r="K59" s="28" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2890,7 +2888,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>한솔테크닉스</t>
+          <t>메리츠제2호스팩</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2905,27 +2903,27 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="29" t="n">
-        <v>-4.87</v>
-      </c>
-      <c r="I60" s="27" t="n">
-        <v>7.83</v>
+      <c r="H60" s="25" t="n">
+        <v/>
+      </c>
+      <c r="I60" s="25" t="n">
+        <v/>
       </c>
       <c r="J60" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +76% / 중요공시 2건</t>
+          <t>네이버 검색 당일 +186%</t>
         </is>
       </c>
       <c r="K60" s="28" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2933,7 +2931,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>삼보산업</t>
+          <t>피앤에스로보틱스</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2949,26 +2947,26 @@
         <v>0</v>
       </c>
       <c r="H61" s="27" t="n">
-        <v>11.54</v>
+        <v>22.04</v>
       </c>
       <c r="I61" s="27" t="n">
-        <v>45.97</v>
+        <v>20.74</v>
       </c>
       <c r="J61" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +61% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +182%</t>
         </is>
       </c>
       <c r="K61" s="28" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2976,7 +2974,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>다스코</t>
+          <t>티웨이홀딩스</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2991,27 +2989,27 @@
       <c r="G62" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H62" s="27" t="n">
-        <v>29.96</v>
+      <c r="H62" s="29" t="n">
+        <v>-7.09</v>
       </c>
       <c r="I62" s="27" t="n">
-        <v>31.44</v>
+        <v>26.88</v>
       </c>
       <c r="J62" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +59% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +181%</t>
         </is>
       </c>
       <c r="K62" s="28" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3019,7 +3017,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>부국철강</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3035,19 +3033,19 @@
         <v>0</v>
       </c>
       <c r="H63" s="29" t="n">
-        <v>-7.41</v>
-      </c>
-      <c r="I63" s="29" t="n">
-        <v>-2.75</v>
+        <v>-13.76</v>
+      </c>
+      <c r="I63" s="27" t="n">
+        <v>3.49</v>
       </c>
       <c r="J63" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +58% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +170%</t>
         </is>
       </c>
       <c r="K63" s="28" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
@@ -3144,22 +3142,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>60</v>
+        <v>82</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>60</v>
+        <v>82</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3175,22 +3173,22 @@
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H4" s="27" t="n">
@@ -3210,22 +3208,22 @@
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H5" s="27" t="n">
@@ -3238,142 +3236,138 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H6" s="29" t="n">
-        <v>-2.34</v>
+        <v>-0.91</v>
       </c>
       <c r="I6" s="27" t="n">
-        <v>9.77</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H7" s="27" t="n">
-        <v>2</v>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H7" s="29" t="n">
+        <v>-2.34</v>
       </c>
       <c r="I7" s="27" t="n">
-        <v>0.99</v>
+        <v>9.77</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H8" s="29" t="n">
-        <v>-3.12</v>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H8" s="27" t="n">
+        <v>2</v>
       </c>
       <c r="I8" s="27" t="n">
-        <v>5.08</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H9" s="27" t="n">
-        <v>3.18</v>
-      </c>
-      <c r="I9" s="27" t="n">
-        <v>32.44</v>
-      </c>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H9" s="25" t="n"/>
+      <c r="I9" s="25" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
@@ -3385,22 +3379,22 @@
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H10" s="25" t="n"/>
@@ -3409,64 +3403,60 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H11" s="29" t="n">
-        <v>-0.91</v>
-      </c>
-      <c r="I11" s="27" t="n">
-        <v>2.25</v>
-      </c>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H11" s="25" t="n"/>
+      <c r="I11" s="25" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H12" s="25" t="n"/>
@@ -3475,73 +3465,77 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>넥써쓰</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H13" s="29" t="n">
-        <v>-27.47</v>
-      </c>
-      <c r="I13" s="29" t="n">
-        <v>-4.83</v>
+        <v>-3.12</v>
+      </c>
+      <c r="I13" s="27" t="n">
+        <v>5.08</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H14" s="25" t="n"/>
-      <c r="I14" s="25" t="n"/>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H14" s="29" t="n">
+        <v>-7.44</v>
+      </c>
+      <c r="I14" s="29" t="n">
+        <v>-6.21</v>
+      </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>삼성E&amp;A</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -3558,25 +3552,25 @@
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H15" s="29" t="n">
-        <v>-1.9</v>
-      </c>
-      <c r="I15" s="29" t="n">
-        <v>-1.56</v>
+        <v>-2.11</v>
+      </c>
+      <c r="I15" s="27" t="n">
+        <v>2.21</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -3593,25 +3587,21 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H16" s="29" t="n">
-        <v>-2.13</v>
-      </c>
-      <c r="I16" s="29" t="n">
-        <v>-0.72</v>
-      </c>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H16" s="25" t="n"/>
+      <c r="I16" s="25" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>보해양조</t>
+          <t>HJ중공업</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -3628,25 +3618,25 @@
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H17" s="27" t="n">
-        <v>29.88</v>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H17" s="29" t="n">
+        <v>-3.67</v>
       </c>
       <c r="I17" s="27" t="n">
-        <v>58.36</v>
+        <v>3.24</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>한화</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -3663,130 +3653,130 @@
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H18" s="29" t="n">
-        <v>-4.71</v>
+        <v>-26.16</v>
       </c>
       <c r="I18" s="29" t="n">
-        <v>-0.95</v>
+        <v>-19.9</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>넥써쓰</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H19" s="29" t="n">
-        <v>-0.37</v>
+        <v>-27.47</v>
       </c>
       <c r="I19" s="29" t="n">
-        <v>-2.74</v>
+        <v>-4.83</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>삼성바이오로직스</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D20" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H20" s="29" t="n">
-        <v>-26.16</v>
-      </c>
-      <c r="I20" s="29" t="n">
-        <v>-19.9</v>
+        <v>-3.92</v>
+      </c>
+      <c r="I20" s="27" t="n">
+        <v>6.1</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>한솔테크닉스</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D21" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E21" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H21" s="29" t="n">
-        <v>-3.85</v>
-      </c>
-      <c r="I21" s="29" t="n">
-        <v>-6.79</v>
+        <v>-4.87</v>
+      </c>
+      <c r="I21" s="27" t="n">
+        <v>7.83</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>삼성SDI</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -3803,21 +3793,25 @@
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H22" s="25" t="n"/>
-      <c r="I22" s="25" t="n"/>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H22" s="27" t="n">
+        <v>6.32</v>
+      </c>
+      <c r="I22" s="27" t="n">
+        <v>2.97</v>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>진원생명과학</t>
+          <t>삼성물산</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3834,25 +3828,25 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H23" s="29" t="n">
-        <v>-17.67</v>
-      </c>
-      <c r="I23" s="29" t="n">
-        <v>-24.4</v>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H23" s="27" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="I23" s="27" t="n">
+        <v>13.77</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3869,297 +3863,305 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H24" s="27" t="n">
-        <v>2.64</v>
+        <v>5.97</v>
       </c>
       <c r="I24" s="27" t="n">
-        <v>13.93</v>
+        <v>28.92</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>HD현대</t>
+          <t>삼성에스디에스</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C25" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D25" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E25" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H25" s="29" t="n">
-        <v>-3.35</v>
+        <v>-4.07</v>
       </c>
       <c r="I25" s="29" t="n">
-        <v>-5.53</v>
+        <v>-10.55</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C26" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D26" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E26" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H26" s="29" t="n">
-        <v>-2.49</v>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H26" s="27" t="n">
+        <v>3.18</v>
       </c>
       <c r="I26" s="27" t="n">
-        <v>2.62</v>
+        <v>32.44</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>HJ중공업</t>
+          <t>삼성전자우</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C27" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D27" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E27" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H27" s="29" t="n">
-        <v>-3.67</v>
+        <v>-2.84</v>
       </c>
       <c r="I27" s="27" t="n">
-        <v>3.24</v>
+        <v>7.25</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>삼성제약</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C28" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D28" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E28" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H28" s="29" t="n">
-        <v>-7.44</v>
-      </c>
-      <c r="I28" s="29" t="n">
-        <v>-6.21</v>
+        <v>-3.9</v>
+      </c>
+      <c r="I28" s="27" t="n">
+        <v>3.92</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>남화토건</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C29" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D29" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E29" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H29" s="27" t="n">
-        <v>12.73</v>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H29" s="29" t="n">
+        <v>-0.54</v>
       </c>
       <c r="I29" s="27" t="n">
-        <v>45.92</v>
+        <v>2.42</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C30" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D30" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E30" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H30" s="25" t="n"/>
-      <c r="I30" s="25" t="n"/>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H30" s="29" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="I30" s="27" t="n">
+        <v>0.08</v>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>씨피시스템</t>
+          <t>진원생명과학</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C31" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D31" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E31" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H31" s="27" t="n">
-        <v>29.88</v>
-      </c>
-      <c r="I31" s="27" t="n">
-        <v>20.79</v>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H31" s="29" t="n">
+        <v>-17.67</v>
+      </c>
+      <c r="I31" s="29" t="n">
+        <v>-24.4</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>한화</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C32" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D32" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E32" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H32" s="25" t="n"/>
-      <c r="I32" s="25" t="n"/>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H32" s="29" t="n">
+        <v>-4.71</v>
+      </c>
+      <c r="I32" s="29" t="n">
+        <v>-0.95</v>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4176,231 +4178,231 @@
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H33" s="25" t="n"/>
-      <c r="I33" s="25" t="n"/>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H33" s="29" t="n">
+        <v>-2.39</v>
+      </c>
+      <c r="I33" s="29" t="n">
+        <v>-6.55</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>JW신약</t>
+          <t>HMM</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C34" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D34" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E34" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H34" s="27" t="n">
-        <v>13.08</v>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H34" s="29" t="n">
+        <v>-1.47</v>
       </c>
       <c r="I34" s="27" t="n">
-        <v>70.94</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>강동씨앤엘</t>
+          <t>남화토건</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D35" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E35" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H35" s="27" t="n">
-        <v>29.91</v>
+        <v>12.73</v>
       </c>
       <c r="I35" s="27" t="n">
-        <v>121.56</v>
+        <v>45.92</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>다스코</t>
+          <t>센서뷰</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C36" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D36" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E36" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H36" s="27" t="n">
-        <v>29.96</v>
-      </c>
-      <c r="I36" s="27" t="n">
-        <v>31.44</v>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H36" s="29" t="n">
+        <v>-5.11</v>
+      </c>
+      <c r="I36" s="29" t="n">
+        <v>-12.29</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C37" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D37" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E37" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H37" s="29" t="n">
-        <v>-7.41</v>
-      </c>
-      <c r="I37" s="29" t="n">
-        <v>-2.75</v>
-      </c>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H37" s="25" t="n"/>
+      <c r="I37" s="25" t="n"/>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>대원전선</t>
+          <t>파두</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C38" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D38" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E38" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H38" s="29" t="n">
-        <v>-3.73</v>
+        <v>-2.5</v>
       </c>
       <c r="I38" s="27" t="n">
-        <v>6.02</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>동일스틸럭스</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C39" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D39" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E39" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H39" s="29" t="n">
-        <v>-11.15</v>
-      </c>
-      <c r="I39" s="27" t="n">
-        <v>29.05</v>
+        <v>-2.13</v>
+      </c>
+      <c r="I39" s="29" t="n">
+        <v>-0.72</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>메리츠제2호스팩</t>
+          <t>JW신약</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4417,21 +4419,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H40" s="25" t="n"/>
-      <c r="I40" s="25" t="n"/>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H40" s="27" t="n">
+        <v>13.08</v>
+      </c>
+      <c r="I40" s="27" t="n">
+        <v>70.94</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>부국철강</t>
+          <t>강동씨앤엘</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4448,25 +4454,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H41" s="29" t="n">
-        <v>-13.76</v>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H41" s="27" t="n">
+        <v>29.91</v>
       </c>
       <c r="I41" s="27" t="n">
-        <v>3.49</v>
+        <v>121.56</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>비엘팜텍</t>
+          <t>메리츠제2호스팩</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4483,25 +4489,21 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H42" s="29" t="n">
-        <v>-20.26</v>
-      </c>
-      <c r="I42" s="27" t="n">
-        <v>4.23</v>
-      </c>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H42" s="25" t="n"/>
+      <c r="I42" s="25" t="n"/>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>삼보산업</t>
+          <t>보해양조</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4518,25 +4520,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H43" s="27" t="n">
-        <v>11.54</v>
+        <v>29.88</v>
       </c>
       <c r="I43" s="27" t="n">
-        <v>45.97</v>
+        <v>58.36</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>삼익제약</t>
+          <t>부국철강</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4553,25 +4555,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H44" s="27" t="n">
-        <v>29.98</v>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H44" s="29" t="n">
+        <v>-13.76</v>
       </c>
       <c r="I44" s="27" t="n">
-        <v>41.82</v>
+        <v>3.49</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>삼화전자</t>
+          <t>삼익제약</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4588,25 +4590,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H45" s="27" t="n">
-        <v>2.81</v>
+        <v>29.98</v>
       </c>
       <c r="I45" s="27" t="n">
-        <v>73.59</v>
+        <v>41.82</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>성문전자</t>
+          <t>삼화전자</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4623,25 +4625,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H46" s="27" t="n">
-        <v>4.43</v>
+        <v>2.81</v>
       </c>
       <c r="I46" s="27" t="n">
-        <v>40.24</v>
+        <v>73.59</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>위더스제약</t>
+          <t>성문전자</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4658,25 +4660,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H47" s="27" t="n">
-        <v>13.59</v>
+        <v>4.43</v>
       </c>
       <c r="I47" s="27" t="n">
-        <v>33.03</v>
+        <v>40.24</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>율촌</t>
+          <t>위더스제약</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4693,25 +4695,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H48" s="29" t="n">
-        <v>-13.55</v>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H48" s="27" t="n">
+        <v>13.59</v>
       </c>
       <c r="I48" s="27" t="n">
-        <v>30.73</v>
+        <v>33.03</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>티웨이홀딩스</t>
+          <t>율촌</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4728,25 +4730,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H49" s="29" t="n">
-        <v>-7.09</v>
+        <v>-13.55</v>
       </c>
       <c r="I49" s="27" t="n">
-        <v>26.88</v>
+        <v>30.73</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>피앤에스로보틱스</t>
+          <t>티웨이홀딩스</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4763,25 +4765,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H50" s="27" t="n">
-        <v>22.04</v>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H50" s="29" t="n">
+        <v>-7.09</v>
       </c>
       <c r="I50" s="27" t="n">
-        <v>20.74</v>
+        <v>26.88</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>한솔테크닉스</t>
+          <t>피앤에스로보틱스</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4798,19 +4800,19 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="H51" s="29" t="n">
-        <v>-4.87</v>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H51" s="27" t="n">
+        <v>22.04</v>
       </c>
       <c r="I51" s="27" t="n">
-        <v>7.83</v>
+        <v>20.74</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
@@ -4833,12 +4835,12 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H52" s="29" t="n">
@@ -4929,19 +4931,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>60</v>
+        <v>82</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>60</v>
+        <v>82</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4960,19 +4962,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4991,19 +4993,19 @@
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5015,26 +5017,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5046,26 +5048,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5077,26 +5079,26 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5108,26 +5110,26 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B9" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5137,40 +5139,36 @@
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="35" t="inlineStr">
-        <is>
-          <t>인공지능</t>
-        </is>
-      </c>
-      <c r="B10" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" s="36" t="n">
-        <v>12</v>
-      </c>
-      <c r="D10" s="36" t="n">
-        <v>12</v>
-      </c>
-      <c r="E10" s="36" t="inlineStr">
-        <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="F10" s="37" t="inlineStr">
-        <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="G10" s="37" t="inlineStr">
-        <is>
-          <t>⚡ 관심</t>
-        </is>
-      </c>
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>이차전지</t>
+        </is>
+      </c>
+      <c r="B10" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" s="28" t="inlineStr">
+        <is>
+          <t>감지 없음</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>이차전지</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
@@ -5197,7 +5195,7 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-06-28 07:07 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-06-27 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-06-28 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-06-27) 상위: 반도체  점수 101.0점</t>
+          <t>⚡ 최신(2026-06-28) 상위: 반도체  점수 104.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-06-27) 상위: SK  점수 50.0점</t>
+          <t>⚡ 최신(2026-06-28) 상위: SK  점수 50.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-06-27) 상위: SK하이닉스  점수 34.0점</t>
+          <t>⚡ 최신(2026-06-28) 상위: SK하이닉스  점수 35.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -990,7 +990,7 @@
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1014,10 +1014,10 @@
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
@@ -1045,7 +1045,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1057,10 +1057,10 @@
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
@@ -1088,7 +1088,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1129,7 +1129,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1137,14 +1137,14 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1160,7 +1160,7 @@
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K19" s="17" t="inlineStr">
@@ -1172,7 +1172,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1180,14 +1180,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1203,7 +1203,7 @@
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K20" s="17" t="inlineStr">
@@ -1215,7 +1215,7 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1223,42 +1223,42 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>파두</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F21" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G21" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H21" s="18" t="n">
-        <v>-5.14</v>
-      </c>
-      <c r="I21" s="18" t="n">
-        <v>-18.15</v>
+        <v>0</v>
+      </c>
+      <c r="H21" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I21" s="15" t="n">
+        <v/>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +50% / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1266,40 +1266,42 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>젠큐릭스</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G22" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I22" s="15" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H22" s="18" t="n">
+        <v>-1.9</v>
+      </c>
+      <c r="I22" s="18" t="n">
+        <v>-12.13</v>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K22" s="17" t="n">
-        <v/>
+          <t>중요공시 3건 / 중요공시 7일 +200% / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K22" s="17" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1307,42 +1309,40 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>젠큐릭스</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F23" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G23" s="15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H23" s="18" t="n">
-        <v>-1.9</v>
+        <v>-2.31</v>
       </c>
       <c r="I23" s="18" t="n">
-        <v>-12.13</v>
+        <v>-18.69</v>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +200% / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K23" s="17" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K23" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>LG이노텍</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
@@ -1366,14 +1366,14 @@
         <v>0</v>
       </c>
       <c r="H24" s="18" t="n">
-        <v>-2.31</v>
+        <v>-3.21</v>
       </c>
       <c r="I24" s="18" t="n">
-        <v>-18.69</v>
+        <v>-12.19</v>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K24" s="17" t="n">
@@ -1383,7 +1383,7 @@
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1391,40 +1391,42 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="F25" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G25" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="18" t="n">
-        <v>-3.21</v>
+        <v>3</v>
+      </c>
+      <c r="H25" s="19" t="n">
+        <v>0.52</v>
       </c>
       <c r="I25" s="18" t="n">
-        <v>-12.19</v>
+        <v>-24.25</v>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K25" s="17" t="n">
-        <v/>
+          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +50%</t>
+        </is>
+      </c>
+      <c r="K25" s="17" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1432,7 +1434,7 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>파두</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
@@ -1447,11 +1449,11 @@
       <c r="G26" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="H26" s="19" t="n">
-        <v>0.52</v>
+      <c r="H26" s="18" t="n">
+        <v>-5.14</v>
       </c>
       <c r="I26" s="18" t="n">
-        <v>-24.25</v>
+        <v>-18.15</v>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
@@ -1467,7 +1469,7 @@
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -1475,7 +1477,7 @@
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>페니트리움바이오</t>
         </is>
       </c>
       <c r="D27" s="15" t="n">
@@ -1491,14 +1493,14 @@
         <v>3</v>
       </c>
       <c r="H27" s="18" t="n">
-        <v>-8.76</v>
+        <v>-2.96</v>
       </c>
       <c r="I27" s="18" t="n">
-        <v>-31.49</v>
+        <v>-11.93</v>
       </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
-          <t>중요공시 5건 / 중요공시 3일 +150% / 중요공시 7일 +67%</t>
+          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +50%</t>
         </is>
       </c>
       <c r="K27" s="17" t="inlineStr">
@@ -1510,7 +1512,7 @@
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B28" s="15" t="n">
@@ -1518,42 +1520,42 @@
       </c>
       <c r="C28" s="16" t="inlineStr">
         <is>
-          <t>페니트리움바이오</t>
+          <t>다스코</t>
         </is>
       </c>
       <c r="D28" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E28" s="15" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F28" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G28" s="15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H28" s="18" t="n">
-        <v>-2.96</v>
+        <v>-16.32</v>
       </c>
       <c r="I28" s="18" t="n">
-        <v>-11.93</v>
+        <v>-1.01</v>
       </c>
       <c r="J28" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +200%</t>
+          <t>네이버 검색 당일 +134% / 중요공시 1건 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K28" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B29" s="15" t="n">
@@ -1561,14 +1563,14 @@
       </c>
       <c r="C29" s="16" t="inlineStr">
         <is>
-          <t>한미반도체</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="D29" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E29" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F29" s="15" t="n">
         <v>0</v>
@@ -1576,154 +1578,154 @@
       <c r="G29" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H29" s="18" t="n">
-        <v>-5.68</v>
-      </c>
-      <c r="I29" s="18" t="n">
-        <v>-12.71</v>
+      <c r="H29" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I29" s="15" t="n">
+        <v/>
       </c>
       <c r="J29" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K29" s="17" t="inlineStr">
+          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K29" s="17" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="n">
+        <v>17</v>
+      </c>
+      <c r="C30" s="21" t="inlineStr">
+        <is>
+          <t>광주신세계</t>
+        </is>
+      </c>
+      <c r="D30" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E30" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="22" t="n">
+        <v>29.98</v>
+      </c>
+      <c r="I30" s="22" t="n">
+        <v>50.71</v>
+      </c>
+      <c r="J30" s="23" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +1339% / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K30" s="23" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="15" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B30" s="15" t="n">
-        <v>17</v>
-      </c>
-      <c r="C30" s="16" t="inlineStr">
-        <is>
-          <t>소룩스</t>
-        </is>
-      </c>
-      <c r="D30" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E30" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F30" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="18" t="n">
-        <v>-4.21</v>
-      </c>
-      <c r="I30" s="19" t="n">
-        <v>19.47</v>
-      </c>
-      <c r="J30" s="17" t="inlineStr">
-        <is>
-          <t>중요공시 3건 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K30" s="17" t="inlineStr">
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B31" s="20" t="n">
+        <v>18</v>
+      </c>
+      <c r="C31" s="21" t="inlineStr">
+        <is>
+          <t>헝셩그룹</t>
+        </is>
+      </c>
+      <c r="D31" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E31" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F31" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G31" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="24" t="n">
+        <v>-2.71</v>
+      </c>
+      <c r="I31" s="22" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="J31" s="23" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +291% / 중요공시 2건 / 중요공시 3일 +100%</t>
+        </is>
+      </c>
+      <c r="K31" s="23" t="inlineStr">
         <is>
           <t>공시, 네이버</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="15" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B31" s="15" t="n">
-        <v>18</v>
-      </c>
-      <c r="C31" s="16" t="inlineStr">
-        <is>
-          <t>원익IPS</t>
-        </is>
-      </c>
-      <c r="D31" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E31" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F31" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" s="19" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="I31" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="J31" s="17" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K31" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="15" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B32" s="15" t="n">
+      <c r="A32" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B32" s="20" t="n">
         <v>19</v>
       </c>
-      <c r="C32" s="16" t="inlineStr">
-        <is>
-          <t>로봇</t>
-        </is>
-      </c>
-      <c r="D32" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E32" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F32" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H32" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I32" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J32" s="17" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K32" s="17" t="n">
-        <v/>
+      <c r="C32" s="21" t="inlineStr">
+        <is>
+          <t>삼호개발</t>
+        </is>
+      </c>
+      <c r="D32" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E32" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F32" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="22" t="n">
+        <v>8.69</v>
+      </c>
+      <c r="I32" s="22" t="n">
+        <v>16.77</v>
+      </c>
+      <c r="J32" s="23" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +132% / 중요공시 3건</t>
+        </is>
+      </c>
+      <c r="K32" s="23" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1731,7 +1733,7 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>광주신세계</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
@@ -1746,27 +1748,25 @@
       <c r="G33" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H33" s="22" t="n">
-        <v>29.98</v>
-      </c>
-      <c r="I33" s="22" t="n">
-        <v>50.71</v>
+      <c r="H33" s="24" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="I33" s="24" t="n">
+        <v>-7.38</v>
       </c>
       <c r="J33" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +654% / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K33" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K33" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>다스코</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
@@ -1790,26 +1790,26 @@
         <v>0</v>
       </c>
       <c r="H34" s="24" t="n">
-        <v>-16.32</v>
-      </c>
-      <c r="I34" s="24" t="n">
-        <v>-1.01</v>
+        <v>-3.61</v>
+      </c>
+      <c r="I34" s="22" t="n">
+        <v>0.36</v>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +58% / 중요공시 1건 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 3건 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K34" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1817,40 +1817,42 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F35" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G35" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H35" s="24" t="n">
-        <v>-3.5</v>
+        <v>-8.41</v>
       </c>
       <c r="I35" s="24" t="n">
-        <v>-7.38</v>
+        <v>-14.4</v>
       </c>
       <c r="J35" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K35" s="23" t="n">
-        <v/>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K35" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1858,30 +1860,30 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F36" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G36" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H36" s="24" t="n">
-        <v>-3.61</v>
-      </c>
-      <c r="I36" s="22" t="n">
-        <v>0.36</v>
+        <v>-8.76</v>
+      </c>
+      <c r="I36" s="24" t="n">
+        <v>-31.49</v>
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 5건 / 중요공시 7일 +150%</t>
         </is>
       </c>
       <c r="K36" s="23" t="inlineStr">
@@ -1893,7 +1895,7 @@
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1901,30 +1903,30 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>KB금융</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E37" s="20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F37" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G37" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H37" s="24" t="n">
-        <v>-8.41</v>
+        <v>-1.71</v>
       </c>
       <c r="I37" s="24" t="n">
-        <v>-14.4</v>
+        <v>-5.69</v>
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K37" s="23" t="inlineStr">
@@ -1936,7 +1938,7 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1944,30 +1946,30 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>에이팩트</t>
+          <t>카카오뱅크</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F38" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G38" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H38" s="24" t="n">
-        <v>-6.74</v>
+        <v>-3.42</v>
       </c>
       <c r="I38" s="24" t="n">
-        <v>-26.62</v>
+        <v>-10.84</v>
       </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 7일 +50%</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K38" s="23" t="inlineStr">
@@ -1979,7 +1981,7 @@
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1987,7 +1989,7 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>KB금융</t>
+          <t>삼성물산</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
@@ -2003,26 +2005,24 @@
         <v>0</v>
       </c>
       <c r="H39" s="24" t="n">
-        <v>-1.71</v>
-      </c>
-      <c r="I39" s="24" t="n">
-        <v>-5.69</v>
+        <v>-4.72</v>
+      </c>
+      <c r="I39" s="22" t="n">
+        <v>0.61</v>
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K39" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K39" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>카카오뱅크</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
@@ -2046,26 +2046,26 @@
         <v>0</v>
       </c>
       <c r="H40" s="24" t="n">
-        <v>-3.42</v>
+        <v>-4.47</v>
       </c>
       <c r="I40" s="24" t="n">
-        <v>-10.84</v>
+        <v>-21.62</v>
       </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K40" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2073,14 +2073,14 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>소룩스</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E41" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F41" s="20" t="n">
         <v>0</v>
@@ -2088,25 +2088,27 @@
       <c r="G41" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I41" s="20" t="n">
-        <v/>
+      <c r="H41" s="24" t="n">
+        <v>-4.21</v>
+      </c>
+      <c r="I41" s="22" t="n">
+        <v>19.47</v>
       </c>
       <c r="J41" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K41" s="23" t="n">
-        <v/>
+          <t>네이버 검색 당일 +76% / 중요공시 3건</t>
+        </is>
+      </c>
+      <c r="K41" s="23" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2114,14 +2116,14 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>리가켐바이오</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E42" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F42" s="20" t="n">
         <v>0</v>
@@ -2129,27 +2131,27 @@
       <c r="G42" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H42" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I42" s="20" t="n">
-        <v/>
+      <c r="H42" s="24" t="n">
+        <v>-8.279999999999999</v>
+      </c>
+      <c r="I42" s="22" t="n">
+        <v>6.17</v>
       </c>
       <c r="J42" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K42" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2157,42 +2159,42 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>차바이오텍</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E43" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F43" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G43" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H43" s="24" t="n">
-        <v>-4.12</v>
-      </c>
-      <c r="I43" s="24" t="n">
-        <v>-12.15</v>
+      <c r="H43" s="22" t="n">
+        <v>30</v>
+      </c>
+      <c r="I43" s="22" t="n">
+        <v>57.86</v>
       </c>
       <c r="J43" s="23" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 중요공시 3일 +300%</t>
+          <t>네이버 검색 당일 +348% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K43" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2200,14 +2202,14 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>리가켐바이오</t>
+          <t>크리스탈신소재</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E44" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F44" s="20" t="n">
         <v>0</v>
@@ -2215,27 +2217,27 @@
       <c r="G44" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="24" t="n">
-        <v>-8.279999999999999</v>
-      </c>
-      <c r="I44" s="22" t="n">
-        <v>6.17</v>
+      <c r="H44" s="22" t="n">
+        <v>18.81</v>
+      </c>
+      <c r="I44" s="24" t="n">
+        <v>-28.03</v>
       </c>
       <c r="J44" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>네이버 검색 당일 +317% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K44" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2243,7 +2245,7 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>헝셩그룹</t>
+          <t>티이엠씨씨엔에스</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
@@ -2258,15 +2260,15 @@
       <c r="G45" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H45" s="24" t="n">
-        <v>-2.71</v>
+      <c r="H45" s="22" t="n">
+        <v>30</v>
       </c>
       <c r="I45" s="22" t="n">
-        <v>15.4</v>
+        <v>10.36</v>
       </c>
       <c r="J45" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +241% / 중요공시 2건</t>
+          <t>네이버 검색 당일 +273% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K45" s="23" t="inlineStr">
@@ -2278,7 +2280,7 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
@@ -2286,7 +2288,7 @@
       </c>
       <c r="C46" s="21" t="inlineStr">
         <is>
-          <t>크리스탈신소재</t>
+          <t>베셀</t>
         </is>
       </c>
       <c r="D46" s="20" t="n">
@@ -2302,14 +2304,14 @@
         <v>0</v>
       </c>
       <c r="H46" s="22" t="n">
-        <v>18.81</v>
-      </c>
-      <c r="I46" s="24" t="n">
-        <v>-28.03</v>
+        <v>9.69</v>
+      </c>
+      <c r="I46" s="22" t="n">
+        <v>34.27</v>
       </c>
       <c r="J46" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +178% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +222% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K46" s="23" t="inlineStr">
@@ -2321,7 +2323,7 @@
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B47" s="20" t="n">
@@ -2329,7 +2331,7 @@
       </c>
       <c r="C47" s="21" t="inlineStr">
         <is>
-          <t>베셀</t>
+          <t>남화토건</t>
         </is>
       </c>
       <c r="D47" s="20" t="n">
@@ -2345,14 +2347,14 @@
         <v>0</v>
       </c>
       <c r="H47" s="22" t="n">
-        <v>9.69</v>
+        <v>29.96</v>
       </c>
       <c r="I47" s="22" t="n">
-        <v>34.27</v>
+        <v>28.96</v>
       </c>
       <c r="J47" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +169% / 중요공시 2건</t>
+          <t>네이버 검색 당일 +162% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K47" s="23" t="inlineStr">
@@ -2364,7 +2366,7 @@
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B48" s="20" t="n">
@@ -2372,7 +2374,7 @@
       </c>
       <c r="C48" s="21" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>뉴인텍</t>
         </is>
       </c>
       <c r="D48" s="20" t="n">
@@ -2388,14 +2390,14 @@
         <v>0</v>
       </c>
       <c r="H48" s="22" t="n">
-        <v>30</v>
+        <v>29.93</v>
       </c>
       <c r="I48" s="22" t="n">
-        <v>57.86</v>
+        <v>47.06</v>
       </c>
       <c r="J48" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +142% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +144% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K48" s="23" t="inlineStr">
@@ -2407,7 +2409,7 @@
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B49" s="20" t="n">
@@ -2415,42 +2417,42 @@
       </c>
       <c r="C49" s="21" t="inlineStr">
         <is>
-          <t>시너지이노베이션</t>
+          <t>에코프로</t>
         </is>
       </c>
       <c r="D49" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E49" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F49" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G49" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H49" s="24" t="n">
-        <v>-1.93</v>
+        <v>-6.47</v>
       </c>
       <c r="I49" s="24" t="n">
-        <v>-7.84</v>
+        <v>-17.76</v>
       </c>
       <c r="J49" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K49" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B50" s="20" t="n">
@@ -2458,7 +2460,7 @@
       </c>
       <c r="C50" s="21" t="inlineStr">
         <is>
-          <t>에코프로</t>
+          <t>SK텔레콤</t>
         </is>
       </c>
       <c r="D50" s="20" t="n">
@@ -2474,26 +2476,26 @@
         <v>0</v>
       </c>
       <c r="H50" s="24" t="n">
-        <v>-6.47</v>
+        <v>-0.88</v>
       </c>
       <c r="I50" s="24" t="n">
-        <v>-17.76</v>
+        <v>-4.53</v>
       </c>
       <c r="J50" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K50" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B51" s="20" t="n">
@@ -2501,7 +2503,7 @@
       </c>
       <c r="C51" s="21" t="inlineStr">
         <is>
-          <t>심텍</t>
+          <t>카카오게임즈</t>
         </is>
       </c>
       <c r="D51" s="20" t="n">
@@ -2517,26 +2519,26 @@
         <v>0</v>
       </c>
       <c r="H51" s="24" t="n">
-        <v>-1.11</v>
-      </c>
-      <c r="I51" s="22" t="n">
-        <v>0.4</v>
+        <v>-9.41</v>
+      </c>
+      <c r="I51" s="24" t="n">
+        <v>-21.34</v>
       </c>
       <c r="J51" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K51" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B52" s="20" t="n">
@@ -2544,7 +2546,7 @@
       </c>
       <c r="C52" s="21" t="inlineStr">
         <is>
-          <t>SK텔레콤</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="D52" s="20" t="n">
@@ -2560,26 +2562,24 @@
         <v>0</v>
       </c>
       <c r="H52" s="24" t="n">
-        <v>-0.88</v>
+        <v>-5.68</v>
       </c>
       <c r="I52" s="24" t="n">
-        <v>-4.53</v>
+        <v>-12.71</v>
       </c>
       <c r="J52" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K52" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K52" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B53" s="20" t="n">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="C53" s="21" t="inlineStr">
         <is>
-          <t>카카오게임즈</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D53" s="20" t="n">
@@ -2602,27 +2602,27 @@
       <c r="G53" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="24" t="n">
-        <v>-9.41</v>
-      </c>
-      <c r="I53" s="24" t="n">
-        <v>-21.34</v>
+      <c r="H53" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I53" s="20" t="n">
+        <v/>
       </c>
       <c r="J53" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K53" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B54" s="20" t="n">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="C54" s="21" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="D54" s="20" t="n">
@@ -2653,60 +2653,60 @@
       </c>
       <c r="J54" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K54" s="23" t="inlineStr">
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K54" s="23" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="25" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B55" s="25" t="n">
+        <v>42</v>
+      </c>
+      <c r="C55" s="26" t="inlineStr">
+        <is>
+          <t>프로브잇</t>
+        </is>
+      </c>
+      <c r="D55" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E55" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F55" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="27" t="n">
+        <v>-40</v>
+      </c>
+      <c r="I55" s="27" t="n">
+        <v>-98.53</v>
+      </c>
+      <c r="J55" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +1980%</t>
+        </is>
+      </c>
+      <c r="K55" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
-      </c>
-    </row>
-    <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="20" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B55" s="20" t="n">
-        <v>42</v>
-      </c>
-      <c r="C55" s="21" t="inlineStr">
-        <is>
-          <t>조선</t>
-        </is>
-      </c>
-      <c r="D55" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E55" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F55" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G55" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H55" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I55" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J55" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K55" s="23" t="n">
-        <v/>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>프로브잇</t>
+          <t>NPX</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2730,14 +2730,14 @@
         <v>0</v>
       </c>
       <c r="H56" s="27" t="n">
-        <v>-40</v>
+        <v>-97.41</v>
       </c>
       <c r="I56" s="27" t="n">
-        <v>-98.53</v>
+        <v>-97.41</v>
       </c>
       <c r="J56" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1853%</t>
+          <t>네이버 검색 당일 +1112%</t>
         </is>
       </c>
       <c r="K56" s="28" t="inlineStr">
@@ -2749,7 +2749,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>노블엠앤비</t>
+          <t>남화산업</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2772,15 +2772,15 @@
       <c r="G57" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H57" s="27" t="n">
-        <v>-7.69</v>
-      </c>
-      <c r="I57" s="27" t="n">
-        <v>-97.08</v>
+      <c r="H57" s="29" t="n">
+        <v>29.97</v>
+      </c>
+      <c r="I57" s="29" t="n">
+        <v>30.84</v>
       </c>
       <c r="J57" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +714%</t>
+          <t>네이버 검색 당일 +858%</t>
         </is>
       </c>
       <c r="K57" s="28" t="inlineStr">
@@ -2792,7 +2792,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>서암기계공업</t>
+          <t>노블엠앤비</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2815,15 +2815,15 @@
       <c r="G58" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="29" t="n">
-        <v>3.72</v>
-      </c>
-      <c r="I58" s="29" t="n">
-        <v>1.52</v>
+      <c r="H58" s="27" t="n">
+        <v>-7.69</v>
+      </c>
+      <c r="I58" s="27" t="n">
+        <v>-97.08</v>
       </c>
       <c r="J58" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +600%</t>
+          <t>네이버 검색 당일 +783%</t>
         </is>
       </c>
       <c r="K58" s="28" t="inlineStr">
@@ -2835,7 +2835,7 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>남화산업</t>
+          <t>삼기에너지솔루션즈</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2858,15 +2858,15 @@
       <c r="G59" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H59" s="29" t="n">
-        <v>29.97</v>
+      <c r="H59" s="27" t="n">
+        <v>-18.39</v>
       </c>
       <c r="I59" s="29" t="n">
-        <v>30.84</v>
+        <v>21.26</v>
       </c>
       <c r="J59" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +548%</t>
+          <t>네이버 검색 당일 +770%</t>
         </is>
       </c>
       <c r="K59" s="28" t="inlineStr">
@@ -2878,7 +2878,7 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>바이온</t>
+          <t>서암기계공업</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2901,15 +2901,15 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="27" t="n">
-        <v>-50</v>
-      </c>
-      <c r="I60" s="27" t="n">
-        <v>-98.84</v>
+      <c r="H60" s="29" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="I60" s="29" t="n">
+        <v>1.52</v>
       </c>
       <c r="J60" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +473%</t>
+          <t>네이버 검색 당일 +748%</t>
         </is>
       </c>
       <c r="K60" s="28" t="inlineStr">
@@ -2921,7 +2921,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>조아제약</t>
+          <t>바이온</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2944,15 +2944,15 @@
       <c r="G61" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H61" s="29" t="n">
-        <v>4.55</v>
-      </c>
-      <c r="I61" s="29" t="n">
-        <v>44.97</v>
+      <c r="H61" s="27" t="n">
+        <v>-50</v>
+      </c>
+      <c r="I61" s="27" t="n">
+        <v>-98.84</v>
       </c>
       <c r="J61" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +410%</t>
+          <t>네이버 검색 당일 +545%</t>
         </is>
       </c>
       <c r="K61" s="28" t="inlineStr">
@@ -2964,7 +2964,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2972,7 +2972,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>삼기에너지솔루션즈</t>
+          <t>디와이에이</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2987,15 +2987,15 @@
       <c r="G62" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H62" s="27" t="n">
-        <v>-18.39</v>
+      <c r="H62" s="29" t="n">
+        <v>25.79</v>
       </c>
       <c r="I62" s="29" t="n">
-        <v>21.26</v>
+        <v>31.47</v>
       </c>
       <c r="J62" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +398%</t>
+          <t>네이버 검색 당일 +495%</t>
         </is>
       </c>
       <c r="K62" s="28" t="inlineStr">
@@ -3007,7 +3007,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3015,7 +3015,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>보해양조</t>
+          <t>조아제약</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3030,15 +3030,15 @@
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="27" t="n">
-        <v>-15.91</v>
+      <c r="H63" s="29" t="n">
+        <v>4.55</v>
       </c>
       <c r="I63" s="29" t="n">
-        <v>9.15</v>
+        <v>44.97</v>
       </c>
       <c r="J63" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +354%</t>
+          <t>네이버 검색 당일 +475%</t>
         </is>
       </c>
       <c r="K63" s="28" t="inlineStr">
@@ -3140,22 +3140,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3181,12 +3181,12 @@
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H4" s="27" t="n">
@@ -3206,22 +3206,22 @@
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H5" s="27" t="n">
@@ -3241,22 +3241,22 @@
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H6" s="27" t="n">
@@ -3286,12 +3286,12 @@
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H7" s="27" t="n">
@@ -3304,29 +3304,29 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H8" s="25" t="n"/>
@@ -3335,29 +3335,29 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H9" s="25" t="n"/>
@@ -3366,68 +3366,68 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>파두</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="H10" s="27" t="n">
-        <v>-5.14</v>
-      </c>
-      <c r="I10" s="27" t="n">
-        <v>-18.15</v>
-      </c>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="H10" s="25" t="n"/>
+      <c r="I10" s="25" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="H11" s="25" t="n"/>
-      <c r="I11" s="25" t="n"/>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="H11" s="27" t="n">
+        <v>-2.31</v>
+      </c>
+      <c r="I11" s="27" t="n">
+        <v>-18.69</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
@@ -3439,22 +3439,22 @@
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H12" s="27" t="n">
@@ -3467,7 +3467,7 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>LG이노텍</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -3484,60 +3484,60 @@
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H13" s="27" t="n">
-        <v>-2.31</v>
+        <v>-3.21</v>
       </c>
       <c r="I13" s="27" t="n">
-        <v>-18.69</v>
+        <v>-12.19</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="H14" s="27" t="n">
-        <v>-3.21</v>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="H14" s="29" t="n">
+        <v>0.52</v>
       </c>
       <c r="I14" s="27" t="n">
-        <v>-12.19</v>
+        <v>-24.25</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>파두</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -3554,25 +3554,25 @@
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="H15" s="29" t="n">
-        <v>0.52</v>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="H15" s="27" t="n">
+        <v>-5.14</v>
       </c>
       <c r="I15" s="27" t="n">
-        <v>-24.25</v>
+        <v>-18.15</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>페니트리움바이오</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -3589,196 +3589,196 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H16" s="27" t="n">
-        <v>-8.76</v>
+        <v>-2.96</v>
       </c>
       <c r="I16" s="27" t="n">
-        <v>-31.49</v>
+        <v>-11.93</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>페니트리움바이오</t>
+          <t>다스코</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E17" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H17" s="27" t="n">
-        <v>-2.96</v>
+        <v>-16.32</v>
       </c>
       <c r="I17" s="27" t="n">
-        <v>-11.93</v>
+        <v>-1.01</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>한미반도체</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E18" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="H18" s="27" t="n">
-        <v>-5.68</v>
-      </c>
-      <c r="I18" s="27" t="n">
-        <v>-12.71</v>
-      </c>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="H18" s="25" t="n"/>
+      <c r="I18" s="25" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>KB금융</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="H19" s="25" t="n"/>
-      <c r="I19" s="25" t="n"/>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="H19" s="27" t="n">
+        <v>-1.71</v>
+      </c>
+      <c r="I19" s="27" t="n">
+        <v>-5.69</v>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>소룩스</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D20" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H20" s="27" t="n">
-        <v>-4.21</v>
-      </c>
-      <c r="I20" s="29" t="n">
-        <v>19.47</v>
+        <v>-3.5</v>
+      </c>
+      <c r="I20" s="27" t="n">
+        <v>-7.38</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>원익IPS</t>
+          <t>광주신세계</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D21" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E21" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H21" s="29" t="n">
-        <v>5.88</v>
+        <v>29.98</v>
       </c>
       <c r="I21" s="29" t="n">
-        <v>5</v>
+        <v>50.71</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>KB금융</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -3795,25 +3795,25 @@
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H22" s="27" t="n">
-        <v>-1.71</v>
+        <v>-8.41</v>
       </c>
       <c r="I22" s="27" t="n">
-        <v>-5.69</v>
+        <v>-14.4</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3830,25 +3830,25 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H23" s="27" t="n">
-        <v>-3.5</v>
-      </c>
-      <c r="I23" s="27" t="n">
-        <v>-7.38</v>
+        <v>-3.61</v>
+      </c>
+      <c r="I23" s="29" t="n">
+        <v>0.36</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>삼성물산</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3865,21 +3865,25 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="H24" s="25" t="n"/>
-      <c r="I24" s="25" t="n"/>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="H24" s="27" t="n">
+        <v>-4.72</v>
+      </c>
+      <c r="I24" s="29" t="n">
+        <v>0.61</v>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>광주신세계</t>
+          <t>삼호개발</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3896,25 +3900,25 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H25" s="29" t="n">
-        <v>29.98</v>
+        <v>8.69</v>
       </c>
       <c r="I25" s="29" t="n">
-        <v>50.71</v>
+        <v>16.77</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>다스코</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
@@ -3931,25 +3935,25 @@
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H26" s="27" t="n">
-        <v>-16.32</v>
+        <v>-8.76</v>
       </c>
       <c r="I26" s="27" t="n">
-        <v>-1.01</v>
+        <v>-31.49</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>카카오뱅크</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
@@ -3966,25 +3970,25 @@
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H27" s="27" t="n">
-        <v>-8.41</v>
+        <v>-3.42</v>
       </c>
       <c r="I27" s="27" t="n">
-        <v>-14.4</v>
+        <v>-10.84</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>헝셩그룹</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
@@ -4001,25 +4005,25 @@
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H28" s="27" t="n">
-        <v>-3.61</v>
+        <v>-2.71</v>
       </c>
       <c r="I28" s="29" t="n">
-        <v>0.36</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>에이팩트</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
@@ -4036,161 +4040,165 @@
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H29" s="27" t="n">
-        <v>-6.74</v>
+        <v>-4.47</v>
       </c>
       <c r="I29" s="27" t="n">
-        <v>-26.62</v>
+        <v>-21.62</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>리가켐바이오</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C30" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D30" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E30" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="H30" s="25" t="n"/>
-      <c r="I30" s="25" t="n"/>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="H30" s="27" t="n">
+        <v>-8.279999999999999</v>
+      </c>
+      <c r="I30" s="29" t="n">
+        <v>6.17</v>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>카카오뱅크</t>
+          <t>소룩스</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C31" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D31" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E31" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H31" s="27" t="n">
-        <v>-3.42</v>
-      </c>
-      <c r="I31" s="27" t="n">
-        <v>-10.84</v>
+        <v>-4.21</v>
+      </c>
+      <c r="I31" s="29" t="n">
+        <v>19.47</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>리가켐바이오</t>
+          <t>SK텔레콤</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C32" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D32" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E32" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H32" s="27" t="n">
-        <v>-8.279999999999999</v>
-      </c>
-      <c r="I32" s="29" t="n">
-        <v>6.17</v>
+        <v>-0.88</v>
+      </c>
+      <c r="I32" s="27" t="n">
+        <v>-4.53</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>차바이오텍</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C33" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D33" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E33" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="H33" s="27" t="n">
-        <v>-4.12</v>
-      </c>
-      <c r="I33" s="27" t="n">
-        <v>-12.15</v>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="H33" s="29" t="n">
+        <v>30</v>
+      </c>
+      <c r="I33" s="29" t="n">
+        <v>57.86</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>SK텔레콤</t>
+          <t>남화토건</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4207,25 +4215,25 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="H34" s="27" t="n">
-        <v>-0.88</v>
-      </c>
-      <c r="I34" s="27" t="n">
-        <v>-4.53</v>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="H34" s="29" t="n">
+        <v>29.96</v>
+      </c>
+      <c r="I34" s="29" t="n">
+        <v>28.96</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>뉴인텍</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -4242,25 +4250,25 @@
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H35" s="29" t="n">
-        <v>30</v>
+        <v>29.93</v>
       </c>
       <c r="I35" s="29" t="n">
-        <v>57.86</v>
+        <v>47.06</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>베셀</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
@@ -4277,21 +4285,25 @@
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="H36" s="25" t="n"/>
-      <c r="I36" s="25" t="n"/>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="H36" s="29" t="n">
+        <v>9.69</v>
+      </c>
+      <c r="I36" s="29" t="n">
+        <v>34.27</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>베셀</t>
+          <t>에코프로</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
@@ -4308,25 +4320,25 @@
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="H37" s="29" t="n">
-        <v>9.69</v>
-      </c>
-      <c r="I37" s="29" t="n">
-        <v>34.27</v>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="H37" s="27" t="n">
+        <v>-6.47</v>
+      </c>
+      <c r="I37" s="27" t="n">
+        <v>-17.76</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>시너지이노베이션</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4343,25 +4355,21 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="H38" s="27" t="n">
-        <v>-1.93</v>
-      </c>
-      <c r="I38" s="27" t="n">
-        <v>-7.84</v>
-      </c>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="H38" s="25" t="n"/>
+      <c r="I38" s="25" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>심텍</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4378,25 +4386,21 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="H39" s="27" t="n">
-        <v>-1.11</v>
-      </c>
-      <c r="I39" s="29" t="n">
-        <v>0.4</v>
-      </c>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="H39" s="25" t="n"/>
+      <c r="I39" s="25" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>에코프로</t>
+          <t>카카오게임즈</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4413,25 +4417,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H40" s="27" t="n">
-        <v>-6.47</v>
+        <v>-9.41</v>
       </c>
       <c r="I40" s="27" t="n">
-        <v>-17.76</v>
+        <v>-21.34</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>크리스탈신소재</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4448,21 +4452,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="H41" s="25" t="n"/>
-      <c r="I41" s="25" t="n"/>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="H41" s="29" t="n">
+        <v>18.81</v>
+      </c>
+      <c r="I41" s="27" t="n">
+        <v>-28.03</v>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>카카오게임즈</t>
+          <t>티이엠씨씨엔에스</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4479,25 +4487,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="H42" s="27" t="n">
-        <v>-9.41</v>
-      </c>
-      <c r="I42" s="27" t="n">
-        <v>-21.34</v>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="H42" s="29" t="n">
+        <v>30</v>
+      </c>
+      <c r="I42" s="29" t="n">
+        <v>10.36</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>크리스탈신소재</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4514,54 +4522,54 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="H43" s="29" t="n">
-        <v>18.81</v>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="H43" s="27" t="n">
+        <v>-5.68</v>
       </c>
       <c r="I43" s="27" t="n">
-        <v>-28.03</v>
+        <v>-12.71</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>헝셩그룹</t>
+          <t>NPX</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C44" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D44" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E44" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H44" s="27" t="n">
-        <v>-2.71</v>
-      </c>
-      <c r="I44" s="29" t="n">
-        <v>15.4</v>
+        <v>-97.41</v>
+      </c>
+      <c r="I44" s="27" t="n">
+        <v>-97.41</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
@@ -4584,12 +4592,12 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H45" s="29" t="n">
@@ -4619,12 +4627,12 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H46" s="27" t="n">
@@ -4637,7 +4645,7 @@
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>바이온</t>
+          <t>디와이에이</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4654,25 +4662,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="H47" s="27" t="n">
-        <v>-50</v>
-      </c>
-      <c r="I47" s="27" t="n">
-        <v>-98.84</v>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="H47" s="29" t="n">
+        <v>25.79</v>
+      </c>
+      <c r="I47" s="29" t="n">
+        <v>31.47</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>보해양조</t>
+          <t>바이온</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4689,19 +4697,19 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H48" s="27" t="n">
-        <v>-15.91</v>
-      </c>
-      <c r="I48" s="29" t="n">
-        <v>9.15</v>
+        <v>-50</v>
+      </c>
+      <c r="I48" s="27" t="n">
+        <v>-98.84</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
@@ -4724,12 +4732,12 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H49" s="27" t="n">
@@ -4759,12 +4767,12 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H50" s="29" t="n">
@@ -4794,12 +4802,12 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H51" s="29" t="n">
@@ -4829,12 +4837,12 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="H52" s="27" t="n">
@@ -4925,19 +4933,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4956,19 +4964,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4987,19 +4995,19 @@
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5011,26 +5019,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5042,26 +5050,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5073,26 +5081,26 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5104,26 +5112,26 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B9" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5133,71 +5141,63 @@
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="35" t="inlineStr">
-        <is>
-          <t>제약</t>
-        </is>
-      </c>
-      <c r="B10" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" s="36" t="n">
-        <v>6</v>
-      </c>
-      <c r="D10" s="36" t="n">
-        <v>6</v>
-      </c>
-      <c r="E10" s="36" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="F10" s="37" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="G10" s="37" t="inlineStr">
-        <is>
-          <t>⚡ 관심</t>
-        </is>
-      </c>
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>이차전지</t>
+        </is>
+      </c>
+      <c r="B10" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" s="28" t="inlineStr">
+        <is>
+          <t>감지 없음</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="35" t="inlineStr">
-        <is>
-          <t>인공지능</t>
-        </is>
-      </c>
-      <c r="B11" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" s="36" t="n">
-        <v>19</v>
-      </c>
-      <c r="D11" s="36" t="n">
-        <v>19</v>
-      </c>
-      <c r="E11" s="36" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="F11" s="37" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="G11" s="37" t="inlineStr">
-        <is>
-          <t>⚡ 관심</t>
-        </is>
-      </c>
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>AI반도체</t>
+        </is>
+      </c>
+      <c r="B11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F11" s="28" t="inlineStr">
+        <is>
+          <t>감지 없음</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>이차전지</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
@@ -5224,7 +5224,7 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -5251,7 +5251,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5278,7 +5278,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5305,7 +5305,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-06-29 07:09 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-06-28 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-06-29 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-06-28) 상위: 반도체  점수 104.0점</t>
+          <t>⚡ 최신(2026-06-29) 상위: 반도체  점수 101.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-06-28) 상위: SK  점수 50.0점</t>
+          <t>⚡ 최신(2026-06-29) 상위: SK  점수 44.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-06-28) 상위: SK하이닉스  점수 35.0점</t>
+          <t>⚡ 최신(2026-06-29) 상위: 바이오  점수 39.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -971,10 +971,10 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -990,7 +990,7 @@
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1010,14 +1010,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1025,27 +1025,27 @@
       <c r="G16" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="18" t="n">
-        <v>-8.359999999999999</v>
-      </c>
-      <c r="I16" s="18" t="n">
-        <v>-3.29</v>
+      <c r="H16" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I16" s="15" t="n">
+        <v/>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>Google 급상승 검색어 등장 (KR) / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, Google</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1057,10 +1057,10 @@
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
@@ -1088,7 +1088,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1096,14 +1096,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1112,24 +1112,26 @@
         <v>0</v>
       </c>
       <c r="H18" s="18" t="n">
-        <v>-0.8</v>
+        <v>-8.359999999999999</v>
       </c>
       <c r="I18" s="18" t="n">
-        <v>-9.460000000000001</v>
+        <v>-3.29</v>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K18" s="17" t="n">
-        <v/>
+          <t>중요공시 1건 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K18" s="17" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1141,10 +1143,10 @@
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1160,7 +1162,7 @@
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K19" s="17" t="inlineStr">
@@ -1172,7 +1174,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1180,14 +1182,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1195,27 +1197,25 @@
       <c r="G20" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="15" t="n">
+      <c r="H20" s="18" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="I20" s="18" t="n">
+        <v>-9.460000000000001</v>
+      </c>
+      <c r="J20" s="17" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K20" s="17" t="n">
         <v/>
-      </c>
-      <c r="I20" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J20" s="17" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K20" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1227,10 +1227,10 @@
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
@@ -1246,7 +1246,7 @@
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
@@ -1258,7 +1258,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1266,42 +1266,42 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>젠큐릭스</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G22" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H22" s="18" t="n">
-        <v>-1.9</v>
-      </c>
-      <c r="I22" s="18" t="n">
-        <v>-12.13</v>
+        <v>0</v>
+      </c>
+      <c r="H22" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I22" s="15" t="n">
+        <v/>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 7일 +200% / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1309,14 +1309,14 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>LG이노텍</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F23" s="15" t="n">
         <v>0</v>
@@ -1324,15 +1324,15 @@
       <c r="G23" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="18" t="n">
-        <v>-2.31</v>
-      </c>
-      <c r="I23" s="18" t="n">
-        <v>-18.69</v>
+      <c r="H23" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I23" s="15" t="n">
+        <v/>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K23" s="17" t="n">
@@ -1342,7 +1342,7 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1350,40 +1350,42 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>젠큐릭스</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
         <v>9</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G24" s="15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H24" s="18" t="n">
-        <v>-3.21</v>
+        <v>-1.9</v>
       </c>
       <c r="I24" s="18" t="n">
-        <v>-12.19</v>
+        <v>-12.13</v>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K24" s="17" t="n">
-        <v/>
+          <t>중요공시 3건 / 중요공시 7일 +200% / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K24" s="17" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1391,42 +1393,40 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="F25" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G25" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H25" s="19" t="n">
-        <v>0.52</v>
+        <v>0</v>
+      </c>
+      <c r="H25" s="18" t="n">
+        <v>-2.31</v>
       </c>
       <c r="I25" s="18" t="n">
-        <v>-24.25</v>
+        <v>-18.69</v>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +50%</t>
-        </is>
-      </c>
-      <c r="K25" s="17" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K25" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1434,7 +1434,7 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>파두</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
@@ -1449,15 +1449,15 @@
       <c r="G26" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="H26" s="18" t="n">
-        <v>-5.14</v>
+      <c r="H26" s="19" t="n">
+        <v>0.52</v>
       </c>
       <c r="I26" s="18" t="n">
-        <v>-18.15</v>
+        <v>-24.25</v>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +50%</t>
+          <t>중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +200%</t>
         </is>
       </c>
       <c r="K26" s="17" t="inlineStr">
@@ -1467,136 +1467,136 @@
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="15" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="B27" s="15" t="n">
+      <c r="A27" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B27" s="20" t="n">
         <v>14</v>
       </c>
-      <c r="C27" s="16" t="inlineStr">
-        <is>
-          <t>페니트리움바이오</t>
-        </is>
-      </c>
-      <c r="D27" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="E27" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="F27" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="G27" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H27" s="18" t="n">
-        <v>-2.96</v>
-      </c>
-      <c r="I27" s="18" t="n">
-        <v>-11.93</v>
-      </c>
-      <c r="J27" s="17" t="inlineStr">
-        <is>
-          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +50%</t>
-        </is>
-      </c>
-      <c r="K27" s="17" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C27" s="21" t="inlineStr">
+        <is>
+          <t>삼호개발</t>
+        </is>
+      </c>
+      <c r="D27" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E27" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F27" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="22" t="n">
+        <v>8.69</v>
+      </c>
+      <c r="I27" s="22" t="n">
+        <v>16.77</v>
+      </c>
+      <c r="J27" s="23" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +171% / 중요공시 3건</t>
+        </is>
+      </c>
+      <c r="K27" s="23" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="15" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="B28" s="15" t="n">
+      <c r="A28" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="C28" s="16" t="inlineStr">
-        <is>
-          <t>다스코</t>
-        </is>
-      </c>
-      <c r="D28" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E28" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F28" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="18" t="n">
-        <v>-16.32</v>
-      </c>
-      <c r="I28" s="18" t="n">
-        <v>-1.01</v>
-      </c>
-      <c r="J28" s="17" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +134% / 중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K28" s="17" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
+      <c r="C28" s="21" t="inlineStr">
+        <is>
+          <t>샤페론</t>
+        </is>
+      </c>
+      <c r="D28" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E28" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F28" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="24" t="n">
+        <v>-25.16</v>
+      </c>
+      <c r="I28" s="24" t="n">
+        <v>-56.14</v>
+      </c>
+      <c r="J28" s="23" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +61% / 중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K28" s="23" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="15" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="B29" s="15" t="n">
+      <c r="A29" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B29" s="20" t="n">
         <v>16</v>
       </c>
-      <c r="C29" s="16" t="inlineStr">
-        <is>
-          <t>전기차</t>
-        </is>
-      </c>
-      <c r="D29" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E29" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F29" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I29" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J29" s="17" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K29" s="17" t="n">
+      <c r="C29" s="21" t="inlineStr">
+        <is>
+          <t>LG전자</t>
+        </is>
+      </c>
+      <c r="D29" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E29" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F29" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="24" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="I29" s="24" t="n">
+        <v>-7.38</v>
+      </c>
+      <c r="J29" s="23" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K29" s="23" t="n">
         <v/>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
@@ -1604,42 +1604,42 @@
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>광주신세계</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="D30" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E30" s="20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F30" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G30" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="22" t="n">
-        <v>29.98</v>
-      </c>
-      <c r="I30" s="22" t="n">
-        <v>50.71</v>
+        <v>3</v>
+      </c>
+      <c r="H30" s="24" t="n">
+        <v>-8.41</v>
+      </c>
+      <c r="I30" s="24" t="n">
+        <v>-14.4</v>
       </c>
       <c r="J30" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1339% / 매일경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K30" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1647,42 +1647,42 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>헝셩그룹</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F31" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G31" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H31" s="24" t="n">
-        <v>-2.71</v>
-      </c>
-      <c r="I31" s="22" t="n">
-        <v>15.4</v>
+        <v>-8.76</v>
+      </c>
+      <c r="I31" s="24" t="n">
+        <v>-31.49</v>
       </c>
       <c r="J31" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +291% / 중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>중요공시 5건 / 중요공시 7일 +67%</t>
         </is>
       </c>
       <c r="K31" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1690,42 +1690,42 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>삼호개발</t>
+          <t>차바이오텍</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F32" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G32" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H32" s="22" t="n">
-        <v>8.69</v>
-      </c>
-      <c r="I32" s="22" t="n">
-        <v>16.77</v>
+      <c r="H32" s="24" t="n">
+        <v>-4.12</v>
+      </c>
+      <c r="I32" s="24" t="n">
+        <v>-12.15</v>
       </c>
       <c r="J32" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +132% / 중요공시 3건</t>
+          <t>중요공시 4건 / 중요공시 3일 +300% / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K32" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1733,40 +1733,42 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>에이팩트</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F33" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G33" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H33" s="24" t="n">
-        <v>-3.5</v>
+        <v>-6.74</v>
       </c>
       <c r="I33" s="24" t="n">
-        <v>-7.38</v>
+        <v>-26.62</v>
       </c>
       <c r="J33" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K33" s="23" t="n">
-        <v/>
+          <t>중요공시 3건 / 중요공시 7일 +200%</t>
+        </is>
+      </c>
+      <c r="K33" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1774,30 +1776,30 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>페니트리움바이오</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F34" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G34" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H34" s="24" t="n">
-        <v>-3.61</v>
-      </c>
-      <c r="I34" s="22" t="n">
-        <v>0.36</v>
+        <v>-2.96</v>
+      </c>
+      <c r="I34" s="24" t="n">
+        <v>-11.93</v>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 3건 / 중요공시 7일 +200%</t>
         </is>
       </c>
       <c r="K34" s="23" t="inlineStr">
@@ -1809,7 +1811,7 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1817,42 +1819,42 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>삼성바이오로직스</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F35" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G35" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H35" s="24" t="n">
-        <v>-8.41</v>
+        <v>-3.1</v>
       </c>
       <c r="I35" s="24" t="n">
-        <v>-14.4</v>
+        <v>-2.26</v>
       </c>
       <c r="J35" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+          <t>중요공시 1건 / Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K35" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>공시, Google</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1860,42 +1862,42 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>오텍</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F36" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G36" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H36" s="24" t="n">
-        <v>-8.76</v>
-      </c>
-      <c r="I36" s="24" t="n">
-        <v>-31.49</v>
+        <v>0</v>
+      </c>
+      <c r="H36" s="22" t="n">
+        <v>13.75</v>
+      </c>
+      <c r="I36" s="22" t="n">
+        <v>32.47</v>
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>중요공시 5건 / 중요공시 7일 +150%</t>
+          <t>네이버 검색 당일 +88% / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K36" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1903,14 +1905,14 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>KB금융</t>
+          <t>소룩스</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E37" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F37" s="20" t="n">
         <v>0</v>
@@ -1919,26 +1921,26 @@
         <v>0</v>
       </c>
       <c r="H37" s="24" t="n">
-        <v>-1.71</v>
-      </c>
-      <c r="I37" s="24" t="n">
-        <v>-5.69</v>
+        <v>-4.21</v>
+      </c>
+      <c r="I37" s="22" t="n">
+        <v>19.47</v>
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>네이버 검색 당일 +84% / 중요공시 3건</t>
         </is>
       </c>
       <c r="K37" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1946,30 +1948,30 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>카카오뱅크</t>
+          <t>에이프릴바이오</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F38" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H38" s="24" t="n">
-        <v>-3.42</v>
-      </c>
-      <c r="I38" s="24" t="n">
-        <v>-10.84</v>
+        <v>-0.13</v>
+      </c>
+      <c r="I38" s="22" t="n">
+        <v>1.72</v>
       </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 5건 / 중요공시 3일 +400%</t>
         </is>
       </c>
       <c r="K38" s="23" t="inlineStr">
@@ -1981,7 +1983,7 @@
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1989,40 +1991,42 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>파두</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F39" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G39" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H39" s="24" t="n">
-        <v>-4.72</v>
-      </c>
-      <c r="I39" s="22" t="n">
-        <v>0.61</v>
+        <v>-5.14</v>
+      </c>
+      <c r="I39" s="24" t="n">
+        <v>-18.15</v>
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K39" s="23" t="n">
-        <v/>
+          <t>중요공시 3건 / 중요공시 3일 +200%</t>
+        </is>
+      </c>
+      <c r="K39" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2030,14 +2034,14 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>리가켐바이오</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F40" s="20" t="n">
         <v>0</v>
@@ -2046,26 +2050,26 @@
         <v>0</v>
       </c>
       <c r="H40" s="24" t="n">
-        <v>-4.47</v>
-      </c>
-      <c r="I40" s="24" t="n">
-        <v>-21.62</v>
+        <v>-8.279999999999999</v>
+      </c>
+      <c r="I40" s="22" t="n">
+        <v>6.17</v>
       </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K40" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2073,7 +2077,7 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>소룩스</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
@@ -2089,26 +2093,26 @@
         <v>0</v>
       </c>
       <c r="H41" s="24" t="n">
-        <v>-4.21</v>
-      </c>
-      <c r="I41" s="22" t="n">
-        <v>19.47</v>
+        <v>-2.67</v>
+      </c>
+      <c r="I41" s="24" t="n">
+        <v>-11.52</v>
       </c>
       <c r="J41" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +76% / 중요공시 3건</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K41" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2116,7 +2120,7 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>리가켐바이오</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
@@ -2132,26 +2136,26 @@
         <v>0</v>
       </c>
       <c r="H42" s="24" t="n">
-        <v>-8.279999999999999</v>
-      </c>
-      <c r="I42" s="22" t="n">
-        <v>6.17</v>
+        <v>-3.21</v>
+      </c>
+      <c r="I42" s="24" t="n">
+        <v>-12.19</v>
       </c>
       <c r="J42" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K42" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2159,14 +2163,14 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E43" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F43" s="20" t="n">
         <v>0</v>
@@ -2174,27 +2178,27 @@
       <c r="G43" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H43" s="22" t="n">
-        <v>30</v>
-      </c>
-      <c r="I43" s="22" t="n">
-        <v>57.86</v>
+      <c r="H43" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I43" s="20" t="n">
+        <v/>
       </c>
       <c r="J43" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +348% / 중요공시 1건</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K43" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2202,14 +2206,14 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>크리스탈신소재</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E44" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F44" s="20" t="n">
         <v>0</v>
@@ -2217,27 +2221,25 @@
       <c r="G44" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="22" t="n">
-        <v>18.81</v>
-      </c>
-      <c r="I44" s="24" t="n">
-        <v>-28.03</v>
+      <c r="H44" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I44" s="20" t="n">
+        <v/>
       </c>
       <c r="J44" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +317% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K44" s="23" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K44" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2245,7 +2247,7 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>티이엠씨씨엔에스</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
@@ -2264,23 +2266,23 @@
         <v>30</v>
       </c>
       <c r="I45" s="22" t="n">
-        <v>10.36</v>
+        <v>57.86</v>
       </c>
       <c r="J45" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +273% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +397% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K45" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
@@ -2288,7 +2290,7 @@
       </c>
       <c r="C46" s="21" t="inlineStr">
         <is>
-          <t>베셀</t>
+          <t>티이엠씨씨엔에스</t>
         </is>
       </c>
       <c r="D46" s="20" t="n">
@@ -2304,26 +2306,26 @@
         <v>0</v>
       </c>
       <c r="H46" s="22" t="n">
-        <v>9.69</v>
+        <v>30</v>
       </c>
       <c r="I46" s="22" t="n">
-        <v>34.27</v>
+        <v>10.36</v>
       </c>
       <c r="J46" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +222% / 중요공시 2건</t>
+          <t>네이버 검색 당일 +388% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K46" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B47" s="20" t="n">
@@ -2331,7 +2333,7 @@
       </c>
       <c r="C47" s="21" t="inlineStr">
         <is>
-          <t>남화토건</t>
+          <t>크리스탈신소재</t>
         </is>
       </c>
       <c r="D47" s="20" t="n">
@@ -2347,26 +2349,26 @@
         <v>0</v>
       </c>
       <c r="H47" s="22" t="n">
-        <v>29.96</v>
-      </c>
-      <c r="I47" s="22" t="n">
-        <v>28.96</v>
+        <v>18.81</v>
+      </c>
+      <c r="I47" s="24" t="n">
+        <v>-28.03</v>
       </c>
       <c r="J47" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +162% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +336% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K47" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B48" s="20" t="n">
@@ -2374,7 +2376,7 @@
       </c>
       <c r="C48" s="21" t="inlineStr">
         <is>
-          <t>뉴인텍</t>
+          <t>헝셩그룹</t>
         </is>
       </c>
       <c r="D48" s="20" t="n">
@@ -2389,27 +2391,27 @@
       <c r="G48" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H48" s="22" t="n">
-        <v>29.93</v>
+      <c r="H48" s="24" t="n">
+        <v>-2.71</v>
       </c>
       <c r="I48" s="22" t="n">
-        <v>47.06</v>
+        <v>15.4</v>
       </c>
       <c r="J48" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +144% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +299% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K48" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B49" s="20" t="n">
@@ -2417,7 +2419,7 @@
       </c>
       <c r="C49" s="21" t="inlineStr">
         <is>
-          <t>에코프로</t>
+          <t>베셀</t>
         </is>
       </c>
       <c r="D49" s="20" t="n">
@@ -2432,27 +2434,27 @@
       <c r="G49" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="24" t="n">
-        <v>-6.47</v>
-      </c>
-      <c r="I49" s="24" t="n">
-        <v>-17.76</v>
+      <c r="H49" s="22" t="n">
+        <v>9.69</v>
+      </c>
+      <c r="I49" s="22" t="n">
+        <v>34.27</v>
       </c>
       <c r="J49" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버 검색 당일 +235% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K49" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B50" s="20" t="n">
@@ -2460,7 +2462,7 @@
       </c>
       <c r="C50" s="21" t="inlineStr">
         <is>
-          <t>SK텔레콤</t>
+          <t>남화토건</t>
         </is>
       </c>
       <c r="D50" s="20" t="n">
@@ -2475,27 +2477,27 @@
       <c r="G50" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H50" s="24" t="n">
-        <v>-0.88</v>
-      </c>
-      <c r="I50" s="24" t="n">
-        <v>-4.53</v>
+      <c r="H50" s="22" t="n">
+        <v>29.96</v>
+      </c>
+      <c r="I50" s="22" t="n">
+        <v>28.96</v>
       </c>
       <c r="J50" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +181% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K50" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B51" s="20" t="n">
@@ -2503,7 +2505,7 @@
       </c>
       <c r="C51" s="21" t="inlineStr">
         <is>
-          <t>카카오게임즈</t>
+          <t>뉴인텍</t>
         </is>
       </c>
       <c r="D51" s="20" t="n">
@@ -2518,27 +2520,27 @@
       <c r="G51" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H51" s="24" t="n">
-        <v>-9.41</v>
-      </c>
-      <c r="I51" s="24" t="n">
-        <v>-21.34</v>
+      <c r="H51" s="22" t="n">
+        <v>29.93</v>
+      </c>
+      <c r="I51" s="22" t="n">
+        <v>47.06</v>
       </c>
       <c r="J51" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +165% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K51" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B52" s="20" t="n">
@@ -2546,7 +2548,7 @@
       </c>
       <c r="C52" s="21" t="inlineStr">
         <is>
-          <t>한미반도체</t>
+          <t>다스코</t>
         </is>
       </c>
       <c r="D52" s="20" t="n">
@@ -2562,24 +2564,26 @@
         <v>0</v>
       </c>
       <c r="H52" s="24" t="n">
-        <v>-5.68</v>
+        <v>-16.32</v>
       </c>
       <c r="I52" s="24" t="n">
-        <v>-12.71</v>
+        <v>-1.01</v>
       </c>
       <c r="J52" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K52" s="23" t="n">
-        <v/>
+          <t>네이버 검색 당일 +146% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K52" s="23" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B53" s="20" t="n">
@@ -2587,7 +2591,7 @@
       </c>
       <c r="C53" s="21" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>남광토건</t>
         </is>
       </c>
       <c r="D53" s="20" t="n">
@@ -2602,27 +2606,27 @@
       <c r="G53" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I53" s="20" t="n">
-        <v/>
+      <c r="H53" s="22" t="n">
+        <v>6.41</v>
+      </c>
+      <c r="I53" s="22" t="n">
+        <v>5.06</v>
       </c>
       <c r="J53" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>중요공시 3건</t>
         </is>
       </c>
       <c r="K53" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B54" s="20" t="n">
@@ -2630,7 +2634,7 @@
       </c>
       <c r="C54" s="21" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>SK텔레콤</t>
         </is>
       </c>
       <c r="D54" s="20" t="n">
@@ -2645,240 +2649,238 @@
       <c r="G54" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H54" s="20" t="n">
+      <c r="H54" s="24" t="n">
+        <v>-0.88</v>
+      </c>
+      <c r="I54" s="24" t="n">
+        <v>-4.53</v>
+      </c>
+      <c r="J54" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K54" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B55" s="20" t="n">
+        <v>42</v>
+      </c>
+      <c r="C55" s="21" t="inlineStr">
+        <is>
+          <t>카카오게임즈</t>
+        </is>
+      </c>
+      <c r="D55" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E55" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F55" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="24" t="n">
+        <v>-9.41</v>
+      </c>
+      <c r="I55" s="24" t="n">
+        <v>-21.34</v>
+      </c>
+      <c r="J55" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K55" s="23" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B56" s="20" t="n">
+        <v>43</v>
+      </c>
+      <c r="C56" s="21" t="inlineStr">
+        <is>
+          <t>셀트리온</t>
+        </is>
+      </c>
+      <c r="D56" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E56" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F56" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="24" t="n">
+        <v>-4.16</v>
+      </c>
+      <c r="I56" s="24" t="n">
+        <v>-2.58</v>
+      </c>
+      <c r="J56" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K56" s="23" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B57" s="20" t="n">
+        <v>44</v>
+      </c>
+      <c r="C57" s="21" t="inlineStr">
+        <is>
+          <t>게임</t>
+        </is>
+      </c>
+      <c r="D57" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E57" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F57" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" s="20" t="n">
         <v/>
       </c>
-      <c r="I54" s="20" t="n">
+      <c r="I57" s="20" t="n">
         <v/>
       </c>
-      <c r="J54" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K54" s="23" t="n">
+      <c r="J57" s="23" t="inlineStr">
+        <is>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K57" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B58" s="20" t="n">
+        <v>45</v>
+      </c>
+      <c r="C58" s="21" t="inlineStr">
+        <is>
+          <t>한미반도체</t>
+        </is>
+      </c>
+      <c r="D58" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E58" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F58" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" s="24" t="n">
+        <v>-5.68</v>
+      </c>
+      <c r="I58" s="24" t="n">
+        <v>-12.71</v>
+      </c>
+      <c r="J58" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K58" s="23" t="n">
         <v/>
       </c>
     </row>
-    <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="25" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="B55" s="25" t="n">
-        <v>42</v>
-      </c>
-      <c r="C55" s="26" t="inlineStr">
-        <is>
-          <t>프로브잇</t>
-        </is>
-      </c>
-      <c r="D55" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E55" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F55" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G55" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H55" s="27" t="n">
-        <v>-40</v>
-      </c>
-      <c r="I55" s="27" t="n">
-        <v>-98.53</v>
-      </c>
-      <c r="J55" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +1980%</t>
-        </is>
-      </c>
-      <c r="K55" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="18" customHeight="1">
-      <c r="A56" s="25" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="B56" s="25" t="n">
-        <v>43</v>
-      </c>
-      <c r="C56" s="26" t="inlineStr">
-        <is>
-          <t>NPX</t>
-        </is>
-      </c>
-      <c r="D56" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E56" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F56" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G56" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H56" s="27" t="n">
-        <v>-97.41</v>
-      </c>
-      <c r="I56" s="27" t="n">
-        <v>-97.41</v>
-      </c>
-      <c r="J56" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +1112%</t>
-        </is>
-      </c>
-      <c r="K56" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="25" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="B57" s="25" t="n">
-        <v>44</v>
-      </c>
-      <c r="C57" s="26" t="inlineStr">
-        <is>
-          <t>남화산업</t>
-        </is>
-      </c>
-      <c r="D57" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E57" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F57" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G57" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H57" s="29" t="n">
-        <v>29.97</v>
-      </c>
-      <c r="I57" s="29" t="n">
-        <v>30.84</v>
-      </c>
-      <c r="J57" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +858%</t>
-        </is>
-      </c>
-      <c r="K57" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="25" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="B58" s="25" t="n">
-        <v>45</v>
-      </c>
-      <c r="C58" s="26" t="inlineStr">
-        <is>
-          <t>노블엠앤비</t>
-        </is>
-      </c>
-      <c r="D58" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E58" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F58" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G58" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H58" s="27" t="n">
-        <v>-7.69</v>
-      </c>
-      <c r="I58" s="27" t="n">
-        <v>-97.08</v>
-      </c>
-      <c r="J58" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +783%</t>
-        </is>
-      </c>
-      <c r="K58" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
     <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="25" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="B59" s="25" t="n">
+      <c r="A59" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B59" s="20" t="n">
         <v>46</v>
       </c>
-      <c r="C59" s="26" t="inlineStr">
-        <is>
-          <t>삼기에너지솔루션즈</t>
-        </is>
-      </c>
-      <c r="D59" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E59" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F59" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G59" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H59" s="27" t="n">
-        <v>-18.39</v>
-      </c>
-      <c r="I59" s="29" t="n">
-        <v>21.26</v>
-      </c>
-      <c r="J59" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +770%</t>
-        </is>
-      </c>
-      <c r="K59" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+      <c r="C59" s="21" t="inlineStr">
+        <is>
+          <t>전기차</t>
+        </is>
+      </c>
+      <c r="D59" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E59" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F59" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I59" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J59" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K59" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2886,7 +2888,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>서암기계공업</t>
+          <t>프로브잇</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2901,15 +2903,15 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="29" t="n">
-        <v>3.72</v>
-      </c>
-      <c r="I60" s="29" t="n">
-        <v>1.52</v>
+      <c r="H60" s="27" t="n">
+        <v>-40</v>
+      </c>
+      <c r="I60" s="27" t="n">
+        <v>-98.53</v>
       </c>
       <c r="J60" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +748%</t>
+          <t>네이버 검색 당일 +2008%</t>
         </is>
       </c>
       <c r="K60" s="28" t="inlineStr">
@@ -2921,7 +2923,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2929,7 +2931,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>바이온</t>
+          <t>광주신세계</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2944,15 +2946,15 @@
       <c r="G61" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H61" s="27" t="n">
-        <v>-50</v>
-      </c>
-      <c r="I61" s="27" t="n">
-        <v>-98.84</v>
+      <c r="H61" s="29" t="n">
+        <v>29.98</v>
+      </c>
+      <c r="I61" s="29" t="n">
+        <v>50.71</v>
       </c>
       <c r="J61" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +545%</t>
+          <t>네이버 검색 당일 +1484%</t>
         </is>
       </c>
       <c r="K61" s="28" t="inlineStr">
@@ -2964,7 +2966,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2972,7 +2974,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>디와이에이</t>
+          <t>NPX</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2987,15 +2989,15 @@
       <c r="G62" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H62" s="29" t="n">
-        <v>25.79</v>
-      </c>
-      <c r="I62" s="29" t="n">
-        <v>31.47</v>
+      <c r="H62" s="27" t="n">
+        <v>-97.41</v>
+      </c>
+      <c r="I62" s="27" t="n">
+        <v>-97.41</v>
       </c>
       <c r="J62" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +495%</t>
+          <t>네이버 검색 당일 +1237%</t>
         </is>
       </c>
       <c r="K62" s="28" t="inlineStr">
@@ -3007,7 +3009,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3015,7 +3017,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>조아제약</t>
+          <t>남화산업</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3031,14 +3033,14 @@
         <v>0</v>
       </c>
       <c r="H63" s="29" t="n">
-        <v>4.55</v>
+        <v>29.97</v>
       </c>
       <c r="I63" s="29" t="n">
-        <v>44.97</v>
+        <v>30.84</v>
       </c>
       <c r="J63" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +475%</t>
+          <t>네이버 검색 당일 +931%</t>
         </is>
       </c>
       <c r="K63" s="28" t="inlineStr">
@@ -3140,22 +3142,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3171,22 +3173,22 @@
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H4" s="27" t="n">
@@ -3199,37 +3201,33 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H5" s="27" t="n">
-        <v>-8.359999999999999</v>
-      </c>
-      <c r="I5" s="27" t="n">
-        <v>-3.29</v>
-      </c>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H5" s="25" t="n"/>
+      <c r="I5" s="25" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
@@ -3241,22 +3239,22 @@
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H6" s="27" t="n">
@@ -3269,36 +3267,36 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H7" s="27" t="n">
-        <v>-0.8</v>
+        <v>-8.359999999999999</v>
       </c>
       <c r="I7" s="27" t="n">
-        <v>-9.460000000000001</v>
+        <v>-3.29</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
@@ -3311,22 +3309,22 @@
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H8" s="25" t="n"/>
@@ -3335,33 +3333,37 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H9" s="25" t="n"/>
-      <c r="I9" s="25" t="n"/>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H9" s="27" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="I9" s="27" t="n">
+        <v>-9.460000000000001</v>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
@@ -3373,22 +3375,22 @@
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H10" s="25" t="n"/>
@@ -3397,77 +3399,69 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>LG이노텍</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H11" s="27" t="n">
-        <v>-2.31</v>
-      </c>
-      <c r="I11" s="27" t="n">
-        <v>-18.69</v>
-      </c>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H11" s="25" t="n"/>
+      <c r="I11" s="25" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>젠큐릭스</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H12" s="27" t="n">
-        <v>-1.9</v>
-      </c>
-      <c r="I12" s="27" t="n">
-        <v>-12.13</v>
-      </c>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H12" s="25" t="n"/>
+      <c r="I12" s="25" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -3484,60 +3478,60 @@
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H13" s="27" t="n">
-        <v>-3.21</v>
+        <v>-2.31</v>
       </c>
       <c r="I13" s="27" t="n">
-        <v>-12.19</v>
+        <v>-18.69</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>젠큐릭스</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H14" s="29" t="n">
-        <v>0.52</v>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H14" s="27" t="n">
+        <v>-1.9</v>
       </c>
       <c r="I14" s="27" t="n">
-        <v>-24.25</v>
+        <v>-12.13</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>파두</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -3554,126 +3548,130 @@
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H15" s="27" t="n">
-        <v>-5.14</v>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H15" s="29" t="n">
+        <v>0.52</v>
       </c>
       <c r="I15" s="27" t="n">
-        <v>-18.15</v>
+        <v>-24.25</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>페니트리움바이오</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C16" s="25" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D16" s="25" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E16" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H16" s="27" t="n">
-        <v>-2.96</v>
+        <v>-3.5</v>
       </c>
       <c r="I16" s="27" t="n">
-        <v>-11.93</v>
+        <v>-7.38</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>다스코</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E17" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H17" s="27" t="n">
-        <v>-16.32</v>
+        <v>-8.41</v>
       </c>
       <c r="I17" s="27" t="n">
-        <v>-1.01</v>
+        <v>-14.4</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>삼성바이오로직스</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E18" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H18" s="25" t="n"/>
-      <c r="I18" s="25" t="n"/>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H18" s="27" t="n">
+        <v>-3.1</v>
+      </c>
+      <c r="I18" s="27" t="n">
+        <v>-2.26</v>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>KB금융</t>
+          <t>삼호개발</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -3690,25 +3688,25 @@
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H19" s="27" t="n">
-        <v>-1.71</v>
-      </c>
-      <c r="I19" s="27" t="n">
-        <v>-5.69</v>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H19" s="29" t="n">
+        <v>8.69</v>
+      </c>
+      <c r="I19" s="29" t="n">
+        <v>16.77</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>샤페론</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
@@ -3725,25 +3723,25 @@
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H20" s="27" t="n">
-        <v>-3.5</v>
+        <v>-25.16</v>
       </c>
       <c r="I20" s="27" t="n">
-        <v>-7.38</v>
+        <v>-56.14</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>광주신세계</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -3760,25 +3758,25 @@
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H21" s="29" t="n">
-        <v>29.98</v>
-      </c>
-      <c r="I21" s="29" t="n">
-        <v>50.71</v>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H21" s="27" t="n">
+        <v>-8.76</v>
+      </c>
+      <c r="I21" s="27" t="n">
+        <v>-31.49</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>에이팩트</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -3795,25 +3793,25 @@
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H22" s="27" t="n">
-        <v>-8.41</v>
+        <v>-6.74</v>
       </c>
       <c r="I22" s="27" t="n">
-        <v>-14.4</v>
+        <v>-26.62</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>차바이오텍</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3830,25 +3828,25 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H23" s="27" t="n">
-        <v>-3.61</v>
-      </c>
-      <c r="I23" s="29" t="n">
-        <v>0.36</v>
+        <v>-4.12</v>
+      </c>
+      <c r="I23" s="27" t="n">
+        <v>-12.15</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>페니트리움바이오</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3865,200 +3863,200 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H24" s="27" t="n">
-        <v>-4.72</v>
-      </c>
-      <c r="I24" s="29" t="n">
-        <v>0.61</v>
+        <v>-2.96</v>
+      </c>
+      <c r="I24" s="27" t="n">
+        <v>-11.93</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>삼호개발</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C25" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D25" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E25" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H25" s="29" t="n">
-        <v>8.69</v>
-      </c>
-      <c r="I25" s="29" t="n">
-        <v>16.77</v>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H25" s="27" t="n">
+        <v>-2.67</v>
+      </c>
+      <c r="I25" s="27" t="n">
+        <v>-11.52</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>리가켐바이오</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C26" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D26" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E26" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H26" s="27" t="n">
-        <v>-8.76</v>
-      </c>
-      <c r="I26" s="27" t="n">
-        <v>-31.49</v>
+        <v>-8.279999999999999</v>
+      </c>
+      <c r="I26" s="29" t="n">
+        <v>6.17</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>카카오뱅크</t>
+          <t>소룩스</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C27" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D27" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E27" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H27" s="27" t="n">
-        <v>-3.42</v>
-      </c>
-      <c r="I27" s="27" t="n">
-        <v>-10.84</v>
+        <v>-4.21</v>
+      </c>
+      <c r="I27" s="29" t="n">
+        <v>19.47</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>헝셩그룹</t>
+          <t>에이프릴바이오</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C28" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D28" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E28" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H28" s="27" t="n">
-        <v>-2.71</v>
+        <v>-0.13</v>
       </c>
       <c r="I28" s="29" t="n">
-        <v>15.4</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>오텍</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C29" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D29" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E29" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H29" s="27" t="n">
-        <v>-4.47</v>
-      </c>
-      <c r="I29" s="27" t="n">
-        <v>-21.62</v>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H29" s="29" t="n">
+        <v>13.75</v>
+      </c>
+      <c r="I29" s="29" t="n">
+        <v>32.47</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>리가켐바이오</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -4075,25 +4073,21 @@
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H30" s="27" t="n">
-        <v>-8.279999999999999</v>
-      </c>
-      <c r="I30" s="29" t="n">
-        <v>6.17</v>
-      </c>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H30" s="25" t="n"/>
+      <c r="I30" s="25" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>소룩스</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
@@ -4110,95 +4104,91 @@
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H31" s="27" t="n">
-        <v>-4.21</v>
-      </c>
-      <c r="I31" s="29" t="n">
-        <v>19.47</v>
+        <v>-3.21</v>
+      </c>
+      <c r="I31" s="27" t="n">
+        <v>-12.19</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>SK텔레콤</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C32" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D32" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E32" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H32" s="27" t="n">
-        <v>-0.88</v>
-      </c>
-      <c r="I32" s="27" t="n">
-        <v>-4.53</v>
-      </c>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H32" s="25" t="n"/>
+      <c r="I32" s="25" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>파두</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C33" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D33" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E33" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H33" s="29" t="n">
-        <v>30</v>
-      </c>
-      <c r="I33" s="29" t="n">
-        <v>57.86</v>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H33" s="27" t="n">
+        <v>-5.14</v>
+      </c>
+      <c r="I33" s="27" t="n">
+        <v>-18.15</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>남화토건</t>
+          <t>SK텔레콤</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4215,25 +4205,25 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H34" s="29" t="n">
-        <v>29.96</v>
-      </c>
-      <c r="I34" s="29" t="n">
-        <v>28.96</v>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H34" s="27" t="n">
+        <v>-0.88</v>
+      </c>
+      <c r="I34" s="27" t="n">
+        <v>-4.53</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>뉴인텍</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -4250,25 +4240,21 @@
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H35" s="29" t="n">
-        <v>29.93</v>
-      </c>
-      <c r="I35" s="29" t="n">
-        <v>47.06</v>
-      </c>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H35" s="25" t="n"/>
+      <c r="I35" s="25" t="n"/>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>베셀</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
@@ -4285,25 +4271,25 @@
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H36" s="29" t="n">
-        <v>9.69</v>
+        <v>30</v>
       </c>
       <c r="I36" s="29" t="n">
-        <v>34.27</v>
+        <v>57.86</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>에코프로</t>
+          <t>남광토건</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
@@ -4320,25 +4306,25 @@
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H37" s="27" t="n">
-        <v>-6.47</v>
-      </c>
-      <c r="I37" s="27" t="n">
-        <v>-17.76</v>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H37" s="29" t="n">
+        <v>6.41</v>
+      </c>
+      <c r="I37" s="29" t="n">
+        <v>5.06</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>남화토건</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4355,21 +4341,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H38" s="25" t="n"/>
-      <c r="I38" s="25" t="n"/>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H38" s="29" t="n">
+        <v>29.96</v>
+      </c>
+      <c r="I38" s="29" t="n">
+        <v>28.96</v>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>뉴인텍</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4386,21 +4376,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H39" s="25" t="n"/>
-      <c r="I39" s="25" t="n"/>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H39" s="29" t="n">
+        <v>29.93</v>
+      </c>
+      <c r="I39" s="29" t="n">
+        <v>47.06</v>
+      </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>카카오게임즈</t>
+          <t>다스코</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4417,25 +4411,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H40" s="27" t="n">
-        <v>-9.41</v>
+        <v>-16.32</v>
       </c>
       <c r="I40" s="27" t="n">
-        <v>-21.34</v>
+        <v>-1.01</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>크리스탈신소재</t>
+          <t>베셀</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4452,25 +4446,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H41" s="29" t="n">
-        <v>18.81</v>
-      </c>
-      <c r="I41" s="27" t="n">
-        <v>-28.03</v>
+        <v>9.69</v>
+      </c>
+      <c r="I41" s="29" t="n">
+        <v>34.27</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>티이엠씨씨엔에스</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4487,25 +4481,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H42" s="29" t="n">
-        <v>30</v>
-      </c>
-      <c r="I42" s="29" t="n">
-        <v>10.36</v>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H42" s="27" t="n">
+        <v>-4.16</v>
+      </c>
+      <c r="I42" s="27" t="n">
+        <v>-2.58</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>한미반도체</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4522,200 +4516,196 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H43" s="27" t="n">
-        <v>-5.68</v>
-      </c>
-      <c r="I43" s="27" t="n">
-        <v>-12.71</v>
-      </c>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H43" s="25" t="n"/>
+      <c r="I43" s="25" t="n"/>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>NPX</t>
+          <t>카카오게임즈</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C44" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D44" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E44" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H44" s="27" t="n">
-        <v>-97.41</v>
+        <v>-9.41</v>
       </c>
       <c r="I44" s="27" t="n">
-        <v>-97.41</v>
+        <v>-21.34</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>남화산업</t>
+          <t>크리스탈신소재</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C45" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D45" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E45" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H45" s="29" t="n">
-        <v>29.97</v>
-      </c>
-      <c r="I45" s="29" t="n">
-        <v>30.84</v>
+        <v>18.81</v>
+      </c>
+      <c r="I45" s="27" t="n">
+        <v>-28.03</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>노블엠앤비</t>
+          <t>티이엠씨씨엔에스</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C46" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D46" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E46" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H46" s="27" t="n">
-        <v>-7.69</v>
-      </c>
-      <c r="I46" s="27" t="n">
-        <v>-97.08</v>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H46" s="29" t="n">
+        <v>30</v>
+      </c>
+      <c r="I46" s="29" t="n">
+        <v>10.36</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>디와이에이</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C47" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D47" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E47" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="H47" s="29" t="n">
-        <v>25.79</v>
-      </c>
-      <c r="I47" s="29" t="n">
-        <v>31.47</v>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H47" s="27" t="n">
+        <v>-5.68</v>
+      </c>
+      <c r="I47" s="27" t="n">
+        <v>-12.71</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>바이온</t>
+          <t>헝셩그룹</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C48" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D48" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E48" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H48" s="27" t="n">
-        <v>-50</v>
-      </c>
-      <c r="I48" s="27" t="n">
-        <v>-98.84</v>
+        <v>-2.71</v>
+      </c>
+      <c r="I48" s="29" t="n">
+        <v>15.4</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>삼기에너지솔루션즈</t>
+          <t>NPX</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4732,25 +4722,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H49" s="27" t="n">
-        <v>-18.39</v>
-      </c>
-      <c r="I49" s="29" t="n">
-        <v>21.26</v>
+        <v>-97.41</v>
+      </c>
+      <c r="I49" s="27" t="n">
+        <v>-97.41</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>서암기계공업</t>
+          <t>광주신세계</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4767,25 +4757,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H50" s="29" t="n">
-        <v>3.72</v>
+        <v>29.98</v>
       </c>
       <c r="I50" s="29" t="n">
-        <v>1.52</v>
+        <v>50.71</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>조아제약</t>
+          <t>남화산업</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4802,19 +4792,19 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H51" s="29" t="n">
-        <v>4.55</v>
+        <v>29.97</v>
       </c>
       <c r="I51" s="29" t="n">
-        <v>44.97</v>
+        <v>30.84</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
@@ -4837,12 +4827,12 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H52" s="27" t="n">
@@ -4933,19 +4923,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4964,19 +4954,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4995,19 +4985,19 @@
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5019,26 +5009,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5050,26 +5040,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5081,26 +5071,26 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5112,119 +5102,131 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
+          <t>게임</t>
+        </is>
+      </c>
+      <c r="B9" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" s="36" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="F9" s="37" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="G9" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>조선</t>
+        </is>
+      </c>
+      <c r="B10" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" s="36" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="F10" s="37" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="G10" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>제약</t>
+        </is>
+      </c>
+      <c r="B11" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="36" t="n">
+        <v>13</v>
+      </c>
+      <c r="D11" s="36" t="n">
+        <v>13</v>
+      </c>
+      <c r="E11" s="36" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="F11" s="37" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="G11" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="35" t="inlineStr">
+        <is>
           <t>인공지능</t>
         </is>
       </c>
-      <c r="B9" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" s="36" t="n">
-        <v>18</v>
-      </c>
-      <c r="D9" s="36" t="n">
-        <v>18</v>
-      </c>
-      <c r="E9" s="36" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="F9" s="37" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="G9" s="37" t="inlineStr">
+      <c r="B12" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="36" t="n">
+        <v>21</v>
+      </c>
+      <c r="D12" s="36" t="n">
+        <v>21</v>
+      </c>
+      <c r="E12" s="36" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="F12" s="37" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="G12" s="37" t="inlineStr">
         <is>
           <t>⚡ 관심</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="26" t="inlineStr">
-        <is>
-          <t>이차전지</t>
-        </is>
-      </c>
-      <c r="B10" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" s="28" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="inlineStr"/>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="26" t="inlineStr">
-        <is>
-          <t>AI반도체</t>
-        </is>
-      </c>
-      <c r="B11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F11" s="28" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="inlineStr"/>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="26" t="inlineStr">
-        <is>
-          <t>방산</t>
-        </is>
-      </c>
-      <c r="B12" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F12" s="28" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>이차전지</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -5251,7 +5253,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5278,7 +5280,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5305,7 +5307,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-06-30 07:10 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -258,13 +258,13 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-06-29 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-06-30 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-06-29) 상위: 반도체  점수 101.0점</t>
+          <t>⚡ 최신(2026-06-30) 상위: 반도체  점수 121.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-06-29) 상위: SK  점수 44.0점</t>
+          <t>⚡ 최신(2026-06-30) 상위: SK  점수 40.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-06-29) 상위: 바이오  점수 39.0점</t>
+          <t>⚡ 최신(2026-06-30) 상위: 삼성전자  점수 30.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>101</v>
+        <v>121</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>101</v>
+        <v>121</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -971,10 +971,10 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -983,14 +983,14 @@
         <v>0</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>-5.01</v>
+        <v>-3.68</v>
       </c>
       <c r="I15" s="19" t="n">
-        <v>12.57</v>
+        <v>7.53</v>
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1010,14 +1010,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1025,27 +1025,27 @@
       <c r="G16" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I16" s="15" t="n">
-        <v/>
+      <c r="H16" s="18" t="n">
+        <v>-4.86</v>
+      </c>
+      <c r="I16" s="18" t="n">
+        <v>-8.630000000000001</v>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR) / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
         <is>
-          <t>네이버, Google</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1053,14 +1053,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1068,15 +1068,15 @@
       <c r="G17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="18" t="n">
-        <v>-5.3</v>
-      </c>
-      <c r="I17" s="18" t="n">
-        <v>-4.1</v>
+      <c r="H17" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I17" s="15" t="n">
+        <v/>
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
@@ -1088,7 +1088,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1096,14 +1096,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1111,27 +1111,27 @@
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="18" t="n">
-        <v>-8.359999999999999</v>
-      </c>
-      <c r="I18" s="18" t="n">
-        <v>-3.29</v>
+      <c r="H18" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I18" s="15" t="n">
+        <v/>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K18" s="17" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1139,14 +1139,14 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1154,15 +1154,15 @@
       <c r="G19" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I19" s="15" t="n">
-        <v/>
+      <c r="H19" s="19" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="I19" s="18" t="n">
+        <v>-8.279999999999999</v>
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K19" s="17" t="inlineStr">
@@ -1174,7 +1174,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1182,14 +1182,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1198,24 +1198,26 @@
         <v>0</v>
       </c>
       <c r="H20" s="18" t="n">
-        <v>-0.8</v>
+        <v>-1.68</v>
       </c>
       <c r="I20" s="18" t="n">
-        <v>-9.460000000000001</v>
+        <v>-9.970000000000001</v>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K20" s="17" t="n">
-        <v/>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K20" s="17" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1227,10 +1229,10 @@
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
@@ -1246,19 +1248,17 @@
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K21" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K21" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1270,10 +1270,10 @@
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="inlineStr">
@@ -1301,7 +1301,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1309,14 +1309,14 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F23" s="15" t="n">
         <v>0</v>
@@ -1332,17 +1332,19 @@
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K23" s="17" t="n">
-        <v/>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K23" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1350,42 +1352,42 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>젠큐릭스</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G24" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H24" s="18" t="n">
-        <v>-1.9</v>
+        <v>0</v>
+      </c>
+      <c r="H24" s="19" t="n">
+        <v>3.43</v>
       </c>
       <c r="I24" s="18" t="n">
-        <v>-12.13</v>
+        <v>-14.46</v>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 7일 +200% / 매일경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K24" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1393,7 +1395,7 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>LG이노텍</t>
+          <t>삼호개발</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
@@ -1409,24 +1411,26 @@
         <v>0</v>
       </c>
       <c r="H25" s="18" t="n">
-        <v>-2.31</v>
-      </c>
-      <c r="I25" s="18" t="n">
-        <v>-18.69</v>
+        <v>-2.17</v>
+      </c>
+      <c r="I25" s="19" t="n">
+        <v>17.02</v>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K25" s="17" t="n">
-        <v/>
+          <t>네이버 검색 당일 +208% / 중요공시 3건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K25" s="17" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1434,203 +1438,201 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
+          <t>LG화학</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="E26" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="F26" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="19" t="n">
+        <v>13.65</v>
+      </c>
+      <c r="I26" s="18" t="n">
+        <v>-4.64</v>
+      </c>
+      <c r="J26" s="17" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K26" s="17" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>원전</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="E27" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="F27" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I27" s="15" t="n">
+        <v/>
+      </c>
+      <c r="J27" s="17" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K27" s="17" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
           <t>성호전자</t>
         </is>
       </c>
-      <c r="D26" s="15" t="n">
+      <c r="D28" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="E26" s="15" t="n">
+      <c r="E28" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="F26" s="15" t="n">
+      <c r="F28" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="G26" s="15" t="n">
+      <c r="G28" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="H26" s="19" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="I26" s="18" t="n">
-        <v>-24.25</v>
-      </c>
-      <c r="J26" s="17" t="inlineStr">
-        <is>
-          <t>중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +200%</t>
-        </is>
-      </c>
-      <c r="K26" s="17" t="inlineStr">
+      <c r="H28" s="18" t="n">
+        <v>-1.56</v>
+      </c>
+      <c r="I28" s="18" t="n">
+        <v>-22.9</v>
+      </c>
+      <c r="J28" s="17" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +200%</t>
+        </is>
+      </c>
+      <c r="K28" s="17" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="20" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B27" s="20" t="n">
-        <v>14</v>
-      </c>
-      <c r="C27" s="21" t="inlineStr">
-        <is>
-          <t>삼호개발</t>
-        </is>
-      </c>
-      <c r="D27" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E27" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="F27" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="22" t="n">
-        <v>8.69</v>
-      </c>
-      <c r="I27" s="22" t="n">
-        <v>16.77</v>
-      </c>
-      <c r="J27" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +171% / 중요공시 3건</t>
-        </is>
-      </c>
-      <c r="K27" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="20" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B28" s="20" t="n">
-        <v>15</v>
-      </c>
-      <c r="C28" s="21" t="inlineStr">
-        <is>
-          <t>샤페론</t>
-        </is>
-      </c>
-      <c r="D28" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E28" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="F28" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="24" t="n">
-        <v>-25.16</v>
-      </c>
-      <c r="I28" s="24" t="n">
-        <v>-56.14</v>
-      </c>
-      <c r="J28" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +61% / 중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K28" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
-      </c>
-    </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="20" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B29" s="20" t="n">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="n">
         <v>16</v>
       </c>
-      <c r="C29" s="21" t="inlineStr">
-        <is>
-          <t>LG전자</t>
-        </is>
-      </c>
-      <c r="D29" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E29" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="F29" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="24" t="n">
-        <v>-3.5</v>
-      </c>
-      <c r="I29" s="24" t="n">
-        <v>-7.38</v>
-      </c>
-      <c r="J29" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K29" s="23" t="n">
-        <v/>
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>스피어</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E29" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F29" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G29" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="H29" s="19" t="n">
+        <v>17.63</v>
+      </c>
+      <c r="I29" s="18" t="n">
+        <v>-8.130000000000001</v>
+      </c>
+      <c r="J29" s="17" t="inlineStr">
+        <is>
+          <t>중요공시 7건 / 중요공시 3일 +133% / 중요공시 7일 +250%</t>
+        </is>
+      </c>
+      <c r="K29" s="17" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="20" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B30" s="20" t="n">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="n">
         <v>17</v>
       </c>
-      <c r="C30" s="21" t="inlineStr">
-        <is>
-          <t>대우건설</t>
-        </is>
-      </c>
-      <c r="D30" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E30" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F30" s="20" t="n">
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>파두</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F30" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="G30" s="20" t="n">
+      <c r="G30" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="H30" s="24" t="n">
-        <v>-8.41</v>
-      </c>
-      <c r="I30" s="24" t="n">
-        <v>-14.4</v>
-      </c>
-      <c r="J30" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K30" s="23" t="inlineStr">
+      <c r="H30" s="19" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="I30" s="18" t="n">
+        <v>-26.06</v>
+      </c>
+      <c r="J30" s="17" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +50%</t>
+        </is>
+      </c>
+      <c r="K30" s="17" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
@@ -1639,7 +1641,7 @@
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1647,42 +1649,42 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>아크솔루션스</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F31" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G31" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H31" s="24" t="n">
-        <v>-8.76</v>
-      </c>
-      <c r="I31" s="24" t="n">
-        <v>-31.49</v>
+        <v>0</v>
+      </c>
+      <c r="H31" s="22" t="n">
+        <v>-97.40000000000001</v>
+      </c>
+      <c r="I31" s="22" t="n">
+        <v>-97.40000000000001</v>
       </c>
       <c r="J31" s="23" t="inlineStr">
         <is>
-          <t>중요공시 5건 / 중요공시 7일 +67%</t>
+          <t>네이버 검색 당일 +197% / 중요공시 3건</t>
         </is>
       </c>
       <c r="K31" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1690,7 +1692,7 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>차바이오텍</t>
+          <t>뉴인텍</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
@@ -1705,27 +1707,27 @@
       <c r="G32" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H32" s="24" t="n">
-        <v>-4.12</v>
+      <c r="H32" s="22" t="n">
+        <v>-20.41</v>
       </c>
       <c r="I32" s="24" t="n">
-        <v>-12.15</v>
+        <v>17.04</v>
       </c>
       <c r="J32" s="23" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 중요공시 3일 +300% / 네이버뉴스 기사 언급</t>
+          <t>네이버 검색 당일 +181% / 중요공시 2건 / 중요공시 3일 +100%</t>
         </is>
       </c>
       <c r="K32" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1733,42 +1735,42 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>에이팩트</t>
+          <t>앱튼</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F33" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G33" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H33" s="24" t="n">
-        <v>-6.74</v>
+        <v>29.98</v>
       </c>
       <c r="I33" s="24" t="n">
-        <v>-26.62</v>
+        <v>109.15</v>
       </c>
       <c r="J33" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 7일 +200%</t>
+          <t>네이버 검색 당일 +138% / 중요공시 5건</t>
         </is>
       </c>
       <c r="K33" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1776,42 +1778,40 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>페니트리움바이오</t>
+          <t>원익IPS</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F34" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G34" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H34" s="24" t="n">
-        <v>-2.96</v>
-      </c>
-      <c r="I34" s="24" t="n">
-        <v>-11.93</v>
+        <v>0</v>
+      </c>
+      <c r="H34" s="22" t="n">
+        <v>-2.93</v>
+      </c>
+      <c r="I34" s="22" t="n">
+        <v>-7.83</v>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 7일 +200%</t>
-        </is>
-      </c>
-      <c r="K34" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K34" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1819,7 +1819,7 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>삼성바이오로직스</t>
+          <t>한화생명</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
@@ -1835,26 +1835,24 @@
         <v>0</v>
       </c>
       <c r="H35" s="24" t="n">
-        <v>-3.1</v>
-      </c>
-      <c r="I35" s="24" t="n">
-        <v>-2.26</v>
+        <v>2.71</v>
+      </c>
+      <c r="I35" s="22" t="n">
+        <v>-9.199999999999999</v>
       </c>
       <c r="J35" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / Google 급상승 검색어 등장 (KR)</t>
-        </is>
-      </c>
-      <c r="K35" s="23" t="inlineStr">
-        <is>
-          <t>공시, Google</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K35" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1862,42 +1860,42 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>오텍</t>
+          <t>차바이오텍</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F36" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G36" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H36" s="22" t="n">
-        <v>13.75</v>
-      </c>
-      <c r="I36" s="22" t="n">
-        <v>32.47</v>
+        <v>3</v>
+      </c>
+      <c r="H36" s="24" t="n">
+        <v>10.78</v>
+      </c>
+      <c r="I36" s="24" t="n">
+        <v>0.26</v>
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +88% / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>중요공시 4건 / 중요공시 7일 +300%</t>
         </is>
       </c>
       <c r="K36" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1905,42 +1903,42 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>소룩스</t>
+          <t>페니트리움바이오</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E37" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F37" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G37" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H37" s="24" t="n">
-        <v>-4.21</v>
+        <v>2.16</v>
       </c>
       <c r="I37" s="22" t="n">
-        <v>19.47</v>
+        <v>-7.21</v>
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +84% / 중요공시 3건</t>
+          <t>중요공시 3건 / 중요공시 7일 +200%</t>
         </is>
       </c>
       <c r="K37" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1948,42 +1946,40 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>에이프릴바이오</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F38" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H38" s="24" t="n">
-        <v>-0.13</v>
-      </c>
-      <c r="I38" s="22" t="n">
-        <v>1.72</v>
+      <c r="H38" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I38" s="20" t="n">
+        <v/>
       </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
-          <t>중요공시 5건 / 중요공시 3일 +400%</t>
-        </is>
-      </c>
-      <c r="K38" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K38" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1991,42 +1987,42 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>파두</t>
+          <t>소룩스</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F39" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G39" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H39" s="24" t="n">
-        <v>-5.14</v>
+      <c r="H39" s="22" t="n">
+        <v>-4.76</v>
       </c>
       <c r="I39" s="24" t="n">
-        <v>-18.15</v>
+        <v>18.99</v>
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200%</t>
+          <t>네이버 검색 당일 +92% / 중요공시 3건</t>
         </is>
       </c>
       <c r="K39" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2034,30 +2030,30 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>리가켐바이오</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F40" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G40" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H40" s="24" t="n">
-        <v>-8.279999999999999</v>
-      </c>
-      <c r="I40" s="22" t="n">
-        <v>6.17</v>
+        <v>1.07</v>
+      </c>
+      <c r="I40" s="24" t="n">
+        <v>4.81</v>
       </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 3건 / 중요공시 3일 +200%</t>
         </is>
       </c>
       <c r="K40" s="23" t="inlineStr">
@@ -2069,7 +2065,7 @@
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2077,42 +2073,42 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>남광토건</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E41" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F41" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G41" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H41" s="24" t="n">
-        <v>-2.67</v>
+        <v>2.41</v>
       </c>
       <c r="I41" s="24" t="n">
-        <v>-11.52</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="J41" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 3건 / 중요공시 3일 +50%</t>
         </is>
       </c>
       <c r="K41" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2120,7 +2116,7 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>KB금융</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
@@ -2136,26 +2132,26 @@
         <v>0</v>
       </c>
       <c r="H42" s="24" t="n">
-        <v>-3.21</v>
-      </c>
-      <c r="I42" s="24" t="n">
-        <v>-12.19</v>
+        <v>2.95</v>
+      </c>
+      <c r="I42" s="22" t="n">
+        <v>-2.1</v>
       </c>
       <c r="J42" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K42" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2163,7 +2159,7 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>채비</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
@@ -2178,27 +2174,27 @@
       <c r="G43" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H43" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I43" s="20" t="n">
-        <v/>
+      <c r="H43" s="24" t="n">
+        <v>16.69</v>
+      </c>
+      <c r="I43" s="22" t="n">
+        <v>-3.89</v>
       </c>
       <c r="J43" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K43" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2206,7 +2202,7 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
@@ -2221,25 +2217,27 @@
       <c r="G44" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I44" s="20" t="n">
-        <v/>
+      <c r="H44" s="24" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="I44" s="22" t="n">
+        <v>-7.13</v>
       </c>
       <c r="J44" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K44" s="23" t="n">
-        <v/>
+          <t>Google 급상승 검색어 등장 (KR)</t>
+        </is>
+      </c>
+      <c r="K44" s="23" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2247,14 +2245,14 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E45" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F45" s="20" t="n">
         <v>0</v>
@@ -2262,27 +2260,25 @@
       <c r="G45" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H45" s="22" t="n">
-        <v>30</v>
-      </c>
-      <c r="I45" s="22" t="n">
-        <v>57.86</v>
+      <c r="H45" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I45" s="20" t="n">
+        <v/>
       </c>
       <c r="J45" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +397% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K45" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K45" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
@@ -2290,14 +2286,14 @@
       </c>
       <c r="C46" s="21" t="inlineStr">
         <is>
-          <t>티이엠씨씨엔에스</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="D46" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E46" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F46" s="20" t="n">
         <v>0</v>
@@ -2305,27 +2301,27 @@
       <c r="G46" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H46" s="22" t="n">
-        <v>30</v>
-      </c>
-      <c r="I46" s="22" t="n">
-        <v>10.36</v>
+      <c r="H46" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I46" s="20" t="n">
+        <v/>
       </c>
       <c r="J46" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +388% / 중요공시 1건</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K46" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B47" s="20" t="n">
@@ -2333,14 +2329,14 @@
       </c>
       <c r="C47" s="21" t="inlineStr">
         <is>
-          <t>크리스탈신소재</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D47" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E47" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F47" s="20" t="n">
         <v>0</v>
@@ -2348,27 +2344,25 @@
       <c r="G47" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H47" s="22" t="n">
-        <v>18.81</v>
-      </c>
-      <c r="I47" s="24" t="n">
-        <v>-28.03</v>
+      <c r="H47" s="24" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="I47" s="22" t="n">
+        <v>-8.529999999999999</v>
       </c>
       <c r="J47" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +336% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K47" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K47" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B48" s="20" t="n">
@@ -2376,7 +2370,7 @@
       </c>
       <c r="C48" s="21" t="inlineStr">
         <is>
-          <t>헝셩그룹</t>
+          <t>티이엠씨씨엔에스</t>
         </is>
       </c>
       <c r="D48" s="20" t="n">
@@ -2391,27 +2385,27 @@
       <c r="G48" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H48" s="24" t="n">
-        <v>-2.71</v>
-      </c>
-      <c r="I48" s="22" t="n">
-        <v>15.4</v>
+      <c r="H48" s="22" t="n">
+        <v>-0.31</v>
+      </c>
+      <c r="I48" s="24" t="n">
+        <v>14.49</v>
       </c>
       <c r="J48" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +299% / 중요공시 2건</t>
+          <t>네이버 검색 당일 +524% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K48" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B49" s="20" t="n">
@@ -2434,27 +2428,27 @@
       <c r="G49" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="22" t="n">
-        <v>9.69</v>
-      </c>
-      <c r="I49" s="22" t="n">
-        <v>34.27</v>
+      <c r="H49" s="24" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="I49" s="24" t="n">
+        <v>13.91</v>
       </c>
       <c r="J49" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +235% / 중요공시 2건</t>
+          <t>네이버 검색 당일 +244% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K49" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B50" s="20" t="n">
@@ -2462,7 +2456,7 @@
       </c>
       <c r="C50" s="21" t="inlineStr">
         <is>
-          <t>남화토건</t>
+          <t>다스코</t>
         </is>
       </c>
       <c r="D50" s="20" t="n">
@@ -2477,27 +2471,27 @@
       <c r="G50" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H50" s="22" t="n">
-        <v>29.96</v>
-      </c>
-      <c r="I50" s="22" t="n">
-        <v>28.96</v>
+      <c r="H50" s="24" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="I50" s="24" t="n">
+        <v>52.65</v>
       </c>
       <c r="J50" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +181% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +159% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K50" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B51" s="20" t="n">
@@ -2505,7 +2499,7 @@
       </c>
       <c r="C51" s="21" t="inlineStr">
         <is>
-          <t>뉴인텍</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="D51" s="20" t="n">
@@ -2520,27 +2514,25 @@
       <c r="G51" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H51" s="22" t="n">
-        <v>29.93</v>
+      <c r="H51" s="24" t="n">
+        <v>8.140000000000001</v>
       </c>
       <c r="I51" s="22" t="n">
-        <v>47.06</v>
+        <v>-2.58</v>
       </c>
       <c r="J51" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +165% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K51" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K51" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B52" s="20" t="n">
@@ -2548,7 +2540,7 @@
       </c>
       <c r="C52" s="21" t="inlineStr">
         <is>
-          <t>다스코</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="D52" s="20" t="n">
@@ -2564,26 +2556,24 @@
         <v>0</v>
       </c>
       <c r="H52" s="24" t="n">
-        <v>-16.32</v>
-      </c>
-      <c r="I52" s="24" t="n">
-        <v>-1.01</v>
+        <v>0.41</v>
+      </c>
+      <c r="I52" s="22" t="n">
+        <v>-13.54</v>
       </c>
       <c r="J52" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +146% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K52" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K52" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B53" s="20" t="n">
@@ -2591,30 +2581,30 @@
       </c>
       <c r="C53" s="21" t="inlineStr">
         <is>
-          <t>남광토건</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="D53" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E53" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F53" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G53" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H53" s="22" t="n">
-        <v>6.41</v>
+        <v>3</v>
+      </c>
+      <c r="H53" s="24" t="n">
+        <v>8.91</v>
       </c>
       <c r="I53" s="22" t="n">
-        <v>5.06</v>
+        <v>-9.130000000000001</v>
       </c>
       <c r="J53" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K53" s="23" t="inlineStr">
@@ -2626,7 +2616,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B54" s="20" t="n">
@@ -2634,7 +2624,7 @@
       </c>
       <c r="C54" s="21" t="inlineStr">
         <is>
-          <t>SK텔레콤</t>
+          <t>올릭스</t>
         </is>
       </c>
       <c r="D54" s="20" t="n">
@@ -2650,14 +2640,14 @@
         <v>0</v>
       </c>
       <c r="H54" s="24" t="n">
-        <v>-0.88</v>
+        <v>24.22</v>
       </c>
       <c r="I54" s="24" t="n">
-        <v>-4.53</v>
+        <v>27.93</v>
       </c>
       <c r="J54" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K54" s="23" t="inlineStr">
@@ -2669,7 +2659,7 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B55" s="20" t="n">
@@ -2677,42 +2667,42 @@
       </c>
       <c r="C55" s="21" t="inlineStr">
         <is>
-          <t>카카오게임즈</t>
+          <t>시너지이노베이션</t>
         </is>
       </c>
       <c r="D55" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E55" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F55" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G55" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H55" s="24" t="n">
-        <v>-9.41</v>
+        <v>7.34</v>
       </c>
       <c r="I55" s="24" t="n">
-        <v>-21.34</v>
+        <v>0.06</v>
       </c>
       <c r="J55" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K55" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B56" s="20" t="n">
@@ -2720,42 +2710,42 @@
       </c>
       <c r="C56" s="21" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>모바일어플라이언스</t>
         </is>
       </c>
       <c r="D56" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E56" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F56" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G56" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H56" s="24" t="n">
-        <v>-4.16</v>
-      </c>
-      <c r="I56" s="24" t="n">
-        <v>-2.58</v>
+        <v>3</v>
+      </c>
+      <c r="H56" s="22" t="n">
+        <v>-3.64</v>
+      </c>
+      <c r="I56" s="22" t="n">
+        <v>-13.13</v>
       </c>
       <c r="J56" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K56" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B57" s="20" t="n">
@@ -2763,42 +2753,42 @@
       </c>
       <c r="C57" s="21" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>에임드바이오</t>
         </is>
       </c>
       <c r="D57" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E57" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F57" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G57" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H57" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I57" s="20" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H57" s="24" t="n">
+        <v>16.04</v>
+      </c>
+      <c r="I57" s="24" t="n">
+        <v>6.11</v>
       </c>
       <c r="J57" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K57" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B58" s="20" t="n">
@@ -2806,7 +2796,7 @@
       </c>
       <c r="C58" s="21" t="inlineStr">
         <is>
-          <t>한미반도체</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="D58" s="20" t="n">
@@ -2822,24 +2812,26 @@
         <v>0</v>
       </c>
       <c r="H58" s="24" t="n">
-        <v>-5.68</v>
-      </c>
-      <c r="I58" s="24" t="n">
-        <v>-12.71</v>
+        <v>8.890000000000001</v>
+      </c>
+      <c r="I58" s="22" t="n">
+        <v>-9.140000000000001</v>
       </c>
       <c r="J58" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K58" s="23" t="n">
-        <v/>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K58" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B59" s="20" t="n">
@@ -2847,7 +2839,7 @@
       </c>
       <c r="C59" s="21" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="D59" s="20" t="n">
@@ -2862,15 +2854,15 @@
       <c r="G59" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H59" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I59" s="20" t="n">
-        <v/>
+      <c r="H59" s="24" t="n">
+        <v>7.68</v>
+      </c>
+      <c r="I59" s="22" t="n">
+        <v>-0.44</v>
       </c>
       <c r="J59" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K59" s="23" t="n">
@@ -2878,52 +2870,50 @@
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="25" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B60" s="25" t="n">
+      <c r="A60" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B60" s="20" t="n">
         <v>47</v>
       </c>
-      <c r="C60" s="26" t="inlineStr">
-        <is>
-          <t>프로브잇</t>
-        </is>
-      </c>
-      <c r="D60" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E60" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F60" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G60" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H60" s="27" t="n">
-        <v>-40</v>
-      </c>
-      <c r="I60" s="27" t="n">
-        <v>-98.53</v>
-      </c>
-      <c r="J60" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +2008%</t>
-        </is>
-      </c>
-      <c r="K60" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+      <c r="C60" s="21" t="inlineStr">
+        <is>
+          <t>하이브</t>
+        </is>
+      </c>
+      <c r="D60" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E60" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F60" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" s="24" t="n">
+        <v>9.84</v>
+      </c>
+      <c r="I60" s="22" t="n">
+        <v>-8.31</v>
+      </c>
+      <c r="J60" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K60" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2931,7 +2921,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>광주신세계</t>
+          <t>프로브잇</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2946,15 +2936,15 @@
       <c r="G61" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H61" s="29" t="n">
-        <v>29.98</v>
-      </c>
-      <c r="I61" s="29" t="n">
-        <v>50.71</v>
+      <c r="H61" s="27" t="n">
+        <v>-44.44</v>
+      </c>
+      <c r="I61" s="27" t="n">
+        <v>-72.22</v>
       </c>
       <c r="J61" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1484%</t>
+          <t>네이버 검색 당일 +2031%</t>
         </is>
       </c>
       <c r="K61" s="28" t="inlineStr">
@@ -2966,7 +2956,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2974,7 +2964,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>NPX</t>
+          <t>광주신세계</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2990,14 +2980,14 @@
         <v>0</v>
       </c>
       <c r="H62" s="27" t="n">
-        <v>-97.41</v>
-      </c>
-      <c r="I62" s="27" t="n">
-        <v>-97.41</v>
+        <v>-4.73</v>
+      </c>
+      <c r="I62" s="29" t="n">
+        <v>44.83</v>
       </c>
       <c r="J62" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1237%</t>
+          <t>네이버 검색 당일 +1608%</t>
         </is>
       </c>
       <c r="K62" s="28" t="inlineStr">
@@ -3009,7 +2999,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3017,7 +3007,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>남화산업</t>
+          <t>NPX</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3032,15 +3022,15 @@
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="29" t="n">
-        <v>29.97</v>
-      </c>
-      <c r="I63" s="29" t="n">
-        <v>30.84</v>
+      <c r="H63" s="27" t="n">
+        <v>-49.52</v>
+      </c>
+      <c r="I63" s="27" t="n">
+        <v>-98.69</v>
       </c>
       <c r="J63" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +931%</t>
+          <t>네이버 검색 당일 +1347%</t>
         </is>
       </c>
       <c r="K63" s="28" t="inlineStr">
@@ -3142,22 +3132,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>101</v>
+        <v>121</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>101</v>
+        <v>121</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3173,196 +3163,196 @@
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H4" s="27" t="n">
-        <v>-5.01</v>
+        <v>-3.68</v>
       </c>
       <c r="I4" s="29" t="n">
-        <v>12.57</v>
+        <v>7.53</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H5" s="25" t="n"/>
-      <c r="I5" s="25" t="n"/>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H5" s="27" t="n">
+        <v>-4.86</v>
+      </c>
+      <c r="I5" s="27" t="n">
+        <v>-8.630000000000001</v>
+      </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H6" s="27" t="n">
-        <v>-5.3</v>
-      </c>
-      <c r="I6" s="27" t="n">
-        <v>-4.1</v>
-      </c>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H6" s="25" t="n"/>
+      <c r="I6" s="25" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H7" s="27" t="n">
-        <v>-8.359999999999999</v>
-      </c>
-      <c r="I7" s="27" t="n">
-        <v>-3.29</v>
-      </c>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H7" s="25" t="n"/>
+      <c r="I7" s="25" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H8" s="25" t="n"/>
-      <c r="I8" s="25" t="n"/>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H8" s="29" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="I8" s="27" t="n">
+        <v>-8.279999999999999</v>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H9" s="27" t="n">
-        <v>-0.8</v>
+        <v>-1.68</v>
       </c>
       <c r="I9" s="27" t="n">
-        <v>-9.460000000000001</v>
+        <v>-9.970000000000001</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
@@ -3375,22 +3365,22 @@
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H10" s="25" t="n"/>
@@ -3406,22 +3396,22 @@
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H11" s="25" t="n"/>
@@ -3430,29 +3420,29 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H12" s="25" t="n"/>
@@ -3461,42 +3451,42 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>LG이노텍</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H13" s="27" t="n">
-        <v>-2.31</v>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H13" s="29" t="n">
+        <v>3.43</v>
       </c>
       <c r="I13" s="27" t="n">
-        <v>-18.69</v>
+        <v>-14.46</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>젠큐릭스</t>
+          <t>LG화학</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -3513,200 +3503,196 @@
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H14" s="27" t="n">
-        <v>-1.9</v>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H14" s="29" t="n">
+        <v>13.65</v>
       </c>
       <c r="I14" s="27" t="n">
-        <v>-12.13</v>
+        <v>-4.64</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>삼호개발</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="25" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E15" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H15" s="29" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="I15" s="27" t="n">
-        <v>-24.25</v>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H15" s="27" t="n">
+        <v>-2.17</v>
+      </c>
+      <c r="I15" s="29" t="n">
+        <v>17.02</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C16" s="25" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D16" s="25" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E16" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H16" s="27" t="n">
-        <v>-3.5</v>
-      </c>
-      <c r="I16" s="27" t="n">
-        <v>-7.38</v>
-      </c>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H16" s="25" t="n"/>
+      <c r="I16" s="25" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E17" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H17" s="27" t="n">
-        <v>-8.41</v>
+        <v>-1.56</v>
       </c>
       <c r="I17" s="27" t="n">
-        <v>-14.4</v>
+        <v>-22.9</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>삼성바이오로직스</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E18" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H18" s="27" t="n">
-        <v>-3.1</v>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H18" s="29" t="n">
+        <v>17.63</v>
       </c>
       <c r="I18" s="27" t="n">
-        <v>-2.26</v>
+        <v>-8.130000000000001</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>삼호개발</t>
+          <t>파두</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H19" s="29" t="n">
-        <v>8.69</v>
-      </c>
-      <c r="I19" s="29" t="n">
-        <v>16.77</v>
+        <v>3.25</v>
+      </c>
+      <c r="I19" s="27" t="n">
+        <v>-26.06</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>샤페론</t>
+          <t>뉴인텍</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
@@ -3723,25 +3709,25 @@
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H20" s="27" t="n">
-        <v>-25.16</v>
-      </c>
-      <c r="I20" s="27" t="n">
-        <v>-56.14</v>
+        <v>-20.41</v>
+      </c>
+      <c r="I20" s="29" t="n">
+        <v>17.04</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -3758,25 +3744,21 @@
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H21" s="27" t="n">
-        <v>-8.76</v>
-      </c>
-      <c r="I21" s="27" t="n">
-        <v>-31.49</v>
-      </c>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H21" s="25" t="n"/>
+      <c r="I21" s="25" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>에이팩트</t>
+          <t>아크솔루션스</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -3793,25 +3775,25 @@
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H22" s="27" t="n">
-        <v>-6.74</v>
+        <v>-97.40000000000001</v>
       </c>
       <c r="I22" s="27" t="n">
-        <v>-26.62</v>
+        <v>-97.40000000000001</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>차바이오텍</t>
+          <t>앱튼</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3828,25 +3810,25 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H23" s="27" t="n">
-        <v>-4.12</v>
-      </c>
-      <c r="I23" s="27" t="n">
-        <v>-12.15</v>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H23" s="29" t="n">
+        <v>29.98</v>
+      </c>
+      <c r="I23" s="29" t="n">
+        <v>109.15</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>페니트리움바이오</t>
+          <t>원익IPS</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3863,130 +3845,130 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H24" s="27" t="n">
-        <v>-2.96</v>
+        <v>-2.93</v>
       </c>
       <c r="I24" s="27" t="n">
-        <v>-11.93</v>
+        <v>-7.83</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>차바이오텍</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C25" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D25" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E25" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H25" s="27" t="n">
-        <v>-2.67</v>
-      </c>
-      <c r="I25" s="27" t="n">
-        <v>-11.52</v>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H25" s="29" t="n">
+        <v>10.78</v>
+      </c>
+      <c r="I25" s="29" t="n">
+        <v>0.26</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>리가켐바이오</t>
+          <t>페니트리움바이오</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C26" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D26" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E26" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H26" s="27" t="n">
-        <v>-8.279999999999999</v>
-      </c>
-      <c r="I26" s="29" t="n">
-        <v>6.17</v>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H26" s="29" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="I26" s="27" t="n">
+        <v>-7.21</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>소룩스</t>
+          <t>한화생명</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C27" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D27" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E27" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H27" s="27" t="n">
-        <v>-4.21</v>
-      </c>
-      <c r="I27" s="29" t="n">
-        <v>19.47</v>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H27" s="29" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="I27" s="27" t="n">
+        <v>-9.199999999999999</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>에이프릴바이오</t>
+          <t>KB금융</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
@@ -4003,25 +3985,25 @@
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H28" s="27" t="n">
-        <v>-0.13</v>
-      </c>
-      <c r="I28" s="29" t="n">
-        <v>1.72</v>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H28" s="29" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="I28" s="27" t="n">
+        <v>-2.1</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>오텍</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
@@ -4038,25 +4020,25 @@
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H29" s="29" t="n">
-        <v>13.75</v>
-      </c>
-      <c r="I29" s="29" t="n">
-        <v>32.47</v>
+        <v>3.92</v>
+      </c>
+      <c r="I29" s="27" t="n">
+        <v>-7.13</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>남광토건</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -4073,21 +4055,25 @@
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H30" s="25" t="n"/>
-      <c r="I30" s="25" t="n"/>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H30" s="29" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="I30" s="29" t="n">
+        <v>9.539999999999999</v>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
@@ -4104,25 +4090,21 @@
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H31" s="27" t="n">
-        <v>-3.21</v>
-      </c>
-      <c r="I31" s="27" t="n">
-        <v>-12.19</v>
-      </c>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H31" s="25" t="n"/>
+      <c r="I31" s="25" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -4139,21 +4121,25 @@
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H32" s="25" t="n"/>
-      <c r="I32" s="25" t="n"/>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H32" s="29" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="I32" s="29" t="n">
+        <v>4.81</v>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>파두</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4170,126 +4156,126 @@
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H33" s="27" t="n">
-        <v>-5.14</v>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H33" s="29" t="n">
+        <v>2.26</v>
       </c>
       <c r="I33" s="27" t="n">
-        <v>-18.15</v>
+        <v>-8.529999999999999</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>SK텔레콤</t>
+          <t>소룩스</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C34" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D34" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E34" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H34" s="27" t="n">
-        <v>-0.88</v>
-      </c>
-      <c r="I34" s="27" t="n">
-        <v>-4.53</v>
+        <v>-4.76</v>
+      </c>
+      <c r="I34" s="29" t="n">
+        <v>18.99</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>채비</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D35" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E35" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H35" s="25" t="n"/>
-      <c r="I35" s="25" t="n"/>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H35" s="29" t="n">
+        <v>16.69</v>
+      </c>
+      <c r="I35" s="27" t="n">
+        <v>-3.89</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C36" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D36" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E36" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H36" s="29" t="n">
-        <v>30</v>
-      </c>
-      <c r="I36" s="29" t="n">
-        <v>57.86</v>
-      </c>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H36" s="25" t="n"/>
+      <c r="I36" s="25" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>남광토건</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
@@ -4306,25 +4292,25 @@
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H37" s="29" t="n">
-        <v>6.41</v>
-      </c>
-      <c r="I37" s="29" t="n">
-        <v>5.06</v>
+        <v>7.68</v>
+      </c>
+      <c r="I37" s="27" t="n">
+        <v>-0.44</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>남화토건</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4341,25 +4327,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H38" s="29" t="n">
-        <v>29.96</v>
-      </c>
-      <c r="I38" s="29" t="n">
-        <v>28.96</v>
+        <v>0.41</v>
+      </c>
+      <c r="I38" s="27" t="n">
+        <v>-13.54</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>뉴인텍</t>
+          <t>다스코</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4376,25 +4362,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H39" s="29" t="n">
-        <v>29.93</v>
+        <v>29.99</v>
       </c>
       <c r="I39" s="29" t="n">
-        <v>47.06</v>
+        <v>52.65</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>다스코</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4411,25 +4397,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H40" s="27" t="n">
-        <v>-16.32</v>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H40" s="29" t="n">
+        <v>8.91</v>
       </c>
       <c r="I40" s="27" t="n">
-        <v>-1.01</v>
+        <v>-9.130000000000001</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>베셀</t>
+          <t>모바일어플라이언스</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4446,25 +4432,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H41" s="29" t="n">
-        <v>9.69</v>
-      </c>
-      <c r="I41" s="29" t="n">
-        <v>34.27</v>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H41" s="27" t="n">
+        <v>-3.64</v>
+      </c>
+      <c r="I41" s="27" t="n">
+        <v>-13.13</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>베셀</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4481,25 +4467,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H42" s="27" t="n">
-        <v>-4.16</v>
-      </c>
-      <c r="I42" s="27" t="n">
-        <v>-2.58</v>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H42" s="29" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="I42" s="29" t="n">
+        <v>13.91</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>시너지이노베이션</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4516,21 +4502,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H43" s="25" t="n"/>
-      <c r="I43" s="25" t="n"/>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H43" s="29" t="n">
+        <v>7.34</v>
+      </c>
+      <c r="I43" s="29" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>카카오게임즈</t>
+          <t>에임드바이오</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4547,25 +4537,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H44" s="27" t="n">
-        <v>-9.41</v>
-      </c>
-      <c r="I44" s="27" t="n">
-        <v>-21.34</v>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H44" s="29" t="n">
+        <v>16.04</v>
+      </c>
+      <c r="I44" s="29" t="n">
+        <v>6.11</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>크리스탈신소재</t>
+          <t>올릭스</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4582,25 +4572,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H45" s="29" t="n">
-        <v>18.81</v>
-      </c>
-      <c r="I45" s="27" t="n">
-        <v>-28.03</v>
+        <v>24.22</v>
+      </c>
+      <c r="I45" s="29" t="n">
+        <v>27.93</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>티이엠씨씨엔에스</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4617,25 +4607,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H46" s="29" t="n">
-        <v>30</v>
-      </c>
-      <c r="I46" s="29" t="n">
-        <v>10.36</v>
+        <v>8.140000000000001</v>
+      </c>
+      <c r="I46" s="27" t="n">
+        <v>-2.58</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>한미반도체</t>
+          <t>티이엠씨씨엔에스</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4652,25 +4642,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H47" s="27" t="n">
-        <v>-5.68</v>
-      </c>
-      <c r="I47" s="27" t="n">
-        <v>-12.71</v>
+        <v>-0.31</v>
+      </c>
+      <c r="I47" s="29" t="n">
+        <v>14.49</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>헝셩그룹</t>
+          <t>하이브</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4687,60 +4677,60 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H48" s="27" t="n">
-        <v>-2.71</v>
-      </c>
-      <c r="I48" s="29" t="n">
-        <v>15.4</v>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H48" s="29" t="n">
+        <v>9.84</v>
+      </c>
+      <c r="I48" s="27" t="n">
+        <v>-8.31</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>NPX</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C49" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D49" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E49" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H49" s="27" t="n">
-        <v>-97.41</v>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H49" s="29" t="n">
+        <v>8.890000000000001</v>
       </c>
       <c r="I49" s="27" t="n">
-        <v>-97.41</v>
+        <v>-9.140000000000001</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>광주신세계</t>
+          <t>NPX</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4757,25 +4747,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H50" s="29" t="n">
-        <v>29.98</v>
-      </c>
-      <c r="I50" s="29" t="n">
-        <v>50.71</v>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H50" s="27" t="n">
+        <v>-49.52</v>
+      </c>
+      <c r="I50" s="27" t="n">
+        <v>-98.69</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>남화산업</t>
+          <t>광주신세계</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4792,19 +4782,19 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="H51" s="29" t="n">
-        <v>29.97</v>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H51" s="27" t="n">
+        <v>-4.73</v>
       </c>
       <c r="I51" s="29" t="n">
-        <v>30.84</v>
+        <v>44.83</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
@@ -4827,19 +4817,19 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H52" s="27" t="n">
-        <v>-40</v>
+        <v>-44.44</v>
       </c>
       <c r="I52" s="27" t="n">
-        <v>-98.53</v>
+        <v>-72.22</v>
       </c>
     </row>
   </sheetData>
@@ -4923,19 +4913,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>101</v>
+        <v>121</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>101</v>
+        <v>121</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4954,19 +4944,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4985,19 +4975,19 @@
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5016,19 +5006,19 @@
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5040,26 +5030,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5071,26 +5061,26 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5102,26 +5092,26 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B9" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5133,26 +5123,26 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="35" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B10" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="36" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="D10" s="36" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="E10" s="36" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F10" s="37" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G10" s="37" t="inlineStr">
@@ -5164,26 +5154,26 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="35" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B11" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="36" t="n">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="D11" s="36" t="n">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="E11" s="36" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F11" s="37" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G11" s="37" t="inlineStr">
@@ -5193,40 +5183,36 @@
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="35" t="inlineStr">
-        <is>
-          <t>인공지능</t>
-        </is>
-      </c>
-      <c r="B12" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="36" t="n">
-        <v>21</v>
-      </c>
-      <c r="D12" s="36" t="n">
-        <v>21</v>
-      </c>
-      <c r="E12" s="36" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="F12" s="37" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="G12" s="37" t="inlineStr">
-        <is>
-          <t>⚡ 관심</t>
-        </is>
-      </c>
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>이차전지</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F12" s="28" t="inlineStr">
+        <is>
+          <t>감지 없음</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>이차전지</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -5253,7 +5239,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5280,7 +5266,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5307,7 +5293,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -5334,7 +5320,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>핀테크</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -5361,7 +5347,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>핀테크</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -5388,7 +5374,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-07-05 07:16 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-07-04 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-07-05 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-04) 상위: 반도체  점수 106.0점</t>
+          <t>⚡ 최신(2026-07-05) 상위: 반도체  점수 83.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-04) 상위: SK  점수 54.0점</t>
+          <t>⚡ 최신(2026-07-05) 상위: SK  점수 53.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-04) 상위: 현대차  점수 33.0점</t>
+          <t>⚡ 최신(2026-07-05) 상위: 삼성전자  점수 28.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>106</v>
+        <v>83</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>106</v>
+        <v>83</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -971,10 +971,10 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -990,7 +990,7 @@
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1010,14 +1010,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1026,14 +1026,14 @@
         <v>0</v>
       </c>
       <c r="H16" s="18" t="n">
-        <v>2.07</v>
-      </c>
-      <c r="I16" s="18" t="n">
-        <v>2.39</v>
+        <v>8.220000000000001</v>
+      </c>
+      <c r="I16" s="19" t="n">
+        <v>-8.84</v>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
@@ -1045,7 +1045,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1057,10 +1057,10 @@
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1076,17 +1076,19 @@
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K17" s="17" t="n">
-        <v/>
+          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K17" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1094,14 +1096,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1110,14 +1112,14 @@
         <v>0</v>
       </c>
       <c r="H18" s="18" t="n">
-        <v>8.220000000000001</v>
-      </c>
-      <c r="I18" s="19" t="n">
-        <v>-8.84</v>
+        <v>2.07</v>
+      </c>
+      <c r="I18" s="18" t="n">
+        <v>2.39</v>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K18" s="17" t="inlineStr">
@@ -1129,7 +1131,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1141,10 +1143,10 @@
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1172,7 +1174,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1184,10 +1186,10 @@
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1203,17 +1205,19 @@
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K20" s="17" t="n">
-        <v/>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K20" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1225,10 +1229,10 @@
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
@@ -1244,7 +1248,7 @@
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
@@ -1256,7 +1260,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1268,10 +1272,10 @@
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -1287,7 +1291,7 @@
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="inlineStr">
@@ -1299,7 +1303,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1307,40 +1311,42 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F23" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G23" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="19" t="n">
-        <v>-1.1</v>
-      </c>
-      <c r="I23" s="18" t="n">
-        <v>2.87</v>
+      <c r="H23" s="18" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="I23" s="19" t="n">
+        <v>-0.2</v>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K23" s="17" t="n">
-        <v/>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K23" s="17" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1352,10 +1358,10 @@
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>0</v>
@@ -1371,17 +1377,19 @@
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K24" s="17" t="n">
-        <v/>
+          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K24" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1389,42 +1397,40 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>HJ중공업</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
         <v>8</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F25" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G25" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H25" s="18" t="n">
-        <v>2.05</v>
-      </c>
-      <c r="I25" s="19" t="n">
-        <v>-5.81</v>
+        <v>0</v>
+      </c>
+      <c r="H25" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I25" s="15" t="n">
+        <v/>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 중요공시 3일 +300% / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K25" s="17" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K25" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1432,42 +1438,42 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>에코프로</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F26" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G26" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I26" s="15" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H26" s="18" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="I26" s="19" t="n">
+        <v>-8.49</v>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +121% / 중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K26" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -1475,14 +1481,14 @@
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>콘텐트리중앙</t>
         </is>
       </c>
       <c r="D27" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E27" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F27" s="15" t="n">
         <v>0</v>
@@ -1490,27 +1496,27 @@
       <c r="G27" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H27" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I27" s="15" t="n">
-        <v/>
+      <c r="H27" s="19" t="n">
+        <v>-28.9</v>
+      </c>
+      <c r="I27" s="19" t="n">
+        <v>-65.13</v>
       </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>네이버 검색 당일 +66% / 중요공시 5건 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K27" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B28" s="15" t="n">
@@ -1518,30 +1524,30 @@
       </c>
       <c r="C28" s="16" t="inlineStr">
         <is>
-          <t>기아</t>
+          <t>파라다이스</t>
         </is>
       </c>
       <c r="D28" s="15" t="n">
         <v>7</v>
       </c>
       <c r="E28" s="15" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F28" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G28" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="18" t="n">
-        <v>4.68</v>
+        <v>3</v>
+      </c>
+      <c r="H28" s="19" t="n">
+        <v>-11.77</v>
       </c>
       <c r="I28" s="18" t="n">
-        <v>12.34</v>
+        <v>3.3</v>
       </c>
       <c r="J28" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K28" s="17" t="inlineStr">
@@ -1553,7 +1559,7 @@
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B29" s="15" t="n">
@@ -1561,7 +1567,7 @@
       </c>
       <c r="C29" s="16" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="D29" s="15" t="n">
@@ -1577,67 +1583,67 @@
         <v>0</v>
       </c>
       <c r="H29" s="18" t="n">
+        <v>4.68</v>
+      </c>
+      <c r="I29" s="18" t="n">
+        <v>12.34</v>
+      </c>
+      <c r="J29" s="17" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K29" s="17" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="F30" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="18" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="I29" s="19" t="n">
+      <c r="I30" s="19" t="n">
         <v>-2.46</v>
       </c>
-      <c r="J29" s="17" t="inlineStr">
+      <c r="J30" s="17" t="inlineStr">
         <is>
           <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
-      <c r="K29" s="17" t="n">
+      <c r="K30" s="17" t="n">
         <v/>
-      </c>
-    </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="20" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="B30" s="20" t="n">
-        <v>17</v>
-      </c>
-      <c r="C30" s="21" t="inlineStr">
-        <is>
-          <t>코퍼스코리아</t>
-        </is>
-      </c>
-      <c r="D30" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E30" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="F30" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="22" t="n">
-        <v>18.24</v>
-      </c>
-      <c r="I30" s="22" t="n">
-        <v>90.31999999999999</v>
-      </c>
-      <c r="J30" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +304% / 중요공시 6건</t>
-        </is>
-      </c>
-      <c r="K30" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1645,7 +1651,7 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>삼호개발</t>
+          <t>코퍼스코리아</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
@@ -1660,15 +1666,15 @@
       <c r="G31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="24" t="n">
-        <v>-13.27</v>
+      <c r="H31" s="22" t="n">
+        <v>18.24</v>
       </c>
       <c r="I31" s="22" t="n">
-        <v>2.71</v>
+        <v>90.31999999999999</v>
       </c>
       <c r="J31" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +186% / 중요공시 4건</t>
+          <t>네이버 검색 당일 +392% / 중요공시 6건</t>
         </is>
       </c>
       <c r="K31" s="23" t="inlineStr">
@@ -1680,7 +1686,7 @@
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1688,42 +1694,42 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>모바일어플라이언스</t>
+          <t>삼호개발</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F32" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G32" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H32" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" s="24" t="n">
-        <v>-22.19</v>
+      <c r="H32" s="24" t="n">
+        <v>-13.27</v>
+      </c>
+      <c r="I32" s="22" t="n">
+        <v>2.71</v>
       </c>
       <c r="J32" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +50%</t>
+          <t>네이버 검색 당일 +260% / 중요공시 4건</t>
         </is>
       </c>
       <c r="K32" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1731,40 +1737,42 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>진흥기업</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F33" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G33" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H33" s="22" t="n">
-        <v>6.48</v>
+      <c r="H33" s="24" t="n">
+        <v>-18.04</v>
       </c>
       <c r="I33" s="22" t="n">
-        <v>6.21</v>
+        <v>30</v>
       </c>
       <c r="J33" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K33" s="23" t="n">
-        <v/>
+          <t>네이버 검색 당일 +174% / 중요공시 2건 / 중요공시 3일 +100%</t>
+        </is>
+      </c>
+      <c r="K33" s="23" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1772,7 +1780,7 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>광진실업</t>
+          <t>다보링크</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
@@ -1788,26 +1796,26 @@
         <v>0</v>
       </c>
       <c r="H34" s="24" t="n">
-        <v>-10</v>
-      </c>
-      <c r="I34" s="22" t="n">
-        <v>42.16</v>
+        <v>-9.92</v>
+      </c>
+      <c r="I34" s="24" t="n">
+        <v>-36.8</v>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>중요공시 5건 / 매일경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +113% / 중요공시 3건</t>
         </is>
       </c>
       <c r="K34" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1815,7 +1823,7 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
@@ -1831,26 +1839,24 @@
         <v>0</v>
       </c>
       <c r="H35" s="22" t="n">
-        <v>3.27</v>
-      </c>
-      <c r="I35" s="24" t="n">
-        <v>-0.2</v>
+        <v>6.48</v>
+      </c>
+      <c r="I35" s="22" t="n">
+        <v>6.21</v>
       </c>
       <c r="J35" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K35" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K35" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1858,42 +1864,42 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>광진실업</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F36" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G36" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H36" s="22" t="n">
-        <v>3.96</v>
+      <c r="H36" s="24" t="n">
+        <v>-10</v>
       </c>
       <c r="I36" s="22" t="n">
-        <v>10.67</v>
+        <v>42.16</v>
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 5건 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K36" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1901,40 +1907,42 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>HJ중공업</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E37" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F37" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G37" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H37" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I37" s="20" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H37" s="22" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="I37" s="24" t="n">
+        <v>-5.81</v>
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K37" s="23" t="n">
-        <v/>
+          <t>중요공시 4건 / 중요공시 7일 +300%</t>
+        </is>
+      </c>
+      <c r="K37" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1942,7 +1950,7 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>스테이블코인</t>
+          <t>코오롱티슈진</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
@@ -1957,25 +1965,27 @@
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H38" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I38" s="20" t="n">
-        <v/>
+      <c r="H38" s="22" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="I38" s="24" t="n">
+        <v>-5.25</v>
       </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K38" s="23" t="n">
-        <v/>
+          <t>중요공시 2건 / Google 급상승 검색어 등장 (KR)</t>
+        </is>
+      </c>
+      <c r="K38" s="23" t="inlineStr">
+        <is>
+          <t>Google, 공시</t>
+        </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1983,42 +1993,40 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>에코프로</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F39" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G39" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H39" s="22" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="I39" s="24" t="n">
-        <v>-8.49</v>
+      <c r="H39" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I39" s="20" t="n">
+        <v/>
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +94% / 중요공시 2건 / 중요공시 3일 +100%</t>
-        </is>
-      </c>
-      <c r="K39" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K39" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2026,42 +2034,42 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>진흥기업</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F40" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G40" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H40" s="24" t="n">
-        <v>-18.04</v>
-      </c>
-      <c r="I40" s="22" t="n">
-        <v>30</v>
+      <c r="H40" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I40" s="20" t="n">
+        <v/>
       </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +66% / 중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>한국경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K40" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2069,7 +2077,7 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>콘텐트리중앙</t>
+          <t>모바일어플라이언스</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
@@ -2084,27 +2092,27 @@
       <c r="G41" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="24" t="n">
-        <v>-28.9</v>
+      <c r="H41" s="20" t="n">
+        <v>0</v>
       </c>
       <c r="I41" s="24" t="n">
-        <v>-65.13</v>
+        <v>-22.19</v>
       </c>
       <c r="J41" s="23" t="inlineStr">
         <is>
-          <t>중요공시 5건 / 한국경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +52% / 중요공시 3건</t>
         </is>
       </c>
       <c r="K41" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2145,7 +2153,7 @@
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2188,7 +2196,7 @@
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2219,7 +2227,7 @@
       </c>
       <c r="J44" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200%</t>
+          <t>중요공시 3건 / 중요공시 3일 +50%</t>
         </is>
       </c>
       <c r="K44" s="23" t="inlineStr">
@@ -2231,7 +2239,7 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2239,7 +2247,7 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>슈어소프트테크</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
@@ -2254,25 +2262,27 @@
       <c r="G45" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H45" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I45" s="20" t="n">
-        <v/>
+      <c r="H45" s="22" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="I45" s="22" t="n">
+        <v>5.04</v>
       </c>
       <c r="J45" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K45" s="23" t="n">
-        <v/>
+          <t>Google 급상승 검색어 등장 (KR)</t>
+        </is>
+      </c>
+      <c r="K45" s="23" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
@@ -2280,14 +2290,14 @@
       </c>
       <c r="C46" s="21" t="inlineStr">
         <is>
-          <t>골프존홀딩스</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="D46" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E46" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F46" s="20" t="n">
         <v>0</v>
@@ -2295,27 +2305,27 @@
       <c r="G46" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H46" s="22" t="n">
-        <v>0.15</v>
+      <c r="H46" s="24" t="n">
+        <v>-5.07</v>
       </c>
       <c r="I46" s="22" t="n">
-        <v>56.05</v>
+        <v>16.8</v>
       </c>
       <c r="J46" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +869% / 중요공시 1건</t>
+          <t>Google 급상승 검색어 등장 (US)</t>
         </is>
       </c>
       <c r="K46" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B47" s="20" t="n">
@@ -2323,14 +2333,14 @@
       </c>
       <c r="C47" s="21" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="D47" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E47" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F47" s="20" t="n">
         <v>0</v>
@@ -2338,27 +2348,27 @@
       <c r="G47" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H47" s="24" t="n">
-        <v>-19.01</v>
-      </c>
-      <c r="I47" s="22" t="n">
-        <v>43.29</v>
+      <c r="H47" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I47" s="20" t="n">
+        <v/>
       </c>
       <c r="J47" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +333% / 중요공시 1건</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K47" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B48" s="20" t="n">
@@ -2366,14 +2376,14 @@
       </c>
       <c r="C48" s="21" t="inlineStr">
         <is>
-          <t>금호전기</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="D48" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E48" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F48" s="20" t="n">
         <v>0</v>
@@ -2381,27 +2391,25 @@
       <c r="G48" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H48" s="24" t="n">
-        <v>-24.62</v>
-      </c>
-      <c r="I48" s="24" t="n">
-        <v>-12.31</v>
+      <c r="H48" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I48" s="20" t="n">
+        <v/>
       </c>
       <c r="J48" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +211% / 중요공시 2건</t>
-        </is>
-      </c>
-      <c r="K48" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K48" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B49" s="20" t="n">
@@ -2409,7 +2417,7 @@
       </c>
       <c r="C49" s="21" t="inlineStr">
         <is>
-          <t>신원종합개발</t>
+          <t>골프존홀딩스</t>
         </is>
       </c>
       <c r="D49" s="20" t="n">
@@ -2424,15 +2432,15 @@
       <c r="G49" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="24" t="n">
-        <v>-16.77</v>
+      <c r="H49" s="22" t="n">
+        <v>0.15</v>
       </c>
       <c r="I49" s="22" t="n">
-        <v>23.49</v>
+        <v>56.05</v>
       </c>
       <c r="J49" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +177% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +932% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K49" s="23" t="inlineStr">
@@ -2444,7 +2452,7 @@
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B50" s="20" t="n">
@@ -2452,7 +2460,7 @@
       </c>
       <c r="C50" s="21" t="inlineStr">
         <is>
-          <t>다보링크</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="D50" s="20" t="n">
@@ -2468,26 +2476,26 @@
         <v>0</v>
       </c>
       <c r="H50" s="24" t="n">
-        <v>-9.92</v>
-      </c>
-      <c r="I50" s="24" t="n">
-        <v>-36.8</v>
+        <v>-19.01</v>
+      </c>
+      <c r="I50" s="22" t="n">
+        <v>43.29</v>
       </c>
       <c r="J50" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>네이버 검색 당일 +417% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K50" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B51" s="20" t="n">
@@ -2495,42 +2503,42 @@
       </c>
       <c r="C51" s="21" t="inlineStr">
         <is>
-          <t>파라다이스</t>
+          <t>신원종합개발</t>
         </is>
       </c>
       <c r="D51" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E51" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F51" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G51" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H51" s="24" t="n">
-        <v>-11.77</v>
+        <v>-16.77</v>
       </c>
       <c r="I51" s="22" t="n">
-        <v>3.3</v>
+        <v>23.49</v>
       </c>
       <c r="J51" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+          <t>네이버 검색 당일 +291% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K51" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B52" s="20" t="n">
@@ -2538,7 +2546,7 @@
       </c>
       <c r="C52" s="21" t="inlineStr">
         <is>
-          <t>팸텍</t>
+          <t>금호전기</t>
         </is>
       </c>
       <c r="D52" s="20" t="n">
@@ -2553,27 +2561,27 @@
       <c r="G52" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H52" s="22" t="n">
-        <v>10.35</v>
-      </c>
-      <c r="I52" s="22" t="n">
-        <v>6.84</v>
+      <c r="H52" s="24" t="n">
+        <v>-24.62</v>
+      </c>
+      <c r="I52" s="24" t="n">
+        <v>-12.31</v>
       </c>
       <c r="J52" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +252% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K52" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B53" s="20" t="n">
@@ -2581,7 +2589,7 @@
       </c>
       <c r="C53" s="21" t="inlineStr">
         <is>
-          <t>KB금융</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D53" s="20" t="n">
@@ -2597,239 +2605,237 @@
         <v>0</v>
       </c>
       <c r="H53" s="22" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="I53" s="22" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="J53" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K53" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B54" s="20" t="n">
+        <v>41</v>
+      </c>
+      <c r="C54" s="21" t="inlineStr">
+        <is>
+          <t>DL이앤씨</t>
+        </is>
+      </c>
+      <c r="D54" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E54" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H54" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="22" t="n">
+        <v>7.36</v>
+      </c>
+      <c r="J54" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K54" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B55" s="20" t="n">
+        <v>42</v>
+      </c>
+      <c r="C55" s="21" t="inlineStr">
+        <is>
+          <t>팸텍</t>
+        </is>
+      </c>
+      <c r="D55" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E55" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F55" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="22" t="n">
+        <v>10.35</v>
+      </c>
+      <c r="I55" s="22" t="n">
+        <v>6.84</v>
+      </c>
+      <c r="J55" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K55" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B56" s="20" t="n">
+        <v>43</v>
+      </c>
+      <c r="C56" s="21" t="inlineStr">
+        <is>
+          <t>방산</t>
+        </is>
+      </c>
+      <c r="D56" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E56" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F56" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I56" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J56" s="23" t="inlineStr">
+        <is>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K56" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B57" s="20" t="n">
+        <v>44</v>
+      </c>
+      <c r="C57" s="21" t="inlineStr">
+        <is>
+          <t>KB금융</t>
+        </is>
+      </c>
+      <c r="D57" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E57" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F57" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" s="22" t="n">
         <v>3.09</v>
       </c>
-      <c r="I53" s="22" t="n">
+      <c r="I57" s="22" t="n">
         <v>13.93</v>
       </c>
-      <c r="J53" s="23" t="inlineStr">
+      <c r="J57" s="23" t="inlineStr">
         <is>
           <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
-      <c r="K53" s="23" t="n">
+      <c r="K57" s="23" t="n">
         <v/>
       </c>
     </row>
-    <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="25" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="B54" s="25" t="n">
-        <v>41</v>
-      </c>
-      <c r="C54" s="26" t="inlineStr">
-        <is>
-          <t>져스텍</t>
-        </is>
-      </c>
-      <c r="D54" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E54" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F54" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G54" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H54" s="27" t="n">
-        <v>29.96</v>
-      </c>
-      <c r="I54" s="28" t="n">
-        <v>-9.93</v>
-      </c>
-      <c r="J54" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +699%</t>
-        </is>
-      </c>
-      <c r="K54" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="25" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="B55" s="25" t="n">
-        <v>42</v>
-      </c>
-      <c r="C55" s="26" t="inlineStr">
-        <is>
-          <t>스트라드비젼</t>
-        </is>
-      </c>
-      <c r="D55" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E55" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F55" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G55" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H55" s="28" t="n">
-        <v>-0.76</v>
-      </c>
-      <c r="I55" s="28" t="n">
-        <v>-36.39</v>
-      </c>
-      <c r="J55" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +477%</t>
-        </is>
-      </c>
-      <c r="K55" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="18" customHeight="1">
-      <c r="A56" s="25" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="B56" s="25" t="n">
-        <v>43</v>
-      </c>
-      <c r="C56" s="26" t="inlineStr">
-        <is>
-          <t>에스폴리텍</t>
-        </is>
-      </c>
-      <c r="D56" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E56" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F56" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G56" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H56" s="28" t="n">
-        <v>-1.56</v>
-      </c>
-      <c r="I56" s="27" t="n">
-        <v>35.61</v>
-      </c>
-      <c r="J56" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +391%</t>
-        </is>
-      </c>
-      <c r="K56" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="25" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="B57" s="25" t="n">
-        <v>44</v>
-      </c>
-      <c r="C57" s="26" t="inlineStr">
-        <is>
-          <t>HC보광산업</t>
-        </is>
-      </c>
-      <c r="D57" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E57" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F57" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G57" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H57" s="27" t="n">
-        <v>9.039999999999999</v>
-      </c>
-      <c r="I57" s="27" t="n">
-        <v>40.38</v>
-      </c>
-      <c r="J57" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +311%</t>
-        </is>
-      </c>
-      <c r="K57" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
     <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="25" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="B58" s="25" t="n">
+      <c r="A58" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B58" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="C58" s="26" t="inlineStr">
-        <is>
-          <t>아크솔루션스</t>
-        </is>
-      </c>
-      <c r="D58" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E58" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F58" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G58" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H58" s="27" t="n">
-        <v>27.37</v>
-      </c>
-      <c r="I58" s="28" t="n">
-        <v>-97.27</v>
-      </c>
-      <c r="J58" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +280%</t>
-        </is>
-      </c>
-      <c r="K58" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+      <c r="C58" s="21" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="D58" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E58" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F58" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" s="24" t="n">
+        <v>-1.1</v>
+      </c>
+      <c r="I58" s="22" t="n">
+        <v>2.87</v>
+      </c>
+      <c r="J58" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K58" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2837,7 +2843,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>계룡건설</t>
+          <t>져스텍</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2852,15 +2858,15 @@
       <c r="G59" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H59" s="28" t="n">
-        <v>-11.43</v>
-      </c>
-      <c r="I59" s="27" t="n">
-        <v>22.78</v>
+      <c r="H59" s="27" t="n">
+        <v>29.96</v>
+      </c>
+      <c r="I59" s="28" t="n">
+        <v>-9.93</v>
       </c>
       <c r="J59" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +191%</t>
+          <t>네이버 검색 당일 +763%</t>
         </is>
       </c>
       <c r="K59" s="29" t="inlineStr">
@@ -2872,7 +2878,7 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2880,7 +2886,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>덕신이피씨</t>
+          <t>스트라드비젼</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2896,14 +2902,14 @@
         <v>0</v>
       </c>
       <c r="H60" s="28" t="n">
-        <v>-17.83</v>
-      </c>
-      <c r="I60" s="27" t="n">
-        <v>65.5</v>
+        <v>-0.76</v>
+      </c>
+      <c r="I60" s="28" t="n">
+        <v>-36.39</v>
       </c>
       <c r="J60" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +185%</t>
+          <t>네이버 검색 당일 +525%</t>
         </is>
       </c>
       <c r="K60" s="29" t="inlineStr">
@@ -2915,7 +2921,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2923,7 +2929,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>한성크린텍</t>
+          <t>에스폴리텍</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2938,15 +2944,15 @@
       <c r="G61" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H61" s="27" t="n">
-        <v>2.02</v>
+      <c r="H61" s="28" t="n">
+        <v>-1.56</v>
       </c>
       <c r="I61" s="27" t="n">
-        <v>41.96</v>
+        <v>35.61</v>
       </c>
       <c r="J61" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +168%</t>
+          <t>네이버 검색 당일 +512%</t>
         </is>
       </c>
       <c r="K61" s="29" t="inlineStr">
@@ -2958,7 +2964,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2966,7 +2972,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>우원개발</t>
+          <t>HC보광산업</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2982,14 +2988,14 @@
         <v>0</v>
       </c>
       <c r="H62" s="27" t="n">
-        <v>4.47</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="I62" s="27" t="n">
-        <v>42.99</v>
+        <v>40.38</v>
       </c>
       <c r="J62" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +134%</t>
+          <t>네이버 검색 당일 +494%</t>
         </is>
       </c>
       <c r="K62" s="29" t="inlineStr">
@@ -3001,7 +3007,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3009,7 +3015,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>아크솔루션스</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3025,19 +3031,19 @@
         <v>0</v>
       </c>
       <c r="H63" s="27" t="n">
-        <v>2.05</v>
-      </c>
-      <c r="I63" s="27" t="n">
-        <v>43.93</v>
+        <v>27.37</v>
+      </c>
+      <c r="I63" s="28" t="n">
+        <v>-97.27</v>
       </c>
       <c r="J63" s="29" t="inlineStr">
         <is>
-          <t>중요공시 5건</t>
+          <t>네이버 검색 당일 +337%</t>
         </is>
       </c>
       <c r="K63" s="29" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
@@ -3134,22 +3140,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>106</v>
+        <v>83</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>106</v>
+        <v>83</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3165,22 +3171,22 @@
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H4" s="27" t="n">
@@ -3193,36 +3199,36 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H5" s="27" t="n">
-        <v>2.07</v>
-      </c>
-      <c r="I5" s="27" t="n">
-        <v>2.39</v>
+        <v>8.220000000000001</v>
+      </c>
+      <c r="I5" s="28" t="n">
+        <v>-8.84</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
@@ -3235,22 +3241,22 @@
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H6" s="27" t="n">
@@ -3263,36 +3269,36 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H7" s="27" t="n">
-        <v>8.220000000000001</v>
-      </c>
-      <c r="I7" s="28" t="n">
-        <v>-8.84</v>
+        <v>2.07</v>
+      </c>
+      <c r="I7" s="27" t="n">
+        <v>2.39</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
@@ -3305,22 +3311,22 @@
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H8" s="25" t="n"/>
@@ -3336,22 +3342,22 @@
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H9" s="27" t="n">
@@ -3371,22 +3377,22 @@
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H10" s="25" t="n"/>
@@ -3402,22 +3408,22 @@
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H11" s="25" t="n"/>
@@ -3426,36 +3432,36 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H12" s="28" t="n">
-        <v>-1.1</v>
-      </c>
-      <c r="I12" s="27" t="n">
-        <v>2.87</v>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H12" s="27" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="I12" s="28" t="n">
+        <v>-0.2</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
@@ -3468,22 +3474,22 @@
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H13" s="25" t="n"/>
@@ -3492,7 +3498,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>HJ중공업</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -3509,87 +3515,91 @@
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H14" s="27" t="n">
-        <v>2.05</v>
-      </c>
-      <c r="I14" s="28" t="n">
-        <v>-5.81</v>
-      </c>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H14" s="25" t="n"/>
+      <c r="I14" s="25" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E15" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H15" s="25" t="n"/>
-      <c r="I15" s="25" t="n"/>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H15" s="27" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="I15" s="28" t="n">
+        <v>-2.46</v>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C16" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D16" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E16" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H16" s="25" t="n"/>
-      <c r="I16" s="25" t="n"/>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H16" s="27" t="n">
+        <v>4.68</v>
+      </c>
+      <c r="I16" s="27" t="n">
+        <v>12.34</v>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>에코프로</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -3606,25 +3616,25 @@
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H17" s="27" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.46</v>
       </c>
       <c r="I17" s="28" t="n">
-        <v>-2.46</v>
+        <v>-8.49</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>기아</t>
+          <t>콘텐트리중앙</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -3641,60 +3651,60 @@
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H18" s="27" t="n">
-        <v>4.68</v>
-      </c>
-      <c r="I18" s="27" t="n">
-        <v>12.34</v>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H18" s="28" t="n">
+        <v>-28.9</v>
+      </c>
+      <c r="I18" s="28" t="n">
+        <v>-65.13</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>광진실업</t>
+          <t>파라다이스</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H19" s="28" t="n">
-        <v>-10</v>
+        <v>-11.77</v>
       </c>
       <c r="I19" s="27" t="n">
-        <v>42.16</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>모바일어플라이언스</t>
+          <t>HJ중공업</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
@@ -3711,25 +3721,25 @@
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H20" s="25" t="n">
-        <v>0</v>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H20" s="27" t="n">
+        <v>2.05</v>
       </c>
       <c r="I20" s="28" t="n">
-        <v>-22.19</v>
+        <v>-5.81</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>광진실업</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -3746,25 +3756,25 @@
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H21" s="27" t="n">
-        <v>6.48</v>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H21" s="28" t="n">
+        <v>-10</v>
       </c>
       <c r="I21" s="27" t="n">
-        <v>6.21</v>
+        <v>42.16</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>다보링크</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -3781,25 +3791,25 @@
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H22" s="27" t="n">
-        <v>3.27</v>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H22" s="28" t="n">
+        <v>-9.92</v>
       </c>
       <c r="I22" s="28" t="n">
-        <v>-0.2</v>
+        <v>-36.8</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>삼호개발</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3816,25 +3826,21 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H23" s="28" t="n">
-        <v>-13.27</v>
-      </c>
-      <c r="I23" s="27" t="n">
-        <v>2.71</v>
-      </c>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H23" s="25" t="n"/>
+      <c r="I23" s="25" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3851,25 +3857,25 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H24" s="27" t="n">
-        <v>3.96</v>
+        <v>6.48</v>
       </c>
       <c r="I24" s="27" t="n">
-        <v>10.67</v>
+        <v>6.21</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>스테이블코인</t>
+          <t>삼호개발</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3886,21 +3892,25 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H25" s="25" t="n"/>
-      <c r="I25" s="25" t="n"/>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H25" s="28" t="n">
+        <v>-13.27</v>
+      </c>
+      <c r="I25" s="27" t="n">
+        <v>2.71</v>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>진흥기업</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
@@ -3917,21 +3927,25 @@
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H26" s="25" t="n"/>
-      <c r="I26" s="25" t="n"/>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H26" s="28" t="n">
+        <v>-18.04</v>
+      </c>
+      <c r="I26" s="27" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>코퍼스코리아</t>
+          <t>코오롱티슈진</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
@@ -3948,82 +3962,82 @@
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H27" s="27" t="n">
-        <v>18.24</v>
-      </c>
-      <c r="I27" s="27" t="n">
-        <v>90.31999999999999</v>
+        <v>3.67</v>
+      </c>
+      <c r="I27" s="28" t="n">
+        <v>-5.25</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>CSA 코스믹</t>
+          <t>코퍼스코리아</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C28" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D28" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E28" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H28" s="27" t="n">
-        <v>9.130000000000001</v>
+        <v>18.24</v>
       </c>
       <c r="I28" s="27" t="n">
-        <v>22.22</v>
+        <v>90.31999999999999</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C29" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D29" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E29" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H29" s="25" t="n"/>
@@ -4032,7 +4046,7 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>에코프로</t>
+          <t>CSA 코스믹</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -4049,25 +4063,25 @@
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H30" s="27" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="I30" s="28" t="n">
-        <v>-8.49</v>
+        <v>9.130000000000001</v>
+      </c>
+      <c r="I30" s="27" t="n">
+        <v>22.22</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>에코프로비엠</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
@@ -4084,25 +4098,25 @@
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H31" s="28" t="n">
-        <v>-0.88</v>
-      </c>
-      <c r="I31" s="28" t="n">
-        <v>-6.96</v>
+        <v>-5.07</v>
+      </c>
+      <c r="I31" s="27" t="n">
+        <v>16.8</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>진흥기업</t>
+          <t>모바일어플라이언스</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -4119,25 +4133,25 @@
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H32" s="28" t="n">
-        <v>-18.04</v>
-      </c>
-      <c r="I32" s="27" t="n">
-        <v>30</v>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H32" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="28" t="n">
+        <v>-22.19</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>슈어소프트테크</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4154,25 +4168,25 @@
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H33" s="27" t="n">
-        <v>0.71</v>
+        <v>4.27</v>
       </c>
       <c r="I33" s="27" t="n">
-        <v>7.09</v>
+        <v>5.04</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>콘텐트리중앙</t>
+          <t>에코프로비엠</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4189,130 +4203,122 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H34" s="28" t="n">
-        <v>-28.9</v>
+        <v>-0.88</v>
       </c>
       <c r="I34" s="28" t="n">
-        <v>-65.13</v>
+        <v>-6.96</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>KB금융</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D35" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E35" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H35" s="27" t="n">
-        <v>3.09</v>
-      </c>
-      <c r="I35" s="27" t="n">
-        <v>13.93</v>
-      </c>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H35" s="25" t="n"/>
+      <c r="I35" s="25" t="n"/>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>골프존홀딩스</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C36" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D36" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E36" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H36" s="27" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I36" s="27" t="n">
-        <v>56.05</v>
-      </c>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H36" s="25" t="n"/>
+      <c r="I36" s="25" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C37" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D37" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E37" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H37" s="28" t="n">
-        <v>-19.01</v>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H37" s="27" t="n">
+        <v>0.71</v>
       </c>
       <c r="I37" s="27" t="n">
-        <v>43.29</v>
+        <v>7.09</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>금호전기</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4329,25 +4335,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H38" s="28" t="n">
-        <v>-24.62</v>
-      </c>
-      <c r="I38" s="28" t="n">
-        <v>-12.31</v>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H38" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="27" t="n">
+        <v>7.36</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>다보링크</t>
+          <t>KB금융</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4364,25 +4370,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H39" s="28" t="n">
-        <v>-9.92</v>
-      </c>
-      <c r="I39" s="28" t="n">
-        <v>-36.8</v>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H39" s="27" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="I39" s="27" t="n">
+        <v>13.93</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>신원종합개발</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4399,25 +4405,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H40" s="28" t="n">
-        <v>-16.77</v>
+        <v>-1.1</v>
       </c>
       <c r="I40" s="27" t="n">
-        <v>23.49</v>
+        <v>2.87</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>파라다이스</t>
+          <t>골프존홀딩스</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4434,25 +4440,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H41" s="28" t="n">
-        <v>-11.77</v>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H41" s="27" t="n">
+        <v>0.15</v>
       </c>
       <c r="I41" s="27" t="n">
-        <v>3.3</v>
+        <v>56.05</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>팸텍</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4469,200 +4475,196 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H42" s="27" t="n">
-        <v>10.35</v>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H42" s="28" t="n">
+        <v>-19.01</v>
       </c>
       <c r="I42" s="27" t="n">
-        <v>6.84</v>
+        <v>43.29</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>HC보광산업</t>
+          <t>금호전기</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C43" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D43" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E43" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H43" s="27" t="n">
-        <v>9.039999999999999</v>
-      </c>
-      <c r="I43" s="27" t="n">
-        <v>40.38</v>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H43" s="28" t="n">
+        <v>-24.62</v>
+      </c>
+      <c r="I43" s="28" t="n">
+        <v>-12.31</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>계룡건설</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C44" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D44" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E44" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H44" s="28" t="n">
-        <v>-11.43</v>
-      </c>
-      <c r="I44" s="27" t="n">
-        <v>22.78</v>
-      </c>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H44" s="25" t="n"/>
+      <c r="I44" s="25" t="n"/>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>덕신이피씨</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C45" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D45" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E45" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H45" s="28" t="n">
-        <v>-17.83</v>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H45" s="27" t="n">
+        <v>3.96</v>
       </c>
       <c r="I45" s="27" t="n">
-        <v>65.5</v>
+        <v>10.67</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>스트라드비젼</t>
+          <t>신원종합개발</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C46" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D46" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E46" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H46" s="28" t="n">
-        <v>-0.76</v>
-      </c>
-      <c r="I46" s="28" t="n">
-        <v>-36.39</v>
+        <v>-16.77</v>
+      </c>
+      <c r="I46" s="27" t="n">
+        <v>23.49</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>팸텍</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C47" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D47" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E47" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H47" s="27" t="n">
-        <v>2.05</v>
+        <v>10.35</v>
       </c>
       <c r="I47" s="27" t="n">
-        <v>43.93</v>
+        <v>6.84</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>아크솔루션스</t>
+          <t>HC보광산업</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4679,25 +4681,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H48" s="27" t="n">
-        <v>27.37</v>
-      </c>
-      <c r="I48" s="28" t="n">
-        <v>-97.27</v>
+        <v>9.039999999999999</v>
+      </c>
+      <c r="I48" s="27" t="n">
+        <v>40.38</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>에스폴리텍</t>
+          <t>스트라드비젼</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4714,25 +4716,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H49" s="28" t="n">
-        <v>-1.56</v>
-      </c>
-      <c r="I49" s="27" t="n">
-        <v>35.61</v>
+        <v>-0.76</v>
+      </c>
+      <c r="I49" s="28" t="n">
+        <v>-36.39</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>우원개발</t>
+          <t>아크솔루션스</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4749,25 +4751,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H50" s="27" t="n">
-        <v>4.47</v>
-      </c>
-      <c r="I50" s="27" t="n">
-        <v>42.99</v>
+        <v>27.37</v>
+      </c>
+      <c r="I50" s="28" t="n">
+        <v>-97.27</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>져스텍</t>
+          <t>에스폴리텍</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4784,25 +4786,25 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="H51" s="27" t="n">
-        <v>29.96</v>
-      </c>
-      <c r="I51" s="28" t="n">
-        <v>-9.93</v>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H51" s="28" t="n">
+        <v>-1.56</v>
+      </c>
+      <c r="I51" s="27" t="n">
+        <v>35.61</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="26" t="inlineStr">
         <is>
-          <t>한성크린텍</t>
+          <t>져스텍</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -4819,19 +4821,19 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="H52" s="27" t="n">
-        <v>2.02</v>
-      </c>
-      <c r="I52" s="27" t="n">
-        <v>41.96</v>
+        <v>29.96</v>
+      </c>
+      <c r="I52" s="28" t="n">
+        <v>-9.93</v>
       </c>
     </row>
   </sheetData>
@@ -4915,19 +4917,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>106</v>
+        <v>83</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>106</v>
+        <v>83</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4946,19 +4948,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4977,19 +4979,19 @@
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5001,26 +5003,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5032,7 +5034,7 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
@@ -5046,12 +5048,12 @@
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5063,26 +5065,26 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5094,26 +5096,26 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B9" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5125,92 +5127,100 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="35" t="inlineStr">
         <is>
+          <t>철강</t>
+        </is>
+      </c>
+      <c r="B10" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" s="36" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="F10" s="37" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="G10" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>제약</t>
+        </is>
+      </c>
+      <c r="B11" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="36" t="n">
+        <v>13</v>
+      </c>
+      <c r="D11" s="36" t="n">
+        <v>13</v>
+      </c>
+      <c r="E11" s="36" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="F11" s="37" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="G11" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="35" t="inlineStr">
+        <is>
           <t>인공지능</t>
         </is>
       </c>
-      <c r="B10" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" s="36" t="n">
-        <v>19</v>
-      </c>
-      <c r="D10" s="36" t="n">
-        <v>19</v>
-      </c>
-      <c r="E10" s="36" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="F10" s="37" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="G10" s="37" t="inlineStr">
+      <c r="B12" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="D12" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="E12" s="36" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="F12" s="37" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="G12" s="37" t="inlineStr">
         <is>
           <t>⚡ 관심</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="26" t="inlineStr">
-        <is>
-          <t>이차전지</t>
-        </is>
-      </c>
-      <c r="B11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F11" s="29" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G11" s="29" t="inlineStr"/>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="26" t="inlineStr">
-        <is>
-          <t>AI반도체</t>
-        </is>
-      </c>
-      <c r="B12" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F12" s="29" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G12" s="29" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>이차전지</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -5237,7 +5247,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5264,7 +5274,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5291,7 +5301,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -5318,7 +5328,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -5345,7 +5355,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>핀테크</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -5372,7 +5382,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>핀테크</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -5399,7 +5409,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-07-06 07:18 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -258,14 +258,14 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-07-05 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-07-06 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-05) 상위: 반도체  점수 83.0점</t>
+          <t>⚡ 최신(2026-07-06) 상위: 반도체  점수 100.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-05) 상위: SK  점수 53.0점</t>
+          <t>⚡ 최신(2026-07-06) 상위: SK  점수 49.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-05) 상위: 삼성전자  점수 28.0점</t>
+          <t>⚡ 최신(2026-07-06) 상위: 삼성전자  점수 45.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -971,10 +971,10 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -990,7 +990,7 @@
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1014,10 +1014,10 @@
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
@@ -1045,7 +1045,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1057,10 +1057,10 @@
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
@@ -1088,7 +1088,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1096,14 +1096,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1112,26 +1112,24 @@
         <v>0</v>
       </c>
       <c r="H18" s="18" t="n">
-        <v>2.07</v>
+        <v>2.12</v>
       </c>
       <c r="I18" s="18" t="n">
-        <v>2.39</v>
+        <v>2.54</v>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K18" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K18" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1139,14 +1137,14 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1162,7 +1160,7 @@
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K19" s="17" t="inlineStr">
@@ -1174,7 +1172,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1182,14 +1180,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1197,15 +1195,15 @@
       <c r="G20" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="18" t="n">
-        <v>2.12</v>
-      </c>
-      <c r="I20" s="18" t="n">
-        <v>2.54</v>
+      <c r="H20" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I20" s="15" t="n">
+        <v/>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K20" s="17" t="inlineStr">
@@ -1217,7 +1215,7 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1225,42 +1223,42 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>에코프로</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G21" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I21" s="15" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H21" s="18" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="I21" s="19" t="n">
+        <v>-8.49</v>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+          <t>네이버 검색 당일 +126% / 중요공시 2건 / 중요공시 7일 +100% / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1268,14 +1266,14 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -1291,7 +1289,7 @@
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="inlineStr">
@@ -1303,7 +1301,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1311,42 +1309,42 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E23" s="15" t="n">
         <v>9</v>
       </c>
       <c r="F23" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G23" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H23" s="18" t="n">
-        <v>3.27</v>
-      </c>
-      <c r="I23" s="19" t="n">
-        <v>-0.2</v>
+        <v>2.07</v>
+      </c>
+      <c r="I23" s="18" t="n">
+        <v>2.39</v>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K23" s="17" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1354,42 +1352,42 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>코퍼스코리아</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G24" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H24" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I24" s="15" t="n">
-        <v/>
+      <c r="H24" s="18" t="n">
+        <v>18.24</v>
+      </c>
+      <c r="I24" s="18" t="n">
+        <v>90.31999999999999</v>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +407% / 중요공시 6건 / 중요공시 3일 +50%</t>
         </is>
       </c>
       <c r="K24" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1397,7 +1395,7 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
@@ -1420,17 +1418,19 @@
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K25" s="17" t="n">
-        <v/>
+          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K25" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1438,42 +1438,42 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>에코프로</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
         <v>7</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F26" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G26" s="15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H26" s="18" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="I26" s="19" t="n">
-        <v>-8.49</v>
+        <v>1.05</v>
+      </c>
+      <c r="I26" s="18" t="n">
+        <v>2.85</v>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +121% / 중요공시 2건 / 중요공시 7일 +100%</t>
+          <t>Google 급상승 검색어 등장 (KR) / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K26" s="17" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>콘텐트리중앙</t>
+          <t>에코프로비엠</t>
         </is>
       </c>
       <c r="D27" s="15" t="n">
@@ -1497,26 +1497,26 @@
         <v>0</v>
       </c>
       <c r="H27" s="19" t="n">
-        <v>-28.9</v>
+        <v>-0.88</v>
       </c>
       <c r="I27" s="19" t="n">
-        <v>-65.13</v>
+        <v>-6.96</v>
       </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +66% / 중요공시 5건 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 3건 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K27" s="17" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B28" s="15" t="n">
@@ -1524,42 +1524,40 @@
       </c>
       <c r="C28" s="16" t="inlineStr">
         <is>
-          <t>파라다이스</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D28" s="15" t="n">
         <v>7</v>
       </c>
       <c r="E28" s="15" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F28" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G28" s="15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H28" s="19" t="n">
-        <v>-11.77</v>
-      </c>
-      <c r="I28" s="18" t="n">
-        <v>3.3</v>
+        <v>-0.23</v>
+      </c>
+      <c r="I28" s="19" t="n">
+        <v>-6.34</v>
       </c>
       <c r="J28" s="17" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K28" s="17" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K28" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B29" s="15" t="n">
@@ -1567,7 +1565,7 @@
       </c>
       <c r="C29" s="16" t="inlineStr">
         <is>
-          <t>기아</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="D29" s="15" t="n">
@@ -1582,68 +1580,68 @@
       <c r="G29" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H29" s="18" t="n">
-        <v>4.68</v>
+      <c r="H29" s="19" t="n">
+        <v>-2.38</v>
       </c>
       <c r="I29" s="18" t="n">
-        <v>12.34</v>
+        <v>7.8</v>
       </c>
       <c r="J29" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K29" s="17" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K29" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="15" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="B30" s="15" t="n">
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="n">
         <v>17</v>
       </c>
-      <c r="C30" s="16" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="D30" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E30" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F30" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="18" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="I30" s="19" t="n">
-        <v>-2.46</v>
-      </c>
-      <c r="J30" s="17" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K30" s="17" t="n">
-        <v/>
+      <c r="C30" s="21" t="inlineStr">
+        <is>
+          <t>삼호개발</t>
+        </is>
+      </c>
+      <c r="D30" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E30" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="22" t="n">
+        <v>-13.27</v>
+      </c>
+      <c r="I30" s="23" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="J30" s="24" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +272% / 중요공시 4건</t>
+        </is>
+      </c>
+      <c r="K30" s="24" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1651,42 +1649,42 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>코퍼스코리아</t>
+          <t>진흥기업</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F31" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G31" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H31" s="22" t="n">
-        <v>18.24</v>
-      </c>
-      <c r="I31" s="22" t="n">
-        <v>90.31999999999999</v>
-      </c>
-      <c r="J31" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +392% / 중요공시 6건</t>
-        </is>
-      </c>
-      <c r="K31" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
+        <v>-18.04</v>
+      </c>
+      <c r="I31" s="23" t="n">
+        <v>30</v>
+      </c>
+      <c r="J31" s="24" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +187% / 중요공시 2건 / 중요공시 3일 +100%</t>
+        </is>
+      </c>
+      <c r="K31" s="24" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1694,7 +1692,7 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>삼호개발</t>
+          <t>다보링크</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
@@ -1709,27 +1707,27 @@
       <c r="G32" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H32" s="24" t="n">
-        <v>-13.27</v>
+      <c r="H32" s="22" t="n">
+        <v>-9.92</v>
       </c>
       <c r="I32" s="22" t="n">
-        <v>2.71</v>
-      </c>
-      <c r="J32" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +260% / 중요공시 4건</t>
-        </is>
-      </c>
-      <c r="K32" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
+        <v>-36.8</v>
+      </c>
+      <c r="J32" s="24" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +122% / 중요공시 3건</t>
+        </is>
+      </c>
+      <c r="K32" s="24" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1737,42 +1735,42 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>진흥기업</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F33" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G33" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H33" s="24" t="n">
-        <v>-18.04</v>
-      </c>
-      <c r="I33" s="22" t="n">
-        <v>30</v>
-      </c>
-      <c r="J33" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +174% / 중요공시 2건 / 중요공시 3일 +100%</t>
-        </is>
-      </c>
-      <c r="K33" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
+        <v>3</v>
+      </c>
+      <c r="H33" s="23" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="I33" s="23" t="n">
+        <v>43.93</v>
+      </c>
+      <c r="J33" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 5건 / 중요공시 7일 +67%</t>
+        </is>
+      </c>
+      <c r="K33" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1780,7 +1778,7 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>다보링크</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
@@ -1795,27 +1793,25 @@
       <c r="G34" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="24" t="n">
-        <v>-9.92</v>
-      </c>
-      <c r="I34" s="24" t="n">
-        <v>-36.8</v>
-      </c>
-      <c r="J34" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +113% / 중요공시 3건</t>
-        </is>
-      </c>
-      <c r="K34" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
+      <c r="H34" s="23" t="n">
+        <v>6.48</v>
+      </c>
+      <c r="I34" s="23" t="n">
+        <v>6.21</v>
+      </c>
+      <c r="J34" s="24" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K34" s="24" t="n">
+        <v/>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1823,40 +1819,42 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>썸에이지</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F35" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G35" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H35" s="22" t="n">
-        <v>6.48</v>
-      </c>
-      <c r="I35" s="22" t="n">
-        <v>6.21</v>
-      </c>
-      <c r="J35" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K35" s="23" t="n">
-        <v/>
+        <v>-10.87</v>
+      </c>
+      <c r="I35" s="23" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="J35" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 4건 / 중요공시 7일 +300%</t>
+        </is>
+      </c>
+      <c r="K35" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1864,33 +1862,33 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>광진실업</t>
+          <t>다스코</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F36" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G36" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H36" s="24" t="n">
-        <v>-10</v>
-      </c>
-      <c r="I36" s="22" t="n">
-        <v>42.16</v>
-      </c>
-      <c r="J36" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 5건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K36" s="23" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="H36" s="22" t="n">
+        <v>-7.72</v>
+      </c>
+      <c r="I36" s="23" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="J36" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K36" s="24" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
@@ -1899,7 +1897,7 @@
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1907,33 +1905,33 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>HJ중공업</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E37" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F37" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G37" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="H37" s="22" t="n">
-        <v>2.05</v>
-      </c>
-      <c r="I37" s="24" t="n">
-        <v>-5.81</v>
-      </c>
-      <c r="J37" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 4건 / 중요공시 7일 +300%</t>
-        </is>
-      </c>
-      <c r="K37" s="23" t="inlineStr">
+      <c r="H37" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="23" t="n">
+        <v>7.36</v>
+      </c>
+      <c r="J37" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K37" s="24" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
@@ -1942,7 +1940,7 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1950,7 +1948,7 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>코오롱티슈진</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
@@ -1965,27 +1963,27 @@
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H38" s="22" t="n">
-        <v>3.67</v>
-      </c>
-      <c r="I38" s="24" t="n">
-        <v>-5.25</v>
-      </c>
-      <c r="J38" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / Google 급상승 검색어 등장 (KR)</t>
-        </is>
-      </c>
-      <c r="K38" s="23" t="inlineStr">
-        <is>
-          <t>Google, 공시</t>
+      <c r="H38" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I38" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J38" s="24" t="inlineStr">
+        <is>
+          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K38" s="24" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1993,7 +1991,7 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
@@ -2014,19 +2012,19 @@
       <c r="I39" s="20" t="n">
         <v/>
       </c>
-      <c r="J39" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K39" s="23" t="n">
+      <c r="J39" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K39" s="24" t="n">
         <v/>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2034,14 +2032,14 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>콘텐트리중앙</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F40" s="20" t="n">
         <v>0</v>
@@ -2049,27 +2047,27 @@
       <c r="G40" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H40" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I40" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J40" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K40" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
+      <c r="H40" s="22" t="n">
+        <v>-28.9</v>
+      </c>
+      <c r="I40" s="22" t="n">
+        <v>-65.13</v>
+      </c>
+      <c r="J40" s="24" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +78% / 중요공시 5건</t>
+        </is>
+      </c>
+      <c r="K40" s="24" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2095,24 +2093,24 @@
       <c r="H41" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="I41" s="24" t="n">
+      <c r="I41" s="22" t="n">
         <v>-22.19</v>
       </c>
-      <c r="J41" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +52% / 중요공시 3건</t>
-        </is>
-      </c>
-      <c r="K41" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
+      <c r="J41" s="24" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +56% / 중요공시 3건</t>
+        </is>
+      </c>
+      <c r="K41" s="24" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2120,7 +2118,7 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
@@ -2135,25 +2133,27 @@
       <c r="G42" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H42" s="22" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="I42" s="22" t="n">
-        <v>7.09</v>
-      </c>
-      <c r="J42" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K42" s="23" t="n">
-        <v/>
+      <c r="H42" s="23" t="n">
+        <v>4.68</v>
+      </c>
+      <c r="I42" s="23" t="n">
+        <v>12.34</v>
+      </c>
+      <c r="J42" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K42" s="24" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2161,42 +2161,42 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>CSA 코스믹</t>
+          <t>골프존홀딩스</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E43" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F43" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G43" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H43" s="22" t="n">
-        <v>9.130000000000001</v>
-      </c>
-      <c r="I43" s="22" t="n">
-        <v>22.22</v>
-      </c>
-      <c r="J43" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 6건 / 중요공시 3일 +50%</t>
-        </is>
-      </c>
-      <c r="K43" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="H43" s="23" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="I43" s="23" t="n">
+        <v>56.05</v>
+      </c>
+      <c r="J43" s="24" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +956% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K43" s="24" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2204,42 +2204,42 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>에코프로비엠</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E44" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F44" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G44" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="24" t="n">
-        <v>-0.88</v>
-      </c>
-      <c r="I44" s="24" t="n">
-        <v>-6.96</v>
-      </c>
-      <c r="J44" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 3건 / 중요공시 3일 +50%</t>
-        </is>
-      </c>
-      <c r="K44" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="H44" s="22" t="n">
+        <v>-19.01</v>
+      </c>
+      <c r="I44" s="23" t="n">
+        <v>43.29</v>
+      </c>
+      <c r="J44" s="24" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +428% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K44" s="24" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2247,14 +2247,14 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>슈어소프트테크</t>
+          <t>신원종합개발</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E45" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F45" s="20" t="n">
         <v>0</v>
@@ -2263,26 +2263,26 @@
         <v>0</v>
       </c>
       <c r="H45" s="22" t="n">
-        <v>4.27</v>
-      </c>
-      <c r="I45" s="22" t="n">
-        <v>5.04</v>
-      </c>
-      <c r="J45" s="23" t="inlineStr">
-        <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
-        </is>
-      </c>
-      <c r="K45" s="23" t="inlineStr">
-        <is>
-          <t>Google</t>
+        <v>-16.77</v>
+      </c>
+      <c r="I45" s="23" t="n">
+        <v>23.49</v>
+      </c>
+      <c r="J45" s="24" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +306% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K45" s="24" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
@@ -2290,14 +2290,14 @@
       </c>
       <c r="C46" s="21" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>금호전기</t>
         </is>
       </c>
       <c r="D46" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E46" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F46" s="20" t="n">
         <v>0</v>
@@ -2305,27 +2305,27 @@
       <c r="G46" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H46" s="24" t="n">
-        <v>-5.07</v>
+      <c r="H46" s="22" t="n">
+        <v>-24.62</v>
       </c>
       <c r="I46" s="22" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="J46" s="23" t="inlineStr">
-        <is>
-          <t>Google 급상승 검색어 등장 (US)</t>
-        </is>
-      </c>
-      <c r="K46" s="23" t="inlineStr">
-        <is>
-          <t>Google</t>
+        <v>-12.31</v>
+      </c>
+      <c r="J46" s="24" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +258% / 중요공시 2건</t>
+        </is>
+      </c>
+      <c r="K46" s="24" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B47" s="20" t="n">
@@ -2333,42 +2333,42 @@
       </c>
       <c r="C47" s="21" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>파라다이스</t>
         </is>
       </c>
       <c r="D47" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E47" s="20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F47" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G47" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H47" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I47" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J47" s="23" t="inlineStr">
-        <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K47" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
+      <c r="H47" s="22" t="n">
+        <v>-11.77</v>
+      </c>
+      <c r="I47" s="23" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="J47" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+        </is>
+      </c>
+      <c r="K47" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B48" s="20" t="n">
@@ -2376,40 +2376,42 @@
       </c>
       <c r="C48" s="21" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D48" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E48" s="20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F48" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G48" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H48" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I48" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J48" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K48" s="23" t="n">
-        <v/>
+      <c r="H48" s="23" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="I48" s="22" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="J48" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K48" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B49" s="20" t="n">
@@ -2417,7 +2419,7 @@
       </c>
       <c r="C49" s="21" t="inlineStr">
         <is>
-          <t>골프존홀딩스</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D49" s="20" t="n">
@@ -2432,27 +2434,27 @@
       <c r="G49" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="22" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I49" s="22" t="n">
-        <v>56.05</v>
-      </c>
-      <c r="J49" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +932% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K49" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
+      <c r="H49" s="23" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="I49" s="23" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="J49" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K49" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B50" s="20" t="n">
@@ -2460,42 +2462,42 @@
       </c>
       <c r="C50" s="21" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>젠큐릭스</t>
         </is>
       </c>
       <c r="D50" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E50" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F50" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G50" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H50" s="24" t="n">
-        <v>-19.01</v>
+        <v>3</v>
+      </c>
+      <c r="H50" s="22" t="n">
+        <v>-4.53</v>
       </c>
       <c r="I50" s="22" t="n">
-        <v>43.29</v>
-      </c>
-      <c r="J50" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +417% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K50" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
+        <v>-3.15</v>
+      </c>
+      <c r="J50" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K50" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B51" s="20" t="n">
@@ -2503,7 +2505,7 @@
       </c>
       <c r="C51" s="21" t="inlineStr">
         <is>
-          <t>신원종합개발</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="D51" s="20" t="n">
@@ -2518,27 +2520,25 @@
       <c r="G51" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H51" s="24" t="n">
-        <v>-16.77</v>
+      <c r="H51" s="23" t="n">
+        <v>0.07000000000000001</v>
       </c>
       <c r="I51" s="22" t="n">
-        <v>23.49</v>
-      </c>
-      <c r="J51" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +291% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K51" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
+        <v>-2.46</v>
+      </c>
+      <c r="J51" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K51" s="24" t="n">
+        <v/>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B52" s="20" t="n">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="C52" s="21" t="inlineStr">
         <is>
-          <t>금호전기</t>
+          <t>TSMC</t>
         </is>
       </c>
       <c r="D52" s="20" t="n">
@@ -2561,27 +2561,27 @@
       <c r="G52" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H52" s="24" t="n">
-        <v>-24.62</v>
-      </c>
-      <c r="I52" s="24" t="n">
-        <v>-12.31</v>
-      </c>
-      <c r="J52" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +252% / 중요공시 2건</t>
-        </is>
-      </c>
-      <c r="K52" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
+      <c r="H52" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I52" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J52" s="24" t="inlineStr">
+        <is>
+          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K52" s="24" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B53" s="20" t="n">
@@ -2589,7 +2589,7 @@
       </c>
       <c r="C53" s="21" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="D53" s="20" t="n">
@@ -2604,27 +2604,25 @@
       <c r="G53" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="22" t="n">
-        <v>3.96</v>
-      </c>
-      <c r="I53" s="22" t="n">
-        <v>10.67</v>
-      </c>
-      <c r="J53" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K53" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+      <c r="H53" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I53" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J53" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K53" s="24" t="n">
+        <v/>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B54" s="20" t="n">
@@ -2632,42 +2630,40 @@
       </c>
       <c r="C54" s="21" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="D54" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E54" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F54" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G54" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H54" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I54" s="22" t="n">
-        <v>7.36</v>
-      </c>
-      <c r="J54" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K54" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+        <v/>
+      </c>
+      <c r="I54" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J54" s="24" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K54" s="24" t="n">
+        <v/>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B55" s="20" t="n">
@@ -2675,7 +2671,7 @@
       </c>
       <c r="C55" s="21" t="inlineStr">
         <is>
-          <t>팸텍</t>
+          <t>HMM</t>
         </is>
       </c>
       <c r="D55" s="20" t="n">
@@ -2690,27 +2686,25 @@
       <c r="G55" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H55" s="22" t="n">
-        <v>10.35</v>
-      </c>
-      <c r="I55" s="22" t="n">
-        <v>6.84</v>
-      </c>
-      <c r="J55" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K55" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+      <c r="H55" s="23" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="I55" s="23" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="J55" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K55" s="24" t="n">
+        <v/>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B56" s="20" t="n">
@@ -2718,7 +2712,7 @@
       </c>
       <c r="C56" s="21" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="D56" s="20" t="n">
@@ -2733,109 +2727,111 @@
       <c r="G56" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H56" s="20" t="n">
+      <c r="H56" s="22" t="n">
+        <v>-1.1</v>
+      </c>
+      <c r="I56" s="23" t="n">
+        <v>2.87</v>
+      </c>
+      <c r="J56" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K56" s="24" t="n">
         <v/>
       </c>
-      <c r="I56" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J56" s="23" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K56" s="23" t="inlineStr">
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="25" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B57" s="25" t="n">
+        <v>44</v>
+      </c>
+      <c r="C57" s="26" t="inlineStr">
+        <is>
+          <t>져스텍</t>
+        </is>
+      </c>
+      <c r="D57" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E57" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F57" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" s="27" t="n">
+        <v>29.96</v>
+      </c>
+      <c r="I57" s="28" t="n">
+        <v>-9.93</v>
+      </c>
+      <c r="J57" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +778%</t>
+        </is>
+      </c>
+      <c r="K57" s="29" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="20" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="B57" s="20" t="n">
-        <v>44</v>
-      </c>
-      <c r="C57" s="21" t="inlineStr">
-        <is>
-          <t>KB금융</t>
-        </is>
-      </c>
-      <c r="D57" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E57" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F57" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G57" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H57" s="22" t="n">
-        <v>3.09</v>
-      </c>
-      <c r="I57" s="22" t="n">
-        <v>13.93</v>
-      </c>
-      <c r="J57" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K57" s="23" t="n">
-        <v/>
-      </c>
-    </row>
     <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="20" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="B58" s="20" t="n">
+      <c r="A58" s="25" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B58" s="25" t="n">
         <v>45</v>
       </c>
-      <c r="C58" s="21" t="inlineStr">
-        <is>
-          <t>KT</t>
-        </is>
-      </c>
-      <c r="D58" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E58" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F58" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G58" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H58" s="24" t="n">
-        <v>-1.1</v>
-      </c>
-      <c r="I58" s="22" t="n">
-        <v>2.87</v>
-      </c>
-      <c r="J58" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K58" s="23" t="n">
-        <v/>
+      <c r="C58" s="26" t="inlineStr">
+        <is>
+          <t>에스폴리텍</t>
+        </is>
+      </c>
+      <c r="D58" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E58" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F58" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" s="28" t="n">
+        <v>-1.56</v>
+      </c>
+      <c r="I58" s="27" t="n">
+        <v>35.61</v>
+      </c>
+      <c r="J58" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +533%</t>
+        </is>
+      </c>
+      <c r="K58" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2843,7 +2839,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>져스텍</t>
+          <t>스트라드비젼</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2858,15 +2854,15 @@
       <c r="G59" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H59" s="27" t="n">
-        <v>29.96</v>
+      <c r="H59" s="28" t="n">
+        <v>-0.76</v>
       </c>
       <c r="I59" s="28" t="n">
-        <v>-9.93</v>
+        <v>-36.39</v>
       </c>
       <c r="J59" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +763%</t>
+          <t>네이버 검색 당일 +533%</t>
         </is>
       </c>
       <c r="K59" s="29" t="inlineStr">
@@ -2878,7 +2874,7 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2886,7 +2882,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>스트라드비젼</t>
+          <t>HC보광산업</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2901,15 +2897,15 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="28" t="n">
-        <v>-0.76</v>
-      </c>
-      <c r="I60" s="28" t="n">
-        <v>-36.39</v>
+      <c r="H60" s="27" t="n">
+        <v>9.039999999999999</v>
+      </c>
+      <c r="I60" s="27" t="n">
+        <v>40.38</v>
       </c>
       <c r="J60" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +525%</t>
+          <t>네이버 검색 당일 +533%</t>
         </is>
       </c>
       <c r="K60" s="29" t="inlineStr">
@@ -2921,7 +2917,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2929,7 +2925,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>에스폴리텍</t>
+          <t>우원개발</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2944,15 +2940,15 @@
       <c r="G61" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H61" s="28" t="n">
-        <v>-1.56</v>
+      <c r="H61" s="27" t="n">
+        <v>4.47</v>
       </c>
       <c r="I61" s="27" t="n">
-        <v>35.61</v>
+        <v>42.99</v>
       </c>
       <c r="J61" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +512%</t>
+          <t>네이버 검색 당일 +353%</t>
         </is>
       </c>
       <c r="K61" s="29" t="inlineStr">
@@ -2964,7 +2960,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2972,7 +2968,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>HC보광산업</t>
+          <t>아크솔루션스</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2988,14 +2984,14 @@
         <v>0</v>
       </c>
       <c r="H62" s="27" t="n">
-        <v>9.039999999999999</v>
-      </c>
-      <c r="I62" s="27" t="n">
-        <v>40.38</v>
+        <v>27.37</v>
+      </c>
+      <c r="I62" s="28" t="n">
+        <v>-97.27</v>
       </c>
       <c r="J62" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +494%</t>
+          <t>네이버 검색 당일 +350%</t>
         </is>
       </c>
       <c r="K62" s="29" t="inlineStr">
@@ -3007,7 +3003,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3015,7 +3011,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>아크솔루션스</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3031,14 +3027,14 @@
         <v>0</v>
       </c>
       <c r="H63" s="27" t="n">
-        <v>27.37</v>
-      </c>
-      <c r="I63" s="28" t="n">
-        <v>-97.27</v>
+        <v>29.9</v>
+      </c>
+      <c r="I63" s="27" t="n">
+        <v>46.17</v>
       </c>
       <c r="J63" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +337%</t>
+          <t>네이버 검색 당일 +338%</t>
         </is>
       </c>
       <c r="K63" s="29" t="inlineStr">
@@ -3140,22 +3136,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3171,22 +3167,22 @@
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H4" s="27" t="n">
@@ -3206,22 +3202,22 @@
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H5" s="27" t="n">
@@ -3241,22 +3237,22 @@
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H6" s="27" t="n">
@@ -3269,64 +3265,64 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H7" s="27" t="n">
-        <v>2.07</v>
+        <v>2.12</v>
       </c>
       <c r="I7" s="27" t="n">
-        <v>2.39</v>
+        <v>2.54</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H8" s="25" t="n"/>
@@ -3335,95 +3331,95 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H9" s="27" t="n">
-        <v>2.12</v>
-      </c>
-      <c r="I9" s="27" t="n">
-        <v>2.54</v>
-      </c>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H9" s="25" t="n"/>
+      <c r="I9" s="25" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>에코프로</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H10" s="25" t="n"/>
-      <c r="I10" s="25" t="n"/>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H10" s="27" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="I10" s="28" t="n">
+        <v>-8.49</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H11" s="25" t="n"/>
@@ -3432,64 +3428,64 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H12" s="27" t="n">
-        <v>3.27</v>
-      </c>
-      <c r="I12" s="28" t="n">
-        <v>-0.2</v>
+        <v>2.07</v>
+      </c>
+      <c r="I12" s="27" t="n">
+        <v>2.39</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H13" s="25" t="n"/>
@@ -3498,7 +3494,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>코퍼스코리아</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -3515,21 +3511,25 @@
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H14" s="25" t="n"/>
-      <c r="I14" s="25" t="n"/>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H14" s="27" t="n">
+        <v>18.24</v>
+      </c>
+      <c r="I14" s="27" t="n">
+        <v>90.31999999999999</v>
+      </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -3546,25 +3546,25 @@
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H15" s="27" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="I15" s="28" t="n">
-        <v>-2.46</v>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H15" s="28" t="n">
+        <v>-2.38</v>
+      </c>
+      <c r="I15" s="27" t="n">
+        <v>7.8</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>기아</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -3581,25 +3581,25 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H16" s="27" t="n">
-        <v>4.68</v>
-      </c>
-      <c r="I16" s="27" t="n">
-        <v>12.34</v>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H16" s="28" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="I16" s="28" t="n">
+        <v>-6.34</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>에코프로</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -3616,25 +3616,25 @@
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H17" s="27" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="I17" s="28" t="n">
-        <v>-8.49</v>
+        <v>1.05</v>
+      </c>
+      <c r="I17" s="27" t="n">
+        <v>2.85</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>콘텐트리중앙</t>
+          <t>에코프로비엠</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -3651,60 +3651,60 @@
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H18" s="28" t="n">
-        <v>-28.9</v>
+        <v>-0.88</v>
       </c>
       <c r="I18" s="28" t="n">
-        <v>-65.13</v>
+        <v>-6.96</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>파라다이스</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H19" s="28" t="n">
-        <v>-11.77</v>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H19" s="25" t="n">
+        <v>0</v>
       </c>
       <c r="I19" s="27" t="n">
-        <v>3.3</v>
+        <v>7.36</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>HJ중공업</t>
+          <t>다보링크</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
@@ -3721,25 +3721,25 @@
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H20" s="27" t="n">
-        <v>2.05</v>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H20" s="28" t="n">
+        <v>-9.92</v>
       </c>
       <c r="I20" s="28" t="n">
-        <v>-5.81</v>
+        <v>-36.8</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>광진실업</t>
+          <t>다스코</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -3756,25 +3756,25 @@
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H21" s="28" t="n">
-        <v>-10</v>
+        <v>-7.72</v>
       </c>
       <c r="I21" s="27" t="n">
-        <v>42.16</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>다보링크</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -3791,25 +3791,25 @@
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H22" s="28" t="n">
-        <v>-9.92</v>
-      </c>
-      <c r="I22" s="28" t="n">
-        <v>-36.8</v>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H22" s="27" t="n">
+        <v>6.48</v>
+      </c>
+      <c r="I22" s="27" t="n">
+        <v>6.21</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>삼호개발</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3826,21 +3826,25 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H23" s="25" t="n"/>
-      <c r="I23" s="25" t="n"/>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H23" s="28" t="n">
+        <v>-13.27</v>
+      </c>
+      <c r="I23" s="27" t="n">
+        <v>2.71</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3857,25 +3861,25 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H24" s="27" t="n">
-        <v>6.48</v>
+        <v>2.05</v>
       </c>
       <c r="I24" s="27" t="n">
-        <v>6.21</v>
+        <v>43.93</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>삼호개발</t>
+          <t>썸에이지</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3892,25 +3896,25 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H25" s="28" t="n">
-        <v>-13.27</v>
+        <v>-10.87</v>
       </c>
       <c r="I25" s="27" t="n">
-        <v>2.71</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>진흥기업</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
@@ -3927,25 +3931,21 @@
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H26" s="28" t="n">
-        <v>-18.04</v>
-      </c>
-      <c r="I26" s="27" t="n">
-        <v>30</v>
-      </c>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H26" s="25" t="n"/>
+      <c r="I26" s="25" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>코오롱티슈진</t>
+          <t>진흥기업</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
@@ -3962,25 +3962,25 @@
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H27" s="27" t="n">
-        <v>3.67</v>
-      </c>
-      <c r="I27" s="28" t="n">
-        <v>-5.25</v>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H27" s="28" t="n">
+        <v>-18.04</v>
+      </c>
+      <c r="I27" s="27" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>코퍼스코리아</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
@@ -3997,56 +3997,56 @@
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H28" s="27" t="n">
-        <v>18.24</v>
-      </c>
-      <c r="I28" s="27" t="n">
-        <v>90.31999999999999</v>
-      </c>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H28" s="25" t="n"/>
+      <c r="I28" s="25" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C29" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D29" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E29" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H29" s="25" t="n"/>
-      <c r="I29" s="25" t="n"/>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H29" s="27" t="n">
+        <v>4.68</v>
+      </c>
+      <c r="I29" s="27" t="n">
+        <v>12.34</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>CSA 코스믹</t>
+          <t>모바일어플라이언스</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -4063,25 +4063,25 @@
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H30" s="27" t="n">
-        <v>9.130000000000001</v>
-      </c>
-      <c r="I30" s="27" t="n">
-        <v>22.22</v>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H30" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="28" t="n">
+        <v>-22.19</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>콘텐트리중앙</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
@@ -4098,152 +4098,152 @@
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H31" s="28" t="n">
-        <v>-5.07</v>
-      </c>
-      <c r="I31" s="27" t="n">
-        <v>16.8</v>
+        <v>-28.9</v>
+      </c>
+      <c r="I31" s="28" t="n">
+        <v>-65.13</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>모바일어플라이언스</t>
+          <t>HMM</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C32" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D32" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E32" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H32" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" s="28" t="n">
-        <v>-22.19</v>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H32" s="27" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="I32" s="27" t="n">
+        <v>4.7</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>슈어소프트테크</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C33" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D33" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E33" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H33" s="27" t="n">
-        <v>4.27</v>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H33" s="28" t="n">
+        <v>-1.1</v>
       </c>
       <c r="I33" s="27" t="n">
-        <v>5.04</v>
+        <v>2.87</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>에코프로비엠</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C34" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D34" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E34" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H34" s="28" t="n">
-        <v>-0.88</v>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H34" s="27" t="n">
+        <v>0.07000000000000001</v>
       </c>
       <c r="I34" s="28" t="n">
-        <v>-6.96</v>
+        <v>-2.46</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>TSMC</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D35" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E35" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H35" s="25" t="n"/>
@@ -4252,73 +4252,77 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>골프존홀딩스</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C36" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D36" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E36" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H36" s="25" t="n"/>
-      <c r="I36" s="25" t="n"/>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H36" s="27" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="I36" s="27" t="n">
+        <v>56.05</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C37" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D37" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E37" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H37" s="27" t="n">
-        <v>0.71</v>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H37" s="28" t="n">
+        <v>-19.01</v>
       </c>
       <c r="I37" s="27" t="n">
-        <v>7.09</v>
+        <v>43.29</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>금호전기</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4335,25 +4339,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H38" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I38" s="27" t="n">
-        <v>7.36</v>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H38" s="28" t="n">
+        <v>-24.62</v>
+      </c>
+      <c r="I38" s="28" t="n">
+        <v>-12.31</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>KB금융</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4370,25 +4374,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H39" s="27" t="n">
-        <v>3.09</v>
-      </c>
-      <c r="I39" s="27" t="n">
-        <v>13.93</v>
+        <v>3.27</v>
+      </c>
+      <c r="I39" s="28" t="n">
+        <v>-0.2</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4405,25 +4409,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H40" s="28" t="n">
-        <v>-1.1</v>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H40" s="27" t="n">
+        <v>3.96</v>
       </c>
       <c r="I40" s="27" t="n">
-        <v>2.87</v>
+        <v>10.67</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>골프존홀딩스</t>
+          <t>신원종합개발</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4440,25 +4444,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H41" s="27" t="n">
-        <v>0.15</v>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H41" s="28" t="n">
+        <v>-16.77</v>
       </c>
       <c r="I41" s="27" t="n">
-        <v>56.05</v>
+        <v>23.49</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>젠큐릭스</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4475,25 +4479,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H42" s="28" t="n">
-        <v>-19.01</v>
-      </c>
-      <c r="I42" s="27" t="n">
-        <v>43.29</v>
+        <v>-4.53</v>
+      </c>
+      <c r="I42" s="28" t="n">
+        <v>-3.15</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>금호전기</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4510,25 +4514,21 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H43" s="28" t="n">
-        <v>-24.62</v>
-      </c>
-      <c r="I43" s="28" t="n">
-        <v>-12.31</v>
-      </c>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H43" s="25" t="n"/>
+      <c r="I43" s="25" t="n"/>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4545,12 +4545,12 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H44" s="25" t="n"/>
@@ -4559,7 +4559,7 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>파라다이스</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4576,95 +4576,95 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H45" s="27" t="n">
-        <v>3.96</v>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H45" s="28" t="n">
+        <v>-11.77</v>
       </c>
       <c r="I45" s="27" t="n">
-        <v>10.67</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>신원종합개발</t>
+          <t>HC보광산업</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C46" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D46" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E46" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H46" s="28" t="n">
-        <v>-16.77</v>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H46" s="27" t="n">
+        <v>9.039999999999999</v>
       </c>
       <c r="I46" s="27" t="n">
-        <v>23.49</v>
+        <v>40.38</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>팸텍</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C47" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D47" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E47" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H47" s="27" t="n">
-        <v>10.35</v>
+        <v>29.9</v>
       </c>
       <c r="I47" s="27" t="n">
-        <v>6.84</v>
+        <v>46.17</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>HC보광산업</t>
+          <t>스트라드비젼</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4681,25 +4681,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H48" s="27" t="n">
-        <v>9.039999999999999</v>
-      </c>
-      <c r="I48" s="27" t="n">
-        <v>40.38</v>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H48" s="28" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="I48" s="28" t="n">
+        <v>-36.39</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>스트라드비젼</t>
+          <t>아크솔루션스</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4716,25 +4716,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H49" s="28" t="n">
-        <v>-0.76</v>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H49" s="27" t="n">
+        <v>27.37</v>
       </c>
       <c r="I49" s="28" t="n">
-        <v>-36.39</v>
+        <v>-97.27</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>아크솔루션스</t>
+          <t>에스폴리텍</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4751,25 +4751,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H50" s="27" t="n">
-        <v>27.37</v>
-      </c>
-      <c r="I50" s="28" t="n">
-        <v>-97.27</v>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H50" s="28" t="n">
+        <v>-1.56</v>
+      </c>
+      <c r="I50" s="27" t="n">
+        <v>35.61</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>에스폴리텍</t>
+          <t>우원개발</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4786,19 +4786,19 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="H51" s="28" t="n">
-        <v>-1.56</v>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H51" s="27" t="n">
+        <v>4.47</v>
       </c>
       <c r="I51" s="27" t="n">
-        <v>35.61</v>
+        <v>42.99</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
@@ -4821,12 +4821,12 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H52" s="27" t="n">
@@ -4917,19 +4917,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4948,19 +4948,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4972,26 +4972,26 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="35" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B5" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5003,26 +5003,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5034,26 +5034,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5065,26 +5065,26 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5096,7 +5096,7 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B9" s="36" t="n">
@@ -5110,12 +5110,12 @@
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5127,26 +5127,26 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="35" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B10" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="36" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D10" s="36" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="E10" s="36" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F10" s="37" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G10" s="37" t="inlineStr">
@@ -5158,26 +5158,26 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="35" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B11" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="36" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D11" s="36" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E11" s="36" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F11" s="37" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G11" s="37" t="inlineStr">
@@ -5187,40 +5187,36 @@
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="35" t="inlineStr">
-        <is>
-          <t>인공지능</t>
-        </is>
-      </c>
-      <c r="B12" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="36" t="n">
-        <v>20</v>
-      </c>
-      <c r="D12" s="36" t="n">
-        <v>20</v>
-      </c>
-      <c r="E12" s="36" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="F12" s="37" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="G12" s="37" t="inlineStr">
-        <is>
-          <t>⚡ 관심</t>
-        </is>
-      </c>
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>이차전지</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F12" s="29" t="inlineStr">
+        <is>
+          <t>감지 없음</t>
+        </is>
+      </c>
+      <c r="G12" s="29" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>이차전지</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -5247,7 +5243,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5274,7 +5270,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5301,7 +5297,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-07-07 07:19 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -258,10 +258,10 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -273,14 +273,14 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-07-06 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-07-07 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-06) 상위: 반도체  점수 100.0점</t>
+          <t>⚡ 최신(2026-07-07) 상위: 반도체  점수 89.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-06) 상위: SK  점수 49.0점</t>
+          <t>⚡ 최신(2026-07-07) 상위: 삼성전자  점수 35.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-06) 상위: 삼성전자  점수 45.0점</t>
+          <t>⚡ 최신(2026-07-07) 상위: SK하이닉스  점수 22.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -967,14 +967,14 @@
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -983,14 +983,14 @@
         <v>0</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>1.02</v>
+        <v>2.75</v>
       </c>
       <c r="I15" s="19" t="n">
-        <v>-15.34</v>
+        <v>-1.55</v>
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1010,14 +1010,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1025,27 +1025,27 @@
       <c r="G16" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="18" t="n">
-        <v>8.220000000000001</v>
+      <c r="H16" s="19" t="n">
+        <v>-3.38</v>
       </c>
       <c r="I16" s="19" t="n">
-        <v>-8.84</v>
+        <v>-10.84</v>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>중요공시 1건 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1053,14 +1053,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1068,15 +1068,15 @@
       <c r="G17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="18" t="n">
-        <v>10.88</v>
-      </c>
-      <c r="I17" s="19" t="n">
-        <v>-9.279999999999999</v>
+      <c r="H17" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I17" s="15" t="n">
+        <v/>
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
@@ -1088,7 +1088,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1096,14 +1096,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1111,25 +1111,27 @@
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="18" t="n">
-        <v>2.12</v>
-      </c>
-      <c r="I18" s="18" t="n">
-        <v>2.54</v>
+      <c r="H18" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I18" s="15" t="n">
+        <v/>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K18" s="17" t="n">
-        <v/>
+          <t>네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K18" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1137,14 +1139,14 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1152,27 +1154,27 @@
       <c r="G19" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I19" s="15" t="n">
-        <v/>
+      <c r="H19" s="18" t="n">
+        <v>8.609999999999999</v>
+      </c>
+      <c r="I19" s="18" t="n">
+        <v>10.05</v>
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K19" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1180,14 +1182,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1203,19 +1205,17 @@
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K20" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K20" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1223,42 +1223,42 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>에코프로</t>
+          <t>진흥기업</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
         <v>11</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F21" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G21" s="15" t="n">
         <v>3</v>
       </c>
       <c r="H21" s="18" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="I21" s="19" t="n">
-        <v>-8.49</v>
+        <v>14.32</v>
+      </c>
+      <c r="I21" s="18" t="n">
+        <v>37</v>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +126% / 중요공시 2건 / 중요공시 7일 +100% / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>네이버 검색 당일 +196% / 중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +200%</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
@@ -1281,15 +1281,15 @@
       <c r="G22" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I22" s="15" t="n">
-        <v/>
+      <c r="H22" s="18" t="n">
+        <v>4.68</v>
+      </c>
+      <c r="I22" s="18" t="n">
+        <v>2.76</v>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+          <t>한국경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="inlineStr">
@@ -1301,7 +1301,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1309,42 +1309,42 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F23" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G23" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="18" t="n">
-        <v>2.07</v>
-      </c>
-      <c r="I23" s="18" t="n">
-        <v>2.39</v>
+        <v>3</v>
+      </c>
+      <c r="H23" s="19" t="n">
+        <v>-4.19</v>
+      </c>
+      <c r="I23" s="19" t="n">
+        <v>-1.84</v>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +200% / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K23" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1352,42 +1352,40 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>코퍼스코리아</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G24" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H24" s="18" t="n">
-        <v>18.24</v>
+        <v>0.1</v>
       </c>
       <c r="I24" s="18" t="n">
-        <v>90.31999999999999</v>
+        <v>0.4</v>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +407% / 중요공시 6건 / 중요공시 3일 +50%</t>
-        </is>
-      </c>
-      <c r="K24" s="17" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
-        </is>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K24" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1399,10 +1397,10 @@
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F25" s="15" t="n">
         <v>0</v>
@@ -1418,7 +1416,7 @@
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K25" s="17" t="inlineStr">
@@ -1430,7 +1428,7 @@
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1438,14 +1436,14 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F26" s="15" t="n">
         <v>0</v>
@@ -1453,27 +1451,27 @@
       <c r="G26" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H26" s="18" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="I26" s="18" t="n">
-        <v>2.85</v>
+      <c r="H26" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I26" s="15" t="n">
+        <v/>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR) / 한국경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K26" s="17" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -1481,42 +1479,42 @@
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>에코프로비엠</t>
+          <t>삼호개발</t>
         </is>
       </c>
       <c r="D27" s="15" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E27" s="15" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F27" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G27" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="19" t="n">
-        <v>-0.88</v>
-      </c>
-      <c r="I27" s="19" t="n">
-        <v>-6.96</v>
+        <v>3</v>
+      </c>
+      <c r="H27" s="18" t="n">
+        <v>14.25</v>
+      </c>
+      <c r="I27" s="18" t="n">
+        <v>19.94</v>
       </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>네이버 검색 당일 +284% / 중요공시 5건 / 중요공시 7일 +67%</t>
         </is>
       </c>
       <c r="K27" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B28" s="15" t="n">
@@ -1524,14 +1522,14 @@
       </c>
       <c r="C28" s="16" t="inlineStr">
         <is>
-          <t>LG이노텍</t>
+          <t>한화시스템</t>
         </is>
       </c>
       <c r="D28" s="15" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E28" s="15" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F28" s="15" t="n">
         <v>0</v>
@@ -1539,15 +1537,15 @@
       <c r="G28" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H28" s="19" t="n">
-        <v>-0.23</v>
-      </c>
-      <c r="I28" s="19" t="n">
-        <v>-6.34</v>
+      <c r="H28" s="18" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="I28" s="18" t="n">
+        <v>4.39</v>
       </c>
       <c r="J28" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K28" s="17" t="n">
@@ -1557,7 +1555,7 @@
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B29" s="15" t="n">
@@ -1565,7 +1563,7 @@
       </c>
       <c r="C29" s="16" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="D29" s="15" t="n">
@@ -1580,15 +1578,15 @@
       <c r="G29" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H29" s="19" t="n">
-        <v>-2.38</v>
-      </c>
-      <c r="I29" s="18" t="n">
-        <v>7.8</v>
+      <c r="H29" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I29" s="15" t="n">
+        <v/>
       </c>
       <c r="J29" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K29" s="17" t="n">
@@ -1596,52 +1594,50 @@
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="20" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="B30" s="20" t="n">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="n">
         <v>17</v>
       </c>
-      <c r="C30" s="21" t="inlineStr">
-        <is>
-          <t>삼호개발</t>
-        </is>
-      </c>
-      <c r="D30" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E30" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="F30" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="22" t="n">
-        <v>-13.27</v>
-      </c>
-      <c r="I30" s="23" t="n">
-        <v>2.71</v>
-      </c>
-      <c r="J30" s="24" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +272% / 중요공시 4건</t>
-        </is>
-      </c>
-      <c r="K30" s="24" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
-        </is>
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>태양광</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="F30" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I30" s="15" t="n">
+        <v/>
+      </c>
+      <c r="J30" s="17" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K30" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1649,42 +1645,42 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>진흥기업</t>
+          <t>다스코</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F31" s="20" t="n">
         <v>2</v>
       </c>
       <c r="G31" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H31" s="22" t="n">
-        <v>-18.04</v>
+        <v>1.88</v>
       </c>
       <c r="I31" s="23" t="n">
-        <v>30</v>
+        <v>-20.94</v>
       </c>
       <c r="J31" s="24" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +187% / 중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K31" s="24" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1692,42 +1688,42 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>다보링크</t>
+          <t>광진실업</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F32" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G32" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H32" s="22" t="n">
-        <v>-9.92</v>
+        <v>3</v>
+      </c>
+      <c r="H32" s="23" t="n">
+        <v>-12.31</v>
       </c>
       <c r="I32" s="22" t="n">
-        <v>-36.8</v>
+        <v>19.44</v>
       </c>
       <c r="J32" s="24" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +122% / 중요공시 3건</t>
+          <t>중요공시 5건 / 중요공시 7일 +400%</t>
         </is>
       </c>
       <c r="K32" s="24" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1735,30 +1731,30 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>SK스퀘어</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F33" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G33" s="20" t="n">
         <v>3</v>
       </c>
       <c r="H33" s="23" t="n">
-        <v>2.05</v>
+        <v>-5.92</v>
       </c>
       <c r="I33" s="23" t="n">
-        <v>43.93</v>
+        <v>-8.84</v>
       </c>
       <c r="J33" s="24" t="inlineStr">
         <is>
-          <t>중요공시 5건 / 중요공시 7일 +67%</t>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K33" s="24" t="inlineStr">
@@ -1770,7 +1766,7 @@
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1778,40 +1774,42 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>코오롱티슈진</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F34" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G34" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H34" s="23" t="n">
-        <v>6.48</v>
+        <v>-2.21</v>
       </c>
       <c r="I34" s="23" t="n">
-        <v>6.21</v>
+        <v>-9.34</v>
       </c>
       <c r="J34" s="24" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K34" s="24" t="n">
-        <v/>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K34" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1819,42 +1817,42 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>썸에이지</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F35" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G35" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H35" s="22" t="n">
-        <v>-10.87</v>
-      </c>
-      <c r="I35" s="23" t="n">
-        <v>3.7</v>
+        <v>2.03</v>
+      </c>
+      <c r="I35" s="22" t="n">
+        <v>1.01</v>
       </c>
       <c r="J35" s="24" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 중요공시 7일 +300%</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K35" s="24" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1862,42 +1860,42 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>다스코</t>
+          <t>모바일어플라이언스</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F36" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G36" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H36" s="22" t="n">
-        <v>-7.72</v>
+        <v>0</v>
+      </c>
+      <c r="H36" s="20" t="n">
+        <v>0</v>
       </c>
       <c r="I36" s="23" t="n">
-        <v>0.87</v>
+        <v>-19.24</v>
       </c>
       <c r="J36" s="24" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+          <t>네이버 검색 당일 +60% / 중요공시 3건</t>
         </is>
       </c>
       <c r="K36" s="24" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1905,30 +1903,30 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>다보링크</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E37" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F37" s="20" t="n">
         <v>2</v>
       </c>
       <c r="G37" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H37" s="20" t="n">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="H37" s="22" t="n">
+        <v>4.24</v>
       </c>
       <c r="I37" s="23" t="n">
-        <v>7.36</v>
+        <v>-34.17</v>
       </c>
       <c r="J37" s="24" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+          <t>중요공시 4건 / 중요공시 3일 +100%</t>
         </is>
       </c>
       <c r="K37" s="24" t="inlineStr">
@@ -1940,7 +1938,7 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1948,14 +1946,14 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F38" s="20" t="n">
         <v>0</v>
@@ -1963,27 +1961,27 @@
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H38" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I38" s="20" t="n">
-        <v/>
+      <c r="H38" s="23" t="n">
+        <v>-8.09</v>
+      </c>
+      <c r="I38" s="23" t="n">
+        <v>-10.3</v>
       </c>
       <c r="J38" s="24" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K38" s="24" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1991,14 +1989,14 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F39" s="20" t="n">
         <v>0</v>
@@ -2014,17 +2012,19 @@
       </c>
       <c r="J39" s="24" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K39" s="24" t="n">
-        <v/>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K39" s="24" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2032,14 +2032,14 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>콘텐트리중앙</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F40" s="20" t="n">
         <v>0</v>
@@ -2048,26 +2048,26 @@
         <v>0</v>
       </c>
       <c r="H40" s="22" t="n">
-        <v>-28.9</v>
+        <v>30</v>
       </c>
       <c r="I40" s="22" t="n">
-        <v>-65.13</v>
+        <v>43.44</v>
       </c>
       <c r="J40" s="24" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +78% / 중요공시 5건</t>
+          <t>네이버 검색 당일 +438% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K40" s="24" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2075,14 +2075,14 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>모바일어플라이언스</t>
+          <t>동신건설</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E41" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F41" s="20" t="n">
         <v>0</v>
@@ -2090,27 +2090,27 @@
       <c r="G41" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="20" t="n">
-        <v>0</v>
+      <c r="H41" s="22" t="n">
+        <v>15.17</v>
       </c>
       <c r="I41" s="22" t="n">
-        <v>-22.19</v>
+        <v>45.07</v>
       </c>
       <c r="J41" s="24" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +56% / 중요공시 3건</t>
+          <t>네이버 검색 당일 +390% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K41" s="24" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2118,14 +2118,14 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>기아</t>
+          <t>신원종합개발</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E42" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F42" s="20" t="n">
         <v>0</v>
@@ -2133,27 +2133,27 @@
       <c r="G42" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H42" s="23" t="n">
-        <v>4.68</v>
-      </c>
-      <c r="I42" s="23" t="n">
-        <v>12.34</v>
+      <c r="H42" s="22" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="I42" s="22" t="n">
+        <v>20.09</v>
       </c>
       <c r="J42" s="24" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버 검색 당일 +319% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K42" s="24" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2161,7 +2161,7 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>골프존홀딩스</t>
+          <t>금호전기</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
@@ -2176,27 +2176,27 @@
       <c r="G43" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H43" s="23" t="n">
-        <v>0.15</v>
+      <c r="H43" s="22" t="n">
+        <v>29.96</v>
       </c>
       <c r="I43" s="23" t="n">
-        <v>56.05</v>
+        <v>-12.3</v>
       </c>
       <c r="J43" s="24" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +956% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +263% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K43" s="24" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2204,7 +2204,7 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>일성건설</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
@@ -2220,26 +2220,26 @@
         <v>0</v>
       </c>
       <c r="H44" s="22" t="n">
-        <v>-19.01</v>
-      </c>
-      <c r="I44" s="23" t="n">
-        <v>43.29</v>
+        <v>29.74</v>
+      </c>
+      <c r="I44" s="22" t="n">
+        <v>62.89</v>
       </c>
       <c r="J44" s="24" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +428% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +120% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K44" s="24" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2247,7 +2247,7 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>신원종합개발</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
@@ -2262,27 +2262,27 @@
       <c r="G45" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H45" s="22" t="n">
-        <v>-16.77</v>
-      </c>
-      <c r="I45" s="23" t="n">
-        <v>23.49</v>
+      <c r="H45" s="23" t="n">
+        <v>-11.91</v>
+      </c>
+      <c r="I45" s="22" t="n">
+        <v>14.19</v>
       </c>
       <c r="J45" s="24" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +306% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +59% / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K45" s="24" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
@@ -2290,7 +2290,7 @@
       </c>
       <c r="C46" s="21" t="inlineStr">
         <is>
-          <t>금호전기</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="D46" s="20" t="n">
@@ -2306,26 +2306,26 @@
         <v>0</v>
       </c>
       <c r="H46" s="22" t="n">
-        <v>-24.62</v>
+        <v>5.72</v>
       </c>
       <c r="I46" s="22" t="n">
-        <v>-12.31</v>
+        <v>14.3</v>
       </c>
       <c r="J46" s="24" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +258% / 중요공시 2건</t>
+          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K46" s="24" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B47" s="20" t="n">
@@ -2333,30 +2333,30 @@
       </c>
       <c r="C47" s="21" t="inlineStr">
         <is>
-          <t>파라다이스</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="D47" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E47" s="20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F47" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G47" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H47" s="22" t="n">
-        <v>-11.77</v>
+      <c r="H47" s="23" t="n">
+        <v>-0.8100000000000001</v>
       </c>
       <c r="I47" s="23" t="n">
-        <v>3.3</v>
+        <v>-2.84</v>
       </c>
       <c r="J47" s="24" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>중요공시 1건 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K47" s="24" t="inlineStr">
@@ -2368,7 +2368,7 @@
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B48" s="20" t="n">
@@ -2376,30 +2376,30 @@
       </c>
       <c r="C48" s="21" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>에코프로</t>
         </is>
       </c>
       <c r="D48" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E48" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F48" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G48" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H48" s="23" t="n">
-        <v>3.27</v>
-      </c>
-      <c r="I48" s="22" t="n">
-        <v>-0.2</v>
+        <v>-2.06</v>
+      </c>
+      <c r="I48" s="23" t="n">
+        <v>-27.54</v>
       </c>
       <c r="J48" s="24" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 매일경제 기사 언급</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K48" s="24" t="inlineStr">
@@ -2411,7 +2411,7 @@
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B49" s="20" t="n">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="C49" s="21" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>판타지오</t>
         </is>
       </c>
       <c r="D49" s="20" t="n">
@@ -2434,15 +2434,15 @@
       <c r="G49" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="23" t="n">
-        <v>3.96</v>
-      </c>
-      <c r="I49" s="23" t="n">
-        <v>10.67</v>
+      <c r="H49" s="22" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="I49" s="22" t="n">
+        <v>11.08</v>
       </c>
       <c r="J49" s="24" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K49" s="24" t="inlineStr">
@@ -2454,7 +2454,7 @@
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B50" s="20" t="n">
@@ -2462,7 +2462,7 @@
       </c>
       <c r="C50" s="21" t="inlineStr">
         <is>
-          <t>젠큐릭스</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="D50" s="20" t="n">
@@ -2478,10 +2478,10 @@
         <v>3</v>
       </c>
       <c r="H50" s="22" t="n">
-        <v>-4.53</v>
+        <v>3.74</v>
       </c>
       <c r="I50" s="22" t="n">
-        <v>-3.15</v>
+        <v>1.68</v>
       </c>
       <c r="J50" s="24" t="inlineStr">
         <is>
@@ -2497,7 +2497,7 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B51" s="20" t="n">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="C51" s="21" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>아난티</t>
         </is>
       </c>
       <c r="D51" s="20" t="n">
@@ -2521,24 +2521,26 @@
         <v>0</v>
       </c>
       <c r="H51" s="23" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="I51" s="22" t="n">
-        <v>-2.46</v>
+        <v>-0.13</v>
+      </c>
+      <c r="I51" s="23" t="n">
+        <v>-6.04</v>
       </c>
       <c r="J51" s="24" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K51" s="24" t="n">
-        <v/>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K51" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B52" s="20" t="n">
@@ -2546,7 +2548,7 @@
       </c>
       <c r="C52" s="21" t="inlineStr">
         <is>
-          <t>TSMC</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="D52" s="20" t="n">
@@ -2561,27 +2563,25 @@
       <c r="G52" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H52" s="20" t="n">
+      <c r="H52" s="23" t="n">
+        <v>-2.58</v>
+      </c>
+      <c r="I52" s="23" t="n">
+        <v>-12.21</v>
+      </c>
+      <c r="J52" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K52" s="24" t="n">
         <v/>
-      </c>
-      <c r="I52" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J52" s="24" t="inlineStr">
-        <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K52" s="24" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B53" s="20" t="n">
@@ -2589,7 +2589,7 @@
       </c>
       <c r="C53" s="21" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D53" s="20" t="n">
@@ -2612,17 +2612,19 @@
       </c>
       <c r="J53" s="24" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K53" s="24" t="n">
-        <v/>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K53" s="24" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B54" s="20" t="n">
@@ -2630,7 +2632,7 @@
       </c>
       <c r="C54" s="21" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>하이브</t>
         </is>
       </c>
       <c r="D54" s="20" t="n">
@@ -2645,25 +2647,27 @@
       <c r="G54" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H54" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I54" s="20" t="n">
-        <v/>
+      <c r="H54" s="22" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="I54" s="22" t="n">
+        <v>10.09</v>
       </c>
       <c r="J54" s="24" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K54" s="24" t="n">
-        <v/>
+          <t>한국경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K54" s="24" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B55" s="20" t="n">
@@ -2671,7 +2675,7 @@
       </c>
       <c r="C55" s="21" t="inlineStr">
         <is>
-          <t>HMM</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="D55" s="20" t="n">
@@ -2686,15 +2690,15 @@
       <c r="G55" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H55" s="23" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="I55" s="23" t="n">
-        <v>4.7</v>
+      <c r="H55" s="22" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="I55" s="22" t="n">
+        <v>10.57</v>
       </c>
       <c r="J55" s="24" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K55" s="24" t="n">
@@ -2702,50 +2706,52 @@
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
-      <c r="A56" s="20" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="B56" s="20" t="n">
+      <c r="A56" s="25" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B56" s="25" t="n">
         <v>43</v>
       </c>
-      <c r="C56" s="21" t="inlineStr">
-        <is>
-          <t>KT</t>
-        </is>
-      </c>
-      <c r="D56" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E56" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F56" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G56" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H56" s="22" t="n">
-        <v>-1.1</v>
-      </c>
-      <c r="I56" s="23" t="n">
-        <v>2.87</v>
-      </c>
-      <c r="J56" s="24" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K56" s="24" t="n">
-        <v/>
+      <c r="C56" s="26" t="inlineStr">
+        <is>
+          <t>져스텍</t>
+        </is>
+      </c>
+      <c r="D56" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E56" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F56" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="27" t="n">
+        <v>-11.59</v>
+      </c>
+      <c r="I56" s="27" t="n">
+        <v>-20.37</v>
+      </c>
+      <c r="J56" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +790%</t>
+        </is>
+      </c>
+      <c r="K56" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2753,7 +2759,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>져스텍</t>
+          <t>HC보광산업</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2768,18 +2774,18 @@
       <c r="G57" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H57" s="27" t="n">
-        <v>29.96</v>
-      </c>
-      <c r="I57" s="28" t="n">
-        <v>-9.93</v>
-      </c>
-      <c r="J57" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +778%</t>
-        </is>
-      </c>
-      <c r="K57" s="29" t="inlineStr">
+      <c r="H57" s="29" t="n">
+        <v>7.73</v>
+      </c>
+      <c r="I57" s="29" t="n">
+        <v>40.96</v>
+      </c>
+      <c r="J57" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +565%</t>
+        </is>
+      </c>
+      <c r="K57" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -2788,7 +2794,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2811,18 +2817,18 @@
       <c r="G58" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="28" t="n">
-        <v>-1.56</v>
-      </c>
-      <c r="I58" s="27" t="n">
-        <v>35.61</v>
-      </c>
-      <c r="J58" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +533%</t>
-        </is>
-      </c>
-      <c r="K58" s="29" t="inlineStr">
+      <c r="H58" s="29" t="n">
+        <v>13.96</v>
+      </c>
+      <c r="I58" s="29" t="n">
+        <v>55.29</v>
+      </c>
+      <c r="J58" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +550%</t>
+        </is>
+      </c>
+      <c r="K58" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -2831,7 +2837,7 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2854,18 +2860,18 @@
       <c r="G59" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H59" s="28" t="n">
-        <v>-0.76</v>
-      </c>
-      <c r="I59" s="28" t="n">
-        <v>-36.39</v>
-      </c>
-      <c r="J59" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +533%</t>
-        </is>
-      </c>
-      <c r="K59" s="29" t="inlineStr">
+      <c r="H59" s="29" t="n">
+        <v>7.31</v>
+      </c>
+      <c r="I59" s="27" t="n">
+        <v>-31.74</v>
+      </c>
+      <c r="J59" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +540%</t>
+        </is>
+      </c>
+      <c r="K59" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -2874,7 +2880,7 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2882,7 +2888,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>HC보광산업</t>
+          <t>위메이드맥스</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2897,18 +2903,18 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="27" t="n">
-        <v>9.039999999999999</v>
-      </c>
-      <c r="I60" s="27" t="n">
-        <v>40.38</v>
-      </c>
-      <c r="J60" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +533%</t>
-        </is>
-      </c>
-      <c r="K60" s="29" t="inlineStr">
+      <c r="H60" s="29" t="n">
+        <v>20.44</v>
+      </c>
+      <c r="I60" s="29" t="n">
+        <v>43.74</v>
+      </c>
+      <c r="J60" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +532%</t>
+        </is>
+      </c>
+      <c r="K60" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -2917,7 +2923,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2925,7 +2931,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>우원개발</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2941,17 +2947,17 @@
         <v>0</v>
       </c>
       <c r="H61" s="27" t="n">
-        <v>4.47</v>
-      </c>
-      <c r="I61" s="27" t="n">
-        <v>42.99</v>
-      </c>
-      <c r="J61" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +353%</t>
-        </is>
-      </c>
-      <c r="K61" s="29" t="inlineStr">
+        <v>-3.17</v>
+      </c>
+      <c r="I61" s="29" t="n">
+        <v>33.19</v>
+      </c>
+      <c r="J61" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +393%</t>
+        </is>
+      </c>
+      <c r="K61" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -2960,7 +2966,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2968,7 +2974,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>아크솔루션스</t>
+          <t>우원개발</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2983,18 +2989,18 @@
       <c r="G62" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H62" s="27" t="n">
-        <v>27.37</v>
-      </c>
-      <c r="I62" s="28" t="n">
-        <v>-97.27</v>
-      </c>
-      <c r="J62" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +350%</t>
-        </is>
-      </c>
-      <c r="K62" s="29" t="inlineStr">
+      <c r="H62" s="29" t="n">
+        <v>5.91</v>
+      </c>
+      <c r="I62" s="29" t="n">
+        <v>33.86</v>
+      </c>
+      <c r="J62" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +385%</t>
+        </is>
+      </c>
+      <c r="K62" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -3003,7 +3009,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3011,7 +3017,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>아크솔루션스</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3026,18 +3032,18 @@
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="27" t="n">
-        <v>29.9</v>
-      </c>
-      <c r="I63" s="27" t="n">
-        <v>46.17</v>
-      </c>
-      <c r="J63" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +338%</t>
-        </is>
-      </c>
-      <c r="K63" s="29" t="inlineStr">
+      <c r="H63" s="29" t="n">
+        <v>23.14</v>
+      </c>
+      <c r="I63" s="29" t="n">
+        <v>29.57</v>
+      </c>
+      <c r="J63" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +361%</t>
+        </is>
+      </c>
+      <c r="K63" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -3136,22 +3142,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3160,200 +3166,196 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B4" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H4" s="27" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="I4" s="28" t="n">
-        <v>-15.34</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H4" s="29" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="I4" s="27" t="n">
+        <v>-1.55</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="H5" s="27" t="n">
-        <v>8.220000000000001</v>
-      </c>
-      <c r="I5" s="28" t="n">
-        <v>-8.84</v>
+        <v>-3.38</v>
+      </c>
+      <c r="I5" s="27" t="n">
+        <v>-10.84</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H6" s="27" t="n">
-        <v>10.88</v>
-      </c>
-      <c r="I6" s="28" t="n">
-        <v>-9.279999999999999</v>
-      </c>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H6" s="25" t="n"/>
+      <c r="I6" s="25" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H7" s="27" t="n">
-        <v>2.12</v>
-      </c>
-      <c r="I7" s="27" t="n">
-        <v>2.54</v>
-      </c>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H7" s="25" t="n"/>
+      <c r="I7" s="25" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H8" s="25" t="n"/>
-      <c r="I8" s="25" t="n"/>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H8" s="29" t="n">
+        <v>8.609999999999999</v>
+      </c>
+      <c r="I8" s="29" t="n">
+        <v>10.05</v>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="H9" s="25" t="n"/>
@@ -3362,7 +3364,7 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>에코프로</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
@@ -3379,25 +3381,25 @@
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H10" s="27" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="I10" s="28" t="n">
-        <v>-8.49</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H10" s="29" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I10" s="29" t="n">
+        <v>0.4</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
@@ -3414,227 +3416,227 @@
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H11" s="25" t="n"/>
-      <c r="I11" s="25" t="n"/>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H11" s="29" t="n">
+        <v>4.68</v>
+      </c>
+      <c r="I11" s="29" t="n">
+        <v>2.76</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="H12" s="27" t="n">
-        <v>2.07</v>
+        <v>-4.19</v>
       </c>
       <c r="I12" s="27" t="n">
-        <v>2.39</v>
+        <v>-1.84</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>진흥기업</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H13" s="25" t="n"/>
-      <c r="I13" s="25" t="n"/>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H13" s="29" t="n">
+        <v>14.32</v>
+      </c>
+      <c r="I13" s="29" t="n">
+        <v>37</v>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>코퍼스코리아</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H14" s="27" t="n">
-        <v>18.24</v>
-      </c>
-      <c r="I14" s="27" t="n">
-        <v>90.31999999999999</v>
-      </c>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H14" s="25" t="n"/>
+      <c r="I14" s="25" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="25" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E15" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H15" s="28" t="n">
-        <v>-2.38</v>
-      </c>
-      <c r="I15" s="27" t="n">
-        <v>7.8</v>
-      </c>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H15" s="25" t="n"/>
+      <c r="I15" s="25" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>LG이노텍</t>
+          <t>삼호개발</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C16" s="25" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D16" s="25" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E16" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H16" s="28" t="n">
-        <v>-0.23</v>
-      </c>
-      <c r="I16" s="28" t="n">
-        <v>-6.34</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H16" s="29" t="n">
+        <v>14.25</v>
+      </c>
+      <c r="I16" s="29" t="n">
+        <v>19.94</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>한화시스템</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="25" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E17" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H17" s="27" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="I17" s="27" t="n">
-        <v>2.85</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H17" s="29" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="I17" s="29" t="n">
+        <v>4.39</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>에코프로비엠</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -3651,60 +3653,52 @@
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H18" s="28" t="n">
-        <v>-0.88</v>
-      </c>
-      <c r="I18" s="28" t="n">
-        <v>-6.96</v>
-      </c>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H18" s="25" t="n"/>
+      <c r="I18" s="25" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H19" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="27" t="n">
-        <v>7.36</v>
-      </c>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H19" s="25" t="n"/>
+      <c r="I19" s="25" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>다보링크</t>
+          <t>SK스퀘어</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
@@ -3721,25 +3715,25 @@
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H20" s="28" t="n">
-        <v>-9.92</v>
-      </c>
-      <c r="I20" s="28" t="n">
-        <v>-36.8</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H20" s="27" t="n">
+        <v>-5.92</v>
+      </c>
+      <c r="I20" s="27" t="n">
+        <v>-8.84</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>다스코</t>
+          <t>광진실업</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -3756,25 +3750,25 @@
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H21" s="28" t="n">
-        <v>-7.72</v>
-      </c>
-      <c r="I21" s="27" t="n">
-        <v>0.87</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H21" s="27" t="n">
+        <v>-12.31</v>
+      </c>
+      <c r="I21" s="29" t="n">
+        <v>19.44</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>다스코</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -3791,25 +3785,25 @@
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H22" s="27" t="n">
-        <v>6.48</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H22" s="29" t="n">
+        <v>1.88</v>
       </c>
       <c r="I22" s="27" t="n">
-        <v>6.21</v>
+        <v>-20.94</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>삼호개발</t>
+          <t>코오롱티슈진</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3826,25 +3820,25 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H23" s="28" t="n">
-        <v>-13.27</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H23" s="27" t="n">
+        <v>-2.21</v>
       </c>
       <c r="I23" s="27" t="n">
-        <v>2.71</v>
+        <v>-9.34</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3861,262 +3855,266 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H24" s="27" t="n">
-        <v>2.05</v>
-      </c>
-      <c r="I24" s="27" t="n">
-        <v>43.93</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H24" s="29" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="I24" s="29" t="n">
+        <v>1.01</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>썸에이지</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C25" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D25" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E25" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H25" s="28" t="n">
-        <v>-10.87</v>
-      </c>
-      <c r="I25" s="27" t="n">
-        <v>3.7</v>
-      </c>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H25" s="25" t="n"/>
+      <c r="I25" s="25" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>다보링크</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C26" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D26" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E26" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H26" s="25" t="n"/>
-      <c r="I26" s="25" t="n"/>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H26" s="29" t="n">
+        <v>4.24</v>
+      </c>
+      <c r="I26" s="27" t="n">
+        <v>-34.17</v>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>진흥기업</t>
+          <t>모바일어플라이언스</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C27" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D27" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E27" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H27" s="28" t="n">
-        <v>-18.04</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H27" s="25" t="n">
+        <v>0</v>
       </c>
       <c r="I27" s="27" t="n">
-        <v>30</v>
+        <v>-19.24</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C28" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D28" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E28" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H28" s="25" t="n"/>
-      <c r="I28" s="25" t="n"/>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H28" s="27" t="n">
+        <v>-8.09</v>
+      </c>
+      <c r="I28" s="27" t="n">
+        <v>-10.3</v>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>기아</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C29" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D29" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E29" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="H29" s="27" t="n">
-        <v>4.68</v>
-      </c>
-      <c r="I29" s="27" t="n">
-        <v>12.34</v>
+        <v>-11.91</v>
+      </c>
+      <c r="I29" s="29" t="n">
+        <v>14.19</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>모바일어플라이언스</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C30" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D30" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E30" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H30" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" s="28" t="n">
-        <v>-22.19</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H30" s="29" t="n">
+        <v>3.74</v>
+      </c>
+      <c r="I30" s="29" t="n">
+        <v>1.68</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>콘텐트리중앙</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C31" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D31" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E31" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H31" s="28" t="n">
-        <v>-28.9</v>
-      </c>
-      <c r="I31" s="28" t="n">
-        <v>-65.13</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H31" s="29" t="n">
+        <v>30</v>
+      </c>
+      <c r="I31" s="29" t="n">
+        <v>43.44</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>HMM</t>
+          <t>금호전기</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -4133,25 +4131,25 @@
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H32" s="27" t="n">
-        <v>0.37</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H32" s="29" t="n">
+        <v>29.96</v>
       </c>
       <c r="I32" s="27" t="n">
-        <v>4.7</v>
+        <v>-12.3</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4168,25 +4166,25 @@
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H33" s="28" t="n">
-        <v>-1.1</v>
-      </c>
-      <c r="I33" s="27" t="n">
-        <v>2.87</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H33" s="29" t="n">
+        <v>5.72</v>
+      </c>
+      <c r="I33" s="29" t="n">
+        <v>14.3</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>동신건설</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4203,25 +4201,25 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H34" s="27" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="I34" s="28" t="n">
-        <v>-2.46</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H34" s="29" t="n">
+        <v>15.17</v>
+      </c>
+      <c r="I34" s="29" t="n">
+        <v>45.07</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>TSMC</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -4238,21 +4236,25 @@
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H35" s="25" t="n"/>
-      <c r="I35" s="25" t="n"/>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H35" s="27" t="n">
+        <v>-0.8100000000000001</v>
+      </c>
+      <c r="I35" s="27" t="n">
+        <v>-2.84</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>골프존홀딩스</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
@@ -4269,25 +4271,25 @@
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H36" s="27" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I36" s="27" t="n">
-        <v>56.05</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H36" s="29" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="I36" s="29" t="n">
+        <v>10.57</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>신원종합개발</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
@@ -4304,25 +4306,25 @@
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H37" s="28" t="n">
-        <v>-19.01</v>
-      </c>
-      <c r="I37" s="27" t="n">
-        <v>43.29</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H37" s="29" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="I37" s="29" t="n">
+        <v>20.09</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>금호전기</t>
+          <t>아난티</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4339,25 +4341,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H38" s="28" t="n">
-        <v>-24.62</v>
-      </c>
-      <c r="I38" s="28" t="n">
-        <v>-12.31</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H38" s="27" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="I38" s="27" t="n">
+        <v>-6.04</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>에코프로</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4374,25 +4376,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="H39" s="27" t="n">
-        <v>3.27</v>
-      </c>
-      <c r="I39" s="28" t="n">
-        <v>-0.2</v>
+        <v>-2.06</v>
+      </c>
+      <c r="I39" s="27" t="n">
+        <v>-27.54</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>일성건설</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4409,25 +4411,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H40" s="27" t="n">
-        <v>3.96</v>
-      </c>
-      <c r="I40" s="27" t="n">
-        <v>10.67</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H40" s="29" t="n">
+        <v>29.74</v>
+      </c>
+      <c r="I40" s="29" t="n">
+        <v>62.89</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>신원종합개발</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4444,25 +4446,21 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H41" s="28" t="n">
-        <v>-16.77</v>
-      </c>
-      <c r="I41" s="27" t="n">
-        <v>23.49</v>
-      </c>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H41" s="25" t="n"/>
+      <c r="I41" s="25" t="n"/>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>젠큐릭스</t>
+          <t>판타지오</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4479,25 +4477,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H42" s="28" t="n">
-        <v>-4.53</v>
-      </c>
-      <c r="I42" s="28" t="n">
-        <v>-3.15</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H42" s="29" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="I42" s="29" t="n">
+        <v>11.08</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>하이브</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4514,21 +4512,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H43" s="25" t="n"/>
-      <c r="I43" s="25" t="n"/>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H43" s="29" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="I43" s="29" t="n">
+        <v>10.09</v>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4545,56 +4547,60 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H44" s="25" t="n"/>
-      <c r="I44" s="25" t="n"/>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H44" s="27" t="n">
+        <v>-2.58</v>
+      </c>
+      <c r="I44" s="27" t="n">
+        <v>-12.21</v>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>파라다이스</t>
+          <t>HC보광산업</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C45" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D45" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E45" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H45" s="28" t="n">
-        <v>-11.77</v>
-      </c>
-      <c r="I45" s="27" t="n">
-        <v>3.3</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H45" s="29" t="n">
+        <v>7.73</v>
+      </c>
+      <c r="I45" s="29" t="n">
+        <v>40.96</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>HC보광산업</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4611,25 +4617,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="H46" s="27" t="n">
-        <v>9.039999999999999</v>
-      </c>
-      <c r="I46" s="27" t="n">
-        <v>40.38</v>
+        <v>-3.17</v>
+      </c>
+      <c r="I46" s="29" t="n">
+        <v>33.19</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>스트라드비젼</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4646,25 +4652,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H47" s="27" t="n">
-        <v>29.9</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H47" s="29" t="n">
+        <v>7.31</v>
       </c>
       <c r="I47" s="27" t="n">
-        <v>46.17</v>
+        <v>-31.74</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>스트라드비젼</t>
+          <t>아크솔루션스</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4681,25 +4687,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H48" s="28" t="n">
-        <v>-0.76</v>
-      </c>
-      <c r="I48" s="28" t="n">
-        <v>-36.39</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H48" s="29" t="n">
+        <v>23.14</v>
+      </c>
+      <c r="I48" s="29" t="n">
+        <v>29.57</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>아크솔루션스</t>
+          <t>에스폴리텍</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4716,25 +4722,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H49" s="27" t="n">
-        <v>27.37</v>
-      </c>
-      <c r="I49" s="28" t="n">
-        <v>-97.27</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H49" s="29" t="n">
+        <v>13.96</v>
+      </c>
+      <c r="I49" s="29" t="n">
+        <v>55.29</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>에스폴리텍</t>
+          <t>우원개발</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4751,25 +4757,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H50" s="28" t="n">
-        <v>-1.56</v>
-      </c>
-      <c r="I50" s="27" t="n">
-        <v>35.61</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H50" s="29" t="n">
+        <v>5.91</v>
+      </c>
+      <c r="I50" s="29" t="n">
+        <v>33.86</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>우원개발</t>
+          <t>위메이드맥스</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4786,19 +4792,19 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H51" s="27" t="n">
-        <v>4.47</v>
-      </c>
-      <c r="I51" s="27" t="n">
-        <v>42.99</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H51" s="29" t="n">
+        <v>20.44</v>
+      </c>
+      <c r="I51" s="29" t="n">
+        <v>43.74</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
@@ -4821,19 +4827,19 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="H52" s="27" t="n">
-        <v>29.96</v>
-      </c>
-      <c r="I52" s="28" t="n">
-        <v>-9.93</v>
+        <v>-11.59</v>
+      </c>
+      <c r="I52" s="27" t="n">
+        <v>-20.37</v>
       </c>
     </row>
   </sheetData>
@@ -4917,19 +4923,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4948,19 +4954,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4972,26 +4978,26 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="35" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B5" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5003,26 +5009,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5034,26 +5040,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5065,26 +5071,26 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5096,26 +5102,26 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B9" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5134,19 +5140,19 @@
         <v>1</v>
       </c>
       <c r="C10" s="36" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D10" s="36" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="E10" s="36" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F10" s="37" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G10" s="37" t="inlineStr">
@@ -5165,19 +5171,19 @@
         <v>1</v>
       </c>
       <c r="C11" s="36" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D11" s="36" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E11" s="36" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F11" s="37" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G11" s="37" t="inlineStr">
@@ -5206,12 +5212,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F12" s="29" t="inlineStr">
+      <c r="F12" s="28" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G12" s="29" t="inlineStr"/>
+      <c r="G12" s="28" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
@@ -5233,12 +5239,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F13" s="29" t="inlineStr">
+      <c r="F13" s="28" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G13" s="29" t="inlineStr"/>
+      <c r="G13" s="28" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
@@ -5260,17 +5266,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F14" s="29" t="inlineStr">
+      <c r="F14" s="28" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G14" s="29" t="inlineStr"/>
+      <c r="G14" s="28" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5287,17 +5293,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F15" s="29" t="inlineStr">
+      <c r="F15" s="28" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G15" s="29" t="inlineStr"/>
+      <c r="G15" s="28" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -5314,17 +5320,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F16" s="29" t="inlineStr">
+      <c r="F16" s="28" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G16" s="29" t="inlineStr"/>
+      <c r="G16" s="28" t="inlineStr"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>핀테크</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -5341,17 +5347,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F17" s="29" t="inlineStr">
+      <c r="F17" s="28" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G17" s="29" t="inlineStr"/>
+      <c r="G17" s="28" t="inlineStr"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -5368,17 +5374,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F18" s="29" t="inlineStr">
+      <c r="F18" s="28" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G18" s="29" t="inlineStr"/>
+      <c r="G18" s="28" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>핀테크</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -5395,17 +5401,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F19" s="29" t="inlineStr">
+      <c r="F19" s="28" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G19" s="29" t="inlineStr"/>
+      <c r="G19" s="28" t="inlineStr"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
@@ -5422,12 +5428,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F20" s="29" t="inlineStr">
+      <c r="F20" s="28" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G20" s="29" t="inlineStr"/>
+      <c r="G20" s="28" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
@@ -5449,12 +5455,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F21" s="29" t="inlineStr">
+      <c r="F21" s="28" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G21" s="29" t="inlineStr"/>
+      <c r="G21" s="28" t="inlineStr"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
@@ -5476,12 +5482,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F22" s="29" t="inlineStr">
+      <c r="F22" s="28" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G22" s="29" t="inlineStr"/>
+      <c r="G22" s="28" t="inlineStr"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
@@ -5503,12 +5509,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F23" s="29" t="inlineStr">
+      <c r="F23" s="28" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G23" s="29" t="inlineStr"/>
+      <c r="G23" s="28" t="inlineStr"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
@@ -5530,12 +5536,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F24" s="29" t="inlineStr">
+      <c r="F24" s="28" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G24" s="29" t="inlineStr"/>
+      <c r="G24" s="28" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
auto: 2026-07-11 07:04 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-07-10 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-07-11 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-10) 상위: SK  점수 72.0점</t>
+          <t>⚡ 최신(2026-07-11) 상위: SK  점수 132.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-10) 상위: 반도체  점수 70.0점</t>
+          <t>⚡ 최신(2026-07-11) 상위: SK하이닉스  점수 121.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-10) 상위: SK하이닉스  점수 61.0점</t>
+          <t>⚡ 최신(2026-07-11) 상위: 반도체  점수 83.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>72</v>
+        <v>132</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>72</v>
+        <v>132</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -940,14 +940,14 @@
         <v>0</v>
       </c>
       <c r="H14" s="17" t="n">
-        <v>2.35</v>
+        <v>7.7</v>
       </c>
       <c r="I14" s="18" t="n">
-        <v>-10.69</v>
+        <v>-4.78</v>
       </c>
       <c r="J14" s="19" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K14" s="19" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -967,42 +967,42 @@
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>반도체</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>70</v>
+        <v>121</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>70</v>
+        <v>116</v>
       </c>
       <c r="F15" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G15" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I15" s="15" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H15" s="18" t="n">
+        <v>-0.27</v>
+      </c>
+      <c r="I15" s="18" t="n">
+        <v>-10.1</v>
       </c>
       <c r="J15" s="19" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100% / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K15" s="19" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1010,14 +1010,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>반도체</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>61</v>
+        <v>83</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>61</v>
+        <v>83</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1025,27 +1025,27 @@
       <c r="G16" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="17" t="n">
-        <v>5.3</v>
-      </c>
-      <c r="I16" s="18" t="n">
-        <v>-0.05</v>
+      <c r="H16" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I16" s="15" t="n">
+        <v/>
       </c>
       <c r="J16" s="19" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K16" s="19" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1053,14 +1053,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1068,27 +1068,27 @@
       <c r="G17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I17" s="15" t="n">
-        <v/>
+      <c r="H17" s="17" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="I17" s="18" t="n">
+        <v>-7.92</v>
       </c>
       <c r="J17" s="19" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>중요공시 3건 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K17" s="19" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1100,10 +1100,10 @@
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1111,25 +1111,27 @@
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="18" t="n">
-        <v>-1.17</v>
+      <c r="H18" s="15" t="n">
+        <v>0</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>2.32</v>
+        <v>0.2</v>
       </c>
       <c r="J18" s="19" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K18" s="19" t="n">
-        <v/>
+          <t>Google 급상승 검색어 등장 (KR) / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K18" s="19" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1137,14 +1139,14 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1152,27 +1154,27 @@
       <c r="G19" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="17" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="I19" s="18" t="n">
-        <v>-2.8</v>
+      <c r="H19" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I19" s="15" t="n">
+        <v/>
       </c>
       <c r="J19" s="19" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K19" s="19" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1180,14 +1182,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1195,25 +1197,27 @@
       <c r="G20" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="18" t="n">
-        <v>-3.68</v>
-      </c>
-      <c r="I20" s="18" t="n">
-        <v>-7.57</v>
+      <c r="H20" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I20" s="15" t="n">
+        <v/>
       </c>
       <c r="J20" s="19" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K20" s="19" t="n">
-        <v/>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K20" s="19" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1221,7 +1225,7 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
@@ -1236,15 +1240,15 @@
       <c r="G21" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I21" s="15" t="n">
-        <v/>
+      <c r="H21" s="17" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="I21" s="18" t="n">
+        <v>-7.01</v>
       </c>
       <c r="J21" s="19" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K21" s="19" t="inlineStr">
@@ -1256,7 +1260,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1264,7 +1268,7 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
@@ -1287,7 +1291,7 @@
       </c>
       <c r="J22" s="19" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K22" s="19" t="n">
@@ -1297,7 +1301,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1305,14 +1309,14 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F23" s="15" t="n">
         <v>0</v>
@@ -1320,25 +1324,27 @@
       <c r="G23" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="18" t="n">
-        <v>-2.89</v>
-      </c>
-      <c r="I23" s="18" t="n">
-        <v>-4.54</v>
+      <c r="H23" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I23" s="15" t="n">
+        <v/>
       </c>
       <c r="J23" s="19" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K23" s="19" t="n">
-        <v/>
+          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K23" s="19" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1346,7 +1352,7 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
@@ -1369,17 +1375,19 @@
       </c>
       <c r="J24" s="19" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K24" s="19" t="n">
-        <v/>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K24" s="19" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1387,14 +1395,14 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F25" s="15" t="n">
         <v>0</v>
@@ -1410,7 +1418,7 @@
       </c>
       <c r="J25" s="19" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K25" s="19" t="inlineStr">
@@ -1422,7 +1430,7 @@
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1430,40 +1438,42 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>에이피알</t>
+          <t>다스코</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="F26" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G26" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="18" t="n">
-        <v>-5.19</v>
-      </c>
-      <c r="I26" s="18" t="n">
-        <v>-9.08</v>
+        <v>3</v>
+      </c>
+      <c r="H26" s="17" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="I26" s="17" t="n">
+        <v>45.17</v>
       </c>
       <c r="J26" s="19" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K26" s="19" t="n">
-        <v/>
+          <t>중요공시 4건 / 중요공시 3일 +100% / 중요공시 7일 +300%</t>
+        </is>
+      </c>
+      <c r="K26" s="19" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -1471,7 +1481,7 @@
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>다스코</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="D27" s="15" t="n">
@@ -1486,15 +1496,15 @@
       <c r="G27" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="H27" s="18" t="n">
-        <v>-4.62</v>
+      <c r="H27" s="17" t="n">
+        <v>10.97</v>
       </c>
       <c r="I27" s="17" t="n">
-        <v>32.09</v>
+        <v>0.23</v>
       </c>
       <c r="J27" s="19" t="inlineStr">
         <is>
-          <t>중요공시 6건 / 중요공시 3일 +200% / 중요공시 7일 +500%</t>
+          <t>중요공시 5건 / 중요공시 3일 +150% / 중요공시 7일 +67%</t>
         </is>
       </c>
       <c r="K27" s="19" t="inlineStr">
@@ -1506,7 +1516,7 @@
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B28" s="15" t="n">
@@ -1514,14 +1524,14 @@
       </c>
       <c r="C28" s="16" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>리가켐바이오</t>
         </is>
       </c>
       <c r="D28" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E28" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F28" s="15" t="n">
         <v>0</v>
@@ -1529,27 +1539,27 @@
       <c r="G28" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H28" s="18" t="n">
-        <v>-9.09</v>
+      <c r="H28" s="17" t="n">
+        <v>1.78</v>
       </c>
       <c r="I28" s="18" t="n">
-        <v>-7.44</v>
+        <v>-10.02</v>
       </c>
       <c r="J28" s="19" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K28" s="19" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B29" s="15" t="n">
@@ -1557,7 +1567,7 @@
       </c>
       <c r="C29" s="16" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>HLB</t>
         </is>
       </c>
       <c r="D29" s="15" t="n">
@@ -1572,111 +1582,111 @@
       <c r="G29" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H29" s="15" t="n">
+      <c r="H29" s="18" t="n">
+        <v>-29.89</v>
+      </c>
+      <c r="I29" s="18" t="n">
+        <v>-24.3</v>
+      </c>
+      <c r="J29" s="19" t="inlineStr">
+        <is>
+          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K29" s="19" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>원전</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="F30" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="15" t="n">
         <v/>
       </c>
-      <c r="I29" s="15" t="n">
+      <c r="I30" s="15" t="n">
         <v/>
       </c>
-      <c r="J29" s="19" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K29" s="19" t="inlineStr">
+      <c r="J30" s="19" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K30" s="19" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>조선</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="E31" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="F31" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I31" s="15" t="n">
+        <v/>
+      </c>
+      <c r="J31" s="19" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K31" s="19" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
-      </c>
-    </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="20" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="B30" s="20" t="n">
-        <v>17</v>
-      </c>
-      <c r="C30" s="21" t="inlineStr">
-        <is>
-          <t>한성기업</t>
-        </is>
-      </c>
-      <c r="D30" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E30" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="F30" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="22" t="n">
-        <v>29.94</v>
-      </c>
-      <c r="I30" s="22" t="n">
-        <v>52.1</v>
-      </c>
-      <c r="J30" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +2287% / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K30" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="20" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="B31" s="20" t="n">
-        <v>18</v>
-      </c>
-      <c r="C31" s="21" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="D31" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E31" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="F31" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" s="22" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="I31" s="22" t="n">
-        <v>7.65</v>
-      </c>
-      <c r="J31" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K31" s="23" t="n">
-        <v/>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1684,42 +1694,42 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>주성코퍼레이션</t>
+          <t>모아데이타</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F32" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G32" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H32" s="22" t="n">
-        <v>6.15</v>
-      </c>
-      <c r="I32" s="24" t="n">
-        <v>-13.48</v>
+        <v>1.68</v>
+      </c>
+      <c r="I32" s="22" t="n">
+        <v>1.04</v>
       </c>
       <c r="J32" s="23" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 3건 / 중요공시 7일 +200%</t>
         </is>
       </c>
       <c r="K32" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1727,42 +1737,42 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>서남</t>
+          <t>모아라이프플러스</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F33" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G33" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H33" s="24" t="n">
-        <v>-1.97</v>
-      </c>
-      <c r="I33" s="24" t="n">
-        <v>-3.86</v>
+        <v>-2.52</v>
+      </c>
+      <c r="I33" s="22" t="n">
+        <v>3.48</v>
       </c>
       <c r="J33" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K33" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1770,7 +1780,7 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>한화</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
@@ -1785,11 +1795,11 @@
       <c r="G34" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="24" t="n">
-        <v>-1.93</v>
-      </c>
-      <c r="I34" s="24" t="n">
-        <v>-11.67</v>
+      <c r="H34" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I34" s="20" t="n">
+        <v/>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
@@ -1803,7 +1813,7 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1811,7 +1821,7 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>한성기업</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
@@ -1826,25 +1836,27 @@
       <c r="G35" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H35" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I35" s="20" t="n">
-        <v/>
+      <c r="H35" s="22" t="n">
+        <v>29.95</v>
+      </c>
+      <c r="I35" s="22" t="n">
+        <v>100</v>
       </c>
       <c r="J35" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K35" s="23" t="n">
-        <v/>
+          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K35" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1852,7 +1864,7 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>스테이블코인</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
@@ -1875,19 +1887,17 @@
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K36" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K36" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1895,7 +1905,7 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>삼성SDI</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
@@ -1910,15 +1920,15 @@
       <c r="G37" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H37" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I37" s="20" t="n">
-        <v/>
+      <c r="H37" s="22" t="n">
+        <v>8.09</v>
+      </c>
+      <c r="I37" s="24" t="n">
+        <v>-7.17</v>
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K37" s="23" t="n">
@@ -1928,7 +1938,7 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1936,40 +1946,42 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>NH투자증권</t>
+          <t>PS일렉트로닉스</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F38" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H38" s="24" t="n">
-        <v>-4.57</v>
+      <c r="H38" s="22" t="n">
+        <v>9.300000000000001</v>
       </c>
       <c r="I38" s="22" t="n">
-        <v>1.04</v>
+        <v>18.41</v>
       </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K38" s="23" t="n">
-        <v/>
+          <t>중요공시 3건 / 중요공시 3일 +50%</t>
+        </is>
+      </c>
+      <c r="K38" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1977,42 +1989,42 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>일성건설</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F39" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G39" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H39" s="24" t="n">
-        <v>-0.62</v>
+      <c r="H39" s="22" t="n">
+        <v>6.3</v>
       </c>
       <c r="I39" s="22" t="n">
-        <v>0.25</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 3건 / 중요공시 3일 +200%</t>
         </is>
       </c>
       <c r="K39" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2020,42 +2032,40 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>SK증권</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F40" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G40" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H40" s="22" t="n">
-        <v>6.8</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="I40" s="24" t="n">
-        <v>-8.859999999999999</v>
+        <v>-4.65</v>
       </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 중요공시 3일 +300%</t>
-        </is>
-      </c>
-      <c r="K40" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K40" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2063,7 +2073,7 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
@@ -2078,27 +2088,25 @@
       <c r="G41" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="20" t="n">
+      <c r="H41" s="22" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="I41" s="24" t="n">
+        <v>-2.45</v>
+      </c>
+      <c r="J41" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K41" s="23" t="n">
         <v/>
-      </c>
-      <c r="I41" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J41" s="23" t="inlineStr">
-        <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K41" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2106,14 +2114,14 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>데이타솔루션</t>
+          <t>대덕전자</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E42" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F42" s="20" t="n">
         <v>0</v>
@@ -2122,26 +2130,24 @@
         <v>0</v>
       </c>
       <c r="H42" s="22" t="n">
-        <v>29.97</v>
-      </c>
-      <c r="I42" s="22" t="n">
-        <v>70.42</v>
+        <v>7.95</v>
+      </c>
+      <c r="I42" s="24" t="n">
+        <v>-6.71</v>
       </c>
       <c r="J42" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +284% / 중요공시 2건</t>
-        </is>
-      </c>
-      <c r="K42" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K42" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2149,14 +2155,14 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>광무</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E43" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F43" s="20" t="n">
         <v>0</v>
@@ -2164,27 +2170,27 @@
       <c r="G43" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H43" s="24" t="n">
-        <v>-4.94</v>
-      </c>
-      <c r="I43" s="22" t="n">
-        <v>5.77</v>
+      <c r="H43" s="22" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="I43" s="24" t="n">
+        <v>-4.5</v>
       </c>
       <c r="J43" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +155% / 중요공시 1건</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K43" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2192,42 +2198,42 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E44" s="20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F44" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G44" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H44" s="24" t="n">
-        <v>-2.09</v>
-      </c>
-      <c r="I44" s="24" t="n">
-        <v>-1.98</v>
+        <v>0</v>
+      </c>
+      <c r="H44" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I44" s="20" t="n">
+        <v/>
       </c>
       <c r="J44" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K44" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2235,42 +2241,40 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>비츠로셀</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E45" s="20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F45" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G45" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H45" s="24" t="n">
-        <v>-0.16</v>
+        <v>0</v>
+      </c>
+      <c r="H45" s="22" t="n">
+        <v>1.86</v>
       </c>
       <c r="I45" s="24" t="n">
-        <v>-14.65</v>
+        <v>-2.96</v>
       </c>
       <c r="J45" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K45" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K45" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
@@ -2278,42 +2282,40 @@
       </c>
       <c r="C46" s="21" t="inlineStr">
         <is>
-          <t>HJ중공업</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="D46" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E46" s="20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F46" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G46" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H46" s="24" t="n">
-        <v>-1.3</v>
-      </c>
-      <c r="I46" s="24" t="n">
-        <v>-12.49</v>
+        <v>0</v>
+      </c>
+      <c r="H46" s="22" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="I46" s="22" t="n">
+        <v>9.859999999999999</v>
       </c>
       <c r="J46" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K46" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K46" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B47" s="20" t="n">
@@ -2321,7 +2323,7 @@
       </c>
       <c r="C47" s="21" t="inlineStr">
         <is>
-          <t>SK스퀘어</t>
+          <t>데이타솔루션</t>
         </is>
       </c>
       <c r="D47" s="20" t="n">
@@ -2336,27 +2338,27 @@
       <c r="G47" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H47" s="22" t="n">
-        <v>4.49</v>
-      </c>
-      <c r="I47" s="24" t="n">
-        <v>-12.98</v>
+      <c r="H47" s="24" t="n">
+        <v>-5.44</v>
+      </c>
+      <c r="I47" s="22" t="n">
+        <v>54.99</v>
       </c>
       <c r="J47" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>네이버 검색 당일 +773% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K47" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B48" s="20" t="n">
@@ -2364,7 +2366,7 @@
       </c>
       <c r="C48" s="21" t="inlineStr">
         <is>
-          <t>리가켐바이오</t>
+          <t>씨이랩</t>
         </is>
       </c>
       <c r="D48" s="20" t="n">
@@ -2380,14 +2382,14 @@
         <v>0</v>
       </c>
       <c r="H48" s="24" t="n">
-        <v>-1.83</v>
-      </c>
-      <c r="I48" s="24" t="n">
-        <v>-17.28</v>
+        <v>-6.85</v>
+      </c>
+      <c r="I48" s="22" t="n">
+        <v>23.04</v>
       </c>
       <c r="J48" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버 검색 당일 +238% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K48" s="23" t="inlineStr">
@@ -2399,7 +2401,7 @@
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B49" s="20" t="n">
@@ -2407,7 +2409,7 @@
       </c>
       <c r="C49" s="21" t="inlineStr">
         <is>
-          <t>한화에어로스페이스</t>
+          <t>웰킵스하이텍</t>
         </is>
       </c>
       <c r="D49" s="20" t="n">
@@ -2422,27 +2424,27 @@
       <c r="G49" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="24" t="n">
-        <v>-8.449999999999999</v>
-      </c>
-      <c r="I49" s="24" t="n">
-        <v>-14.61</v>
+      <c r="H49" s="22" t="n">
+        <v>23.33</v>
+      </c>
+      <c r="I49" s="22" t="n">
+        <v>66.29000000000001</v>
       </c>
       <c r="J49" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +105% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K49" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B50" s="20" t="n">
@@ -2450,7 +2452,7 @@
       </c>
       <c r="C50" s="21" t="inlineStr">
         <is>
-          <t>모비스</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="D50" s="20" t="n">
@@ -2466,24 +2468,26 @@
         <v>0</v>
       </c>
       <c r="H50" s="22" t="n">
-        <v>0.6</v>
+        <v>3.44</v>
       </c>
       <c r="I50" s="24" t="n">
-        <v>-3.07</v>
+        <v>-23.95</v>
       </c>
       <c r="J50" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K50" s="23" t="n">
-        <v/>
+          <t>네이버 검색 당일 +52% / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K50" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B51" s="20" t="n">
@@ -2491,7 +2495,7 @@
       </c>
       <c r="C51" s="21" t="inlineStr">
         <is>
-          <t>카카오페이</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="D51" s="20" t="n">
@@ -2506,25 +2510,27 @@
       <c r="G51" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H51" s="24" t="n">
-        <v>-1.83</v>
+      <c r="H51" s="22" t="n">
+        <v>0.19</v>
       </c>
       <c r="I51" s="24" t="n">
-        <v>-7.76</v>
+        <v>-7.28</v>
       </c>
       <c r="J51" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K51" s="23" t="n">
-        <v/>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K51" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B52" s="20" t="n">
@@ -2532,40 +2538,42 @@
       </c>
       <c r="C52" s="21" t="inlineStr">
         <is>
-          <t>롯데관광개발</t>
+          <t>유티아이</t>
         </is>
       </c>
       <c r="D52" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E52" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F52" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G52" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H52" s="24" t="n">
-        <v>-6.07</v>
+        <v>-6.91</v>
       </c>
       <c r="I52" s="24" t="n">
-        <v>-4.4</v>
+        <v>-19.29</v>
       </c>
       <c r="J52" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K52" s="23" t="n">
-        <v/>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K52" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B53" s="20" t="n">
@@ -2573,7 +2581,7 @@
       </c>
       <c r="C53" s="21" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>조이웍스앤코</t>
         </is>
       </c>
       <c r="D53" s="20" t="n">
@@ -2588,27 +2596,27 @@
       <c r="G53" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I53" s="20" t="n">
-        <v/>
+      <c r="H53" s="24" t="n">
+        <v>-0.75</v>
+      </c>
+      <c r="I53" s="22" t="n">
+        <v>34.84</v>
       </c>
       <c r="J53" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K53" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B54" s="20" t="n">
@@ -2616,7 +2624,7 @@
       </c>
       <c r="C54" s="21" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>롯데관광개발</t>
         </is>
       </c>
       <c r="D54" s="20" t="n">
@@ -2631,68 +2639,68 @@
       <c r="G54" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H54" s="20" t="n">
+      <c r="H54" s="22" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="I54" s="24" t="n">
+        <v>-1.97</v>
+      </c>
+      <c r="J54" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K54" s="23" t="n">
         <v/>
       </c>
-      <c r="I54" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J54" s="23" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K54" s="23" t="inlineStr">
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="25" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B55" s="25" t="n">
+        <v>42</v>
+      </c>
+      <c r="C55" s="26" t="inlineStr">
+        <is>
+          <t>레몬헬스케어</t>
+        </is>
+      </c>
+      <c r="D55" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E55" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F55" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="27" t="n">
+        <v>-0.51</v>
+      </c>
+      <c r="I55" s="28" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="J55" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +1248%</t>
+        </is>
+      </c>
+      <c r="K55" s="29" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
-      </c>
-    </row>
-    <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="20" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="B55" s="20" t="n">
-        <v>42</v>
-      </c>
-      <c r="C55" s="21" t="inlineStr">
-        <is>
-          <t>현대해상</t>
-        </is>
-      </c>
-      <c r="D55" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E55" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F55" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G55" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H55" s="24" t="n">
-        <v>-5.01</v>
-      </c>
-      <c r="I55" s="22" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="J55" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K55" s="23" t="n">
-        <v/>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2700,7 +2708,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>레몬헬스케어</t>
+          <t>금호에이치티</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2716,14 +2724,14 @@
         <v>0</v>
       </c>
       <c r="H56" s="27" t="n">
-        <v>-3.34</v>
+        <v>-3.36</v>
       </c>
       <c r="I56" s="28" t="n">
-        <v>4.79</v>
+        <v>24.17</v>
       </c>
       <c r="J56" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1144%</t>
+          <t>네이버 검색 당일 +666%</t>
         </is>
       </c>
       <c r="K56" s="29" t="inlineStr">
@@ -2735,7 +2743,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2743,7 +2751,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>금호에이치티</t>
+          <t>흥구석유</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2758,11 +2766,11 @@
       <c r="G57" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H57" s="27" t="n">
-        <v>-1.11</v>
+      <c r="H57" s="28" t="n">
+        <v>0.5600000000000001</v>
       </c>
       <c r="I57" s="28" t="n">
-        <v>28.49</v>
+        <v>16.68</v>
       </c>
       <c r="J57" s="29" t="inlineStr">
         <is>
@@ -2778,7 +2786,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2801,15 +2809,15 @@
       <c r="G58" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="27" t="n">
-        <v>-9.380000000000001</v>
+      <c r="H58" s="25" t="n">
+        <v>0</v>
       </c>
       <c r="I58" s="28" t="n">
-        <v>17.13</v>
+        <v>14.82</v>
       </c>
       <c r="J58" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +199%</t>
+          <t>네이버 검색 당일 +261%</t>
         </is>
       </c>
       <c r="K58" s="29" t="inlineStr">
@@ -2821,7 +2829,7 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2829,7 +2837,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>씨이랩</t>
+          <t>모나미</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2845,26 +2853,26 @@
         <v>0</v>
       </c>
       <c r="H59" s="28" t="n">
-        <v>4.04</v>
+        <v>25.66</v>
       </c>
       <c r="I59" s="28" t="n">
-        <v>45.89</v>
+        <v>62.01</v>
       </c>
       <c r="J59" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +93% / 중요공시 2건</t>
+          <t>네이버 검색 당일 +116%</t>
         </is>
       </c>
       <c r="K59" s="29" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2872,7 +2880,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>PS일렉트로닉스</t>
+          <t>흥아해운</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2887,27 +2895,27 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="27" t="n">
-        <v>-1.58</v>
+      <c r="H60" s="28" t="n">
+        <v>6.06</v>
       </c>
       <c r="I60" s="28" t="n">
-        <v>12.02</v>
+        <v>5.67</v>
       </c>
       <c r="J60" s="29" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>네이버 검색 당일 +116%</t>
         </is>
       </c>
       <c r="K60" s="29" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2915,7 +2923,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>LG디스플레이</t>
+          <t>오픈베이스</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2931,24 +2939,26 @@
         <v>0</v>
       </c>
       <c r="H61" s="27" t="n">
-        <v>-4.98</v>
-      </c>
-      <c r="I61" s="27" t="n">
-        <v>-2.73</v>
+        <v>-7.16</v>
+      </c>
+      <c r="I61" s="28" t="n">
+        <v>6.74</v>
       </c>
       <c r="J61" s="29" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K61" s="29" t="n">
-        <v/>
+          <t>네이버 검색 당일 +104%</t>
+        </is>
+      </c>
+      <c r="K61" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2956,7 +2966,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>HMM</t>
+          <t>레이저쎌</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2971,25 +2981,27 @@
       <c r="G62" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H62" s="27" t="n">
-        <v>-3.64</v>
+      <c r="H62" s="28" t="n">
+        <v>23.8</v>
       </c>
       <c r="I62" s="28" t="n">
-        <v>1.15</v>
+        <v>40.2</v>
       </c>
       <c r="J62" s="29" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K62" s="29" t="n">
-        <v/>
+          <t>네이버 검색 당일 +59% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K62" s="29" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
       </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -2997,7 +3009,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>매드업</t>
+          <t>우리금융지주</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3013,20 +3025,18 @@
         <v>0</v>
       </c>
       <c r="H63" s="28" t="n">
-        <v>8.289999999999999</v>
+        <v>4.66</v>
       </c>
       <c r="I63" s="28" t="n">
-        <v>2.88</v>
+        <v>2.28</v>
       </c>
       <c r="J63" s="29" t="inlineStr">
         <is>
-          <t>중요공시 4건</t>
-        </is>
-      </c>
-      <c r="K63" s="29" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K63" s="29" t="n">
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -3122,96 +3132,96 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>72</v>
+        <v>132</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>72</v>
+        <v>132</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="H3" s="28" t="n">
-        <v>2.35</v>
+        <v>7.7</v>
       </c>
       <c r="I3" s="27" t="n">
-        <v>-10.69</v>
+        <v>-4.78</v>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>반도체</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B4" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>70</v>
+        <v>121</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>70</v>
+        <v>121</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H4" s="25" t="n"/>
-      <c r="I4" s="25" t="n"/>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H4" s="27" t="n">
+        <v>-0.27</v>
+      </c>
+      <c r="I4" s="27" t="n">
+        <v>-10.1</v>
+      </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>반도체</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>61</v>
+        <v>83</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>61</v>
+        <v>83</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H5" s="28" t="n">
-        <v>5.3</v>
-      </c>
-      <c r="I5" s="27" t="n">
-        <v>-0.05</v>
-      </c>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H5" s="25" t="n"/>
+      <c r="I5" s="25" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
@@ -3223,136 +3233,132 @@
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H6" s="27" t="n">
-        <v>-1.17</v>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H6" s="25" t="n">
+        <v>0</v>
       </c>
       <c r="I6" s="28" t="n">
-        <v>2.32</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H7" s="25" t="n"/>
-      <c r="I7" s="25" t="n"/>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H7" s="28" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="I7" s="27" t="n">
+        <v>-7.92</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H8" s="28" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="I8" s="27" t="n">
-        <v>-2.8</v>
-      </c>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H8" s="25" t="n"/>
+      <c r="I8" s="25" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H9" s="27" t="n">
-        <v>-3.68</v>
-      </c>
-      <c r="I9" s="27" t="n">
-        <v>-7.57</v>
-      </c>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H9" s="25" t="n"/>
+      <c r="I9" s="25" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
@@ -3369,16 +3375,20 @@
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H10" s="25" t="n"/>
-      <c r="I10" s="25" t="n"/>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H10" s="28" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="I10" s="27" t="n">
+        <v>-7.01</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
@@ -3400,12 +3410,12 @@
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="H11" s="25" t="n"/>
@@ -3421,22 +3431,22 @@
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="H12" s="25" t="n"/>
@@ -3445,7 +3455,7 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -3462,12 +3472,12 @@
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="H13" s="25" t="n"/>
@@ -3476,77 +3486,73 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H14" s="27" t="n">
-        <v>-2.89</v>
-      </c>
-      <c r="I14" s="27" t="n">
-        <v>-4.54</v>
-      </c>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H14" s="25" t="n"/>
+      <c r="I14" s="25" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>에이피알</t>
+          <t>다스코</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E15" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H15" s="27" t="n">
-        <v>-5.19</v>
-      </c>
-      <c r="I15" s="27" t="n">
-        <v>-9.08</v>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H15" s="28" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="I15" s="28" t="n">
+        <v>45.17</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -3563,60 +3569,60 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H16" s="27" t="n">
-        <v>-9.09</v>
-      </c>
-      <c r="I16" s="27" t="n">
-        <v>-7.44</v>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H16" s="28" t="n">
+        <v>10.97</v>
+      </c>
+      <c r="I16" s="28" t="n">
+        <v>0.23</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>다스코</t>
+          <t>HLB</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E17" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="H17" s="27" t="n">
-        <v>-4.62</v>
-      </c>
-      <c r="I17" s="28" t="n">
-        <v>32.09</v>
+        <v>-29.89</v>
+      </c>
+      <c r="I17" s="27" t="n">
+        <v>-24.3</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>리가켐바이오</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -3633,91 +3639,87 @@
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H18" s="25" t="n"/>
-      <c r="I18" s="25" t="n"/>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H18" s="28" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="I18" s="27" t="n">
+        <v>-10.02</v>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>NH투자증권</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H19" s="27" t="n">
-        <v>-4.57</v>
-      </c>
-      <c r="I19" s="28" t="n">
-        <v>1.04</v>
-      </c>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H19" s="25" t="n"/>
+      <c r="I19" s="25" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D20" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H20" s="28" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="I20" s="28" t="n">
-        <v>7.65</v>
-      </c>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H20" s="25" t="n"/>
+      <c r="I20" s="25" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>모아데이타</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -3734,21 +3736,25 @@
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H21" s="25" t="n"/>
-      <c r="I21" s="25" t="n"/>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H21" s="28" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="I21" s="28" t="n">
+        <v>1.04</v>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>서남</t>
+          <t>모아라이프플러스</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -3765,25 +3771,25 @@
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="H22" s="27" t="n">
-        <v>-1.97</v>
-      </c>
-      <c r="I22" s="27" t="n">
-        <v>-3.86</v>
+        <v>-2.52</v>
+      </c>
+      <c r="I22" s="28" t="n">
+        <v>3.48</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>삼성SDI</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3800,21 +3806,25 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H23" s="25" t="n"/>
-      <c r="I23" s="25" t="n"/>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H23" s="28" t="n">
+        <v>8.09</v>
+      </c>
+      <c r="I23" s="27" t="n">
+        <v>-7.17</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>스테이블코인</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3831,12 +3841,12 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="H24" s="25" t="n"/>
@@ -3845,7 +3855,7 @@
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>주성코퍼레이션</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3862,20 +3872,16 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H25" s="28" t="n">
-        <v>6.15</v>
-      </c>
-      <c r="I25" s="27" t="n">
-        <v>-13.48</v>
-      </c>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H25" s="25" t="n"/>
+      <c r="I25" s="25" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
@@ -3897,60 +3903,60 @@
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="H26" s="28" t="n">
-        <v>29.94</v>
+        <v>29.95</v>
       </c>
       <c r="I26" s="28" t="n">
-        <v>52.1</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>한화</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C27" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D27" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E27" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H27" s="27" t="n">
-        <v>-1.93</v>
-      </c>
-      <c r="I27" s="27" t="n">
-        <v>-11.67</v>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H27" s="28" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="I27" s="28" t="n">
+        <v>9.859999999999999</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
@@ -3967,25 +3973,25 @@
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H28" s="27" t="n">
-        <v>-0.62</v>
-      </c>
-      <c r="I28" s="28" t="n">
-        <v>0.25</v>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H28" s="28" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="I28" s="27" t="n">
+        <v>-4.5</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>PS일렉트로닉스</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
@@ -4002,25 +4008,25 @@
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="H29" s="28" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="I29" s="27" t="n">
-        <v>-8.859999999999999</v>
+        <v>9.300000000000001</v>
+      </c>
+      <c r="I29" s="28" t="n">
+        <v>18.41</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>SK증권</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -4037,196 +4043,196 @@
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H30" s="25" t="n"/>
-      <c r="I30" s="25" t="n"/>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H30" s="28" t="n">
+        <v>8.609999999999999</v>
+      </c>
+      <c r="I30" s="27" t="n">
+        <v>-4.65</v>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>HJ중공업</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C31" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D31" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E31" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H31" s="27" t="n">
-        <v>-1.3</v>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H31" s="28" t="n">
+        <v>1.86</v>
       </c>
       <c r="I31" s="27" t="n">
-        <v>-12.49</v>
+        <v>-2.96</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>SK스퀘어</t>
+          <t>대덕전자</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C32" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D32" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E32" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="H32" s="28" t="n">
-        <v>4.49</v>
+        <v>7.95</v>
       </c>
       <c r="I32" s="27" t="n">
-        <v>-12.98</v>
+        <v>-6.71</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>광무</t>
+          <t>일성건설</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C33" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D33" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E33" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H33" s="27" t="n">
-        <v>-4.94</v>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H33" s="28" t="n">
+        <v>6.3</v>
       </c>
       <c r="I33" s="28" t="n">
-        <v>5.77</v>
+        <v>8.210000000000001</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>데이타솔루션</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C34" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D34" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E34" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H34" s="28" t="n">
-        <v>29.97</v>
-      </c>
-      <c r="I34" s="28" t="n">
-        <v>70.42</v>
-      </c>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H34" s="25" t="n"/>
+      <c r="I34" s="25" t="n"/>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>롯데관광개발</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D35" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E35" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H35" s="27" t="n">
-        <v>-6.07</v>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H35" s="28" t="n">
+        <v>3.57</v>
       </c>
       <c r="I35" s="27" t="n">
-        <v>-4.4</v>
+        <v>-2.45</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>리가켐바이오</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
@@ -4243,25 +4249,25 @@
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H36" s="27" t="n">
-        <v>-1.83</v>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H36" s="28" t="n">
+        <v>0.19</v>
       </c>
       <c r="I36" s="27" t="n">
-        <v>-17.28</v>
+        <v>-7.28</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>모비스</t>
+          <t>데이타솔루션</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
@@ -4278,25 +4284,25 @@
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H37" s="28" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="I37" s="27" t="n">
-        <v>-3.07</v>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H37" s="27" t="n">
+        <v>-5.44</v>
+      </c>
+      <c r="I37" s="28" t="n">
+        <v>54.99</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>비츠로셀</t>
+          <t>롯데관광개발</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4313,25 +4319,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H38" s="27" t="n">
-        <v>-0.16</v>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H38" s="28" t="n">
+        <v>2.48</v>
       </c>
       <c r="I38" s="27" t="n">
-        <v>-14.65</v>
+        <v>-1.97</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>씨이랩</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4348,25 +4354,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="H39" s="27" t="n">
-        <v>-2.09</v>
-      </c>
-      <c r="I39" s="27" t="n">
-        <v>-1.98</v>
+        <v>-6.85</v>
+      </c>
+      <c r="I39" s="28" t="n">
+        <v>23.04</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>웰킵스하이텍</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4383,21 +4389,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H40" s="25" t="n"/>
-      <c r="I40" s="25" t="n"/>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H40" s="28" t="n">
+        <v>23.33</v>
+      </c>
+      <c r="I40" s="28" t="n">
+        <v>66.29000000000001</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>유티아이</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4414,21 +4424,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H41" s="25" t="n"/>
-      <c r="I41" s="25" t="n"/>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H41" s="27" t="n">
+        <v>-6.91</v>
+      </c>
+      <c r="I41" s="27" t="n">
+        <v>-19.29</v>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>카카오페이</t>
+          <t>조이웍스앤코</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4445,25 +4459,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="H42" s="27" t="n">
-        <v>-1.83</v>
-      </c>
-      <c r="I42" s="27" t="n">
-        <v>-7.76</v>
+        <v>-0.75</v>
+      </c>
+      <c r="I42" s="28" t="n">
+        <v>34.84</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>한화에어로스페이스</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4480,60 +4494,60 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H43" s="27" t="n">
-        <v>-8.449999999999999</v>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H43" s="28" t="n">
+        <v>3.44</v>
       </c>
       <c r="I43" s="27" t="n">
-        <v>-14.61</v>
+        <v>-23.95</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>현대해상</t>
+          <t>금호에이치티</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C44" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D44" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E44" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="H44" s="27" t="n">
-        <v>-5.01</v>
+        <v>-3.36</v>
       </c>
       <c r="I44" s="28" t="n">
-        <v>0.14</v>
+        <v>24.17</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>HMM</t>
+          <t>레몬헬스케어</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4550,25 +4564,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="H45" s="27" t="n">
-        <v>-3.64</v>
+        <v>-0.51</v>
       </c>
       <c r="I45" s="28" t="n">
-        <v>1.15</v>
+        <v>4.26</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>LG디스플레이</t>
+          <t>레이저쎌</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4585,25 +4599,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H46" s="27" t="n">
-        <v>-4.98</v>
-      </c>
-      <c r="I46" s="27" t="n">
-        <v>-2.73</v>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H46" s="28" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="I46" s="28" t="n">
+        <v>40.2</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>PS일렉트로닉스</t>
+          <t>모나미</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4620,25 +4634,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H47" s="27" t="n">
-        <v>-1.58</v>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H47" s="28" t="n">
+        <v>25.66</v>
       </c>
       <c r="I47" s="28" t="n">
-        <v>12.02</v>
+        <v>62.01</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>금호에이치티</t>
+          <t>에스와이</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4655,25 +4669,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H48" s="27" t="n">
-        <v>-1.11</v>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H48" s="25" t="n">
+        <v>0</v>
       </c>
       <c r="I48" s="28" t="n">
-        <v>28.49</v>
+        <v>14.82</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>레몬헬스케어</t>
+          <t>오픈베이스</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4690,25 +4704,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="H49" s="27" t="n">
-        <v>-3.34</v>
+        <v>-7.16</v>
       </c>
       <c r="I49" s="28" t="n">
-        <v>4.79</v>
+        <v>6.74</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>매드업</t>
+          <t>우리금융지주</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4725,25 +4739,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="H50" s="28" t="n">
-        <v>8.289999999999999</v>
+        <v>4.66</v>
       </c>
       <c r="I50" s="28" t="n">
-        <v>2.88</v>
+        <v>2.28</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>씨이랩</t>
+          <t>흥구석유</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4760,25 +4774,25 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="H51" s="28" t="n">
-        <v>4.04</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I51" s="28" t="n">
-        <v>45.89</v>
+        <v>16.68</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="26" t="inlineStr">
         <is>
-          <t>에스와이</t>
+          <t>흥아해운</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -4795,19 +4809,19 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="H52" s="27" t="n">
-        <v>-9.380000000000001</v>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H52" s="28" t="n">
+        <v>6.06</v>
       </c>
       <c r="I52" s="28" t="n">
-        <v>17.13</v>
+        <v>5.67</v>
       </c>
     </row>
   </sheetData>
@@ -4891,19 +4905,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4922,19 +4936,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4960,12 +4974,12 @@
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -4984,19 +4998,19 @@
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5015,19 +5029,19 @@
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5053,12 +5067,12 @@
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5084,12 +5098,12 @@
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5101,26 +5115,26 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="35" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B10" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="36" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D10" s="36" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E10" s="36" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="F10" s="37" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G10" s="37" t="inlineStr">
@@ -5132,26 +5146,26 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="35" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B11" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="36" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D11" s="36" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E11" s="36" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="F11" s="37" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G11" s="37" t="inlineStr">
@@ -5163,7 +5177,7 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="35" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B12" s="36" t="n">
@@ -5177,12 +5191,12 @@
       </c>
       <c r="E12" s="36" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="F12" s="37" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="G12" s="37" t="inlineStr">
@@ -5194,65 +5208,69 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="35" t="inlineStr">
         <is>
+          <t>제약</t>
+        </is>
+      </c>
+      <c r="B13" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="36" t="n">
+        <v>9</v>
+      </c>
+      <c r="D13" s="36" t="n">
+        <v>9</v>
+      </c>
+      <c r="E13" s="36" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="F13" s="37" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="G13" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="35" t="inlineStr">
+        <is>
           <t>인공지능</t>
         </is>
       </c>
-      <c r="B13" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C13" s="36" t="n">
-        <v>22</v>
-      </c>
-      <c r="D13" s="36" t="n">
-        <v>22</v>
-      </c>
-      <c r="E13" s="36" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="F13" s="37" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="G13" s="37" t="inlineStr">
+      <c r="B14" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="36" t="n">
+        <v>18</v>
+      </c>
+      <c r="D14" s="36" t="n">
+        <v>18</v>
+      </c>
+      <c r="E14" s="36" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="F14" s="37" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="G14" s="37" t="inlineStr">
         <is>
           <t>⚡ 관심</t>
         </is>
       </c>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="26" t="inlineStr">
-        <is>
-          <t>이차전지</t>
-        </is>
-      </c>
-      <c r="B14" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F14" s="29" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G14" s="29" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>이차전지</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5279,7 +5297,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -5306,7 +5324,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -5333,7 +5351,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>핀테크</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -5360,7 +5378,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>핀테크</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -5387,7 +5405,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-07-12 07:06 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-07-11 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-07-12 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-11) 상위: SK  점수 132.0점</t>
+          <t>⚡ 최신(2026-07-12) 상위: SK  점수 119.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-11) 상위: SK하이닉스  점수 121.0점</t>
+          <t>⚡ 최신(2026-07-12) 상위: SK하이닉스  점수 101.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-11) 상위: 반도체  점수 83.0점</t>
+          <t>⚡ 최신(2026-07-12) 상위: 반도체  점수 69.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>132</v>
+        <v>119</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>132</v>
+        <v>119</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="19" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K14" s="19" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -971,16 +971,16 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>121</v>
+        <v>101</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>2</v>
       </c>
       <c r="G15" s="15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H15" s="18" t="n">
         <v>-0.27</v>
@@ -990,19 +990,19 @@
       </c>
       <c r="J15" s="19" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100% / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K15" s="19" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1014,10 +1014,10 @@
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="J16" s="19" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K16" s="19" t="inlineStr">
@@ -1045,7 +1045,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1057,13 +1057,13 @@
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F17" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G17" s="15" t="n">
         <v>0</v>
@@ -1076,19 +1076,19 @@
       </c>
       <c r="J17" s="19" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 3건 / 중요공시 3일 +50% / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K17" s="19" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1096,14 +1096,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1112,26 +1112,26 @@
         <v>0</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="17" t="n">
-        <v>0.2</v>
+        <v/>
+      </c>
+      <c r="I18" s="15" t="n">
+        <v/>
       </c>
       <c r="J18" s="19" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR) / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K18" s="19" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1143,10 +1143,10 @@
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="J19" s="19" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K19" s="19" t="inlineStr">
@@ -1174,7 +1174,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1182,14 +1182,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1198,26 +1198,24 @@
         <v>0</v>
       </c>
       <c r="H20" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="17" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J20" s="19" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K20" s="19" t="n">
         <v/>
-      </c>
-      <c r="I20" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J20" s="19" t="inlineStr">
-        <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K20" s="19" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1229,10 +1227,10 @@
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
@@ -1248,19 +1246,17 @@
       </c>
       <c r="J21" s="19" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K21" s="19" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K21" s="19" t="n">
+        <v/>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1268,14 +1264,14 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -1291,17 +1287,19 @@
       </c>
       <c r="J22" s="19" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K22" s="19" t="n">
-        <v/>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K22" s="19" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1313,10 +1311,10 @@
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F23" s="15" t="n">
         <v>0</v>
@@ -1332,19 +1330,17 @@
       </c>
       <c r="J23" s="19" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K23" s="19" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K23" s="19" t="n">
+        <v/>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1352,42 +1348,42 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>다스코</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G24" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I24" s="15" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H24" s="17" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="I24" s="17" t="n">
+        <v>45.17</v>
       </c>
       <c r="J24" s="19" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 4건 / 중요공시 3일 +100% / 중요공시 7일 +300%</t>
         </is>
       </c>
       <c r="K24" s="19" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1395,42 +1391,42 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="F25" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G25" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I25" s="15" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H25" s="17" t="n">
+        <v>10.97</v>
+      </c>
+      <c r="I25" s="17" t="n">
+        <v>0.23</v>
       </c>
       <c r="J25" s="19" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+          <t>중요공시 5건 / 중요공시 3일 +150% / 중요공시 7일 +150%</t>
         </is>
       </c>
       <c r="K25" s="19" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1438,42 +1434,42 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>다스코</t>
+          <t>HLB</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F26" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G26" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H26" s="17" t="n">
-        <v>1.41</v>
-      </c>
-      <c r="I26" s="17" t="n">
-        <v>45.17</v>
+        <v>0</v>
+      </c>
+      <c r="H26" s="18" t="n">
+        <v>-29.89</v>
+      </c>
+      <c r="I26" s="18" t="n">
+        <v>-24.3</v>
       </c>
       <c r="J26" s="19" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 중요공시 3일 +100% / 중요공시 7일 +300%</t>
+          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K26" s="19" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -1481,212 +1477,214 @@
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D27" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E27" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="F27" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I27" s="15" t="n">
+        <v/>
+      </c>
+      <c r="J27" s="19" t="inlineStr">
+        <is>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K27" s="19" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="C28" s="21" t="inlineStr">
+        <is>
+          <t>일성건설</t>
+        </is>
+      </c>
+      <c r="D28" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E28" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F28" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G28" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="22" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="I28" s="22" t="n">
+        <v>8.210000000000001</v>
+      </c>
+      <c r="J28" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 3일 +200%</t>
+        </is>
+      </c>
+      <c r="K28" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B29" s="20" t="n">
+        <v>16</v>
+      </c>
+      <c r="C29" s="21" t="inlineStr">
+        <is>
+          <t>서진시스템</t>
+        </is>
+      </c>
+      <c r="D29" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E29" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G29" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="F27" s="15" t="n">
+      <c r="H29" s="22" t="n">
+        <v>13.55</v>
+      </c>
+      <c r="I29" s="24" t="n">
+        <v>-6.97</v>
+      </c>
+      <c r="J29" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K29" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="n">
+        <v>17</v>
+      </c>
+      <c r="C30" s="21" t="inlineStr">
+        <is>
+          <t>SK스퀘어</t>
+        </is>
+      </c>
+      <c r="D30" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E30" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="G27" s="15" t="n">
+      <c r="G30" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="H27" s="17" t="n">
-        <v>10.97</v>
-      </c>
-      <c r="I27" s="17" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="J27" s="19" t="inlineStr">
-        <is>
-          <t>중요공시 5건 / 중요공시 3일 +150% / 중요공시 7일 +67%</t>
-        </is>
-      </c>
-      <c r="K27" s="19" t="inlineStr">
+      <c r="H30" s="22" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="I30" s="24" t="n">
+        <v>-11.33</v>
+      </c>
+      <c r="J30" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K30" s="23" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="15" t="inlineStr">
-        <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="B28" s="15" t="n">
-        <v>15</v>
-      </c>
-      <c r="C28" s="16" t="inlineStr">
-        <is>
-          <t>리가켐바이오</t>
-        </is>
-      </c>
-      <c r="D28" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E28" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F28" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="17" t="n">
-        <v>1.78</v>
-      </c>
-      <c r="I28" s="18" t="n">
-        <v>-10.02</v>
-      </c>
-      <c r="J28" s="19" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K28" s="19" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="15" t="inlineStr">
-        <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="B29" s="15" t="n">
-        <v>16</v>
-      </c>
-      <c r="C29" s="16" t="inlineStr">
-        <is>
-          <t>HLB</t>
-        </is>
-      </c>
-      <c r="D29" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E29" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F29" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="18" t="n">
-        <v>-29.89</v>
-      </c>
-      <c r="I29" s="18" t="n">
-        <v>-24.3</v>
-      </c>
-      <c r="J29" s="19" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K29" s="19" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="15" t="inlineStr">
-        <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="B30" s="15" t="n">
-        <v>17</v>
-      </c>
-      <c r="C30" s="16" t="inlineStr">
-        <is>
-          <t>원전</t>
-        </is>
-      </c>
-      <c r="D30" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E30" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F30" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I30" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J30" s="19" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K30" s="19" t="n">
-        <v/>
-      </c>
-    </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="15" t="inlineStr">
-        <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="B31" s="15" t="n">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B31" s="20" t="n">
         <v>18</v>
       </c>
-      <c r="C31" s="16" t="inlineStr">
-        <is>
-          <t>조선</t>
-        </is>
-      </c>
-      <c r="D31" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E31" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F31" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I31" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J31" s="19" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K31" s="19" t="inlineStr">
-        <is>
-          <t>네이버</t>
+      <c r="C31" s="21" t="inlineStr">
+        <is>
+          <t>현대건설</t>
+        </is>
+      </c>
+      <c r="D31" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E31" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F31" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G31" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="22" t="n">
+        <v>8.390000000000001</v>
+      </c>
+      <c r="I31" s="24" t="n">
+        <v>-7.03</v>
+      </c>
+      <c r="J31" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K31" s="23" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1694,30 +1692,30 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>모아데이타</t>
+          <t>남광토건</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F32" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G32" s="20" t="n">
         <v>3</v>
       </c>
       <c r="H32" s="22" t="n">
-        <v>1.68</v>
+        <v>6.05</v>
       </c>
       <c r="I32" s="22" t="n">
-        <v>1.04</v>
+        <v>12.88</v>
       </c>
       <c r="J32" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 7일 +200%</t>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K32" s="23" t="inlineStr">
@@ -1729,7 +1727,7 @@
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1737,42 +1735,42 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>모아라이프플러스</t>
+          <t>NH투자증권</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F33" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G33" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H33" s="24" t="n">
-        <v>-2.52</v>
+        <v>0</v>
+      </c>
+      <c r="H33" s="22" t="n">
+        <v>8.029999999999999</v>
       </c>
       <c r="I33" s="22" t="n">
-        <v>3.48</v>
+        <v>0.64</v>
       </c>
       <c r="J33" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+          <t>Google 급상승 검색어 등장 (KR) / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K33" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>Google, 네이버</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1780,7 +1778,7 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>TSMC</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
@@ -1803,17 +1801,19 @@
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K34" s="23" t="n">
-        <v/>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K34" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1821,14 +1821,14 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>한성기업</t>
+          <t>모나미</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F35" s="20" t="n">
         <v>0</v>
@@ -1837,14 +1837,14 @@
         <v>0</v>
       </c>
       <c r="H35" s="22" t="n">
-        <v>29.95</v>
+        <v>25.66</v>
       </c>
       <c r="I35" s="22" t="n">
-        <v>100</v>
+        <v>62.01</v>
       </c>
       <c r="J35" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +616% / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K35" s="23" t="inlineStr">
@@ -1856,7 +1856,7 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1864,14 +1864,14 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>PS일렉트로닉스</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F36" s="20" t="n">
         <v>0</v>
@@ -1879,25 +1879,27 @@
       <c r="G36" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H36" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I36" s="20" t="n">
-        <v/>
+      <c r="H36" s="22" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="I36" s="22" t="n">
+        <v>18.41</v>
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K36" s="23" t="n">
-        <v/>
+          <t>네이버 검색 당일 +54% / 중요공시 3건</t>
+        </is>
+      </c>
+      <c r="K36" s="23" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1905,14 +1907,14 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>SK증권</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E37" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F37" s="20" t="n">
         <v>0</v>
@@ -1921,14 +1923,14 @@
         <v>0</v>
       </c>
       <c r="H37" s="22" t="n">
-        <v>8.09</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="I37" s="24" t="n">
-        <v>-7.17</v>
+        <v>-4.65</v>
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K37" s="23" t="n">
@@ -1938,7 +1940,7 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1946,42 +1948,40 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>PS일렉트로닉스</t>
+          <t>대덕전자</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F38" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H38" s="22" t="n">
-        <v>9.300000000000001</v>
-      </c>
-      <c r="I38" s="22" t="n">
-        <v>18.41</v>
+        <v>7.95</v>
+      </c>
+      <c r="I38" s="24" t="n">
+        <v>-6.71</v>
       </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +50%</t>
-        </is>
-      </c>
-      <c r="K38" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K38" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1989,7 +1989,7 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>일성건설</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
@@ -2005,14 +2005,14 @@
         <v>0</v>
       </c>
       <c r="H39" s="22" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="I39" s="22" t="n">
-        <v>8.210000000000001</v>
+        <v>17.27</v>
+      </c>
+      <c r="I39" s="24" t="n">
+        <v>-12.45</v>
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200%</t>
+          <t>중요공시 3건 / 중요공시 3일 +50%</t>
         </is>
       </c>
       <c r="K39" s="23" t="inlineStr">
@@ -2024,7 +2024,7 @@
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2032,40 +2032,42 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>SK증권</t>
+          <t>모아데이타</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F40" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G40" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H40" s="22" t="n">
-        <v>8.609999999999999</v>
-      </c>
-      <c r="I40" s="24" t="n">
-        <v>-4.65</v>
+        <v>1.68</v>
+      </c>
+      <c r="I40" s="22" t="n">
+        <v>1.04</v>
       </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K40" s="23" t="n">
-        <v/>
+          <t>중요공시 3건 / 중요공시 3일 +50%</t>
+        </is>
+      </c>
+      <c r="K40" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2073,7 +2075,7 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>한화투자증권</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
@@ -2089,24 +2091,26 @@
         <v>0</v>
       </c>
       <c r="H41" s="22" t="n">
-        <v>3.57</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="I41" s="24" t="n">
-        <v>-2.45</v>
+        <v>-3.43</v>
       </c>
       <c r="J41" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K41" s="23" t="n">
-        <v/>
+          <t>Google 급상승 검색어 등장 (KR)</t>
+        </is>
+      </c>
+      <c r="K41" s="23" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2114,7 +2118,7 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>대덕전자</t>
+          <t>아주IB투자</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
@@ -2130,24 +2134,26 @@
         <v>0</v>
       </c>
       <c r="H42" s="22" t="n">
-        <v>7.95</v>
+        <v>6.9</v>
       </c>
       <c r="I42" s="24" t="n">
-        <v>-6.71</v>
+        <v>-11.43</v>
       </c>
       <c r="J42" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K42" s="23" t="n">
-        <v/>
+          <t>Google 급상승 검색어 등장 (KR)</t>
+        </is>
+      </c>
+      <c r="K42" s="23" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2155,7 +2161,7 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>유진투자증권</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
@@ -2171,26 +2177,26 @@
         <v>0</v>
       </c>
       <c r="H43" s="22" t="n">
-        <v>2.47</v>
-      </c>
-      <c r="I43" s="24" t="n">
-        <v>-4.5</v>
+        <v>8.02</v>
+      </c>
+      <c r="I43" s="22" t="n">
+        <v>0.34</v>
       </c>
       <c r="J43" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K43" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2198,7 +2204,7 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>우리기술투자</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
@@ -2213,27 +2219,27 @@
       <c r="G44" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I44" s="20" t="n">
-        <v/>
+      <c r="H44" s="22" t="n">
+        <v>8.369999999999999</v>
+      </c>
+      <c r="I44" s="24" t="n">
+        <v>-2.68</v>
       </c>
       <c r="J44" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K44" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2241,7 +2247,7 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>기아</t>
+          <t>미래에셋벤처투자</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
@@ -2257,24 +2263,26 @@
         <v>0</v>
       </c>
       <c r="H45" s="22" t="n">
-        <v>1.86</v>
+        <v>10.56</v>
       </c>
       <c r="I45" s="24" t="n">
-        <v>-2.96</v>
+        <v>-8.06</v>
       </c>
       <c r="J45" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K45" s="23" t="n">
-        <v/>
+          <t>Google 급상승 검색어 등장 (KR)</t>
+        </is>
+      </c>
+      <c r="K45" s="23" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
@@ -2282,7 +2290,7 @@
       </c>
       <c r="C46" s="21" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="D46" s="20" t="n">
@@ -2297,25 +2305,27 @@
       <c r="G46" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H46" s="22" t="n">
-        <v>6.08</v>
-      </c>
-      <c r="I46" s="22" t="n">
-        <v>9.859999999999999</v>
+      <c r="H46" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I46" s="20" t="n">
+        <v/>
       </c>
       <c r="J46" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K46" s="23" t="n">
-        <v/>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K46" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B47" s="20" t="n">
@@ -2346,19 +2356,19 @@
       </c>
       <c r="J47" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +773% / 중요공시 2건</t>
+          <t>네이버 검색 당일 +1304% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K47" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B48" s="20" t="n">
@@ -2389,19 +2399,19 @@
       </c>
       <c r="J48" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +238% / 중요공시 2건</t>
+          <t>네이버 검색 당일 +309% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K48" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B49" s="20" t="n">
@@ -2432,19 +2442,19 @@
       </c>
       <c r="J49" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +105% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +242% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K49" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B50" s="20" t="n">
@@ -2452,7 +2462,7 @@
       </c>
       <c r="C50" s="21" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="D50" s="20" t="n">
@@ -2468,26 +2478,26 @@
         <v>0</v>
       </c>
       <c r="H50" s="22" t="n">
-        <v>3.44</v>
+        <v>0.19</v>
       </c>
       <c r="I50" s="24" t="n">
-        <v>-23.95</v>
+        <v>-7.28</v>
       </c>
       <c r="J50" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +52% / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K50" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B51" s="20" t="n">
@@ -2495,30 +2505,30 @@
       </c>
       <c r="C51" s="21" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>까뮤이앤씨</t>
         </is>
       </c>
       <c r="D51" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E51" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F51" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G51" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H51" s="22" t="n">
-        <v>0.19</v>
+        <v>1.1</v>
       </c>
       <c r="I51" s="24" t="n">
-        <v>-7.28</v>
+        <v>-0.46</v>
       </c>
       <c r="J51" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K51" s="23" t="inlineStr">
@@ -2530,7 +2540,7 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B52" s="20" t="n">
@@ -2573,7 +2583,7 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B53" s="20" t="n">
@@ -2581,30 +2591,30 @@
       </c>
       <c r="C53" s="21" t="inlineStr">
         <is>
-          <t>조이웍스앤코</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="D53" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E53" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F53" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G53" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H53" s="24" t="n">
-        <v>-0.75</v>
-      </c>
-      <c r="I53" s="22" t="n">
-        <v>34.84</v>
+        <v>3</v>
+      </c>
+      <c r="H53" s="22" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="I53" s="24" t="n">
+        <v>-1.4</v>
       </c>
       <c r="J53" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K53" s="23" t="inlineStr">
@@ -2616,7 +2626,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B54" s="20" t="n">
@@ -2624,7 +2634,7 @@
       </c>
       <c r="C54" s="21" t="inlineStr">
         <is>
-          <t>롯데관광개발</t>
+          <t>조이웍스앤코</t>
         </is>
       </c>
       <c r="D54" s="20" t="n">
@@ -2639,111 +2649,109 @@
       <c r="G54" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H54" s="22" t="n">
-        <v>2.48</v>
-      </c>
-      <c r="I54" s="24" t="n">
-        <v>-1.97</v>
+      <c r="H54" s="24" t="n">
+        <v>-0.75</v>
+      </c>
+      <c r="I54" s="22" t="n">
+        <v>34.84</v>
       </c>
       <c r="J54" s="23" t="inlineStr">
         <is>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K54" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B55" s="20" t="n">
+        <v>42</v>
+      </c>
+      <c r="C55" s="21" t="inlineStr">
+        <is>
+          <t>방산</t>
+        </is>
+      </c>
+      <c r="D55" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E55" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F55" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I55" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J55" s="23" t="inlineStr">
+        <is>
           <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
-      <c r="K54" s="23" t="n">
+      <c r="K55" s="23" t="n">
         <v/>
       </c>
     </row>
-    <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="25" t="inlineStr">
-        <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="B55" s="25" t="n">
-        <v>42</v>
-      </c>
-      <c r="C55" s="26" t="inlineStr">
-        <is>
-          <t>레몬헬스케어</t>
-        </is>
-      </c>
-      <c r="D55" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E55" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F55" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G55" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H55" s="27" t="n">
-        <v>-0.51</v>
-      </c>
-      <c r="I55" s="28" t="n">
-        <v>4.26</v>
-      </c>
-      <c r="J55" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +1248%</t>
-        </is>
-      </c>
-      <c r="K55" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
     <row r="56" ht="18" customHeight="1">
-      <c r="A56" s="25" t="inlineStr">
-        <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="B56" s="25" t="n">
+      <c r="A56" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B56" s="20" t="n">
         <v>43</v>
       </c>
-      <c r="C56" s="26" t="inlineStr">
-        <is>
-          <t>금호에이치티</t>
-        </is>
-      </c>
-      <c r="D56" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E56" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F56" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G56" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H56" s="27" t="n">
-        <v>-3.36</v>
-      </c>
-      <c r="I56" s="28" t="n">
-        <v>24.17</v>
-      </c>
-      <c r="J56" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +666%</t>
-        </is>
-      </c>
-      <c r="K56" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+      <c r="C56" s="21" t="inlineStr">
+        <is>
+          <t>전기차</t>
+        </is>
+      </c>
+      <c r="D56" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E56" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F56" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I56" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J56" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K56" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2751,7 +2759,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>흥구석유</t>
+          <t>레몬헬스케어</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2766,15 +2774,15 @@
       <c r="G57" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H57" s="28" t="n">
-        <v>0.5600000000000001</v>
+      <c r="H57" s="27" t="n">
+        <v>-0.51</v>
       </c>
       <c r="I57" s="28" t="n">
-        <v>16.68</v>
+        <v>4.26</v>
       </c>
       <c r="J57" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +268%</t>
+          <t>네이버 검색 당일 +1319%</t>
         </is>
       </c>
       <c r="K57" s="29" t="inlineStr">
@@ -2786,7 +2794,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2794,7 +2802,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>에스와이</t>
+          <t>금호에이치티</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2809,15 +2817,15 @@
       <c r="G58" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="25" t="n">
-        <v>0</v>
+      <c r="H58" s="27" t="n">
+        <v>-3.36</v>
       </c>
       <c r="I58" s="28" t="n">
-        <v>14.82</v>
+        <v>24.17</v>
       </c>
       <c r="J58" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +261%</t>
+          <t>네이버 검색 당일 +854%</t>
         </is>
       </c>
       <c r="K58" s="29" t="inlineStr">
@@ -2829,7 +2837,7 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2837,7 +2845,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>모나미</t>
+          <t>흥구석유</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2853,14 +2861,14 @@
         <v>0</v>
       </c>
       <c r="H59" s="28" t="n">
-        <v>25.66</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I59" s="28" t="n">
-        <v>62.01</v>
+        <v>16.68</v>
       </c>
       <c r="J59" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +116%</t>
+          <t>네이버 검색 당일 +337%</t>
         </is>
       </c>
       <c r="K59" s="29" t="inlineStr">
@@ -2872,7 +2880,7 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2880,7 +2888,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>흥아해운</t>
+          <t>에스와이</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2895,15 +2903,15 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="28" t="n">
-        <v>6.06</v>
+      <c r="H60" s="25" t="n">
+        <v>0</v>
       </c>
       <c r="I60" s="28" t="n">
-        <v>5.67</v>
+        <v>14.82</v>
       </c>
       <c r="J60" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +116%</t>
+          <t>네이버 검색 당일 +299%</t>
         </is>
       </c>
       <c r="K60" s="29" t="inlineStr">
@@ -2915,7 +2923,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2923,7 +2931,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>오픈베이스</t>
+          <t>펩트론</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2939,14 +2947,14 @@
         <v>0</v>
       </c>
       <c r="H61" s="27" t="n">
-        <v>-7.16</v>
-      </c>
-      <c r="I61" s="28" t="n">
-        <v>6.74</v>
+        <v>-29.94</v>
+      </c>
+      <c r="I61" s="27" t="n">
+        <v>-38.24</v>
       </c>
       <c r="J61" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +104%</t>
+          <t>네이버 검색 당일 +280%</t>
         </is>
       </c>
       <c r="K61" s="29" t="inlineStr">
@@ -2958,7 +2966,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2966,7 +2974,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>레이저쎌</t>
+          <t>흥아해운</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2982,26 +2990,26 @@
         <v>0</v>
       </c>
       <c r="H62" s="28" t="n">
-        <v>23.8</v>
+        <v>6.06</v>
       </c>
       <c r="I62" s="28" t="n">
-        <v>40.2</v>
+        <v>5.67</v>
       </c>
       <c r="J62" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +59% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +158%</t>
         </is>
       </c>
       <c r="K62" s="29" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3009,7 +3017,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>우리금융지주</t>
+          <t>오픈베이스</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3024,19 +3032,21 @@
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="28" t="n">
-        <v>4.66</v>
+      <c r="H63" s="27" t="n">
+        <v>-7.16</v>
       </c>
       <c r="I63" s="28" t="n">
-        <v>2.28</v>
+        <v>6.74</v>
       </c>
       <c r="J63" s="29" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K63" s="29" t="n">
-        <v/>
+          <t>네이버 검색 당일 +147%</t>
+        </is>
+      </c>
+      <c r="K63" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3132,22 +3142,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>132</v>
+        <v>119</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>132</v>
+        <v>119</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H3" s="28" t="n">
@@ -3167,22 +3177,22 @@
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>121</v>
+        <v>101</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>121</v>
+        <v>101</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H4" s="27" t="n">
@@ -3202,22 +3212,22 @@
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H5" s="25" t="n"/>
@@ -3226,72 +3236,68 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="H6" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="28" t="n">
-        <v>0.2</v>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="H6" s="28" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="I6" s="27" t="n">
+        <v>-7.92</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="H7" s="28" t="n">
-        <v>2.52</v>
-      </c>
-      <c r="I7" s="27" t="n">
-        <v>-7.92</v>
-      </c>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="H7" s="25" t="n"/>
+      <c r="I7" s="25" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
@@ -3303,22 +3309,22 @@
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H8" s="25" t="n"/>
@@ -3327,33 +3333,37 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="H9" s="25" t="n"/>
-      <c r="I9" s="25" t="n"/>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="H9" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="28" t="n">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
@@ -3365,22 +3375,22 @@
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H10" s="28" t="n">
@@ -3393,29 +3403,29 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H11" s="25" t="n"/>
@@ -3424,29 +3434,29 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H12" s="25" t="n"/>
@@ -3455,231 +3465,235 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>다스코</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="H13" s="25" t="n"/>
-      <c r="I13" s="25" t="n"/>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="H13" s="28" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="I13" s="28" t="n">
+        <v>45.17</v>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="H14" s="25" t="n"/>
-      <c r="I14" s="25" t="n"/>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="H14" s="28" t="n">
+        <v>10.97</v>
+      </c>
+      <c r="I14" s="28" t="n">
+        <v>0.23</v>
+      </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>다스코</t>
+          <t>HLB</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E15" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="H15" s="28" t="n">
-        <v>1.41</v>
-      </c>
-      <c r="I15" s="28" t="n">
-        <v>45.17</v>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="H15" s="27" t="n">
+        <v>-29.89</v>
+      </c>
+      <c r="I15" s="27" t="n">
+        <v>-24.3</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C16" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D16" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E16" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="H16" s="28" t="n">
-        <v>10.97</v>
-      </c>
-      <c r="I16" s="28" t="n">
-        <v>0.23</v>
-      </c>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="H16" s="25" t="n"/>
+      <c r="I16" s="25" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>HLB</t>
+          <t>NH투자증권</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E17" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="H17" s="27" t="n">
-        <v>-29.89</v>
-      </c>
-      <c r="I17" s="27" t="n">
-        <v>-24.3</v>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="H17" s="28" t="n">
+        <v>8.029999999999999</v>
+      </c>
+      <c r="I17" s="28" t="n">
+        <v>0.64</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>리가켐바이오</t>
+          <t>SK스퀘어</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E18" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H18" s="28" t="n">
-        <v>1.78</v>
+        <v>6.18</v>
       </c>
       <c r="I18" s="27" t="n">
-        <v>-10.02</v>
+        <v>-11.33</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>TSMC</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H19" s="25" t="n"/>
@@ -3688,38 +3702,42 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>남광토건</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D20" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="H20" s="25" t="n"/>
-      <c r="I20" s="25" t="n"/>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="H20" s="28" t="n">
+        <v>6.05</v>
+      </c>
+      <c r="I20" s="28" t="n">
+        <v>12.88</v>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>모아데이타</t>
+          <t>서진시스템</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -3736,25 +3754,25 @@
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H21" s="28" t="n">
-        <v>1.68</v>
-      </c>
-      <c r="I21" s="28" t="n">
-        <v>1.04</v>
+        <v>13.55</v>
+      </c>
+      <c r="I21" s="27" t="n">
+        <v>-6.97</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>모아라이프플러스</t>
+          <t>일성건설</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -3771,25 +3789,25 @@
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="H22" s="27" t="n">
-        <v>-2.52</v>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="H22" s="28" t="n">
+        <v>6.3</v>
       </c>
       <c r="I22" s="28" t="n">
-        <v>3.48</v>
+        <v>8.210000000000001</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3806,122 +3824,126 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H23" s="28" t="n">
-        <v>8.09</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="I23" s="27" t="n">
-        <v>-7.17</v>
+        <v>-7.03</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>PS일렉트로닉스</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C24" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D24" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E24" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="H24" s="25" t="n"/>
-      <c r="I24" s="25" t="n"/>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="H24" s="28" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="I24" s="28" t="n">
+        <v>18.41</v>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>SK증권</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C25" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D25" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E25" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="H25" s="25" t="n"/>
-      <c r="I25" s="25" t="n"/>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="H25" s="28" t="n">
+        <v>8.609999999999999</v>
+      </c>
+      <c r="I25" s="27" t="n">
+        <v>-4.65</v>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>한성기업</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C26" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D26" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E26" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="H26" s="28" t="n">
-        <v>29.95</v>
-      </c>
-      <c r="I26" s="28" t="n">
-        <v>100</v>
-      </c>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="H26" s="25" t="n"/>
+      <c r="I26" s="25" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>대덕전자</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
@@ -3938,25 +3960,25 @@
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H27" s="28" t="n">
-        <v>6.08</v>
-      </c>
-      <c r="I27" s="28" t="n">
-        <v>9.859999999999999</v>
+        <v>7.95</v>
+      </c>
+      <c r="I27" s="27" t="n">
+        <v>-6.71</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>모나미</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
@@ -3973,25 +3995,25 @@
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H28" s="28" t="n">
-        <v>2.47</v>
-      </c>
-      <c r="I28" s="27" t="n">
-        <v>-4.5</v>
+        <v>25.66</v>
+      </c>
+      <c r="I28" s="28" t="n">
+        <v>62.01</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>PS일렉트로닉스</t>
+          <t>모아데이타</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
@@ -4008,25 +4030,25 @@
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H29" s="28" t="n">
-        <v>9.300000000000001</v>
+        <v>1.68</v>
       </c>
       <c r="I29" s="28" t="n">
-        <v>18.41</v>
+        <v>1.04</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>SK증권</t>
+          <t>미래에셋벤처투자</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -4043,25 +4065,25 @@
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H30" s="28" t="n">
-        <v>8.609999999999999</v>
+        <v>10.56</v>
       </c>
       <c r="I30" s="27" t="n">
-        <v>-4.65</v>
+        <v>-8.06</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>기아</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
@@ -4078,25 +4100,25 @@
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H31" s="28" t="n">
-        <v>1.86</v>
+        <v>17.27</v>
       </c>
       <c r="I31" s="27" t="n">
-        <v>-2.96</v>
+        <v>-12.45</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>대덕전자</t>
+          <t>아주IB투자</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -4113,25 +4135,25 @@
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H32" s="28" t="n">
-        <v>7.95</v>
+        <v>6.9</v>
       </c>
       <c r="I32" s="27" t="n">
-        <v>-6.71</v>
+        <v>-11.43</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>일성건설</t>
+          <t>우리기술투자</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4148,25 +4170,25 @@
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H33" s="28" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="I33" s="28" t="n">
-        <v>8.210000000000001</v>
+        <v>8.369999999999999</v>
+      </c>
+      <c r="I33" s="27" t="n">
+        <v>-2.68</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>유진투자증권</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4183,21 +4205,25 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="H34" s="25" t="n"/>
-      <c r="I34" s="25" t="n"/>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="H34" s="28" t="n">
+        <v>8.02</v>
+      </c>
+      <c r="I34" s="28" t="n">
+        <v>0.34</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>한화투자증권</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -4214,25 +4240,25 @@
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H35" s="28" t="n">
-        <v>3.57</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="I35" s="27" t="n">
-        <v>-2.45</v>
+        <v>-3.43</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
@@ -4249,25 +4275,25 @@
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H36" s="28" t="n">
-        <v>0.19</v>
+        <v>2.26</v>
       </c>
       <c r="I36" s="27" t="n">
-        <v>-7.28</v>
+        <v>-1.4</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>데이타솔루션</t>
+          <t>까뮤이앤씨</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
@@ -4284,25 +4310,25 @@
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="H37" s="27" t="n">
-        <v>-5.44</v>
-      </c>
-      <c r="I37" s="28" t="n">
-        <v>54.99</v>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="H37" s="28" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="I37" s="27" t="n">
+        <v>-0.46</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>롯데관광개발</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4319,25 +4345,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H38" s="28" t="n">
-        <v>2.48</v>
+        <v>0.19</v>
       </c>
       <c r="I38" s="27" t="n">
-        <v>-1.97</v>
+        <v>-7.28</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>씨이랩</t>
+          <t>데이타솔루션</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4354,25 +4380,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H39" s="27" t="n">
-        <v>-6.85</v>
+        <v>-5.44</v>
       </c>
       <c r="I39" s="28" t="n">
-        <v>23.04</v>
+        <v>54.99</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>웰킵스하이텍</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4389,25 +4415,21 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="H40" s="28" t="n">
-        <v>23.33</v>
-      </c>
-      <c r="I40" s="28" t="n">
-        <v>66.29000000000001</v>
-      </c>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="H40" s="25" t="n"/>
+      <c r="I40" s="25" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>유티아이</t>
+          <t>씨이랩</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4424,25 +4446,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H41" s="27" t="n">
-        <v>-6.91</v>
-      </c>
-      <c r="I41" s="27" t="n">
-        <v>-19.29</v>
+        <v>-6.85</v>
+      </c>
+      <c r="I41" s="28" t="n">
+        <v>23.04</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>조이웍스앤코</t>
+          <t>웰킵스하이텍</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4459,25 +4481,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="H42" s="27" t="n">
-        <v>-0.75</v>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="H42" s="28" t="n">
+        <v>23.33</v>
       </c>
       <c r="I42" s="28" t="n">
-        <v>34.84</v>
+        <v>66.29000000000001</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>유티아이</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4494,95 +4516,91 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="H43" s="28" t="n">
-        <v>3.44</v>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="H43" s="27" t="n">
+        <v>-6.91</v>
       </c>
       <c r="I43" s="27" t="n">
-        <v>-23.95</v>
+        <v>-19.29</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>금호에이치티</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C44" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D44" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E44" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="H44" s="27" t="n">
-        <v>-3.36</v>
-      </c>
-      <c r="I44" s="28" t="n">
-        <v>24.17</v>
-      </c>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="H44" s="25" t="n"/>
+      <c r="I44" s="25" t="n"/>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>레몬헬스케어</t>
+          <t>조이웍스앤코</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C45" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D45" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E45" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H45" s="27" t="n">
-        <v>-0.51</v>
+        <v>-0.75</v>
       </c>
       <c r="I45" s="28" t="n">
-        <v>4.26</v>
+        <v>34.84</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>레이저쎌</t>
+          <t>금호에이치티</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4599,25 +4617,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="H46" s="28" t="n">
-        <v>23.8</v>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="H46" s="27" t="n">
+        <v>-3.36</v>
       </c>
       <c r="I46" s="28" t="n">
-        <v>40.2</v>
+        <v>24.17</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>모나미</t>
+          <t>레몬헬스케어</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4634,19 +4652,19 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="H47" s="28" t="n">
-        <v>25.66</v>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="H47" s="27" t="n">
+        <v>-0.51</v>
       </c>
       <c r="I47" s="28" t="n">
-        <v>62.01</v>
+        <v>4.26</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
@@ -4669,12 +4687,12 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H48" s="25" t="n">
@@ -4704,12 +4722,12 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H49" s="27" t="n">
@@ -4722,7 +4740,7 @@
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>우리금융지주</t>
+          <t>펩트론</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4739,19 +4757,19 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="H50" s="28" t="n">
-        <v>4.66</v>
-      </c>
-      <c r="I50" s="28" t="n">
-        <v>2.28</v>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="H50" s="27" t="n">
+        <v>-29.94</v>
+      </c>
+      <c r="I50" s="27" t="n">
+        <v>-38.24</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
@@ -4774,12 +4792,12 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H51" s="28" t="n">
@@ -4809,12 +4827,12 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="H52" s="28" t="n">
@@ -4905,19 +4923,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4936,19 +4954,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4967,19 +4985,19 @@
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -4998,19 +5016,19 @@
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5029,19 +5047,19 @@
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5060,19 +5078,19 @@
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5084,26 +5102,26 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B9" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5115,26 +5133,26 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="35" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B10" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="36" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D10" s="36" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E10" s="36" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="F10" s="37" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G10" s="37" t="inlineStr">
@@ -5146,26 +5164,26 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="35" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B11" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="36" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D11" s="36" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="E11" s="36" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="F11" s="37" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="G11" s="37" t="inlineStr">
@@ -5175,102 +5193,90 @@
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="35" t="inlineStr">
-        <is>
-          <t>조선</t>
-        </is>
-      </c>
-      <c r="B12" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="36" t="n">
-        <v>7</v>
-      </c>
-      <c r="D12" s="36" t="n">
-        <v>7</v>
-      </c>
-      <c r="E12" s="36" t="inlineStr">
-        <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="F12" s="37" t="inlineStr">
-        <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="G12" s="37" t="inlineStr">
-        <is>
-          <t>⚡ 관심</t>
-        </is>
-      </c>
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>이차전지</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F12" s="29" t="inlineStr">
+        <is>
+          <t>감지 없음</t>
+        </is>
+      </c>
+      <c r="G12" s="29" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="35" t="inlineStr">
-        <is>
-          <t>제약</t>
-        </is>
-      </c>
-      <c r="B13" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C13" s="36" t="n">
-        <v>9</v>
-      </c>
-      <c r="D13" s="36" t="n">
-        <v>9</v>
-      </c>
-      <c r="E13" s="36" t="inlineStr">
-        <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="F13" s="37" t="inlineStr">
-        <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="G13" s="37" t="inlineStr">
-        <is>
-          <t>⚡ 관심</t>
-        </is>
-      </c>
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>AI반도체</t>
+        </is>
+      </c>
+      <c r="B13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F13" s="29" t="inlineStr">
+        <is>
+          <t>감지 없음</t>
+        </is>
+      </c>
+      <c r="G13" s="29" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="35" t="inlineStr">
-        <is>
-          <t>인공지능</t>
-        </is>
-      </c>
-      <c r="B14" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C14" s="36" t="n">
-        <v>18</v>
-      </c>
-      <c r="D14" s="36" t="n">
-        <v>18</v>
-      </c>
-      <c r="E14" s="36" t="inlineStr">
-        <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="F14" s="37" t="inlineStr">
-        <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="G14" s="37" t="inlineStr">
-        <is>
-          <t>⚡ 관심</t>
-        </is>
-      </c>
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>수소</t>
+        </is>
+      </c>
+      <c r="B14" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" s="29" t="inlineStr">
+        <is>
+          <t>감지 없음</t>
+        </is>
+      </c>
+      <c r="G14" s="29" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>이차전지</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5297,7 +5303,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -5324,7 +5330,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>핀테크</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -5351,7 +5357,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>핀테크</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -5378,7 +5384,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-07-16 07:11 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -57,13 +57,13 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="002563EB"/>
+      <color rgb="00E53935"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00E53935"/>
+      <color rgb="002563EB"/>
       <sz val="10"/>
     </font>
     <font>
@@ -273,13 +273,13 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-07-15 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-07-16 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-15) 상위: 반도체  점수 84.0점</t>
+          <t>⚡ 최신(2026-07-16) 상위: 반도체  점수 103.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-15) 상위: SK  점수 47.0점</t>
+          <t>⚡ 최신(2026-07-16) 상위: SK  점수 39.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-15) 상위: 삼성전자  점수 35.0점</t>
+          <t>⚡ 최신(2026-07-16) 상위: SK하이닉스  점수 38.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>84</v>
+        <v>103</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>84</v>
+        <v>103</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -971,10 +971,10 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -983,26 +983,26 @@
         <v>0</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>-3.6</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="I15" s="18" t="n">
-        <v>-10.22</v>
+        <v>2.18</v>
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (US) / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
         <is>
-          <t>네이버, Google</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1010,14 +1010,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1025,27 +1025,27 @@
       <c r="G16" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="19" t="n">
-        <v>3.34</v>
+      <c r="H16" s="18" t="n">
+        <v>8.83</v>
       </c>
       <c r="I16" s="18" t="n">
-        <v>-11.15</v>
+        <v>0.29</v>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 2건 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1053,14 +1053,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1068,27 +1068,27 @@
       <c r="G17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="19" t="n">
-        <v>3.69</v>
-      </c>
-      <c r="I17" s="18" t="n">
-        <v>-13.08</v>
+      <c r="H17" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I17" s="15" t="n">
+        <v/>
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1096,14 +1096,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1111,27 +1111,27 @@
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I18" s="15" t="n">
-        <v/>
+      <c r="H18" s="18" t="n">
+        <v>29.88</v>
+      </c>
+      <c r="I18" s="18" t="n">
+        <v>35.29</v>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K18" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1139,14 +1139,14 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1162,17 +1162,19 @@
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K19" s="17" t="n">
-        <v/>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K19" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1180,14 +1182,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1196,24 +1198,26 @@
         <v>0</v>
       </c>
       <c r="H20" s="18" t="n">
-        <v>-2.84</v>
-      </c>
-      <c r="I20" s="18" t="n">
-        <v>-3.93</v>
+        <v>2.24</v>
+      </c>
+      <c r="I20" s="19" t="n">
+        <v>-6.16</v>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K20" s="17" t="n">
-        <v/>
+          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K20" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1221,14 +1225,14 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
@@ -1237,24 +1241,26 @@
         <v>0</v>
       </c>
       <c r="H21" s="18" t="n">
-        <v>-4.39</v>
+        <v>6.27</v>
       </c>
       <c r="I21" s="18" t="n">
-        <v>-11.47</v>
+        <v>0.72</v>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K21" s="17" t="n">
-        <v/>
+          <t>중요공시 2건 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K21" s="17" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1262,14 +1268,14 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -1277,15 +1283,15 @@
       <c r="G22" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="18" t="n">
-        <v>-2.92</v>
-      </c>
-      <c r="I22" s="18" t="n">
-        <v>-5.77</v>
+      <c r="H22" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I22" s="15" t="n">
+        <v/>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="n">
@@ -1295,7 +1301,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1303,14 +1309,14 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F23" s="15" t="n">
         <v>0</v>
@@ -1326,7 +1332,7 @@
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K23" s="17" t="inlineStr">
@@ -1338,7 +1344,7 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1346,14 +1352,14 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>0</v>
@@ -1361,25 +1367,27 @@
       <c r="G24" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H24" s="18" t="n">
-        <v>-0.11</v>
-      </c>
-      <c r="I24" s="18" t="n">
-        <v>-1.96</v>
+      <c r="H24" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I24" s="15" t="n">
+        <v/>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K24" s="17" t="n">
-        <v/>
+          <t>Google 급상승 검색어 등장 (KR) / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K24" s="17" t="inlineStr">
+        <is>
+          <t>Google, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1387,42 +1395,40 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>서진시스템</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F25" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G25" s="15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H25" s="18" t="n">
-        <v>-3.95</v>
-      </c>
-      <c r="I25" s="18" t="n">
-        <v>-17.6</v>
+        <v>6.22</v>
+      </c>
+      <c r="I25" s="19" t="n">
+        <v>-0.1</v>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +200%</t>
-        </is>
-      </c>
-      <c r="K25" s="17" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K25" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1430,42 +1436,40 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>한화엔진</t>
+          <t>HLB</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="F26" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G26" s="15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H26" s="18" t="n">
-        <v>-5.84</v>
-      </c>
-      <c r="I26" s="18" t="n">
-        <v>-10.95</v>
+        <v>29.96</v>
+      </c>
+      <c r="I26" s="19" t="n">
+        <v>-30.74</v>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +200%</t>
-        </is>
-      </c>
-      <c r="K26" s="17" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K26" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -1473,7 +1477,7 @@
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>서진시스템</t>
         </is>
       </c>
       <c r="D27" s="15" t="n">
@@ -1489,14 +1493,14 @@
         <v>3</v>
       </c>
       <c r="H27" s="18" t="n">
-        <v>-1.33</v>
-      </c>
-      <c r="I27" s="18" t="n">
-        <v>-7.89</v>
+        <v>11.27</v>
+      </c>
+      <c r="I27" s="19" t="n">
+        <v>-3.78</v>
       </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +50%</t>
+          <t>중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +200%</t>
         </is>
       </c>
       <c r="K27" s="17" t="inlineStr">
@@ -1508,7 +1512,7 @@
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B28" s="15" t="n">
@@ -1516,42 +1520,42 @@
       </c>
       <c r="C28" s="16" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="D28" s="15" t="n">
         <v>8</v>
       </c>
       <c r="E28" s="15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F28" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G28" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H28" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I28" s="15" t="n">
-        <v/>
+      <c r="H28" s="18" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="I28" s="19" t="n">
+        <v>-5.33</v>
       </c>
       <c r="J28" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 3건 / 중요공시 3일 +200% / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K28" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B29" s="15" t="n">
@@ -1559,7 +1563,7 @@
       </c>
       <c r="C29" s="16" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D29" s="15" t="n">
@@ -1582,7 +1586,7 @@
       </c>
       <c r="J29" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K29" s="17" t="n">
@@ -1590,136 +1594,136 @@
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="15" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="B30" s="15" t="n">
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="n">
         <v>17</v>
       </c>
-      <c r="C30" s="16" t="inlineStr">
-        <is>
-          <t>한미반도체</t>
-        </is>
-      </c>
-      <c r="D30" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E30" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F30" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="19" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="I30" s="18" t="n">
-        <v>-1.43</v>
-      </c>
-      <c r="J30" s="17" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K30" s="17" t="inlineStr">
+      <c r="C30" s="21" t="inlineStr">
+        <is>
+          <t>이브이첨단소재</t>
+        </is>
+      </c>
+      <c r="D30" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E30" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F30" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="22" t="n">
+        <v>11.19</v>
+      </c>
+      <c r="I30" s="23" t="n">
+        <v>-21.38</v>
+      </c>
+      <c r="J30" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 3일 +200%</t>
+        </is>
+      </c>
+      <c r="K30" s="24" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="15" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="B31" s="15" t="n">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B31" s="20" t="n">
         <v>18</v>
       </c>
-      <c r="C31" s="16" t="inlineStr">
-        <is>
-          <t>원전</t>
-        </is>
-      </c>
-      <c r="D31" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E31" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F31" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" s="15" t="n">
+      <c r="C31" s="21" t="inlineStr">
+        <is>
+          <t>KB금융</t>
+        </is>
+      </c>
+      <c r="D31" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E31" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F31" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="22" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="I31" s="22" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="J31" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K31" s="24" t="n">
         <v/>
       </c>
-      <c r="I31" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J31" s="17" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K31" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="15" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="B32" s="15" t="n">
+      <c r="A32" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B32" s="20" t="n">
         <v>19</v>
       </c>
-      <c r="C32" s="16" t="inlineStr">
-        <is>
-          <t>방산</t>
-        </is>
-      </c>
-      <c r="D32" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E32" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F32" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H32" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I32" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J32" s="17" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K32" s="17" t="n">
-        <v/>
+      <c r="C32" s="21" t="inlineStr">
+        <is>
+          <t>성호전자</t>
+        </is>
+      </c>
+      <c r="D32" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E32" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F32" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H32" s="22" t="n">
+        <v>9.119999999999999</v>
+      </c>
+      <c r="I32" s="22" t="n">
+        <v>7.54</v>
+      </c>
+      <c r="J32" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 7일 +200%</t>
+        </is>
+      </c>
+      <c r="K32" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1727,7 +1731,7 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>다스코</t>
+          <t>수성웹툰</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
@@ -1743,14 +1747,14 @@
         <v>3</v>
       </c>
       <c r="H33" s="22" t="n">
-        <v>-7.87</v>
-      </c>
-      <c r="I33" s="23" t="n">
-        <v>9.75</v>
+        <v>17.76</v>
+      </c>
+      <c r="I33" s="22" t="n">
+        <v>12.56</v>
       </c>
       <c r="J33" s="24" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 중요공시 7일 +100%</t>
+          <t>중요공시 5건 / 중요공시 7일 +400%</t>
         </is>
       </c>
       <c r="K33" s="24" t="inlineStr">
@@ -1762,7 +1766,7 @@
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1770,42 +1774,42 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>수성웹툰</t>
+          <t>비비안</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F34" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G34" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H34" s="23" t="n">
-        <v>4.58</v>
+        <v>0</v>
+      </c>
+      <c r="H34" s="22" t="n">
+        <v>29.99</v>
       </c>
       <c r="I34" s="22" t="n">
-        <v>-8.050000000000001</v>
+        <v>75.83</v>
       </c>
       <c r="J34" s="24" t="inlineStr">
         <is>
-          <t>중요공시 5건 / 중요공시 7일 +400%</t>
+          <t>중요공시 3건 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K34" s="24" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1813,7 +1817,7 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>모아데이타</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
@@ -1829,14 +1833,14 @@
         <v>3</v>
       </c>
       <c r="H35" s="22" t="n">
-        <v>-2.8</v>
-      </c>
-      <c r="I35" s="22" t="n">
-        <v>-5.05</v>
+        <v>1.17</v>
+      </c>
+      <c r="I35" s="23" t="n">
+        <v>-10.19</v>
       </c>
       <c r="J35" s="24" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 중요공시 7일 +300%</t>
+          <t>중요공시 3건 / 중요공시 7일 +200%</t>
         </is>
       </c>
       <c r="K35" s="24" t="inlineStr">
@@ -1848,7 +1852,7 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1856,7 +1860,7 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>에코프로비엠</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
@@ -1871,15 +1875,15 @@
       <c r="G36" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H36" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I36" s="20" t="n">
-        <v/>
+      <c r="H36" s="22" t="n">
+        <v>7.37</v>
+      </c>
+      <c r="I36" s="22" t="n">
+        <v>7.37</v>
       </c>
       <c r="J36" s="24" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K36" s="24" t="n">
@@ -1889,7 +1893,7 @@
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1897,7 +1901,7 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>현대해상</t>
+          <t>에코프로</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
@@ -1913,14 +1917,14 @@
         <v>0</v>
       </c>
       <c r="H37" s="22" t="n">
-        <v>-3.5</v>
+        <v>9.23</v>
       </c>
       <c r="I37" s="22" t="n">
-        <v>-0.93</v>
+        <v>10.77</v>
       </c>
       <c r="J37" s="24" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K37" s="24" t="n">
@@ -1930,7 +1934,7 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1938,42 +1942,40 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>이브이첨단소재</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F38" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H38" s="22" t="n">
-        <v>-5.1</v>
-      </c>
-      <c r="I38" s="22" t="n">
-        <v>-34.66</v>
+        <v>4.64</v>
+      </c>
+      <c r="I38" s="23" t="n">
+        <v>-0.92</v>
       </c>
       <c r="J38" s="24" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200%</t>
-        </is>
-      </c>
-      <c r="K38" s="24" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K38" s="24" t="n">
+        <v/>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1981,7 +1983,7 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>한솔테크닉스</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
@@ -1996,15 +1998,15 @@
       <c r="G39" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H39" s="23" t="n">
-        <v>2.51</v>
+      <c r="H39" s="22" t="n">
+        <v>23.68</v>
       </c>
       <c r="I39" s="22" t="n">
-        <v>-9.09</v>
+        <v>25.79</v>
       </c>
       <c r="J39" s="24" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200%</t>
+          <t>중요공시 3건 / 중요공시 3일 +50%</t>
         </is>
       </c>
       <c r="K39" s="24" t="inlineStr">
@@ -2016,7 +2018,7 @@
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2024,40 +2026,42 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>코세스</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F40" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G40" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H40" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I40" s="20" t="n">
-        <v/>
+      <c r="H40" s="23" t="n">
+        <v>-2.76</v>
+      </c>
+      <c r="I40" s="22" t="n">
+        <v>0.38</v>
       </c>
       <c r="J40" s="24" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K40" s="24" t="n">
-        <v/>
+          <t>중요공시 3건 / 중요공시 3일 +200%</t>
+        </is>
+      </c>
+      <c r="K40" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2065,14 +2069,14 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>고영</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E41" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F41" s="20" t="n">
         <v>0</v>
@@ -2081,26 +2085,26 @@
         <v>0</v>
       </c>
       <c r="H41" s="22" t="n">
-        <v>-3.14</v>
+        <v>12.48</v>
       </c>
       <c r="I41" s="22" t="n">
-        <v>-13.11</v>
+        <v>13.6</v>
       </c>
       <c r="J41" s="24" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K41" s="24" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2108,7 +2112,7 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>스타코링크</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
@@ -2123,27 +2127,27 @@
       <c r="G42" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H42" s="22" t="n">
-        <v>-3.12</v>
-      </c>
-      <c r="I42" s="22" t="n">
-        <v>-9.039999999999999</v>
+      <c r="H42" s="23" t="n">
+        <v>-11.29</v>
+      </c>
+      <c r="I42" s="23" t="n">
+        <v>-88.87</v>
       </c>
       <c r="J42" s="24" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +327% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K42" s="24" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2151,42 +2155,42 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>STX그린로지스</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E43" s="20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F43" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G43" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H43" s="22" t="n">
-        <v>-4.41</v>
+        <v>13.33</v>
       </c>
       <c r="I43" s="22" t="n">
-        <v>-15.58</v>
+        <v>77.25</v>
       </c>
       <c r="J43" s="24" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 매일경제 기사 언급</t>
+          <t>네이버 검색 당일 +147% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K43" s="24" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2194,7 +2198,7 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>뉴인텍</t>
+          <t>모나미</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
@@ -2210,26 +2214,26 @@
         <v>0</v>
       </c>
       <c r="H44" s="22" t="n">
-        <v>-0.29</v>
+        <v>30</v>
       </c>
       <c r="I44" s="22" t="n">
-        <v>-12.44</v>
+        <v>151.64</v>
       </c>
       <c r="J44" s="24" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K44" s="24" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2237,7 +2241,7 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>TSMC</t>
+          <t>서남</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
@@ -2252,25 +2256,27 @@
       <c r="G45" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H45" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I45" s="20" t="n">
-        <v/>
+      <c r="H45" s="22" t="n">
+        <v>9.42</v>
+      </c>
+      <c r="I45" s="22" t="n">
+        <v>7.48</v>
       </c>
       <c r="J45" s="24" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K45" s="24" t="n">
-        <v/>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K45" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
@@ -2278,42 +2284,42 @@
       </c>
       <c r="C46" s="21" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>한화엔진</t>
         </is>
       </c>
       <c r="D46" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E46" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F46" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G46" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I46" s="20" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H46" s="22" t="n">
+        <v>8.619999999999999</v>
+      </c>
+      <c r="I46" s="22" t="n">
+        <v>5.59</v>
       </c>
       <c r="J46" s="24" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K46" s="24" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B47" s="20" t="n">
@@ -2321,208 +2327,208 @@
       </c>
       <c r="C47" s="21" t="inlineStr">
         <is>
-          <t>테스</t>
+          <t>아미코젠</t>
         </is>
       </c>
       <c r="D47" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E47" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H47" s="22" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="I47" s="22" t="n">
+        <v>9.42</v>
+      </c>
+      <c r="J47" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K47" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B48" s="20" t="n">
+        <v>35</v>
+      </c>
+      <c r="C48" s="21" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D48" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="F47" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" s="23" t="n">
-        <v>16.68</v>
-      </c>
-      <c r="I47" s="23" t="n">
-        <v>50</v>
-      </c>
-      <c r="J47" s="24" t="inlineStr">
+      <c r="E48" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F48" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I48" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J48" s="24" t="inlineStr">
+        <is>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K48" s="24" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B49" s="20" t="n">
+        <v>36</v>
+      </c>
+      <c r="C49" s="21" t="inlineStr">
+        <is>
+          <t>TSMC</t>
+        </is>
+      </c>
+      <c r="D49" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E49" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F49" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I49" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J49" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K49" s="24" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B50" s="20" t="n">
+        <v>37</v>
+      </c>
+      <c r="C50" s="21" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="D50" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E50" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F50" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="22" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="I50" s="23" t="n">
+        <v>-7.12</v>
+      </c>
+      <c r="J50" s="24" t="inlineStr">
         <is>
           <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
-      <c r="K47" s="24" t="n">
+      <c r="K50" s="24" t="n">
         <v/>
       </c>
     </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="25" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="B48" s="25" t="n">
-        <v>35</v>
-      </c>
-      <c r="C48" s="26" t="inlineStr">
-        <is>
-          <t>레메디</t>
-        </is>
-      </c>
-      <c r="D48" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E48" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F48" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="27" t="n">
-        <v>-20.64</v>
-      </c>
-      <c r="I48" s="27" t="n">
-        <v>-20.64</v>
-      </c>
-      <c r="J48" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +617%</t>
-        </is>
-      </c>
-      <c r="K48" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="25" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="B49" s="25" t="n">
-        <v>36</v>
-      </c>
-      <c r="C49" s="26" t="inlineStr">
-        <is>
-          <t>모나미</t>
-        </is>
-      </c>
-      <c r="D49" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E49" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F49" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G49" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H49" s="29" t="n">
-        <v>29.9</v>
-      </c>
-      <c r="I49" s="29" t="n">
-        <v>102.29</v>
-      </c>
-      <c r="J49" s="28" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K49" s="28" t="n">
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B51" s="20" t="n">
+        <v>38</v>
+      </c>
+      <c r="C51" s="21" t="inlineStr">
+        <is>
+          <t>전기차</t>
+        </is>
+      </c>
+      <c r="D51" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E51" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F51" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="20" t="n">
         <v/>
       </c>
-    </row>
-    <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="25" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="B50" s="25" t="n">
-        <v>37</v>
-      </c>
-      <c r="C50" s="26" t="inlineStr">
-        <is>
-          <t>카카오</t>
-        </is>
-      </c>
-      <c r="D50" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E50" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F50" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G50" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H50" s="27" t="n">
-        <v>-2.59</v>
-      </c>
-      <c r="I50" s="27" t="n">
-        <v>-4.38</v>
-      </c>
-      <c r="J50" s="28" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K50" s="28" t="n">
+      <c r="I51" s="20" t="n">
         <v/>
       </c>
-    </row>
-    <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="25" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="B51" s="25" t="n">
-        <v>38</v>
-      </c>
-      <c r="C51" s="26" t="inlineStr">
-        <is>
-          <t>우리기술</t>
-        </is>
-      </c>
-      <c r="D51" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E51" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F51" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G51" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H51" s="27" t="n">
-        <v>-3.27</v>
-      </c>
-      <c r="I51" s="27" t="n">
-        <v>-4.88</v>
-      </c>
-      <c r="J51" s="28" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K51" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+      <c r="J51" s="24" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K51" s="24" t="n">
+        <v/>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -2530,7 +2536,7 @@
       </c>
       <c r="C52" s="26" t="inlineStr">
         <is>
-          <t>한성기업</t>
+          <t>레메디</t>
         </is>
       </c>
       <c r="D52" s="25" t="n">
@@ -2545,25 +2551,27 @@
       <c r="G52" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H52" s="29" t="n">
-        <v>20.11</v>
-      </c>
-      <c r="I52" s="29" t="n">
-        <v>132.22</v>
+      <c r="H52" s="27" t="n">
+        <v>-5.33</v>
+      </c>
+      <c r="I52" s="27" t="n">
+        <v>-24.86</v>
       </c>
       <c r="J52" s="28" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K52" s="28" t="n">
-        <v/>
+          <t>네이버 검색 당일 +817%</t>
+        </is>
+      </c>
+      <c r="K52" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2571,7 +2579,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>매드업</t>
+          <t>미래생명자원</t>
         </is>
       </c>
       <c r="D53" s="25" t="n">
@@ -2587,26 +2595,26 @@
         <v>0</v>
       </c>
       <c r="H53" s="27" t="n">
-        <v>-6.94</v>
-      </c>
-      <c r="I53" s="27" t="n">
-        <v>-19.06</v>
+        <v>-11.13</v>
+      </c>
+      <c r="I53" s="29" t="n">
+        <v>23.68</v>
       </c>
       <c r="J53" s="28" t="inlineStr">
         <is>
-          <t>중요공시 4건</t>
+          <t>네이버 검색 당일 +181%</t>
         </is>
       </c>
       <c r="K53" s="28" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2614,7 +2622,7 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>현대약품</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -2630,26 +2638,24 @@
         <v>0</v>
       </c>
       <c r="H54" s="29" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="I54" s="27" t="n">
-        <v>-2.44</v>
+        <v>10.54</v>
+      </c>
+      <c r="I54" s="29" t="n">
+        <v>48.12</v>
       </c>
       <c r="J54" s="28" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
-        </is>
-      </c>
-      <c r="K54" s="28" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K54" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2657,7 +2663,7 @@
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>육일씨엔에쓰</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="D55" s="25" t="n">
@@ -2672,27 +2678,27 @@
       <c r="G55" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H55" s="27" t="n">
-        <v>-4.22</v>
+      <c r="H55" s="29" t="n">
+        <v>7.74</v>
       </c>
       <c r="I55" s="29" t="n">
-        <v>20.81</v>
+        <v>3.09</v>
       </c>
       <c r="J55" s="28" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K55" s="28" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2700,30 +2706,30 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>육일씨엔에쓰</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E56" s="25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F56" s="25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G56" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H56" s="27" t="n">
-        <v>-1.31</v>
-      </c>
-      <c r="I56" s="27" t="n">
-        <v>-3.03</v>
+      <c r="H56" s="29" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="I56" s="29" t="n">
+        <v>28.93</v>
       </c>
       <c r="J56" s="28" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>중요공시 3건</t>
         </is>
       </c>
       <c r="K56" s="28" t="inlineStr">
@@ -2735,7 +2741,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2743,42 +2749,42 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>에코프로</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E57" s="25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F57" s="25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G57" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H57" s="27" t="n">
-        <v>-5.38</v>
+      <c r="H57" s="29" t="n">
+        <v>1.68</v>
       </c>
       <c r="I57" s="27" t="n">
-        <v>-6.28</v>
+        <v>-0.62</v>
       </c>
       <c r="J57" s="28" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 3일 +100%</t>
         </is>
       </c>
       <c r="K57" s="28" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2786,42 +2792,42 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>HD현대중공업</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E58" s="25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F58" s="25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G58" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="27" t="n">
-        <v>-2.09</v>
+      <c r="H58" s="29" t="n">
+        <v>1.07</v>
       </c>
       <c r="I58" s="27" t="n">
-        <v>-7.03</v>
+        <v>-8.9</v>
       </c>
       <c r="J58" s="28" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 3일 +100%</t>
         </is>
       </c>
       <c r="K58" s="28" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2829,7 +2835,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>에넥스</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2844,25 +2850,27 @@
       <c r="G59" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H59" s="27" t="n">
-        <v>-6.34</v>
-      </c>
-      <c r="I59" s="27" t="n">
-        <v>-11.85</v>
+      <c r="H59" s="29" t="n">
+        <v>29.98</v>
+      </c>
+      <c r="I59" s="29" t="n">
+        <v>119.46</v>
       </c>
       <c r="J59" s="28" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K59" s="28" t="n">
-        <v/>
+          <t>네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K59" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2870,7 +2878,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>로킷헬스케어</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2885,11 +2893,11 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="29" t="n">
-        <v>23.16</v>
-      </c>
-      <c r="I60" s="29" t="n">
-        <v>21.18</v>
+      <c r="H60" s="25" t="n">
+        <v/>
+      </c>
+      <c r="I60" s="25" t="n">
+        <v/>
       </c>
       <c r="J60" s="28" t="inlineStr">
         <is>
@@ -2903,7 +2911,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2911,7 +2919,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>한화시스템</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2926,27 +2934,25 @@
       <c r="G61" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H61" s="27" t="n">
-        <v>-4.26</v>
-      </c>
-      <c r="I61" s="27" t="n">
-        <v>-3.19</v>
+      <c r="H61" s="29" t="n">
+        <v>5.11</v>
+      </c>
+      <c r="I61" s="29" t="n">
+        <v>1.39</v>
       </c>
       <c r="J61" s="28" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K61" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K61" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2954,7 +2960,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>서한</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2970,14 +2976,14 @@
         <v>0</v>
       </c>
       <c r="H62" s="29" t="n">
-        <v>1.66</v>
+        <v>3.87</v>
       </c>
       <c r="I62" s="27" t="n">
-        <v>-5.36</v>
+        <v>-7.53</v>
       </c>
       <c r="J62" s="28" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K62" s="28" t="n">
@@ -2987,7 +2993,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -2995,14 +3001,14 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>기업은행</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E63" s="25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F63" s="25" t="n">
         <v>0</v>
@@ -3010,21 +3016,19 @@
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="27" t="n">
-        <v>-0.24</v>
+      <c r="H63" s="29" t="n">
+        <v>0.78</v>
       </c>
       <c r="I63" s="27" t="n">
-        <v>-1.17</v>
+        <v>-6.14</v>
       </c>
       <c r="J63" s="28" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K63" s="28" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K63" s="28" t="n">
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -3120,22 +3124,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>84</v>
+        <v>103</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>84</v>
+        <v>103</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3151,127 +3155,123 @@
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H4" s="27" t="n">
-        <v>-3.6</v>
-      </c>
-      <c r="I4" s="27" t="n">
-        <v>-10.22</v>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H4" s="29" t="n">
+        <v>8.359999999999999</v>
+      </c>
+      <c r="I4" s="29" t="n">
+        <v>2.18</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="H5" s="29" t="n">
-        <v>3.34</v>
-      </c>
-      <c r="I5" s="27" t="n">
-        <v>-11.15</v>
+        <v>8.83</v>
+      </c>
+      <c r="I5" s="29" t="n">
+        <v>0.29</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H6" s="29" t="n">
-        <v>3.69</v>
-      </c>
-      <c r="I6" s="27" t="n">
-        <v>-13.08</v>
-      </c>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H6" s="25" t="n"/>
+      <c r="I6" s="25" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="H7" s="25" t="n"/>
@@ -3280,165 +3280,165 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H8" s="25" t="n"/>
-      <c r="I8" s="25" t="n"/>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H8" s="29" t="n">
+        <v>29.88</v>
+      </c>
+      <c r="I8" s="29" t="n">
+        <v>35.29</v>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H9" s="27" t="n">
-        <v>-2.84</v>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H9" s="29" t="n">
+        <v>2.24</v>
       </c>
       <c r="I9" s="27" t="n">
-        <v>-3.93</v>
+        <v>-6.16</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H10" s="27" t="n">
-        <v>-4.39</v>
-      </c>
-      <c r="I10" s="27" t="n">
-        <v>-11.47</v>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H10" s="29" t="n">
+        <v>6.27</v>
+      </c>
+      <c r="I10" s="29" t="n">
+        <v>0.72</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H11" s="27" t="n">
-        <v>-2.92</v>
-      </c>
-      <c r="I11" s="27" t="n">
-        <v>-5.77</v>
-      </c>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H11" s="25" t="n"/>
+      <c r="I11" s="25" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="H12" s="25" t="n"/>
@@ -3447,108 +3447,108 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H13" s="27" t="n">
-        <v>-1.33</v>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H13" s="29" t="n">
+        <v>6.22</v>
       </c>
       <c r="I13" s="27" t="n">
-        <v>-7.89</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H14" s="27" t="n">
-        <v>-0.11</v>
-      </c>
-      <c r="I14" s="27" t="n">
-        <v>-1.96</v>
-      </c>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H14" s="25" t="n"/>
+      <c r="I14" s="25" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>HLB</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="25" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E15" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H15" s="25" t="n"/>
-      <c r="I15" s="25" t="n"/>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H15" s="29" t="n">
+        <v>29.96</v>
+      </c>
+      <c r="I15" s="27" t="n">
+        <v>-30.74</v>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>서진시스템</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -3565,25 +3565,25 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H16" s="27" t="n">
-        <v>-3.95</v>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H16" s="29" t="n">
+        <v>0.57</v>
       </c>
       <c r="I16" s="27" t="n">
-        <v>-17.6</v>
+        <v>-5.33</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -3600,12 +3600,12 @@
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="H17" s="25" t="n"/>
@@ -3614,7 +3614,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>한화엔진</t>
+          <t>서진시스템</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -3631,122 +3631,130 @@
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H18" s="27" t="n">
-        <v>-5.84</v>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H18" s="29" t="n">
+        <v>11.27</v>
       </c>
       <c r="I18" s="27" t="n">
-        <v>-10.95</v>
+        <v>-3.78</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>KB금융</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H19" s="25" t="n"/>
-      <c r="I19" s="25" t="n"/>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H19" s="29" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="I19" s="29" t="n">
+        <v>6.2</v>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D20" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H20" s="25" t="n"/>
-      <c r="I20" s="25" t="n"/>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H20" s="29" t="n">
+        <v>4.64</v>
+      </c>
+      <c r="I20" s="27" t="n">
+        <v>-0.92</v>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>한미반도체</t>
+          <t>모아데이타</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D21" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E21" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="H21" s="29" t="n">
-        <v>0.97</v>
+        <v>1.17</v>
       </c>
       <c r="I21" s="27" t="n">
-        <v>-1.43</v>
+        <v>-10.19</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>비비안</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -3763,21 +3771,25 @@
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H22" s="25" t="n"/>
-      <c r="I22" s="25" t="n"/>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H22" s="29" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="I22" s="29" t="n">
+        <v>75.83</v>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>다스코</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3794,25 +3806,25 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H23" s="27" t="n">
-        <v>-7.87</v>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H23" s="29" t="n">
+        <v>9.119999999999999</v>
       </c>
       <c r="I23" s="29" t="n">
-        <v>9.75</v>
+        <v>7.54</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>수성웹툰</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3829,25 +3841,25 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H24" s="27" t="n">
-        <v>-2.8</v>
-      </c>
-      <c r="I24" s="27" t="n">
-        <v>-5.05</v>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H24" s="29" t="n">
+        <v>17.76</v>
+      </c>
+      <c r="I24" s="29" t="n">
+        <v>12.56</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>수성웹툰</t>
+          <t>에코프로</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3864,25 +3876,25 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="H25" s="29" t="n">
-        <v>4.58</v>
-      </c>
-      <c r="I25" s="27" t="n">
-        <v>-8.050000000000001</v>
+        <v>9.23</v>
+      </c>
+      <c r="I25" s="29" t="n">
+        <v>10.77</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>현대해상</t>
+          <t>에코프로비엠</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
@@ -3899,60 +3911,60 @@
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H26" s="27" t="n">
-        <v>-3.5</v>
-      </c>
-      <c r="I26" s="27" t="n">
-        <v>-0.93</v>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H26" s="29" t="n">
+        <v>7.37</v>
+      </c>
+      <c r="I26" s="29" t="n">
+        <v>7.37</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>이브이첨단소재</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C27" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D27" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E27" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="H27" s="29" t="n">
-        <v>2.51</v>
+        <v>11.19</v>
       </c>
       <c r="I27" s="27" t="n">
-        <v>-9.09</v>
+        <v>-21.38</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>이브이첨단소재</t>
+          <t>고영</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
@@ -3969,25 +3981,25 @@
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H28" s="27" t="n">
-        <v>-5.1</v>
-      </c>
-      <c r="I28" s="27" t="n">
-        <v>-34.66</v>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H28" s="29" t="n">
+        <v>12.48</v>
+      </c>
+      <c r="I28" s="29" t="n">
+        <v>13.6</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>코세스</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
@@ -4004,56 +4016,60 @@
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H29" s="25" t="n"/>
-      <c r="I29" s="25" t="n"/>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H29" s="27" t="n">
+        <v>-2.76</v>
+      </c>
+      <c r="I29" s="29" t="n">
+        <v>0.38</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>한솔테크닉스</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C30" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D30" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E30" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H30" s="27" t="n">
-        <v>-4.41</v>
-      </c>
-      <c r="I30" s="27" t="n">
-        <v>-15.58</v>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H30" s="29" t="n">
+        <v>23.68</v>
+      </c>
+      <c r="I30" s="29" t="n">
+        <v>25.79</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>TSMC</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
@@ -4070,12 +4086,12 @@
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="H31" s="25" t="n"/>
@@ -4084,7 +4100,7 @@
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>뉴인텍</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -4101,25 +4117,25 @@
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H32" s="27" t="n">
-        <v>-0.29</v>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H32" s="29" t="n">
+        <v>0.88</v>
       </c>
       <c r="I32" s="27" t="n">
-        <v>-12.44</v>
+        <v>-7.12</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>STX그린로지스</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4136,25 +4152,25 @@
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H33" s="27" t="n">
-        <v>-3.14</v>
-      </c>
-      <c r="I33" s="27" t="n">
-        <v>-13.11</v>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H33" s="29" t="n">
+        <v>13.33</v>
+      </c>
+      <c r="I33" s="29" t="n">
+        <v>77.25</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>TSMC</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4171,25 +4187,21 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H34" s="27" t="n">
-        <v>-3.12</v>
-      </c>
-      <c r="I34" s="27" t="n">
-        <v>-9.039999999999999</v>
-      </c>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H34" s="25" t="n"/>
+      <c r="I34" s="25" t="n"/>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>모나미</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -4206,21 +4218,25 @@
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H35" s="25" t="n"/>
-      <c r="I35" s="25" t="n"/>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H35" s="29" t="n">
+        <v>30</v>
+      </c>
+      <c r="I35" s="29" t="n">
+        <v>151.64</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>테스</t>
+          <t>서남</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
@@ -4237,165 +4253,161 @@
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="H36" s="29" t="n">
-        <v>16.68</v>
+        <v>9.42</v>
       </c>
       <c r="I36" s="29" t="n">
-        <v>50</v>
+        <v>7.48</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>스타코링크</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C37" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D37" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E37" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="H37" s="27" t="n">
-        <v>-4.26</v>
+        <v>-11.29</v>
       </c>
       <c r="I37" s="27" t="n">
-        <v>-3.19</v>
+        <v>-88.87</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>아미코젠</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C38" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D38" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E38" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H38" s="27" t="n">
-        <v>-2.09</v>
-      </c>
-      <c r="I38" s="27" t="n">
-        <v>-7.03</v>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H38" s="29" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="I38" s="29" t="n">
+        <v>9.42</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>레메디</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C39" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D39" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E39" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H39" s="27" t="n">
-        <v>-20.64</v>
-      </c>
-      <c r="I39" s="27" t="n">
-        <v>-20.64</v>
-      </c>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H39" s="25" t="n"/>
+      <c r="I39" s="25" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>로킷헬스케어</t>
+          <t>한화엔진</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C40" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D40" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E40" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="H40" s="29" t="n">
-        <v>23.16</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="I40" s="29" t="n">
-        <v>21.18</v>
+        <v>5.59</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>매드업</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4412,25 +4424,21 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H41" s="27" t="n">
-        <v>-6.94</v>
-      </c>
-      <c r="I41" s="27" t="n">
-        <v>-19.06</v>
-      </c>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H41" s="25" t="n"/>
+      <c r="I41" s="25" t="n"/>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>모나미</t>
+          <t>HD현대중공업</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4447,25 +4455,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="H42" s="29" t="n">
-        <v>29.9</v>
-      </c>
-      <c r="I42" s="29" t="n">
-        <v>102.29</v>
+        <v>1.07</v>
+      </c>
+      <c r="I42" s="27" t="n">
+        <v>-8.9</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4482,25 +4490,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H43" s="27" t="n">
-        <v>-6.34</v>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H43" s="29" t="n">
+        <v>0.78</v>
       </c>
       <c r="I43" s="27" t="n">
-        <v>-11.85</v>
+        <v>-6.14</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>서한</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4517,25 +4525,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="H44" s="29" t="n">
-        <v>1.66</v>
+        <v>3.87</v>
       </c>
       <c r="I44" s="27" t="n">
-        <v>-5.36</v>
+        <v>-7.53</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>레메디</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4552,25 +4560,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="H45" s="27" t="n">
-        <v>-1.31</v>
+        <v>-5.33</v>
       </c>
       <c r="I45" s="27" t="n">
-        <v>-3.03</v>
+        <v>-24.86</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>미래생명자원</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4587,25 +4595,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H46" s="29" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="I46" s="27" t="n">
-        <v>-2.44</v>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H46" s="27" t="n">
+        <v>-11.13</v>
+      </c>
+      <c r="I46" s="29" t="n">
+        <v>23.68</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>에코프로</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4622,25 +4630,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H47" s="27" t="n">
-        <v>-5.38</v>
-      </c>
-      <c r="I47" s="27" t="n">
-        <v>-6.28</v>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H47" s="29" t="n">
+        <v>7.74</v>
+      </c>
+      <c r="I47" s="29" t="n">
+        <v>3.09</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>우리기술</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4657,25 +4665,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H48" s="27" t="n">
-        <v>-3.27</v>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H48" s="29" t="n">
+        <v>1.68</v>
       </c>
       <c r="I48" s="27" t="n">
-        <v>-4.88</v>
+        <v>-0.62</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>육일씨엔에쓰</t>
+          <t>에넥스</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4692,25 +4700,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H49" s="27" t="n">
-        <v>-4.22</v>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H49" s="29" t="n">
+        <v>29.98</v>
       </c>
       <c r="I49" s="29" t="n">
-        <v>20.81</v>
+        <v>119.46</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>육일씨엔에쓰</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4727,25 +4735,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H50" s="27" t="n">
-        <v>-2.59</v>
-      </c>
-      <c r="I50" s="27" t="n">
-        <v>-4.38</v>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H50" s="29" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="I50" s="29" t="n">
+        <v>28.93</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>한성기업</t>
+          <t>한화시스템</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4762,54 +4770,54 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="H51" s="29" t="n">
-        <v>20.11</v>
+        <v>5.11</v>
       </c>
       <c r="I51" s="29" t="n">
-        <v>132.22</v>
+        <v>1.39</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="26" t="inlineStr">
         <is>
-          <t>기업은행</t>
+          <t>현대약품</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C52" s="25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D52" s="25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E52" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H52" s="27" t="n">
-        <v>-0.24</v>
-      </c>
-      <c r="I52" s="27" t="n">
-        <v>-1.17</v>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H52" s="29" t="n">
+        <v>10.54</v>
+      </c>
+      <c r="I52" s="29" t="n">
+        <v>48.12</v>
       </c>
     </row>
   </sheetData>
@@ -4893,19 +4901,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>84</v>
+        <v>103</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>84</v>
+        <v>103</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4924,19 +4932,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4948,26 +4956,26 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="35" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B5" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -4979,26 +4987,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5010,26 +5018,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5048,19 +5056,19 @@
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5072,26 +5080,26 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B9" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5103,26 +5111,26 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="35" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B10" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="36" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D10" s="36" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="E10" s="36" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F10" s="37" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G10" s="37" t="inlineStr">
@@ -5134,26 +5142,26 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="35" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B11" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="36" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="D11" s="36" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="E11" s="36" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F11" s="37" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G11" s="37" t="inlineStr">
@@ -5165,26 +5173,26 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="35" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B12" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="36" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="D12" s="36" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="E12" s="36" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F12" s="37" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G12" s="37" t="inlineStr">
@@ -5223,7 +5231,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5304,7 +5312,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -5331,7 +5339,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>핀테크</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -5358,7 +5366,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>핀테크</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -5385,7 +5393,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
@@ -5412,7 +5420,7 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -5439,7 +5447,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -5466,7 +5474,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>Tesla</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -5493,7 +5501,7 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Tesla</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-07-18 07:13 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -258,13 +258,13 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-07-17 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-07-18 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-17) 상위: 반도체  점수 86.0점</t>
+          <t>⚡ 최신(2026-07-18) 상위: 반도체  점수 91.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-17) 상위: SK하이닉스  점수 34.0점</t>
+          <t>⚡ 최신(2026-07-18) 상위: TSMC  점수 21.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-17) 상위: 삼성전자  점수 27.0점</t>
+          <t>⚡ 최신(2026-07-18) 상위: 삼성전자  점수 19.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -967,42 +967,42 @@
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>TSMC</t>
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G15" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H15" s="18" t="n">
-        <v>-11.53</v>
-      </c>
-      <c r="I15" s="18" t="n">
-        <v>-15.74</v>
+        <v>0</v>
+      </c>
+      <c r="H15" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I15" s="15" t="n">
+        <v/>
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100% / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1014,10 +1014,10 @@
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1033,19 +1033,19 @@
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 2건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1053,14 +1053,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1068,27 +1068,27 @@
       <c r="G17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I17" s="15" t="n">
-        <v/>
+      <c r="H17" s="18" t="n">
+        <v>-11.53</v>
+      </c>
+      <c r="I17" s="18" t="n">
+        <v>-15.74</v>
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 1건 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1096,14 +1096,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>TSMC</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1119,7 +1119,7 @@
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K18" s="17" t="inlineStr">
@@ -1131,7 +1131,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1139,14 +1139,14 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1154,15 +1154,15 @@
       <c r="G19" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="18" t="n">
-        <v>-3.52</v>
-      </c>
-      <c r="I19" s="18" t="n">
-        <v>-2.47</v>
+      <c r="H19" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I19" s="15" t="n">
+        <v/>
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K19" s="17" t="n">
@@ -1172,7 +1172,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1184,10 +1184,10 @@
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1203,19 +1203,19 @@
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K20" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1223,14 +1223,14 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
@@ -1238,27 +1238,25 @@
       <c r="G21" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="15" t="n">
+      <c r="H21" s="18" t="n">
+        <v>-3.52</v>
+      </c>
+      <c r="I21" s="18" t="n">
+        <v>-2.47</v>
+      </c>
+      <c r="J21" s="17" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K21" s="17" t="n">
         <v/>
-      </c>
-      <c r="I21" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J21" s="17" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K21" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1266,42 +1264,42 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="F22" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G22" s="15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H22" s="18" t="n">
-        <v>-2.07</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="I22" s="18" t="n">
-        <v>-4.6</v>
+        <v>-0.75</v>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +200%</t>
         </is>
       </c>
       <c r="K22" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1313,10 +1311,10 @@
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F23" s="15" t="n">
         <v>0</v>
@@ -1332,7 +1330,7 @@
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K23" s="17" t="inlineStr">
@@ -1344,7 +1342,7 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1352,42 +1350,42 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>기가레인</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G24" s="15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H24" s="18" t="n">
-        <v>-0.5600000000000001</v>
-      </c>
-      <c r="I24" s="18" t="n">
-        <v>-0.75</v>
+        <v>-3.75</v>
+      </c>
+      <c r="I24" s="19" t="n">
+        <v>145.7</v>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +200%</t>
+          <t>네이버 검색 당일 +226% / 중요공시 1건 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K24" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1395,42 +1393,40 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>서진시스템</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F25" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G25" s="15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H25" s="18" t="n">
-        <v>-6.32</v>
+        <v>-9.619999999999999</v>
       </c>
       <c r="I25" s="18" t="n">
-        <v>-5.76</v>
+        <v>-14.47</v>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +200%</t>
-        </is>
-      </c>
-      <c r="K25" s="17" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K25" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1438,14 +1434,14 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F26" s="15" t="n">
         <v>0</v>
@@ -1461,189 +1457,189 @@
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K26" s="17" t="n">
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K26" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B27" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="C27" s="21" t="inlineStr">
+        <is>
+          <t>현대약품</t>
+        </is>
+      </c>
+      <c r="D27" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E27" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F27" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="22" t="n">
+        <v>13.26</v>
+      </c>
+      <c r="I27" s="22" t="n">
+        <v>65.40000000000001</v>
+      </c>
+      <c r="J27" s="23" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +241% / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K27" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="C28" s="21" t="inlineStr">
+        <is>
+          <t>HD한국조선해양</t>
+        </is>
+      </c>
+      <c r="D28" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E28" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F28" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H28" s="22" t="n">
+        <v>5.67</v>
+      </c>
+      <c r="I28" s="22" t="n">
+        <v>8.09</v>
+      </c>
+      <c r="J28" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 7일 +200%</t>
+        </is>
+      </c>
+      <c r="K28" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B29" s="20" t="n">
+        <v>16</v>
+      </c>
+      <c r="C29" s="21" t="inlineStr">
+        <is>
+          <t>바이오</t>
+        </is>
+      </c>
+      <c r="D29" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E29" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F29" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="20" t="n">
         <v/>
       </c>
-    </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="15" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="B27" s="15" t="n">
-        <v>14</v>
-      </c>
-      <c r="C27" s="16" t="inlineStr">
-        <is>
-          <t>기가레인</t>
-        </is>
-      </c>
-      <c r="D27" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E27" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F27" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="18" t="n">
-        <v>-3.75</v>
-      </c>
-      <c r="I27" s="19" t="n">
-        <v>145.7</v>
-      </c>
-      <c r="J27" s="17" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +118% / 중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K27" s="17" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="15" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="B28" s="15" t="n">
-        <v>15</v>
-      </c>
-      <c r="C28" s="16" t="inlineStr">
-        <is>
-          <t>KB금융</t>
-        </is>
-      </c>
-      <c r="D28" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E28" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F28" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="18" t="n">
-        <v>-0.28</v>
-      </c>
-      <c r="I28" s="19" t="n">
-        <v>5.66</v>
-      </c>
-      <c r="J28" s="17" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K28" s="17" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="15" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="B29" s="15" t="n">
-        <v>16</v>
-      </c>
-      <c r="C29" s="16" t="inlineStr">
-        <is>
-          <t>서남</t>
-        </is>
-      </c>
-      <c r="D29" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E29" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F29" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="18" t="n">
-        <v>-3.66</v>
-      </c>
-      <c r="I29" s="19" t="n">
-        <v>5.62</v>
-      </c>
-      <c r="J29" s="17" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K29" s="17" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
+      <c r="I29" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J29" s="23" t="inlineStr">
+        <is>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K29" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="15" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="B30" s="15" t="n">
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="n">
         <v>17</v>
       </c>
-      <c r="C30" s="16" t="inlineStr">
-        <is>
-          <t>바이오</t>
-        </is>
-      </c>
-      <c r="D30" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E30" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F30" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="15" t="n">
+      <c r="C30" s="21" t="inlineStr">
+        <is>
+          <t>GS</t>
+        </is>
+      </c>
+      <c r="D30" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E30" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="22" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I30" s="22" t="n">
+        <v>9.52</v>
+      </c>
+      <c r="J30" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K30" s="23" t="n">
         <v/>
-      </c>
-      <c r="I30" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J30" s="17" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K30" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1651,7 +1647,7 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
@@ -1666,27 +1662,25 @@
       <c r="G31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="22" t="n">
-        <v>-6.71</v>
-      </c>
-      <c r="I31" s="22" t="n">
-        <v>-5.55</v>
+      <c r="H31" s="24" t="n">
+        <v>-2.07</v>
+      </c>
+      <c r="I31" s="24" t="n">
+        <v>-4.6</v>
       </c>
       <c r="J31" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / Google 급상승 검색어 등장 (KR)</t>
-        </is>
-      </c>
-      <c r="K31" s="23" t="inlineStr">
-        <is>
-          <t>공시, Google</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K31" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1694,30 +1688,30 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>수성웹툰</t>
+          <t>다보링크</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E32" s="20" t="n">
         <v>3</v>
       </c>
       <c r="F32" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G32" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H32" s="24" t="n">
-        <v>11.36</v>
-      </c>
-      <c r="I32" s="24" t="n">
-        <v>47.27</v>
+        <v>0</v>
+      </c>
+      <c r="H32" s="22" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="I32" s="22" t="n">
+        <v>38.35</v>
       </c>
       <c r="J32" s="23" t="inlineStr">
         <is>
-          <t>중요공시 5건 / 중요공시 7일 +400%</t>
+          <t>중요공시 3건 / 중요공시 3일 +200%</t>
         </is>
       </c>
       <c r="K32" s="23" t="inlineStr">
@@ -1729,7 +1723,7 @@
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1737,42 +1731,40 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>파두</t>
+          <t>SK텔레콤</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F33" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G33" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H33" s="22" t="n">
-        <v>-11.89</v>
+        <v>5.53</v>
       </c>
       <c r="I33" s="22" t="n">
-        <v>-1.95</v>
+        <v>3.46</v>
       </c>
       <c r="J33" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K33" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K33" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1780,14 +1772,14 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F34" s="20" t="n">
         <v>0</v>
@@ -1795,15 +1787,15 @@
       <c r="G34" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="24" t="n">
-        <v>1.22</v>
+      <c r="H34" s="22" t="n">
+        <v>0.77</v>
       </c>
       <c r="I34" s="24" t="n">
-        <v>9.52</v>
+        <v>-9.66</v>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K34" s="23" t="n">
@@ -1813,7 +1805,7 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1821,42 +1813,42 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>코세스</t>
+          <t>STX그린로지스</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F35" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G35" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H35" s="22" t="n">
-        <v>-10.04</v>
+      <c r="H35" s="24" t="n">
+        <v>-14.84</v>
       </c>
       <c r="I35" s="22" t="n">
-        <v>-14.57</v>
+        <v>67.45999999999999</v>
       </c>
       <c r="J35" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200%</t>
+          <t>네이버 검색 당일 +438% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K35" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1864,42 +1856,42 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>엔켐</t>
+          <t>엑사이엔씨</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F36" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G36" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H36" s="24" t="n">
-        <v>9.58</v>
-      </c>
-      <c r="I36" s="24" t="n">
-        <v>4.92</v>
+        <v>-9.109999999999999</v>
+      </c>
+      <c r="I36" s="22" t="n">
+        <v>24.49</v>
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200%</t>
+          <t>네이버 검색 당일 +227% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K36" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1907,30 +1899,30 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>다보링크</t>
+          <t>에스아이리소스</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E37" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F37" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G37" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H37" s="24" t="n">
-        <v>4.18</v>
+        <v>-29.78</v>
       </c>
       <c r="I37" s="24" t="n">
-        <v>38.35</v>
+        <v>-29.78</v>
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200%</t>
+          <t>중요공시 5건</t>
         </is>
       </c>
       <c r="K37" s="23" t="inlineStr">
@@ -1942,7 +1934,7 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1950,14 +1942,14 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>진영</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F38" s="20" t="n">
         <v>0</v>
@@ -1965,25 +1957,27 @@
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H38" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I38" s="20" t="n">
-        <v/>
+      <c r="H38" s="22" t="n">
+        <v>29.96</v>
+      </c>
+      <c r="I38" s="22" t="n">
+        <v>32.65</v>
       </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K38" s="23" t="n">
-        <v/>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K38" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1991,14 +1985,14 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>SK증권</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F39" s="20" t="n">
         <v>0</v>
@@ -2006,15 +2000,15 @@
       <c r="G39" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H39" s="22" t="n">
-        <v>-7.73</v>
+      <c r="H39" s="24" t="n">
+        <v>-3.42</v>
       </c>
       <c r="I39" s="24" t="n">
-        <v>0.5600000000000001</v>
+        <v>-0.22</v>
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K39" s="23" t="n">
@@ -2024,7 +2018,7 @@
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2032,40 +2026,42 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>서진시스템</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F40" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G40" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H40" s="24" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="I40" s="22" t="n">
-        <v>-9.66</v>
+        <v>-6.32</v>
+      </c>
+      <c r="I40" s="24" t="n">
+        <v>-5.76</v>
       </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K40" s="23" t="n">
-        <v/>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K40" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2073,7 +2069,7 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>STX그린로지스</t>
+          <t>벡트</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
@@ -2088,27 +2084,27 @@
       <c r="G41" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="22" t="n">
-        <v>-14.84</v>
-      </c>
-      <c r="I41" s="24" t="n">
-        <v>67.45999999999999</v>
+      <c r="H41" s="24" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="I41" s="22" t="n">
+        <v>15.15</v>
       </c>
       <c r="J41" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +320% / 중요공시 1건</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K41" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2116,7 +2112,7 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>엑사이엔씨</t>
+          <t>우성머티리얼스</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
@@ -2132,26 +2128,26 @@
         <v>0</v>
       </c>
       <c r="H42" s="22" t="n">
-        <v>-9.109999999999999</v>
-      </c>
-      <c r="I42" s="24" t="n">
-        <v>24.49</v>
+        <v>0.36</v>
+      </c>
+      <c r="I42" s="22" t="n">
+        <v>10.6</v>
       </c>
       <c r="J42" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +178% / 중요공시 1건</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K42" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2159,7 +2155,7 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>진영</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
@@ -2174,27 +2170,27 @@
       <c r="G43" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H43" s="24" t="n">
-        <v>29.96</v>
-      </c>
-      <c r="I43" s="24" t="n">
-        <v>32.65</v>
+      <c r="H43" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I43" s="20" t="n">
+        <v/>
       </c>
       <c r="J43" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K43" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2202,42 +2198,40 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>한화엔진</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E44" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F44" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G44" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H44" s="22" t="n">
-        <v>-0.74</v>
-      </c>
-      <c r="I44" s="24" t="n">
-        <v>10.09</v>
+        <v>0</v>
+      </c>
+      <c r="H44" s="24" t="n">
+        <v>-7.73</v>
+      </c>
+      <c r="I44" s="22" t="n">
+        <v>0.5600000000000001</v>
       </c>
       <c r="J44" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K44" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K44" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2245,7 +2239,7 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>벡트</t>
+          <t>한화비전</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
@@ -2260,152 +2254,154 @@
       <c r="G45" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H45" s="22" t="n">
-        <v>-2.8</v>
-      </c>
-      <c r="I45" s="24" t="n">
-        <v>15.15</v>
+      <c r="H45" s="24" t="n">
+        <v>-4.58</v>
+      </c>
+      <c r="I45" s="22" t="n">
+        <v>6.14</v>
       </c>
       <c r="J45" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K45" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K45" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="20" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="B46" s="20" t="n">
+      <c r="A46" s="25" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B46" s="25" t="n">
         <v>33</v>
       </c>
-      <c r="C46" s="21" t="inlineStr">
-        <is>
-          <t>우성머티리얼스</t>
-        </is>
-      </c>
-      <c r="D46" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E46" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F46" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G46" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" s="24" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="I46" s="24" t="n">
-        <v>10.6</v>
-      </c>
-      <c r="J46" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K46" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C46" s="26" t="inlineStr">
+        <is>
+          <t>레메디</t>
+        </is>
+      </c>
+      <c r="D46" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E46" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F46" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="27" t="n">
+        <v>-20.15</v>
+      </c>
+      <c r="I46" s="27" t="n">
+        <v>-40</v>
+      </c>
+      <c r="J46" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +1054%</t>
+        </is>
+      </c>
+      <c r="K46" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="20" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="B47" s="20" t="n">
+      <c r="A47" s="25" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B47" s="25" t="n">
         <v>34</v>
       </c>
-      <c r="C47" s="21" t="inlineStr">
-        <is>
-          <t>기아</t>
-        </is>
-      </c>
-      <c r="D47" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E47" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F47" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" s="24" t="n">
-        <v>3.24</v>
-      </c>
-      <c r="I47" s="24" t="n">
-        <v>3.38</v>
-      </c>
-      <c r="J47" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K47" s="23" t="n">
-        <v/>
+      <c r="C47" s="26" t="inlineStr">
+        <is>
+          <t>미래생명자원</t>
+        </is>
+      </c>
+      <c r="D47" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E47" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F47" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="27" t="n">
+        <v>-4.02</v>
+      </c>
+      <c r="I47" s="29" t="n">
+        <v>12.72</v>
+      </c>
+      <c r="J47" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +540%</t>
+        </is>
+      </c>
+      <c r="K47" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="20" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="B48" s="20" t="n">
+      <c r="A48" s="25" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B48" s="25" t="n">
         <v>35</v>
       </c>
-      <c r="C48" s="21" t="inlineStr">
-        <is>
-          <t>한화비전</t>
-        </is>
-      </c>
-      <c r="D48" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E48" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F48" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="22" t="n">
-        <v>-4.58</v>
-      </c>
-      <c r="I48" s="24" t="n">
-        <v>6.14</v>
-      </c>
-      <c r="J48" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K48" s="23" t="n">
-        <v/>
+      <c r="C48" s="26" t="inlineStr">
+        <is>
+          <t>에넥스</t>
+        </is>
+      </c>
+      <c r="D48" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F48" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="29" t="n">
+        <v>29.95</v>
+      </c>
+      <c r="I48" s="29" t="n">
+        <v>196.24</v>
+      </c>
+      <c r="J48" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +385%</t>
+        </is>
+      </c>
+      <c r="K48" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -2413,7 +2409,7 @@
       </c>
       <c r="C49" s="26" t="inlineStr">
         <is>
-          <t>레메디</t>
+          <t>에스씨디</t>
         </is>
       </c>
       <c r="D49" s="25" t="n">
@@ -2428,15 +2424,15 @@
       <c r="G49" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="27" t="n">
-        <v>-20.15</v>
-      </c>
-      <c r="I49" s="27" t="n">
-        <v>-40</v>
+      <c r="H49" s="29" t="n">
+        <v>6.01</v>
+      </c>
+      <c r="I49" s="29" t="n">
+        <v>20.93</v>
       </c>
       <c r="J49" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +946%</t>
+          <t>네이버 검색 당일 +199%</t>
         </is>
       </c>
       <c r="K49" s="28" t="inlineStr">
@@ -2448,7 +2444,7 @@
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -2456,7 +2452,7 @@
       </c>
       <c r="C50" s="26" t="inlineStr">
         <is>
-          <t>미래생명자원</t>
+          <t>씨피시스템</t>
         </is>
       </c>
       <c r="D50" s="25" t="n">
@@ -2471,15 +2467,15 @@
       <c r="G50" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H50" s="27" t="n">
-        <v>-4.02</v>
+      <c r="H50" s="29" t="n">
+        <v>12.37</v>
       </c>
       <c r="I50" s="29" t="n">
-        <v>12.72</v>
+        <v>68.67</v>
       </c>
       <c r="J50" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +372%</t>
+          <t>네이버 검색 당일 +183%</t>
         </is>
       </c>
       <c r="K50" s="28" t="inlineStr">
@@ -2491,7 +2487,7 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -2499,7 +2495,7 @@
       </c>
       <c r="C51" s="26" t="inlineStr">
         <is>
-          <t>에넥스</t>
+          <t>삼성공조</t>
         </is>
       </c>
       <c r="D51" s="25" t="n">
@@ -2515,14 +2511,14 @@
         <v>0</v>
       </c>
       <c r="H51" s="29" t="n">
-        <v>29.95</v>
+        <v>17.07</v>
       </c>
       <c r="I51" s="29" t="n">
-        <v>196.24</v>
+        <v>48.42</v>
       </c>
       <c r="J51" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +220%</t>
+          <t>네이버 검색 당일 +150%</t>
         </is>
       </c>
       <c r="K51" s="28" t="inlineStr">
@@ -2534,7 +2530,7 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -2542,7 +2538,7 @@
       </c>
       <c r="C52" s="26" t="inlineStr">
         <is>
-          <t>현대약품</t>
+          <t>웰크론</t>
         </is>
       </c>
       <c r="D52" s="25" t="n">
@@ -2558,14 +2554,14 @@
         <v>0</v>
       </c>
       <c r="H52" s="29" t="n">
-        <v>13.26</v>
+        <v>6.55</v>
       </c>
       <c r="I52" s="29" t="n">
-        <v>65.40000000000001</v>
+        <v>31.54</v>
       </c>
       <c r="J52" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +121%</t>
+          <t>네이버 검색 당일 +146%</t>
         </is>
       </c>
       <c r="K52" s="28" t="inlineStr">
@@ -2577,7 +2573,7 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2585,7 +2581,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>에스씨디</t>
+          <t>동화약품</t>
         </is>
       </c>
       <c r="D53" s="25" t="n">
@@ -2600,15 +2596,15 @@
       <c r="G53" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="29" t="n">
-        <v>6.01</v>
+      <c r="H53" s="27" t="n">
+        <v>-4.49</v>
       </c>
       <c r="I53" s="29" t="n">
-        <v>20.93</v>
+        <v>15.49</v>
       </c>
       <c r="J53" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +112%</t>
+          <t>네이버 검색 당일 +103%</t>
         </is>
       </c>
       <c r="K53" s="28" t="inlineStr">
@@ -2620,7 +2616,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2651,7 +2647,7 @@
       </c>
       <c r="J54" s="28" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K54" s="28" t="n">
@@ -2661,7 +2657,7 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2702,7 +2698,7 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2710,7 +2706,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>삼성중공업</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2726,24 +2722,26 @@
         <v>0</v>
       </c>
       <c r="H56" s="29" t="n">
-        <v>2.06</v>
-      </c>
-      <c r="I56" s="29" t="n">
-        <v>6.44</v>
+        <v>3.76</v>
+      </c>
+      <c r="I56" s="27" t="n">
+        <v>-3.76</v>
       </c>
       <c r="J56" s="28" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K56" s="28" t="n">
-        <v/>
+          <t>네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K56" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2751,7 +2749,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>에스아이리소스</t>
+          <t>수성웹툰</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2766,11 +2764,11 @@
       <c r="G57" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H57" s="27" t="n">
-        <v>-29.78</v>
-      </c>
-      <c r="I57" s="27" t="n">
-        <v>-29.78</v>
+      <c r="H57" s="29" t="n">
+        <v>11.36</v>
+      </c>
+      <c r="I57" s="29" t="n">
+        <v>47.27</v>
       </c>
       <c r="J57" s="28" t="inlineStr">
         <is>
@@ -2786,7 +2784,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2794,7 +2792,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>대구백화점</t>
+          <t>엔켐</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2810,10 +2808,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="29" t="n">
-        <v>5.96</v>
+        <v>9.58</v>
       </c>
       <c r="I58" s="29" t="n">
-        <v>62.15</v>
+        <v>4.92</v>
       </c>
       <c r="J58" s="28" t="inlineStr">
         <is>
@@ -2829,7 +2827,7 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2837,7 +2835,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>HD한국조선해양</t>
+          <t>대구백화점</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2853,10 +2851,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="29" t="n">
-        <v>5.67</v>
+        <v>5.96</v>
       </c>
       <c r="I59" s="29" t="n">
-        <v>8.09</v>
+        <v>62.15</v>
       </c>
       <c r="J59" s="28" t="inlineStr">
         <is>
@@ -2872,7 +2870,7 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2880,7 +2878,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>이브이첨단소재</t>
+          <t>HJ중공업</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2896,10 +2894,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="27" t="n">
-        <v>-3.4</v>
+        <v>-1.64</v>
       </c>
       <c r="I60" s="27" t="n">
-        <v>-23.74</v>
+        <v>-6.71</v>
       </c>
       <c r="J60" s="28" t="inlineStr">
         <is>
@@ -2915,7 +2913,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2923,7 +2921,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>HJ중공업</t>
+          <t>HD현대중공업</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2938,11 +2936,11 @@
       <c r="G61" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H61" s="27" t="n">
-        <v>-1.64</v>
+      <c r="H61" s="29" t="n">
+        <v>2.76</v>
       </c>
       <c r="I61" s="27" t="n">
-        <v>-6.71</v>
+        <v>-4.54</v>
       </c>
       <c r="J61" s="28" t="inlineStr">
         <is>
@@ -2958,7 +2956,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2966,7 +2964,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>리가켐바이오</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2981,11 +2979,11 @@
       <c r="G62" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H62" s="29" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="I62" s="29" t="n">
-        <v>1.56</v>
+      <c r="H62" s="27" t="n">
+        <v>-6.58</v>
+      </c>
+      <c r="I62" s="27" t="n">
+        <v>-12.27</v>
       </c>
       <c r="J62" s="28" t="inlineStr">
         <is>
@@ -3001,7 +2999,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3009,36 +3007,34 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E63" s="25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F63" s="25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="29" t="n">
-        <v>2.76</v>
-      </c>
-      <c r="I63" s="27" t="n">
-        <v>-4.54</v>
+      <c r="H63" s="25" t="n">
+        <v/>
+      </c>
+      <c r="I63" s="25" t="n">
+        <v/>
       </c>
       <c r="J63" s="28" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
-        </is>
-      </c>
-      <c r="K63" s="28" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K63" s="28" t="n">
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -3134,22 +3130,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3158,37 +3154,33 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>TSMC</t>
         </is>
       </c>
       <c r="B4" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H4" s="27" t="n">
-        <v>-11.53</v>
-      </c>
-      <c r="I4" s="27" t="n">
-        <v>-15.74</v>
-      </c>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H4" s="25" t="n"/>
+      <c r="I4" s="25" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
@@ -3200,22 +3192,22 @@
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H5" s="27" t="n">
@@ -3228,60 +3220,64 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H6" s="25" t="n"/>
-      <c r="I6" s="25" t="n"/>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H6" s="27" t="n">
+        <v>-11.53</v>
+      </c>
+      <c r="I6" s="27" t="n">
+        <v>-15.74</v>
+      </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>TSMC</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H7" s="25" t="n"/>
@@ -3290,37 +3286,33 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H8" s="27" t="n">
-        <v>-3.52</v>
-      </c>
-      <c r="I8" s="27" t="n">
-        <v>-2.47</v>
-      </c>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H8" s="25" t="n"/>
+      <c r="I8" s="25" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
@@ -3332,22 +3324,22 @@
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H9" s="27" t="n">
@@ -3360,67 +3352,71 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H10" s="25" t="n"/>
-      <c r="I10" s="25" t="n"/>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H10" s="27" t="n">
+        <v>-3.52</v>
+      </c>
+      <c r="I10" s="27" t="n">
+        <v>-2.47</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H11" s="27" t="n">
-        <v>-2.07</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="I11" s="27" t="n">
-        <v>-4.6</v>
+        <v>-0.75</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
@@ -3433,22 +3429,22 @@
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H12" s="27" t="n">
@@ -3461,172 +3457,172 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>기가레인</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H13" s="27" t="n">
-        <v>-0.5600000000000001</v>
-      </c>
-      <c r="I13" s="27" t="n">
-        <v>-0.75</v>
+        <v>-3.75</v>
+      </c>
+      <c r="I13" s="29" t="n">
+        <v>145.7</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H14" s="25" t="n"/>
-      <c r="I14" s="25" t="n"/>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H14" s="27" t="n">
+        <v>-9.619999999999999</v>
+      </c>
+      <c r="I14" s="27" t="n">
+        <v>-14.47</v>
+      </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>서진시스템</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E15" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H15" s="27" t="n">
-        <v>-6.32</v>
-      </c>
-      <c r="I15" s="27" t="n">
-        <v>-5.76</v>
-      </c>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H15" s="25" t="n"/>
+      <c r="I15" s="25" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>KB금융</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C16" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D16" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E16" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H16" s="27" t="n">
-        <v>-0.28</v>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H16" s="29" t="n">
+        <v>1.22</v>
       </c>
       <c r="I16" s="29" t="n">
-        <v>5.66</v>
+        <v>9.52</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>기가레인</t>
+          <t>HD한국조선해양</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E17" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H17" s="27" t="n">
-        <v>-3.75</v>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H17" s="29" t="n">
+        <v>5.67</v>
       </c>
       <c r="I17" s="29" t="n">
-        <v>145.7</v>
+        <v>8.09</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
@@ -3639,22 +3635,22 @@
         <v>1</v>
       </c>
       <c r="C18" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E18" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H18" s="25" t="n"/>
@@ -3663,42 +3659,42 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>서남</t>
+          <t>현대약품</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H19" s="27" t="n">
-        <v>-3.66</v>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H19" s="29" t="n">
+        <v>13.26</v>
       </c>
       <c r="I19" s="29" t="n">
-        <v>5.62</v>
+        <v>65.40000000000001</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
@@ -3715,336 +3711,340 @@
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H20" s="29" t="n">
-        <v>1.22</v>
-      </c>
-      <c r="I20" s="29" t="n">
-        <v>9.52</v>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H20" s="27" t="n">
+        <v>-2.07</v>
+      </c>
+      <c r="I20" s="27" t="n">
+        <v>-4.6</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D21" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E21" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H21" s="27" t="n">
-        <v>-6.71</v>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H21" s="29" t="n">
+        <v>0.77</v>
       </c>
       <c r="I21" s="27" t="n">
-        <v>-5.55</v>
+        <v>-9.66</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>수성웹툰</t>
+          <t>SK텔레콤</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D22" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E22" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H22" s="29" t="n">
-        <v>11.36</v>
+        <v>5.53</v>
       </c>
       <c r="I22" s="29" t="n">
-        <v>47.27</v>
+        <v>3.46</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>파두</t>
+          <t>다보링크</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D23" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E23" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H23" s="27" t="n">
-        <v>-11.89</v>
-      </c>
-      <c r="I23" s="27" t="n">
-        <v>-1.95</v>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H23" s="29" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="I23" s="29" t="n">
+        <v>38.35</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C24" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D24" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E24" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H24" s="29" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="I24" s="27" t="n">
-        <v>-9.66</v>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H24" s="27" t="n">
+        <v>-7.73</v>
+      </c>
+      <c r="I24" s="29" t="n">
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>SK증권</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C25" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D25" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E25" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H25" s="27" t="n">
-        <v>-7.73</v>
-      </c>
-      <c r="I25" s="29" t="n">
-        <v>0.5600000000000001</v>
+        <v>-3.42</v>
+      </c>
+      <c r="I25" s="27" t="n">
+        <v>-0.22</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>다보링크</t>
+          <t>STX그린로지스</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C26" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D26" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E26" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H26" s="29" t="n">
-        <v>4.18</v>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H26" s="27" t="n">
+        <v>-14.84</v>
       </c>
       <c r="I26" s="29" t="n">
-        <v>38.35</v>
+        <v>67.45999999999999</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>엔켐</t>
+          <t>벡트</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C27" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D27" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E27" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H27" s="29" t="n">
-        <v>9.58</v>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H27" s="27" t="n">
+        <v>-2.8</v>
       </c>
       <c r="I27" s="29" t="n">
-        <v>4.92</v>
+        <v>15.15</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>코세스</t>
+          <t>서진시스템</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C28" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D28" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E28" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H28" s="27" t="n">
-        <v>-10.04</v>
+        <v>-6.32</v>
       </c>
       <c r="I28" s="27" t="n">
-        <v>-14.57</v>
+        <v>-5.76</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>에스아이리소스</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C29" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D29" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E29" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H29" s="25" t="n"/>
-      <c r="I29" s="25" t="n"/>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H29" s="27" t="n">
+        <v>-29.78</v>
+      </c>
+      <c r="I29" s="27" t="n">
+        <v>-29.78</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>STX그린로지스</t>
+          <t>엑사이엔씨</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -4061,25 +4061,25 @@
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H30" s="27" t="n">
-        <v>-14.84</v>
+        <v>-9.109999999999999</v>
       </c>
       <c r="I30" s="29" t="n">
-        <v>67.45999999999999</v>
+        <v>24.49</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>기아</t>
+          <t>우성머티리얼스</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
@@ -4096,25 +4096,25 @@
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H31" s="29" t="n">
-        <v>3.24</v>
+        <v>0.36</v>
       </c>
       <c r="I31" s="29" t="n">
-        <v>3.38</v>
+        <v>10.6</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>벡트</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -4131,25 +4131,21 @@
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H32" s="27" t="n">
-        <v>-2.8</v>
-      </c>
-      <c r="I32" s="29" t="n">
-        <v>15.15</v>
-      </c>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H32" s="25" t="n"/>
+      <c r="I32" s="25" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>엑사이엔씨</t>
+          <t>진영</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4166,25 +4162,25 @@
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H33" s="27" t="n">
-        <v>-9.109999999999999</v>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H33" s="29" t="n">
+        <v>29.96</v>
       </c>
       <c r="I33" s="29" t="n">
-        <v>24.49</v>
+        <v>32.65</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>우성머티리얼스</t>
+          <t>한화비전</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4201,130 +4197,130 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H34" s="29" t="n">
-        <v>0.36</v>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H34" s="27" t="n">
+        <v>-4.58</v>
       </c>
       <c r="I34" s="29" t="n">
-        <v>10.6</v>
+        <v>6.14</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>진영</t>
+          <t>HD현대중공업</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D35" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E35" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H35" s="29" t="n">
-        <v>29.96</v>
-      </c>
-      <c r="I35" s="29" t="n">
-        <v>32.65</v>
+        <v>2.76</v>
+      </c>
+      <c r="I35" s="27" t="n">
+        <v>-4.54</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>한화비전</t>
+          <t>HJ중공업</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C36" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D36" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E36" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H36" s="27" t="n">
-        <v>-4.58</v>
-      </c>
-      <c r="I36" s="29" t="n">
-        <v>6.14</v>
+        <v>-1.64</v>
+      </c>
+      <c r="I36" s="27" t="n">
+        <v>-6.71</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>한화엔진</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C37" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D37" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E37" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H37" s="27" t="n">
-        <v>-0.74</v>
-      </c>
-      <c r="I37" s="29" t="n">
-        <v>10.09</v>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H37" s="29" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="I37" s="27" t="n">
+        <v>-3.76</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>HD한국조선해양</t>
+          <t>대구백화점</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4341,25 +4337,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H38" s="29" t="n">
-        <v>5.67</v>
+        <v>5.96</v>
       </c>
       <c r="I38" s="29" t="n">
-        <v>8.09</v>
+        <v>62.15</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>동화약품</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4376,25 +4372,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H39" s="29" t="n">
-        <v>2.76</v>
-      </c>
-      <c r="I39" s="27" t="n">
-        <v>-4.54</v>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H39" s="27" t="n">
+        <v>-4.49</v>
+      </c>
+      <c r="I39" s="29" t="n">
+        <v>15.49</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>HJ중공업</t>
+          <t>레메디</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4411,25 +4407,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H40" s="27" t="n">
-        <v>-1.64</v>
+        <v>-20.15</v>
       </c>
       <c r="I40" s="27" t="n">
-        <v>-6.71</v>
+        <v>-40</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>대구백화점</t>
+          <t>리가켐바이오</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4446,25 +4442,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H41" s="29" t="n">
-        <v>5.96</v>
-      </c>
-      <c r="I41" s="29" t="n">
-        <v>62.15</v>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H41" s="27" t="n">
+        <v>-6.58</v>
+      </c>
+      <c r="I41" s="27" t="n">
+        <v>-12.27</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>레메디</t>
+          <t>미래생명자원</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4481,25 +4477,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H42" s="27" t="n">
-        <v>-20.15</v>
-      </c>
-      <c r="I42" s="27" t="n">
-        <v>-40</v>
+        <v>-4.02</v>
+      </c>
+      <c r="I42" s="29" t="n">
+        <v>12.72</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>미래생명자원</t>
+          <t>삼성공조</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4516,25 +4512,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H43" s="27" t="n">
-        <v>-4.02</v>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H43" s="29" t="n">
+        <v>17.07</v>
       </c>
       <c r="I43" s="29" t="n">
-        <v>12.72</v>
+        <v>48.42</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>삼성중공업</t>
+          <t>수성웹툰</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4551,25 +4547,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H44" s="29" t="n">
-        <v>2.06</v>
+        <v>11.36</v>
       </c>
       <c r="I44" s="29" t="n">
-        <v>6.44</v>
+        <v>47.27</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>씨피시스템</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4586,19 +4582,19 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H45" s="29" t="n">
-        <v>0.06</v>
+        <v>12.37</v>
       </c>
       <c r="I45" s="29" t="n">
-        <v>1.56</v>
+        <v>68.67</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
@@ -4621,12 +4617,12 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H46" s="29" t="n">
@@ -4656,12 +4652,12 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H47" s="29" t="n">
@@ -4674,7 +4670,7 @@
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>에스아이리소스</t>
+          <t>엔켐</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4691,25 +4687,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H48" s="27" t="n">
-        <v>-29.78</v>
-      </c>
-      <c r="I48" s="27" t="n">
-        <v>-29.78</v>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H48" s="29" t="n">
+        <v>9.58</v>
+      </c>
+      <c r="I48" s="29" t="n">
+        <v>4.92</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>이브이첨단소재</t>
+          <t>웰크론</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4726,19 +4722,19 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H49" s="27" t="n">
-        <v>-3.4</v>
-      </c>
-      <c r="I49" s="27" t="n">
-        <v>-23.74</v>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H49" s="29" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="I49" s="29" t="n">
+        <v>31.54</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
@@ -4761,12 +4757,12 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="H50" s="29" t="n">
@@ -4779,7 +4775,7 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4796,25 +4792,21 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H51" s="27" t="n">
-        <v>-10.39</v>
-      </c>
-      <c r="I51" s="27" t="n">
-        <v>-10.39</v>
-      </c>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H51" s="25" t="n"/>
+      <c r="I51" s="25" t="n"/>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="26" t="inlineStr">
         <is>
-          <t>현대약품</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -4831,19 +4823,19 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="H52" s="29" t="n">
-        <v>13.26</v>
-      </c>
-      <c r="I52" s="29" t="n">
-        <v>65.40000000000001</v>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H52" s="27" t="n">
+        <v>-10.39</v>
+      </c>
+      <c r="I52" s="27" t="n">
+        <v>-10.39</v>
       </c>
     </row>
   </sheetData>
@@ -4927,19 +4919,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4958,19 +4950,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4982,26 +4974,26 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="35" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B5" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5013,26 +5005,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5044,26 +5036,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5075,65 +5067,69 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
+          <t>제약</t>
+        </is>
+      </c>
+      <c r="B8" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="36" t="n">
+        <v>7</v>
+      </c>
+      <c r="D8" s="36" t="n">
+        <v>7</v>
+      </c>
+      <c r="E8" s="36" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="F8" s="37" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="G8" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="35" t="inlineStr">
+        <is>
           <t>인공지능</t>
         </is>
       </c>
-      <c r="B8" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" s="36" t="n">
-        <v>17</v>
-      </c>
-      <c r="D8" s="36" t="n">
-        <v>17</v>
-      </c>
-      <c r="E8" s="36" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="F8" s="37" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="G8" s="37" t="inlineStr">
+      <c r="B9" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="36" t="n">
+        <v>13</v>
+      </c>
+      <c r="D9" s="36" t="n">
+        <v>13</v>
+      </c>
+      <c r="E9" s="36" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="F9" s="37" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="G9" s="37" t="inlineStr">
         <is>
           <t>⚡ 관심</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="26" t="inlineStr">
-        <is>
-          <t>이차전지</t>
-        </is>
-      </c>
-      <c r="B9" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F9" s="28" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>이차전지</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
@@ -5160,7 +5156,7 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-07-21 07:17 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -258,14 +258,14 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-07-20 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-07-21 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-20) 상위: 반도체  점수 86.0점</t>
+          <t>⚡ 최신(2026-07-21) 상위: 반도체  점수 78.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-20) 상위: SK하이닉스  점수 33.0점</t>
+          <t>⚡ 최신(2026-07-21) 상위: SK하이닉스  점수 29.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-20) 상위: 삼성전자  점수 27.0점</t>
+          <t>⚡ 최신(2026-07-21) 상위: 삼성전자  점수 21.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -971,10 +971,10 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -983,26 +983,26 @@
         <v>0</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>-11.53</v>
+        <v>-4.23</v>
       </c>
       <c r="I15" s="18" t="n">
-        <v>-15.5</v>
+        <v>-4.39</v>
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 1건 / Google 급상승 검색어 등장 (KR) / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>Google, 네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1014,10 +1014,10 @@
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1026,26 +1026,26 @@
         <v>0</v>
       </c>
       <c r="H16" s="18" t="n">
-        <v>-8.77</v>
+        <v>-4.31</v>
       </c>
       <c r="I16" s="18" t="n">
-        <v>-10.53</v>
+        <v>-4.13</v>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1053,14 +1053,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1068,15 +1068,15 @@
       <c r="G17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I17" s="15" t="n">
-        <v/>
+      <c r="H17" s="18" t="n">
+        <v>-3.85</v>
+      </c>
+      <c r="I17" s="18" t="n">
+        <v>-4.33</v>
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
@@ -1088,7 +1088,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1096,14 +1096,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1119,7 +1119,7 @@
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K18" s="17" t="inlineStr">
@@ -1131,7 +1131,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>TSMC</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K19" s="17" t="inlineStr">
@@ -1174,7 +1174,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1182,14 +1182,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1205,17 +1205,19 @@
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K20" s="17" t="n">
-        <v/>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K20" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1223,7 +1225,7 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
@@ -1246,17 +1248,19 @@
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K21" s="17" t="n">
-        <v/>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K21" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1264,42 +1268,42 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>엑시온그룹</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
         <v>9</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F22" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G22" s="15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H22" s="19" t="n">
-        <v>2.76</v>
-      </c>
-      <c r="I22" s="18" t="n">
-        <v>-3.97</v>
+        <v>29.93</v>
+      </c>
+      <c r="I22" s="19" t="n">
+        <v>137.57</v>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100% / Google 급상승 검색어 등장 (KR)</t>
+          <t>중요공시 3건 / 중요공시 3일 +50% / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="inlineStr">
         <is>
-          <t>공시, Google</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1307,14 +1311,14 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>TSMC</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F23" s="15" t="n">
         <v>0</v>
@@ -1322,15 +1326,15 @@
       <c r="G23" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="18" t="n">
-        <v>-2.07</v>
-      </c>
-      <c r="I23" s="18" t="n">
-        <v>-7.1</v>
+      <c r="H23" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I23" s="15" t="n">
+        <v/>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K23" s="17" t="inlineStr">
@@ -1342,7 +1346,7 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1350,42 +1354,42 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>다보링크</t>
+          <t>에스아이리소스</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>2</v>
       </c>
       <c r="G24" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H24" s="19" t="n">
-        <v>4.18</v>
-      </c>
-      <c r="I24" s="19" t="n">
-        <v>38.35</v>
+        <v>0</v>
+      </c>
+      <c r="H24" s="18" t="n">
+        <v>-21.6</v>
+      </c>
+      <c r="I24" s="18" t="n">
+        <v>-44.94</v>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +50%</t>
+          <t>네이버 검색 당일 +76% / 중요공시 8건 / 중요공시 3일 +60%</t>
         </is>
       </c>
       <c r="K24" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1393,14 +1397,14 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>KB금융</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F25" s="15" t="n">
         <v>0</v>
@@ -1409,24 +1413,26 @@
         <v>0</v>
       </c>
       <c r="H25" s="18" t="n">
-        <v>-3.52</v>
+        <v>-6.79</v>
       </c>
       <c r="I25" s="18" t="n">
-        <v>-2.47</v>
+        <v>-9.34</v>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K25" s="17" t="n">
-        <v/>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K25" s="17" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1434,42 +1440,42 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>파두</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F26" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G26" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I26" s="15" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H26" s="19" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="I26" s="19" t="n">
+        <v>1.42</v>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+          <t>중요공시 2건 / 중요공시 7일 +100% / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K26" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -1477,7 +1483,7 @@
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>진영</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D27" s="15" t="n">
@@ -1492,111 +1498,111 @@
       <c r="G27" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H27" s="19" t="n">
-        <v>29.96</v>
-      </c>
-      <c r="I27" s="19" t="n">
-        <v>28.14</v>
+      <c r="H27" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I27" s="15" t="n">
+        <v/>
       </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K27" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="15" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="B28" s="15" t="n">
+      <c r="A28" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="C28" s="16" t="inlineStr">
-        <is>
-          <t>알테오젠</t>
-        </is>
-      </c>
-      <c r="D28" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E28" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F28" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="18" t="n">
-        <v>-4.16</v>
-      </c>
-      <c r="I28" s="18" t="n">
-        <v>-14.66</v>
-      </c>
-      <c r="J28" s="17" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K28" s="17" t="inlineStr">
+      <c r="C28" s="21" t="inlineStr">
+        <is>
+          <t>하나마이크론</t>
+        </is>
+      </c>
+      <c r="D28" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E28" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F28" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="22" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="I28" s="23" t="n">
+        <v>-4.06</v>
+      </c>
+      <c r="J28" s="24" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K28" s="24" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B29" s="20" t="n">
+        <v>16</v>
+      </c>
+      <c r="C29" s="21" t="inlineStr">
+        <is>
+          <t>삼기에너지솔루션즈</t>
+        </is>
+      </c>
+      <c r="D29" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E29" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G29" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H29" s="23" t="n">
+        <v>-7.31</v>
+      </c>
+      <c r="I29" s="23" t="n">
+        <v>-14.98</v>
+      </c>
+      <c r="J29" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K29" s="24" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
-      </c>
-    </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="15" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="B29" s="15" t="n">
-        <v>16</v>
-      </c>
-      <c r="C29" s="16" t="inlineStr">
-        <is>
-          <t>삼성전기</t>
-        </is>
-      </c>
-      <c r="D29" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E29" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F29" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="18" t="n">
-        <v>-9.619999999999999</v>
-      </c>
-      <c r="I29" s="18" t="n">
-        <v>-19.38</v>
-      </c>
-      <c r="J29" s="17" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K29" s="17" t="n">
-        <v/>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
@@ -1604,42 +1610,42 @@
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>제이케이시냅스</t>
         </is>
       </c>
       <c r="D30" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E30" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F30" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G30" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H30" s="22" t="n">
-        <v>-0.5600000000000001</v>
+        <v>16.74</v>
       </c>
       <c r="I30" s="22" t="n">
-        <v>-0.93</v>
-      </c>
-      <c r="J30" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 3건 / 중요공시 7일 +200%</t>
-        </is>
-      </c>
-      <c r="K30" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+        <v>32.42</v>
+      </c>
+      <c r="J30" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K30" s="24" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1647,42 +1653,40 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>수성웹툰</t>
+          <t>금호타이어</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F31" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G31" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H31" s="24" t="n">
-        <v>11.36</v>
-      </c>
-      <c r="I31" s="24" t="n">
-        <v>41.1</v>
-      </c>
-      <c r="J31" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 5건 / 중요공시 7일 +400%</t>
-        </is>
-      </c>
-      <c r="K31" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="H31" s="22" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="I31" s="23" t="n">
+        <v>-14.8</v>
+      </c>
+      <c r="J31" s="24" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K31" s="24" t="n">
+        <v/>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1690,33 +1694,33 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>리가켐바이오</t>
+          <t>GS건설</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F32" s="20" t="n">
         <v>2</v>
       </c>
       <c r="G32" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H32" s="22" t="n">
-        <v>-6.58</v>
-      </c>
-      <c r="I32" s="22" t="n">
-        <v>-13.8</v>
-      </c>
-      <c r="J32" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K32" s="23" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="H32" s="23" t="n">
+        <v>-4.58</v>
+      </c>
+      <c r="I32" s="23" t="n">
+        <v>-11.54</v>
+      </c>
+      <c r="J32" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 3일 +50%</t>
+        </is>
+      </c>
+      <c r="K32" s="24" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
@@ -1725,7 +1729,7 @@
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1733,42 +1737,42 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F33" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G33" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H33" s="22" t="n">
-        <v>-11.29</v>
-      </c>
-      <c r="I33" s="22" t="n">
-        <v>-19.5</v>
-      </c>
-      <c r="J33" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K33" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
+      <c r="H33" s="23" t="n">
+        <v>-5.08</v>
+      </c>
+      <c r="I33" s="23" t="n">
+        <v>-9.85</v>
+      </c>
+      <c r="J33" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 3일 +50%</t>
+        </is>
+      </c>
+      <c r="K33" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1776,40 +1780,42 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F34" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G34" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="24" t="n">
-        <v>1.22</v>
-      </c>
-      <c r="I34" s="24" t="n">
-        <v>3.24</v>
-      </c>
-      <c r="J34" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K34" s="23" t="n">
-        <v/>
+      <c r="H34" s="23" t="n">
+        <v>-2.53</v>
+      </c>
+      <c r="I34" s="23" t="n">
+        <v>-14.85</v>
+      </c>
+      <c r="J34" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 3일 +50%</t>
+        </is>
+      </c>
+      <c r="K34" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1817,7 +1823,7 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>에스아이리소스</t>
+          <t>defense stock</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
@@ -1832,27 +1838,27 @@
       <c r="G35" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H35" s="22" t="n">
-        <v>-29.78</v>
-      </c>
-      <c r="I35" s="22" t="n">
-        <v>-29.78</v>
-      </c>
-      <c r="J35" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +66% / 중요공시 5건</t>
-        </is>
-      </c>
-      <c r="K35" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
+      <c r="H35" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I35" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J35" s="24" t="inlineStr">
+        <is>
+          <t>Google 급상승 검색어 등장 (US)</t>
+        </is>
+      </c>
+      <c r="K35" s="24" t="inlineStr">
+        <is>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1860,42 +1866,42 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>대구백화점</t>
+          <t>기가레인</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F36" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G36" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H36" s="24" t="n">
-        <v>5.96</v>
-      </c>
-      <c r="I36" s="24" t="n">
-        <v>24.76</v>
-      </c>
-      <c r="J36" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 3건 / 중요공시 3일 +200%</t>
-        </is>
-      </c>
-      <c r="K36" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="H36" s="22" t="n">
+        <v>15.06</v>
+      </c>
+      <c r="I36" s="22" t="n">
+        <v>67.40000000000001</v>
+      </c>
+      <c r="J36" s="24" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +255% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K36" s="24" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1903,7 +1909,7 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>STX그린로지스</t>
+          <t>엑사이엔씨</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
@@ -1918,18 +1924,18 @@
       <c r="G37" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H37" s="22" t="n">
-        <v>-14.84</v>
-      </c>
-      <c r="I37" s="24" t="n">
-        <v>63</v>
-      </c>
-      <c r="J37" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +471% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K37" s="23" t="inlineStr">
+      <c r="H37" s="23" t="n">
+        <v>-6.35</v>
+      </c>
+      <c r="I37" s="22" t="n">
+        <v>12.16</v>
+      </c>
+      <c r="J37" s="24" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +253% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K37" s="24" t="inlineStr">
         <is>
           <t>네이버, 공시</t>
         </is>
@@ -1938,7 +1944,7 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1946,42 +1952,42 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>기가레인</t>
+          <t>다보링크</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F38" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G38" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H38" s="22" t="n">
-        <v>-3.75</v>
-      </c>
-      <c r="I38" s="24" t="n">
-        <v>89.11</v>
-      </c>
-      <c r="J38" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +247% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K38" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
+        <v>3</v>
+      </c>
+      <c r="H38" s="23" t="n">
+        <v>-3.89</v>
+      </c>
+      <c r="I38" s="22" t="n">
+        <v>28.48</v>
+      </c>
+      <c r="J38" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K38" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1989,42 +1995,42 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>엑사이엔씨</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F39" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G39" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H39" s="22" t="n">
-        <v>-9.109999999999999</v>
-      </c>
-      <c r="I39" s="24" t="n">
-        <v>19.58</v>
-      </c>
-      <c r="J39" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +246% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K39" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
+        <v>3</v>
+      </c>
+      <c r="H39" s="23" t="n">
+        <v>-1.82</v>
+      </c>
+      <c r="I39" s="23" t="n">
+        <v>-1.43</v>
+      </c>
+      <c r="J39" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K39" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2032,42 +2038,42 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>흥구석유</t>
+          <t>HD현대중공업</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F40" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G40" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H40" s="22" t="n">
-        <v>-4.53</v>
-      </c>
-      <c r="I40" s="24" t="n">
-        <v>10.79</v>
-      </c>
-      <c r="J40" s="23" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K40" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
+        <v>3</v>
+      </c>
+      <c r="H40" s="23" t="n">
+        <v>-7.33</v>
+      </c>
+      <c r="I40" s="23" t="n">
+        <v>-8</v>
+      </c>
+      <c r="J40" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K40" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2075,7 +2081,7 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>이브이첨단소재</t>
+          <t>리가켐바이오</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
@@ -2090,18 +2096,18 @@
       <c r="G41" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="H41" s="22" t="n">
-        <v>-3.4</v>
-      </c>
-      <c r="I41" s="22" t="n">
-        <v>-28.6</v>
-      </c>
-      <c r="J41" s="23" t="inlineStr">
+      <c r="H41" s="23" t="n">
+        <v>-6.36</v>
+      </c>
+      <c r="I41" s="23" t="n">
+        <v>-14.3</v>
+      </c>
+      <c r="J41" s="24" t="inlineStr">
         <is>
           <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
-      <c r="K41" s="23" t="inlineStr">
+      <c r="K41" s="24" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
@@ -2110,7 +2116,7 @@
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2118,42 +2124,42 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>서진시스템</t>
+          <t>SK이노베이션</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E42" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F42" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G42" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H42" s="22" t="n">
-        <v>-6.32</v>
+        <v>0</v>
+      </c>
+      <c r="H42" s="23" t="n">
+        <v>-3.71</v>
       </c>
       <c r="I42" s="22" t="n">
-        <v>-17</v>
-      </c>
-      <c r="J42" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K42" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+        <v>6.08</v>
+      </c>
+      <c r="J42" s="24" t="inlineStr">
+        <is>
+          <t>네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K42" s="24" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2161,7 +2167,7 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>벡트</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
@@ -2176,27 +2182,27 @@
       <c r="G43" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H43" s="22" t="n">
-        <v>-2.8</v>
-      </c>
-      <c r="I43" s="22" t="n">
-        <v>-3.14</v>
-      </c>
-      <c r="J43" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K43" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="H43" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I43" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J43" s="24" t="inlineStr">
+        <is>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K43" s="24" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2204,7 +2210,7 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>우성머티리얼스</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
@@ -2219,27 +2225,25 @@
       <c r="G44" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="24" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="I44" s="24" t="n">
-        <v>10.38</v>
-      </c>
-      <c r="J44" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K44" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+      <c r="H44" s="23" t="n">
+        <v>-6.12</v>
+      </c>
+      <c r="I44" s="23" t="n">
+        <v>-7.09</v>
+      </c>
+      <c r="J44" s="24" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K44" s="24" t="n">
+        <v/>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2247,7 +2251,7 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
@@ -2262,27 +2266,25 @@
       <c r="G45" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H45" s="20" t="n">
+      <c r="H45" s="23" t="n">
+        <v>-6.48</v>
+      </c>
+      <c r="I45" s="23" t="n">
+        <v>-2.44</v>
+      </c>
+      <c r="J45" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K45" s="24" t="n">
         <v/>
-      </c>
-      <c r="I45" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J45" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K45" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
@@ -2290,7 +2292,7 @@
       </c>
       <c r="C46" s="21" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>현대모비스</t>
         </is>
       </c>
       <c r="D46" s="20" t="n">
@@ -2305,66 +2307,68 @@
       <c r="G46" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H46" s="22" t="n">
-        <v>-7.73</v>
-      </c>
-      <c r="I46" s="22" t="n">
-        <v>-1.86</v>
-      </c>
-      <c r="J46" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K46" s="23" t="n">
+      <c r="H46" s="23" t="n">
+        <v>-1.97</v>
+      </c>
+      <c r="I46" s="23" t="n">
+        <v>-3.08</v>
+      </c>
+      <c r="J46" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K46" s="24" t="n">
         <v/>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="20" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="B47" s="20" t="n">
+      <c r="A47" s="25" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B47" s="25" t="n">
         <v>34</v>
       </c>
-      <c r="C47" s="21" t="inlineStr">
-        <is>
-          <t>SK텔레콤</t>
-        </is>
-      </c>
-      <c r="D47" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E47" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F47" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" s="24" t="n">
-        <v>5.53</v>
-      </c>
-      <c r="I47" s="24" t="n">
-        <v>1.13</v>
-      </c>
-      <c r="J47" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K47" s="23" t="n">
-        <v/>
+      <c r="C47" s="26" t="inlineStr">
+        <is>
+          <t>레메디</t>
+        </is>
+      </c>
+      <c r="D47" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E47" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F47" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="27" t="n">
+        <v>-6.29</v>
+      </c>
+      <c r="I47" s="27" t="n">
+        <v>-43.77</v>
+      </c>
+      <c r="J47" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +1101%</t>
+        </is>
+      </c>
+      <c r="K47" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -2372,7 +2376,7 @@
       </c>
       <c r="C48" s="26" t="inlineStr">
         <is>
-          <t>레메디</t>
+          <t>미래생명자원</t>
         </is>
       </c>
       <c r="D48" s="25" t="n">
@@ -2387,15 +2391,15 @@
       <c r="G48" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H48" s="27" t="n">
-        <v>-20.15</v>
-      </c>
-      <c r="I48" s="27" t="n">
-        <v>-40</v>
+      <c r="H48" s="29" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="I48" s="29" t="n">
+        <v>43.75</v>
       </c>
       <c r="J48" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1088%</t>
+          <t>네이버 검색 당일 +611%</t>
         </is>
       </c>
       <c r="K48" s="28" t="inlineStr">
@@ -2407,7 +2411,7 @@
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -2415,7 +2419,7 @@
       </c>
       <c r="C49" s="26" t="inlineStr">
         <is>
-          <t>미래생명자원</t>
+          <t>에넥스</t>
         </is>
       </c>
       <c r="D49" s="25" t="n">
@@ -2431,14 +2435,14 @@
         <v>0</v>
       </c>
       <c r="H49" s="27" t="n">
-        <v>-4.02</v>
+        <v>-29.95</v>
       </c>
       <c r="I49" s="29" t="n">
-        <v>12.53</v>
+        <v>53.78</v>
       </c>
       <c r="J49" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +587%</t>
+          <t>네이버 검색 당일 +466%</t>
         </is>
       </c>
       <c r="K49" s="28" t="inlineStr">
@@ -2450,7 +2454,7 @@
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -2458,7 +2462,7 @@
       </c>
       <c r="C50" s="26" t="inlineStr">
         <is>
-          <t>에넥스</t>
+          <t>현대약품</t>
         </is>
       </c>
       <c r="D50" s="25" t="n">
@@ -2473,15 +2477,15 @@
       <c r="G50" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H50" s="29" t="n">
-        <v>29.95</v>
+      <c r="H50" s="27" t="n">
+        <v>-18.16</v>
       </c>
       <c r="I50" s="29" t="n">
-        <v>185.2</v>
+        <v>33.05</v>
       </c>
       <c r="J50" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +445%</t>
+          <t>네이버 검색 당일 +290%</t>
         </is>
       </c>
       <c r="K50" s="28" t="inlineStr">
@@ -2493,7 +2497,7 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -2501,7 +2505,7 @@
       </c>
       <c r="C51" s="26" t="inlineStr">
         <is>
-          <t>현대약품</t>
+          <t>씨피시스템</t>
         </is>
       </c>
       <c r="D51" s="25" t="n">
@@ -2516,15 +2520,15 @@
       <c r="G51" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H51" s="29" t="n">
-        <v>13.26</v>
+      <c r="H51" s="27" t="n">
+        <v>-0.45</v>
       </c>
       <c r="I51" s="29" t="n">
-        <v>55.58</v>
+        <v>39.38</v>
       </c>
       <c r="J51" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +276%</t>
+          <t>네이버 검색 당일 +241%</t>
         </is>
       </c>
       <c r="K51" s="28" t="inlineStr">
@@ -2536,7 +2540,7 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -2559,15 +2563,15 @@
       <c r="G52" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H52" s="29" t="n">
-        <v>6.01</v>
-      </c>
-      <c r="I52" s="29" t="n">
-        <v>18.3</v>
+      <c r="H52" s="27" t="n">
+        <v>-5.67</v>
+      </c>
+      <c r="I52" s="27" t="n">
+        <v>-1.36</v>
       </c>
       <c r="J52" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +226%</t>
+          <t>네이버 검색 당일 +239%</t>
         </is>
       </c>
       <c r="K52" s="28" t="inlineStr">
@@ -2579,7 +2583,7 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2587,7 +2591,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>씨피시스템</t>
+          <t>삼성공조</t>
         </is>
       </c>
       <c r="D53" s="25" t="n">
@@ -2602,15 +2606,15 @@
       <c r="G53" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="29" t="n">
-        <v>12.37</v>
+      <c r="H53" s="27" t="n">
+        <v>-7.51</v>
       </c>
       <c r="I53" s="29" t="n">
-        <v>54.84</v>
+        <v>24.6</v>
       </c>
       <c r="J53" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +223%</t>
+          <t>네이버 검색 당일 +190%</t>
         </is>
       </c>
       <c r="K53" s="28" t="inlineStr">
@@ -2622,7 +2626,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2630,7 +2634,7 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>삼성공조</t>
+          <t>동화약품</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -2645,15 +2649,15 @@
       <c r="G54" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H54" s="29" t="n">
-        <v>17.07</v>
+      <c r="H54" s="27" t="n">
+        <v>-11.85</v>
       </c>
       <c r="I54" s="29" t="n">
-        <v>42.65</v>
+        <v>0.6</v>
       </c>
       <c r="J54" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +177%</t>
+          <t>네이버 검색 당일 +138%</t>
         </is>
       </c>
       <c r="K54" s="28" t="inlineStr">
@@ -2665,7 +2669,7 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2673,7 +2677,7 @@
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>웰크론</t>
+          <t>모나리자</t>
         </is>
       </c>
       <c r="D55" s="25" t="n">
@@ -2688,15 +2692,15 @@
       <c r="G55" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H55" s="29" t="n">
-        <v>6.55</v>
+      <c r="H55" s="27" t="n">
+        <v>-19.82</v>
       </c>
       <c r="I55" s="29" t="n">
-        <v>29.09</v>
+        <v>29.27</v>
       </c>
       <c r="J55" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +172%</t>
+          <t>네이버 검색 당일 +136%</t>
         </is>
       </c>
       <c r="K55" s="28" t="inlineStr">
@@ -2708,7 +2712,7 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2716,7 +2720,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>동화약품</t>
+          <t>PN풍년</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2732,14 +2736,14 @@
         <v>0</v>
       </c>
       <c r="H56" s="27" t="n">
-        <v>-4.49</v>
+        <v>-13.52</v>
       </c>
       <c r="I56" s="29" t="n">
-        <v>11.24</v>
+        <v>16.17</v>
       </c>
       <c r="J56" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +127%</t>
+          <t>네이버 검색 당일 +132%</t>
         </is>
       </c>
       <c r="K56" s="28" t="inlineStr">
@@ -2751,7 +2755,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2759,7 +2763,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>모나리자</t>
+          <t>한탑</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2775,14 +2779,14 @@
         <v>0</v>
       </c>
       <c r="H57" s="29" t="n">
-        <v>29.94</v>
+        <v>13.79</v>
       </c>
       <c r="I57" s="29" t="n">
-        <v>54.23</v>
+        <v>82.98999999999999</v>
       </c>
       <c r="J57" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +116%</t>
+          <t>네이버 검색 당일 +114%</t>
         </is>
       </c>
       <c r="K57" s="28" t="inlineStr">
@@ -2794,7 +2798,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2802,7 +2806,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>명문제약</t>
+          <t>고려산업</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2818,14 +2822,14 @@
         <v>0</v>
       </c>
       <c r="H58" s="29" t="n">
-        <v>5.78</v>
+        <v>29.99</v>
       </c>
       <c r="I58" s="29" t="n">
-        <v>10.91</v>
+        <v>36.65</v>
       </c>
       <c r="J58" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +114%</t>
+          <t>네이버 검색 당일 +100%</t>
         </is>
       </c>
       <c r="K58" s="28" t="inlineStr">
@@ -2837,7 +2841,7 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2845,7 +2849,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>한탑</t>
+          <t>한일사료</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2861,14 +2865,14 @@
         <v>0</v>
       </c>
       <c r="H59" s="29" t="n">
-        <v>14.62</v>
+        <v>14.94</v>
       </c>
       <c r="I59" s="29" t="n">
-        <v>51.4</v>
+        <v>11.69</v>
       </c>
       <c r="J59" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +108%</t>
+          <t>네이버 검색 당일 +100%</t>
         </is>
       </c>
       <c r="K59" s="28" t="inlineStr">
@@ -2880,7 +2884,7 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2888,7 +2892,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>코아스</t>
+          <t>엔피</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2903,15 +2907,15 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="29" t="n">
-        <v>29.27</v>
+      <c r="H60" s="27" t="n">
+        <v>-7.8</v>
       </c>
       <c r="I60" s="29" t="n">
-        <v>42.56</v>
+        <v>21.86</v>
       </c>
       <c r="J60" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +73% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +95% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K60" s="28" t="inlineStr">
@@ -2923,7 +2927,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2931,7 +2935,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>온코닉테라퓨틱스</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2946,27 +2950,27 @@
       <c r="G61" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H61" s="29" t="n">
-        <v>20.33</v>
-      </c>
-      <c r="I61" s="29" t="n">
-        <v>23.93</v>
+      <c r="H61" s="27" t="n">
+        <v>-3.08</v>
+      </c>
+      <c r="I61" s="27" t="n">
+        <v>-16.41</v>
       </c>
       <c r="J61" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +70% / 중요공시 1건</t>
+          <t>중요공시 2건 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K61" s="28" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2974,40 +2978,42 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>SK증권</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E62" s="25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F62" s="25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G62" s="25" t="n">
         <v>0</v>
       </c>
       <c r="H62" s="27" t="n">
-        <v>-3.42</v>
+        <v>-4.03</v>
       </c>
       <c r="I62" s="27" t="n">
-        <v>-8.130000000000001</v>
+        <v>-9.18</v>
       </c>
       <c r="J62" s="28" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K62" s="28" t="n">
-        <v/>
+          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+        </is>
+      </c>
+      <c r="K62" s="28" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3015,7 +3021,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>엔켐</t>
+          <t>비비안</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3030,11 +3036,11 @@
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="29" t="n">
-        <v>9.58</v>
+      <c r="H63" s="27" t="n">
+        <v>-30</v>
       </c>
       <c r="I63" s="29" t="n">
-        <v>1.52</v>
+        <v>53.58</v>
       </c>
       <c r="J63" s="28" t="inlineStr">
         <is>
@@ -3140,22 +3146,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3171,29 +3177,29 @@
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H4" s="27" t="n">
-        <v>-11.53</v>
+        <v>-4.23</v>
       </c>
       <c r="I4" s="27" t="n">
-        <v>-15.5</v>
+        <v>-4.39</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
@@ -3206,88 +3212,92 @@
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H5" s="27" t="n">
-        <v>-8.77</v>
+        <v>-4.31</v>
       </c>
       <c r="I5" s="27" t="n">
-        <v>-10.53</v>
+        <v>-4.13</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H6" s="25" t="n"/>
-      <c r="I6" s="25" t="n"/>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H6" s="27" t="n">
+        <v>-3.85</v>
+      </c>
+      <c r="I6" s="27" t="n">
+        <v>-4.33</v>
+      </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H7" s="25" t="n"/>
@@ -3296,7 +3306,7 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>TSMC</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
@@ -3313,12 +3323,12 @@
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H8" s="25" t="n"/>
@@ -3327,29 +3337,29 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H9" s="25" t="n"/>
@@ -3358,7 +3368,7 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
@@ -3375,12 +3385,12 @@
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H10" s="25" t="n"/>
@@ -3389,7 +3399,7 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>엑시온그룹</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
@@ -3406,161 +3416,157 @@
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H11" s="29" t="n">
-        <v>2.76</v>
-      </c>
-      <c r="I11" s="27" t="n">
-        <v>-3.97</v>
+        <v>29.93</v>
+      </c>
+      <c r="I11" s="29" t="n">
+        <v>137.57</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>TSMC</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H12" s="27" t="n">
-        <v>-2.07</v>
-      </c>
-      <c r="I12" s="27" t="n">
-        <v>-7.1</v>
-      </c>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H12" s="25" t="n"/>
+      <c r="I12" s="25" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>KB금융</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H13" s="27" t="n">
-        <v>-3.52</v>
+        <v>-6.79</v>
       </c>
       <c r="I13" s="27" t="n">
-        <v>-2.47</v>
+        <v>-9.34</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>다보링크</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H14" s="29" t="n">
-        <v>4.18</v>
-      </c>
-      <c r="I14" s="29" t="n">
-        <v>38.35</v>
-      </c>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H14" s="25" t="n"/>
+      <c r="I14" s="25" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>에스아이리소스</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E15" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H15" s="25" t="n"/>
-      <c r="I15" s="25" t="n"/>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H15" s="27" t="n">
+        <v>-21.6</v>
+      </c>
+      <c r="I15" s="27" t="n">
+        <v>-44.94</v>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>파두</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -3577,270 +3583,266 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H16" s="27" t="n">
-        <v>-9.619999999999999</v>
-      </c>
-      <c r="I16" s="27" t="n">
-        <v>-19.38</v>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H16" s="29" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="I16" s="29" t="n">
+        <v>1.42</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>알테오젠</t>
+          <t>삼기에너지솔루션즈</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E17" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H17" s="27" t="n">
-        <v>-4.16</v>
+        <v>-7.31</v>
       </c>
       <c r="I17" s="27" t="n">
-        <v>-14.66</v>
+        <v>-14.98</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>진영</t>
+          <t>하나마이크론</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E18" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H18" s="29" t="n">
-        <v>29.96</v>
-      </c>
-      <c r="I18" s="29" t="n">
-        <v>28.14</v>
+        <v>2.52</v>
+      </c>
+      <c r="I18" s="27" t="n">
+        <v>-4.06</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>GS건설</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H19" s="29" t="n">
-        <v>1.22</v>
-      </c>
-      <c r="I19" s="29" t="n">
-        <v>3.24</v>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H19" s="27" t="n">
+        <v>-4.58</v>
+      </c>
+      <c r="I19" s="27" t="n">
+        <v>-11.54</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>defense stock</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D20" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H20" s="27" t="n">
-        <v>-0.5600000000000001</v>
-      </c>
-      <c r="I20" s="27" t="n">
-        <v>-0.93</v>
-      </c>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H20" s="25" t="n"/>
+      <c r="I20" s="25" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>리가켐바이오</t>
+          <t>금호타이어</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D21" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E21" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H21" s="27" t="n">
-        <v>-6.58</v>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H21" s="29" t="n">
+        <v>4.27</v>
       </c>
       <c r="I21" s="27" t="n">
-        <v>-13.8</v>
+        <v>-14.8</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D22" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E22" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H22" s="27" t="n">
-        <v>-11.29</v>
+        <v>-5.08</v>
       </c>
       <c r="I22" s="27" t="n">
-        <v>-19.5</v>
+        <v>-9.85</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>수성웹툰</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D23" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E23" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H23" s="29" t="n">
-        <v>11.36</v>
-      </c>
-      <c r="I23" s="29" t="n">
-        <v>41.1</v>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H23" s="27" t="n">
+        <v>-2.53</v>
+      </c>
+      <c r="I23" s="27" t="n">
+        <v>-14.85</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>대구백화점</t>
+          <t>제이케이시냅스</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3857,60 +3859,60 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H24" s="29" t="n">
-        <v>5.96</v>
+        <v>16.74</v>
       </c>
       <c r="I24" s="29" t="n">
-        <v>24.76</v>
+        <v>32.42</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>에스아이리소스</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C25" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D25" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E25" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H25" s="27" t="n">
-        <v>-29.78</v>
+        <v>-6.12</v>
       </c>
       <c r="I25" s="27" t="n">
-        <v>-29.78</v>
+        <v>-7.09</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>HD현대중공업</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
@@ -3927,25 +3929,25 @@
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H26" s="27" t="n">
-        <v>-7.73</v>
+        <v>-7.33</v>
       </c>
       <c r="I26" s="27" t="n">
-        <v>-1.86</v>
+        <v>-8</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>SK텔레콤</t>
+          <t>SK이노베이션</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
@@ -3962,25 +3964,25 @@
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H27" s="29" t="n">
-        <v>5.53</v>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H27" s="27" t="n">
+        <v>-3.71</v>
       </c>
       <c r="I27" s="29" t="n">
-        <v>1.13</v>
+        <v>6.08</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>STX그린로지스</t>
+          <t>기가레인</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
@@ -3997,25 +3999,25 @@
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H28" s="27" t="n">
-        <v>-14.84</v>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H28" s="29" t="n">
+        <v>15.06</v>
       </c>
       <c r="I28" s="29" t="n">
-        <v>63</v>
+        <v>67.40000000000001</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>기가레인</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
@@ -4032,25 +4034,25 @@
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H29" s="27" t="n">
-        <v>-3.75</v>
-      </c>
-      <c r="I29" s="29" t="n">
-        <v>89.11</v>
+        <v>-6.48</v>
+      </c>
+      <c r="I29" s="27" t="n">
+        <v>-2.44</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>벡트</t>
+          <t>다보링크</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -4067,25 +4069,25 @@
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H30" s="27" t="n">
-        <v>-2.8</v>
-      </c>
-      <c r="I30" s="27" t="n">
-        <v>-3.14</v>
+        <v>-3.89</v>
+      </c>
+      <c r="I30" s="29" t="n">
+        <v>28.48</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>서진시스템</t>
+          <t>리가켐바이오</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
@@ -4102,25 +4104,25 @@
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H31" s="27" t="n">
-        <v>-6.32</v>
+        <v>-6.36</v>
       </c>
       <c r="I31" s="27" t="n">
-        <v>-17</v>
+        <v>-14.3</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>엑사이엔씨</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -4137,25 +4139,21 @@
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H32" s="27" t="n">
-        <v>-9.109999999999999</v>
-      </c>
-      <c r="I32" s="29" t="n">
-        <v>19.58</v>
-      </c>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H32" s="25" t="n"/>
+      <c r="I32" s="25" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4172,21 +4170,25 @@
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H33" s="25" t="n"/>
-      <c r="I33" s="25" t="n"/>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H33" s="27" t="n">
+        <v>-1.82</v>
+      </c>
+      <c r="I33" s="27" t="n">
+        <v>-1.43</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>우성머티리얼스</t>
+          <t>엑사이엔씨</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4203,25 +4205,25 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H34" s="29" t="n">
-        <v>0.36</v>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H34" s="27" t="n">
+        <v>-6.35</v>
       </c>
       <c r="I34" s="29" t="n">
-        <v>10.38</v>
+        <v>12.16</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>이브이첨단소재</t>
+          <t>현대모비스</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -4238,60 +4240,60 @@
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H35" s="27" t="n">
-        <v>-3.4</v>
+        <v>-1.97</v>
       </c>
       <c r="I35" s="27" t="n">
-        <v>-28.6</v>
+        <v>-3.08</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>흥구석유</t>
+          <t>PN풍년</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C36" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D36" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E36" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H36" s="27" t="n">
-        <v>-4.53</v>
+        <v>-13.52</v>
       </c>
       <c r="I36" s="29" t="n">
-        <v>10.79</v>
+        <v>16.17</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>SK증권</t>
+          <t>고려산업</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
@@ -4308,25 +4310,25 @@
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H37" s="27" t="n">
-        <v>-3.42</v>
-      </c>
-      <c r="I37" s="27" t="n">
-        <v>-8.130000000000001</v>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H37" s="29" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="I37" s="29" t="n">
+        <v>36.65</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>동화약품</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4343,25 +4345,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H38" s="27" t="n">
-        <v>-4.49</v>
-      </c>
-      <c r="I38" s="29" t="n">
-        <v>11.24</v>
+        <v>-4.03</v>
+      </c>
+      <c r="I38" s="27" t="n">
+        <v>-9.18</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>레메디</t>
+          <t>동화약품</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4378,25 +4380,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H39" s="27" t="n">
-        <v>-20.15</v>
-      </c>
-      <c r="I39" s="27" t="n">
-        <v>-40</v>
+        <v>-11.85</v>
+      </c>
+      <c r="I39" s="29" t="n">
+        <v>0.6</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>명문제약</t>
+          <t>레메디</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4413,19 +4415,19 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H40" s="29" t="n">
-        <v>5.78</v>
-      </c>
-      <c r="I40" s="29" t="n">
-        <v>10.91</v>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H40" s="27" t="n">
+        <v>-6.29</v>
+      </c>
+      <c r="I40" s="27" t="n">
+        <v>-43.77</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
@@ -4448,19 +4450,19 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H41" s="29" t="n">
-        <v>29.94</v>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H41" s="27" t="n">
+        <v>-19.82</v>
       </c>
       <c r="I41" s="29" t="n">
-        <v>54.23</v>
+        <v>29.27</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
@@ -4483,25 +4485,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H42" s="27" t="n">
-        <v>-4.02</v>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H42" s="29" t="n">
+        <v>29.8</v>
       </c>
       <c r="I42" s="29" t="n">
-        <v>12.53</v>
+        <v>43.75</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>삼성공조</t>
+          <t>비비안</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4518,25 +4520,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H43" s="29" t="n">
-        <v>17.07</v>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H43" s="27" t="n">
+        <v>-30</v>
       </c>
       <c r="I43" s="29" t="n">
-        <v>42.65</v>
+        <v>53.58</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>씨피시스템</t>
+          <t>삼성공조</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4553,25 +4555,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H44" s="29" t="n">
-        <v>12.37</v>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H44" s="27" t="n">
+        <v>-7.51</v>
       </c>
       <c r="I44" s="29" t="n">
-        <v>54.84</v>
+        <v>24.6</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>에넥스</t>
+          <t>씨피시스템</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4588,25 +4590,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H45" s="29" t="n">
-        <v>29.95</v>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H45" s="27" t="n">
+        <v>-0.45</v>
       </c>
       <c r="I45" s="29" t="n">
-        <v>185.2</v>
+        <v>39.38</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>에스씨디</t>
+          <t>에넥스</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4623,25 +4625,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H46" s="29" t="n">
-        <v>6.01</v>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H46" s="27" t="n">
+        <v>-29.95</v>
       </c>
       <c r="I46" s="29" t="n">
-        <v>18.3</v>
+        <v>53.78</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>엔켐</t>
+          <t>에스씨디</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4658,25 +4660,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H47" s="29" t="n">
-        <v>9.58</v>
-      </c>
-      <c r="I47" s="29" t="n">
-        <v>1.52</v>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H47" s="27" t="n">
+        <v>-5.67</v>
+      </c>
+      <c r="I47" s="27" t="n">
+        <v>-1.36</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>온코닉테라퓨틱스</t>
+          <t>엔피</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4693,25 +4695,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H48" s="29" t="n">
-        <v>20.33</v>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H48" s="27" t="n">
+        <v>-7.8</v>
       </c>
       <c r="I48" s="29" t="n">
-        <v>23.93</v>
+        <v>21.86</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>웰크론</t>
+          <t>한일사료</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4728,25 +4730,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H49" s="29" t="n">
-        <v>6.55</v>
+        <v>14.94</v>
       </c>
       <c r="I49" s="29" t="n">
-        <v>29.09</v>
+        <v>11.69</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>코아스</t>
+          <t>한탑</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4763,25 +4765,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H50" s="29" t="n">
-        <v>29.27</v>
+        <v>13.79</v>
       </c>
       <c r="I50" s="29" t="n">
-        <v>42.56</v>
+        <v>82.98999999999999</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>한탑</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4798,19 +4800,19 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H51" s="29" t="n">
-        <v>14.62</v>
-      </c>
-      <c r="I51" s="29" t="n">
-        <v>51.4</v>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H51" s="27" t="n">
+        <v>-3.08</v>
+      </c>
+      <c r="I51" s="27" t="n">
+        <v>-16.41</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
@@ -4833,19 +4835,19 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="H52" s="29" t="n">
-        <v>13.26</v>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="H52" s="27" t="n">
+        <v>-18.16</v>
       </c>
       <c r="I52" s="29" t="n">
-        <v>55.58</v>
+        <v>33.05</v>
       </c>
     </row>
   </sheetData>
@@ -4929,19 +4931,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4960,19 +4962,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4984,26 +4986,26 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="35" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B5" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5015,26 +5017,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5053,19 +5055,19 @@
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5084,19 +5086,19 @@
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5115,19 +5117,19 @@
         <v>1</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5220,7 +5222,7 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -5247,7 +5249,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5274,7 +5276,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5301,7 +5303,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -5328,7 +5330,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-08-01 07:04 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -57,13 +57,13 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="002563EB"/>
+      <color rgb="00E53935"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00E53935"/>
+      <color rgb="002563EB"/>
       <sz val="10"/>
     </font>
     <font>
@@ -258,10 +258,10 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -276,11 +276,11 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-07-31 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-08-01 06:54</t>
         </is>
       </c>
     </row>
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-31) 상위: 반도체  점수 77.0점</t>
+          <t>⚡ 최신(2026-08-01) 상위: 반도체  점수 72.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-31) 상위: 삼성전자  점수 67.0점</t>
+          <t>⚡ 최신(2026-08-01) 상위: SK  점수 58.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-07-31) 상위: LG  점수 33.0점</t>
+          <t>⚡ 최신(2026-08-01) 상위: SK하이닉스  점수 35.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -967,42 +967,40 @@
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>SK</t>
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G15" s="15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>-0.72</v>
-      </c>
-      <c r="I15" s="18" t="n">
-        <v>-23.33</v>
+        <v>18.89</v>
+      </c>
+      <c r="I15" s="19" t="n">
+        <v>-11.59</v>
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 7일 +200% / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K15" s="17" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K15" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1010,14 +1008,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1025,25 +1023,27 @@
       <c r="G16" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="19" t="n">
-        <v>4.56</v>
-      </c>
-      <c r="I16" s="18" t="n">
-        <v>-5.12</v>
+      <c r="H16" s="18" t="n">
+        <v>29.95</v>
+      </c>
+      <c r="I16" s="19" t="n">
+        <v>-2.33</v>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K16" s="17" t="n">
-        <v/>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K16" s="17" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1051,14 +1051,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1067,26 +1067,26 @@
         <v>0</v>
       </c>
       <c r="H17" s="18" t="n">
-        <v>-5.64</v>
+        <v>26.81</v>
       </c>
       <c r="I17" s="18" t="n">
-        <v>-31.11</v>
+        <v>5.21</v>
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 3건 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1098,10 +1098,10 @@
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K18" s="17" t="inlineStr">
@@ -1129,7 +1129,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1137,14 +1137,14 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1152,27 +1152,25 @@
       <c r="G19" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="15" t="n">
+      <c r="H19" s="18" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="I19" s="18" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="J19" s="17" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K19" s="17" t="n">
         <v/>
-      </c>
-      <c r="I19" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J19" s="17" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K19" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1180,14 +1178,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1195,27 +1193,27 @@
       <c r="G20" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="18" t="n">
-        <v>-1.66</v>
-      </c>
-      <c r="I20" s="18" t="n">
-        <v>-21.07</v>
+      <c r="H20" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I20" s="15" t="n">
+        <v/>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K20" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1223,14 +1221,14 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
@@ -1238,27 +1236,27 @@
       <c r="G21" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="18" t="n">
-        <v>-14.58</v>
-      </c>
-      <c r="I21" s="18" t="n">
-        <v>-39.3</v>
+      <c r="H21" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I21" s="15" t="n">
+        <v/>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1266,14 +1264,14 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -1281,27 +1279,27 @@
       <c r="G22" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I22" s="15" t="n">
-        <v/>
+      <c r="H22" s="18" t="n">
+        <v>29.92</v>
+      </c>
+      <c r="I22" s="19" t="n">
+        <v>-13.88</v>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 1건 / 매일경제 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1313,10 +1311,10 @@
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F23" s="15" t="n">
         <v>0</v>
@@ -1332,7 +1330,7 @@
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K23" s="17" t="n">
@@ -1342,7 +1340,7 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1350,30 +1348,30 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>LG생활건강</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G24" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="19" t="n">
-        <v>11.03</v>
+        <v>3</v>
+      </c>
+      <c r="H24" s="18" t="n">
+        <v>14.11</v>
       </c>
       <c r="I24" s="19" t="n">
-        <v>17.74</v>
+        <v>-16.47</v>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 5건 / 중요공시 3일 +400% / 중요공시 7일 +150% / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K24" s="17" t="inlineStr">
@@ -1385,7 +1383,7 @@
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1393,14 +1391,14 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F25" s="15" t="n">
         <v>0</v>
@@ -1408,15 +1406,15 @@
       <c r="G25" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H25" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I25" s="15" t="n">
-        <v/>
+      <c r="H25" s="18" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="I25" s="18" t="n">
+        <v>3.31</v>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K25" s="17" t="n">
@@ -1426,7 +1424,7 @@
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1434,40 +1432,42 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="F26" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G26" s="15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H26" s="18" t="n">
-        <v>-0.71</v>
-      </c>
-      <c r="I26" s="18" t="n">
-        <v>-18.75</v>
+        <v>7.44</v>
+      </c>
+      <c r="I26" s="19" t="n">
+        <v>-3.07</v>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K26" s="17" t="n">
-        <v/>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100% / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K26" s="17" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -1475,42 +1475,42 @@
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D27" s="15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E27" s="15" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="F27" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G27" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H27" s="19" t="n">
-        <v>5.56</v>
-      </c>
-      <c r="I27" s="19" t="n">
-        <v>10.34</v>
+        <v>0</v>
+      </c>
+      <c r="H27" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I27" s="15" t="n">
+        <v/>
       </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
-          <t>중요공시 6건 / 중요공시 3일 +50% / 중요공시 7일 +200%</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K27" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B28" s="15" t="n">
@@ -1518,30 +1518,30 @@
       </c>
       <c r="C28" s="16" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>기업은행</t>
         </is>
       </c>
       <c r="D28" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E28" s="15" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F28" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G28" s="15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H28" s="18" t="n">
-        <v>-6.82</v>
-      </c>
-      <c r="I28" s="18" t="n">
-        <v>-31.46</v>
+        <v>0.98</v>
+      </c>
+      <c r="I28" s="19" t="n">
+        <v>-3.28</v>
       </c>
       <c r="J28" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +50%</t>
+          <t>중요공시 1건 / 매일경제 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K28" s="17" t="inlineStr">
@@ -1553,7 +1553,7 @@
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B29" s="15" t="n">
@@ -1561,42 +1561,40 @@
       </c>
       <c r="C29" s="16" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="D29" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E29" s="15" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F29" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G29" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H29" s="19" t="n">
-        <v>2.98</v>
-      </c>
-      <c r="I29" s="18" t="n">
-        <v>-18.33</v>
+        <v>0</v>
+      </c>
+      <c r="H29" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I29" s="15" t="n">
+        <v/>
       </c>
       <c r="J29" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +200%</t>
-        </is>
-      </c>
-      <c r="K29" s="17" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K29" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B30" s="15" t="n">
@@ -1604,7 +1602,7 @@
       </c>
       <c r="C30" s="16" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D30" s="15" t="n">
@@ -1619,15 +1617,15 @@
       <c r="G30" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H30" s="19" t="n">
-        <v>2.73</v>
-      </c>
-      <c r="I30" s="18" t="n">
-        <v>-13.92</v>
+      <c r="H30" s="18" t="n">
+        <v>10.54</v>
+      </c>
+      <c r="I30" s="19" t="n">
+        <v>-3.24</v>
       </c>
       <c r="J30" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K30" s="17" t="n">
@@ -1637,7 +1635,7 @@
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1645,30 +1643,30 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>BNK금융지주</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F31" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G31" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H31" s="22" t="n">
-        <v>2.84</v>
+        <v>2.5</v>
       </c>
       <c r="I31" s="23" t="n">
-        <v>-21.67</v>
+        <v>-15.91</v>
       </c>
       <c r="J31" s="24" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 중요공시 7일 +100%</t>
+          <t>중요공시 6건 / 중요공시 3일 +500%</t>
         </is>
       </c>
       <c r="K31" s="24" t="inlineStr">
@@ -1680,7 +1678,7 @@
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1688,7 +1686,7 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
@@ -1704,24 +1702,26 @@
         <v>0</v>
       </c>
       <c r="H32" s="22" t="n">
-        <v>2.41</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="I32" s="23" t="n">
-        <v>-2.69</v>
+        <v>-4.2</v>
       </c>
       <c r="J32" s="24" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K32" s="24" t="n">
-        <v/>
+          <t>중요공시 4건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K32" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1729,30 +1729,30 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F33" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G33" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="23" t="n">
-        <v>-0.6</v>
+      <c r="H33" s="22" t="n">
+        <v>26.08</v>
       </c>
       <c r="I33" s="23" t="n">
-        <v>-4.27</v>
+        <v>-14.38</v>
       </c>
       <c r="J33" s="24" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+          <t>중요공시 3건 / 중요공시 7일 +200%</t>
         </is>
       </c>
       <c r="K33" s="24" t="inlineStr">
@@ -1764,7 +1764,7 @@
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1772,30 +1772,30 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>HD한국조선해양</t>
+          <t>삼성물산</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F34" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G34" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H34" s="22" t="n">
-        <v>10</v>
-      </c>
-      <c r="I34" s="23" t="n">
-        <v>-3.28</v>
+        <v>19.56</v>
+      </c>
+      <c r="I34" s="22" t="n">
+        <v>2.78</v>
       </c>
       <c r="J34" s="24" t="inlineStr">
         <is>
-          <t>중요공시 9건 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K34" s="24" t="inlineStr">
@@ -1807,7 +1807,7 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1815,42 +1815,40 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>BNK금융지주</t>
+          <t>스테이블코인</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F35" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G35" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H35" s="23" t="n">
-        <v>-1.07</v>
-      </c>
-      <c r="I35" s="23" t="n">
-        <v>-16.71</v>
+      <c r="H35" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I35" s="20" t="n">
+        <v/>
       </c>
       <c r="J35" s="24" t="inlineStr">
         <is>
-          <t>중요공시 7건 / 중요공시 3일 +600% / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K35" s="24" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K35" s="24" t="n">
+        <v/>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1858,42 +1856,42 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F36" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G36" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H36" s="22" t="n">
-        <v>3.49</v>
-      </c>
-      <c r="I36" s="23" t="n">
-        <v>-4.52</v>
+        <v>0</v>
+      </c>
+      <c r="H36" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I36" s="20" t="n">
+        <v/>
       </c>
       <c r="J36" s="24" t="inlineStr">
         <is>
-          <t>중요공시 7건 / 중요공시 7일 +600%</t>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K36" s="24" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1901,42 +1899,40 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>카카오뱅크</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E37" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F37" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G37" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H37" s="22" t="n">
-        <v>3.23</v>
-      </c>
-      <c r="I37" s="23" t="n">
-        <v>-10.04</v>
+        <v>1.38</v>
+      </c>
+      <c r="I37" s="22" t="n">
+        <v>0.23</v>
       </c>
       <c r="J37" s="24" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K37" s="24" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K37" s="24" t="n">
+        <v/>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1944,30 +1940,30 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>한솔테크닉스</t>
+          <t>미래산업</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E38" s="20" t="n">
         <v>3</v>
       </c>
       <c r="F38" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G38" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H38" s="23" t="n">
-        <v>-3.59</v>
+        <v>0</v>
+      </c>
+      <c r="H38" s="22" t="n">
+        <v>18.43</v>
       </c>
       <c r="I38" s="23" t="n">
-        <v>-35.4</v>
+        <v>-20.72</v>
       </c>
       <c r="J38" s="24" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 7일 +200%</t>
+          <t>중요공시 3건 / 중요공시 3일 +50%</t>
         </is>
       </c>
       <c r="K38" s="24" t="inlineStr">
@@ -1979,7 +1975,7 @@
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1987,30 +1983,30 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>지엔씨에너지</t>
+          <t>파두</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F39" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G39" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H39" s="22" t="n">
-        <v>4.02</v>
+        <v>29.92</v>
       </c>
       <c r="I39" s="23" t="n">
-        <v>-34.69</v>
+        <v>-1.71</v>
       </c>
       <c r="J39" s="24" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+          <t>중요공시 1건 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K39" s="24" t="inlineStr">
@@ -2022,7 +2018,7 @@
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2030,42 +2026,42 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F40" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G40" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H40" s="22" t="n">
-        <v>3.14</v>
-      </c>
-      <c r="I40" s="23" t="n">
-        <v>-12.11</v>
+      <c r="H40" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I40" s="20" t="n">
+        <v/>
       </c>
       <c r="J40" s="24" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +50%</t>
+          <t>Google 급상승 검색어 등장 (US)</t>
         </is>
       </c>
       <c r="K40" s="24" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2073,7 +2069,7 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>Netflix</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
@@ -2088,27 +2084,27 @@
       <c r="G41" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="23" t="n">
-        <v>-1.51</v>
-      </c>
-      <c r="I41" s="23" t="n">
-        <v>-23.23</v>
+      <c r="H41" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I41" s="20" t="n">
+        <v/>
       </c>
       <c r="J41" s="24" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>Google 급상승 검색어 등장 (US)</t>
         </is>
       </c>
       <c r="K41" s="24" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2116,7 +2112,7 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
@@ -2131,25 +2127,27 @@
       <c r="G42" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H42" s="22" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="I42" s="23" t="n">
-        <v>-11</v>
+      <c r="H42" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I42" s="20" t="n">
+        <v/>
       </c>
       <c r="J42" s="24" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K42" s="24" t="n">
-        <v/>
+          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K42" s="24" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2173,26 +2171,26 @@
         <v>0</v>
       </c>
       <c r="H43" s="22" t="n">
-        <v>29.97</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="I43" s="23" t="n">
-        <v>-32.45</v>
+        <v>-26.2</v>
       </c>
       <c r="J43" s="24" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +166% / 중요공시 2건</t>
+          <t>네이버 검색 당일 +298% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K43" s="24" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2200,7 +2198,7 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>대한전선</t>
+          <t>주성엔지니어링</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
@@ -2215,11 +2213,11 @@
       <c r="G44" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="23" t="n">
-        <v>-6.31</v>
+      <c r="H44" s="22" t="n">
+        <v>26.65</v>
       </c>
       <c r="I44" s="23" t="n">
-        <v>-32.9</v>
+        <v>-11.7</v>
       </c>
       <c r="J44" s="24" t="inlineStr">
         <is>
@@ -2228,14 +2226,14 @@
       </c>
       <c r="K44" s="24" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2258,11 +2256,11 @@
       <c r="G45" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H45" s="23" t="n">
-        <v>-0.35</v>
+      <c r="H45" s="22" t="n">
+        <v>7.85</v>
       </c>
       <c r="I45" s="23" t="n">
-        <v>-18.51</v>
+        <v>-6.02</v>
       </c>
       <c r="J45" s="24" t="inlineStr">
         <is>
@@ -2278,7 +2276,7 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
@@ -2286,30 +2284,30 @@
       </c>
       <c r="C46" s="21" t="inlineStr">
         <is>
-          <t>HD현대일렉트릭</t>
+          <t>HD현대마린엔진</t>
         </is>
       </c>
       <c r="D46" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E46" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F46" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G46" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" s="23" t="n">
-        <v>-0.51</v>
+        <v>3</v>
+      </c>
+      <c r="H46" s="22" t="n">
+        <v>3.24</v>
       </c>
       <c r="I46" s="23" t="n">
-        <v>-32.91</v>
+        <v>-26.85</v>
       </c>
       <c r="J46" s="24" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 매일경제 기사 언급</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K46" s="24" t="inlineStr">
@@ -2321,7 +2319,7 @@
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B47" s="20" t="n">
@@ -2329,7 +2327,7 @@
       </c>
       <c r="C47" s="21" t="inlineStr">
         <is>
-          <t>현대모비스</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="D47" s="20" t="n">
@@ -2344,15 +2342,15 @@
       <c r="G47" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H47" s="20" t="n">
-        <v>0</v>
+      <c r="H47" s="22" t="n">
+        <v>15.79</v>
       </c>
       <c r="I47" s="23" t="n">
-        <v>-15.08</v>
+        <v>-10.92</v>
       </c>
       <c r="J47" s="24" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 매일경제 기사 언급</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K47" s="24" t="inlineStr">
@@ -2364,7 +2362,7 @@
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B48" s="20" t="n">
@@ -2372,7 +2370,7 @@
       </c>
       <c r="C48" s="21" t="inlineStr">
         <is>
-          <t>LG이노텍</t>
+          <t>네이처셀</t>
         </is>
       </c>
       <c r="D48" s="20" t="n">
@@ -2388,26 +2386,26 @@
         <v>0</v>
       </c>
       <c r="H48" s="23" t="n">
-        <v>-7.42</v>
+        <v>-3.51</v>
       </c>
       <c r="I48" s="23" t="n">
-        <v>-37.56</v>
+        <v>-8.710000000000001</v>
       </c>
       <c r="J48" s="24" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K48" s="24" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B49" s="20" t="n">
@@ -2415,7 +2413,7 @@
       </c>
       <c r="C49" s="21" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>호텔신라</t>
         </is>
       </c>
       <c r="D49" s="20" t="n">
@@ -2430,27 +2428,27 @@
       <c r="G49" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I49" s="20" t="n">
-        <v/>
+      <c r="H49" s="22" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="I49" s="23" t="n">
+        <v>-7.54</v>
       </c>
       <c r="J49" s="24" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K49" s="24" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B50" s="20" t="n">
@@ -2458,7 +2456,7 @@
       </c>
       <c r="C50" s="21" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>넥스트아이</t>
         </is>
       </c>
       <c r="D50" s="20" t="n">
@@ -2473,68 +2471,70 @@
       <c r="G50" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H50" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I50" s="20" t="n">
-        <v/>
+      <c r="H50" s="22" t="n">
+        <v>10.96</v>
+      </c>
+      <c r="I50" s="22" t="n">
+        <v>1.28</v>
       </c>
       <c r="J50" s="24" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K50" s="24" t="n">
-        <v/>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K50" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="25" t="inlineStr">
-        <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="B51" s="25" t="n">
+      <c r="A51" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B51" s="20" t="n">
         <v>38</v>
       </c>
-      <c r="C51" s="26" t="inlineStr">
-        <is>
-          <t>더테크놀로지</t>
-        </is>
-      </c>
-      <c r="D51" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E51" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F51" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G51" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H51" s="27" t="n">
-        <v>-80</v>
-      </c>
-      <c r="I51" s="27" t="n">
-        <v>-80</v>
-      </c>
-      <c r="J51" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +59% / 중요공시 2건</t>
-        </is>
-      </c>
-      <c r="K51" s="28" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
+      <c r="C51" s="21" t="inlineStr">
+        <is>
+          <t>LG화학</t>
+        </is>
+      </c>
+      <c r="D51" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E51" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F51" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="22" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="I51" s="23" t="n">
+        <v>-0.39</v>
+      </c>
+      <c r="J51" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K51" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -2542,7 +2542,7 @@
       </c>
       <c r="C52" s="26" t="inlineStr">
         <is>
-          <t>우리금융지주</t>
+          <t>두산퓨얼셀</t>
         </is>
       </c>
       <c r="D52" s="25" t="n">
@@ -2557,27 +2557,27 @@
       <c r="G52" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H52" s="29" t="n">
-        <v>2.03</v>
-      </c>
-      <c r="I52" s="29" t="n">
-        <v>5.83</v>
-      </c>
-      <c r="J52" s="28" t="inlineStr">
-        <is>
-          <t>중요공시 5건</t>
-        </is>
-      </c>
-      <c r="K52" s="28" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="H52" s="27" t="n">
+        <v>29.89</v>
+      </c>
+      <c r="I52" s="28" t="n">
+        <v>-42.64</v>
+      </c>
+      <c r="J52" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +154%</t>
+        </is>
+      </c>
+      <c r="K52" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2585,7 +2585,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>LG유플러스</t>
+          <t>셀리드</t>
         </is>
       </c>
       <c r="D53" s="25" t="n">
@@ -2600,27 +2600,27 @@
       <c r="G53" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="29" t="n">
-        <v>6.59</v>
-      </c>
-      <c r="I53" s="29" t="n">
-        <v>3.85</v>
-      </c>
-      <c r="J53" s="28" t="inlineStr">
-        <is>
-          <t>중요공시 3건</t>
-        </is>
-      </c>
-      <c r="K53" s="28" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="H53" s="27" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="I53" s="27" t="n">
+        <v>62.26</v>
+      </c>
+      <c r="J53" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +150%</t>
+        </is>
+      </c>
+      <c r="K53" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2628,42 +2628,42 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>삼성중공업</t>
+          <t>아이씨에이치</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E54" s="25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F54" s="25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G54" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H54" s="29" t="n">
-        <v>5.93</v>
+      <c r="H54" s="27" t="n">
+        <v>5.96</v>
       </c>
       <c r="I54" s="27" t="n">
-        <v>-13.11</v>
-      </c>
-      <c r="J54" s="28" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
-        </is>
-      </c>
-      <c r="K54" s="28" t="inlineStr">
-        <is>
-          <t>공시</t>
+        <v>34.09</v>
+      </c>
+      <c r="J54" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +149%</t>
+        </is>
+      </c>
+      <c r="K54" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2671,7 +2671,7 @@
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>iM금융지주</t>
+          <t>동성제약</t>
         </is>
       </c>
       <c r="D55" s="25" t="n">
@@ -2686,27 +2686,27 @@
       <c r="G55" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H55" s="29" t="n">
-        <v>5.03</v>
-      </c>
-      <c r="I55" s="27" t="n">
-        <v>-7.97</v>
-      </c>
-      <c r="J55" s="28" t="inlineStr">
-        <is>
-          <t>중요공시 4건</t>
-        </is>
-      </c>
-      <c r="K55" s="28" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="H55" s="27" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="I55" s="28" t="n">
+        <v>-5.14</v>
+      </c>
+      <c r="J55" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +129%</t>
+        </is>
+      </c>
+      <c r="K55" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>엑시온그룹</t>
+          <t>씨피시스템</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2730,26 +2730,26 @@
         <v>0</v>
       </c>
       <c r="H56" s="27" t="n">
-        <v>-3.76</v>
-      </c>
-      <c r="I56" s="29" t="n">
-        <v>35.09</v>
-      </c>
-      <c r="J56" s="28" t="inlineStr">
-        <is>
-          <t>중요공시 4건</t>
-        </is>
-      </c>
-      <c r="K56" s="28" t="inlineStr">
-        <is>
-          <t>공시</t>
+        <v>8.869999999999999</v>
+      </c>
+      <c r="I56" s="27" t="n">
+        <v>23.48</v>
+      </c>
+      <c r="J56" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +113%</t>
+        </is>
+      </c>
+      <c r="K56" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>알엔티엑스</t>
+          <t>세아메카닉스</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2773,26 +2773,26 @@
         <v>0</v>
       </c>
       <c r="H57" s="27" t="n">
-        <v>-3.89</v>
+        <v>6.48</v>
       </c>
       <c r="I57" s="27" t="n">
-        <v>-24.6</v>
-      </c>
-      <c r="J57" s="28" t="inlineStr">
-        <is>
-          <t>중요공시 4건</t>
-        </is>
-      </c>
-      <c r="K57" s="28" t="inlineStr">
-        <is>
-          <t>공시</t>
+        <v>17.76</v>
+      </c>
+      <c r="J57" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +61% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K57" s="29" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>미래산업</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2816,17 +2816,17 @@
         <v>0</v>
       </c>
       <c r="H58" s="27" t="n">
-        <v>-9.25</v>
-      </c>
-      <c r="I58" s="27" t="n">
-        <v>-33.05</v>
-      </c>
-      <c r="J58" s="28" t="inlineStr">
+        <v>8.51</v>
+      </c>
+      <c r="I58" s="28" t="n">
+        <v>-15</v>
+      </c>
+      <c r="J58" s="29" t="inlineStr">
         <is>
           <t>중요공시 3건</t>
         </is>
       </c>
-      <c r="K58" s="28" t="inlineStr">
+      <c r="K58" s="29" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
@@ -2835,7 +2835,7 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>시선AI</t>
+          <t>한화생명</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2858,27 +2858,25 @@
       <c r="G59" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H59" s="29" t="n">
-        <v>9.19</v>
-      </c>
-      <c r="I59" s="29" t="n">
-        <v>13.79</v>
-      </c>
-      <c r="J59" s="28" t="inlineStr">
-        <is>
-          <t>중요공시 3건</t>
-        </is>
-      </c>
-      <c r="K59" s="28" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+      <c r="H59" s="27" t="n">
+        <v>5.11</v>
+      </c>
+      <c r="I59" s="28" t="n">
+        <v>-3.7</v>
+      </c>
+      <c r="J59" s="29" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K59" s="29" t="n">
+        <v/>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2886,42 +2884,42 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>제주반도체</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E60" s="25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F60" s="25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="29" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="I60" s="27" t="n">
-        <v>-27.63</v>
-      </c>
-      <c r="J60" s="28" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
-        </is>
-      </c>
-      <c r="K60" s="28" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="H60" s="27" t="n">
+        <v>29.94</v>
+      </c>
+      <c r="I60" s="28" t="n">
+        <v>-7.4</v>
+      </c>
+      <c r="J60" s="29" t="inlineStr">
+        <is>
+          <t>네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K60" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2929,7 +2927,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>SK이노베이션</t>
+          <t>서한</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2944,18 +2942,18 @@
       <c r="G61" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H61" s="29" t="n">
-        <v>6.48</v>
-      </c>
-      <c r="I61" s="27" t="n">
-        <v>-11.8</v>
-      </c>
-      <c r="J61" s="28" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K61" s="28" t="inlineStr">
+      <c r="H61" s="27" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="I61" s="28" t="n">
+        <v>-6.69</v>
+      </c>
+      <c r="J61" s="29" t="inlineStr">
+        <is>
+          <t>중요공시 3건</t>
+        </is>
+      </c>
+      <c r="K61" s="29" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
@@ -2964,7 +2962,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2972,33 +2970,33 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>동국제강</t>
+          <t>GS건설</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E62" s="25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F62" s="25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G62" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H62" s="29" t="n">
-        <v>3.34</v>
-      </c>
-      <c r="I62" s="27" t="n">
-        <v>-5.56</v>
-      </c>
-      <c r="J62" s="28" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K62" s="28" t="inlineStr">
+      <c r="H62" s="27" t="n">
+        <v>5.39</v>
+      </c>
+      <c r="I62" s="28" t="n">
+        <v>-22.48</v>
+      </c>
+      <c r="J62" s="29" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+        </is>
+      </c>
+      <c r="K62" s="29" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
@@ -3007,7 +3005,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3015,7 +3013,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>한미반도체</t>
+          <t>SK오션플랜트</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3030,19 +3028,21 @@
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I63" s="27" t="n">
-        <v>-22.41</v>
-      </c>
-      <c r="J63" s="28" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K63" s="28" t="n">
-        <v/>
+      <c r="H63" s="27" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="I63" s="28" t="n">
+        <v>-31.77</v>
+      </c>
+      <c r="J63" s="29" t="inlineStr">
+        <is>
+          <t>중요공시 3건</t>
+        </is>
+      </c>
+      <c r="K63" s="29" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3138,22 +3138,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3162,165 +3162,169 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>SK</t>
         </is>
       </c>
       <c r="B4" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H4" s="27" t="n">
-        <v>-0.72</v>
-      </c>
-      <c r="I4" s="27" t="n">
-        <v>-23.33</v>
+        <v>18.89</v>
+      </c>
+      <c r="I4" s="28" t="n">
+        <v>-11.59</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H5" s="29" t="n">
-        <v>4.56</v>
-      </c>
-      <c r="I5" s="27" t="n">
-        <v>-5.12</v>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H5" s="27" t="n">
+        <v>29.95</v>
+      </c>
+      <c r="I5" s="28" t="n">
+        <v>-2.33</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H6" s="27" t="n">
-        <v>-5.64</v>
+        <v>26.81</v>
       </c>
       <c r="I6" s="27" t="n">
-        <v>-31.11</v>
+        <v>5.21</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H7" s="25" t="n"/>
-      <c r="I7" s="25" t="n"/>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H7" s="27" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="I7" s="27" t="n">
+        <v>3.27</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H8" s="25" t="n"/>
@@ -3329,103 +3333,99 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H9" s="27" t="n">
-        <v>-1.66</v>
-      </c>
-      <c r="I9" s="27" t="n">
-        <v>-21.07</v>
-      </c>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H9" s="25" t="n"/>
+      <c r="I9" s="25" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H10" s="27" t="n">
-        <v>-14.58</v>
-      </c>
-      <c r="I10" s="27" t="n">
-        <v>-39.3</v>
-      </c>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H10" s="25" t="n"/>
+      <c r="I10" s="25" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H11" s="25" t="n"/>
-      <c r="I11" s="25" t="n"/>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H11" s="27" t="n">
+        <v>29.92</v>
+      </c>
+      <c r="I11" s="28" t="n">
+        <v>-13.88</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
@@ -3437,22 +3437,22 @@
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H12" s="25" t="n"/>
@@ -3461,36 +3461,36 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>LG생활건강</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H13" s="29" t="n">
-        <v>11.03</v>
-      </c>
-      <c r="I13" s="29" t="n">
-        <v>17.74</v>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H13" s="27" t="n">
+        <v>14.11</v>
+      </c>
+      <c r="I13" s="28" t="n">
+        <v>-16.47</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
@@ -3503,22 +3503,22 @@
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H14" s="25" t="n"/>
@@ -3527,147 +3527,143 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E15" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H15" s="27" t="n">
-        <v>-0.71</v>
+        <v>3.46</v>
       </c>
       <c r="I15" s="27" t="n">
-        <v>-18.75</v>
+        <v>3.31</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C16" s="25" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D16" s="25" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E16" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H16" s="27" t="n">
-        <v>-6.82</v>
-      </c>
-      <c r="I16" s="27" t="n">
-        <v>-31.46</v>
+        <v>7.44</v>
+      </c>
+      <c r="I16" s="28" t="n">
+        <v>-3.07</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>기업은행</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E17" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H17" s="29" t="n">
-        <v>2.98</v>
-      </c>
-      <c r="I17" s="27" t="n">
-        <v>-18.33</v>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H17" s="27" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I17" s="28" t="n">
+        <v>-3.28</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E18" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H18" s="29" t="n">
-        <v>5.56</v>
-      </c>
-      <c r="I18" s="29" t="n">
-        <v>10.34</v>
-      </c>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H18" s="25" t="n"/>
+      <c r="I18" s="25" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -3684,19 +3680,19 @@
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H19" s="29" t="n">
-        <v>2.73</v>
-      </c>
-      <c r="I19" s="27" t="n">
-        <v>-13.92</v>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H19" s="27" t="n">
+        <v>10.54</v>
+      </c>
+      <c r="I19" s="28" t="n">
+        <v>-3.24</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
@@ -3719,25 +3715,25 @@
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H20" s="27" t="n">
-        <v>-1.07</v>
-      </c>
-      <c r="I20" s="27" t="n">
-        <v>-16.71</v>
+        <v>2.5</v>
+      </c>
+      <c r="I20" s="28" t="n">
+        <v>-15.91</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>HD한국조선해양</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -3754,25 +3750,25 @@
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H21" s="29" t="n">
-        <v>10</v>
-      </c>
-      <c r="I21" s="27" t="n">
-        <v>-3.28</v>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H21" s="27" t="n">
+        <v>9.529999999999999</v>
+      </c>
+      <c r="I21" s="28" t="n">
+        <v>-4.2</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>삼성물산</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -3789,25 +3785,25 @@
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H22" s="29" t="n">
-        <v>3.23</v>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H22" s="27" t="n">
+        <v>19.56</v>
       </c>
       <c r="I22" s="27" t="n">
-        <v>-10.04</v>
+        <v>2.78</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3824,25 +3820,25 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H23" s="27" t="n">
-        <v>-0.6</v>
-      </c>
-      <c r="I23" s="27" t="n">
-        <v>-4.27</v>
+        <v>26.08</v>
+      </c>
+      <c r="I23" s="28" t="n">
+        <v>-14.38</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>지엔씨에너지</t>
+          <t>스테이블코인</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3859,25 +3855,21 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H24" s="29" t="n">
-        <v>4.02</v>
-      </c>
-      <c r="I24" s="27" t="n">
-        <v>-34.69</v>
-      </c>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H24" s="25" t="n"/>
+      <c r="I24" s="25" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>카카오뱅크</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3894,25 +3886,25 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H25" s="29" t="n">
-        <v>2.41</v>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H25" s="27" t="n">
+        <v>1.38</v>
       </c>
       <c r="I25" s="27" t="n">
-        <v>-2.69</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
@@ -3929,95 +3921,83 @@
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H26" s="29" t="n">
-        <v>3.49</v>
-      </c>
-      <c r="I26" s="27" t="n">
-        <v>-4.52</v>
-      </c>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H26" s="25" t="n"/>
+      <c r="I26" s="25" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>한솔테크닉스</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C27" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D27" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E27" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H27" s="27" t="n">
-        <v>-3.59</v>
-      </c>
-      <c r="I27" s="27" t="n">
-        <v>-35.4</v>
-      </c>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H27" s="25" t="n"/>
+      <c r="I27" s="25" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>Netflix</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C28" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D28" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E28" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H28" s="29" t="n">
-        <v>2.84</v>
-      </c>
-      <c r="I28" s="27" t="n">
-        <v>-21.67</v>
-      </c>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H28" s="25" t="n"/>
+      <c r="I28" s="25" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>미래산업</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
@@ -4034,25 +4014,25 @@
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H29" s="29" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="I29" s="27" t="n">
-        <v>-11</v>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H29" s="27" t="n">
+        <v>18.43</v>
+      </c>
+      <c r="I29" s="28" t="n">
+        <v>-20.72</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -4069,25 +4049,21 @@
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H30" s="29" t="n">
-        <v>3.14</v>
-      </c>
-      <c r="I30" s="27" t="n">
-        <v>-12.11</v>
-      </c>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H30" s="25" t="n"/>
+      <c r="I30" s="25" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>파두</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
@@ -4104,25 +4080,25 @@
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H31" s="27" t="n">
-        <v>-1.51</v>
-      </c>
-      <c r="I31" s="27" t="n">
-        <v>-23.23</v>
+        <v>29.92</v>
+      </c>
+      <c r="I31" s="28" t="n">
+        <v>-1.71</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>HD현대일렉트릭</t>
+          <t>HD현대마린엔진</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -4139,19 +4115,19 @@
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H32" s="27" t="n">
-        <v>-0.51</v>
-      </c>
-      <c r="I32" s="27" t="n">
-        <v>-32.91</v>
+        <v>3.24</v>
+      </c>
+      <c r="I32" s="28" t="n">
+        <v>-26.85</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
@@ -4174,25 +4150,25 @@
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H33" s="27" t="n">
-        <v>-0.35</v>
-      </c>
-      <c r="I33" s="27" t="n">
-        <v>-18.51</v>
+        <v>7.85</v>
+      </c>
+      <c r="I33" s="28" t="n">
+        <v>-6.02</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>LG이노텍</t>
+          <t>LG화학</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4209,25 +4185,25 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H34" s="27" t="n">
-        <v>-7.42</v>
-      </c>
-      <c r="I34" s="27" t="n">
-        <v>-37.56</v>
+        <v>5.09</v>
+      </c>
+      <c r="I34" s="28" t="n">
+        <v>-0.39</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>대한전선</t>
+          <t>네이처셀</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -4244,25 +4220,25 @@
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H35" s="27" t="n">
-        <v>-6.31</v>
-      </c>
-      <c r="I35" s="27" t="n">
-        <v>-32.9</v>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H35" s="28" t="n">
+        <v>-3.51</v>
+      </c>
+      <c r="I35" s="28" t="n">
+        <v>-8.710000000000001</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>야스</t>
+          <t>넥스트아이</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
@@ -4279,25 +4255,25 @@
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H36" s="29" t="n">
-        <v>29.97</v>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H36" s="27" t="n">
+        <v>10.96</v>
       </c>
       <c r="I36" s="27" t="n">
-        <v>-32.45</v>
+        <v>1.28</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>야스</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
@@ -4314,21 +4290,25 @@
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H37" s="25" t="n"/>
-      <c r="I37" s="25" t="n"/>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H37" s="27" t="n">
+        <v>8.359999999999999</v>
+      </c>
+      <c r="I37" s="28" t="n">
+        <v>-26.2</v>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>주성엔지니어링</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4345,21 +4325,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H38" s="25" t="n"/>
-      <c r="I38" s="25" t="n"/>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H38" s="27" t="n">
+        <v>26.65</v>
+      </c>
+      <c r="I38" s="28" t="n">
+        <v>-11.7</v>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>현대모비스</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4376,60 +4360,60 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H39" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" s="27" t="n">
-        <v>-15.08</v>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H39" s="27" t="n">
+        <v>15.79</v>
+      </c>
+      <c r="I39" s="28" t="n">
+        <v>-10.92</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>LG유플러스</t>
+          <t>호텔신라</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C40" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D40" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E40" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H40" s="29" t="n">
-        <v>6.59</v>
-      </c>
-      <c r="I40" s="29" t="n">
-        <v>3.85</v>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H40" s="27" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="I40" s="28" t="n">
+        <v>-7.54</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>SK이노베이션</t>
+          <t>GS건설</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4446,25 +4430,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H41" s="29" t="n">
-        <v>6.48</v>
-      </c>
-      <c r="I41" s="27" t="n">
-        <v>-11.8</v>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H41" s="27" t="n">
+        <v>5.39</v>
+      </c>
+      <c r="I41" s="28" t="n">
+        <v>-22.48</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>iM금융지주</t>
+          <t>SK오션플랜트</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4481,25 +4465,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H42" s="29" t="n">
-        <v>5.03</v>
-      </c>
-      <c r="I42" s="27" t="n">
-        <v>-7.97</v>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H42" s="27" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="I42" s="28" t="n">
+        <v>-31.77</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>더테크놀로지</t>
+          <t>동성제약</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4516,25 +4500,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H43" s="27" t="n">
-        <v>-80</v>
-      </c>
-      <c r="I43" s="27" t="n">
-        <v>-80</v>
+        <v>2.56</v>
+      </c>
+      <c r="I43" s="28" t="n">
+        <v>-5.14</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>동국제강</t>
+          <t>두산퓨얼셀</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4551,25 +4535,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H44" s="29" t="n">
-        <v>3.34</v>
-      </c>
-      <c r="I44" s="27" t="n">
-        <v>-5.56</v>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H44" s="27" t="n">
+        <v>29.89</v>
+      </c>
+      <c r="I44" s="28" t="n">
+        <v>-42.64</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>미래산업</t>
+          <t>서한</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4586,25 +4570,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H45" s="27" t="n">
-        <v>-9.25</v>
-      </c>
-      <c r="I45" s="27" t="n">
-        <v>-33.05</v>
+        <v>2.26</v>
+      </c>
+      <c r="I45" s="28" t="n">
+        <v>-6.69</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>삼성중공업</t>
+          <t>세아메카닉스</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4621,25 +4605,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H46" s="29" t="n">
-        <v>5.93</v>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H46" s="27" t="n">
+        <v>6.48</v>
       </c>
       <c r="I46" s="27" t="n">
-        <v>-13.11</v>
+        <v>17.76</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>시선AI</t>
+          <t>셀리드</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4656,25 +4640,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H47" s="29" t="n">
-        <v>9.19</v>
-      </c>
-      <c r="I47" s="29" t="n">
-        <v>13.79</v>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H47" s="27" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="I47" s="27" t="n">
+        <v>62.26</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>알엔티엑스</t>
+          <t>씨피시스템</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4691,25 +4675,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H48" s="27" t="n">
-        <v>-3.89</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="I48" s="27" t="n">
-        <v>-24.6</v>
+        <v>23.48</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>엑시온그룹</t>
+          <t>아이씨에이치</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4726,25 +4710,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H49" s="27" t="n">
-        <v>-3.76</v>
-      </c>
-      <c r="I49" s="29" t="n">
-        <v>35.09</v>
+        <v>5.96</v>
+      </c>
+      <c r="I49" s="27" t="n">
+        <v>34.09</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>우리금융지주</t>
+          <t>제주반도체</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4761,25 +4745,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H50" s="29" t="n">
-        <v>2.03</v>
-      </c>
-      <c r="I50" s="29" t="n">
-        <v>5.83</v>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H50" s="27" t="n">
+        <v>29.94</v>
+      </c>
+      <c r="I50" s="28" t="n">
+        <v>-7.4</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>한미반도체</t>
+          <t>한화생명</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4796,25 +4780,25 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H51" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I51" s="27" t="n">
-        <v>-22.41</v>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H51" s="27" t="n">
+        <v>5.11</v>
+      </c>
+      <c r="I51" s="28" t="n">
+        <v>-3.7</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="26" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -4831,19 +4815,19 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="H52" s="29" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="I52" s="27" t="n">
-        <v>-27.63</v>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="H52" s="27" t="n">
+        <v>8.51</v>
+      </c>
+      <c r="I52" s="28" t="n">
+        <v>-15</v>
       </c>
     </row>
   </sheetData>
@@ -4927,19 +4911,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4958,19 +4942,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4989,19 +4973,19 @@
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5013,26 +4997,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5044,26 +5028,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5075,26 +5059,26 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5106,26 +5090,26 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B9" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5137,7 +5121,7 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="35" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B10" s="36" t="n">
@@ -5151,12 +5135,12 @@
       </c>
       <c r="E10" s="36" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="F10" s="37" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G10" s="37" t="inlineStr">
@@ -5166,36 +5150,40 @@
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="26" t="inlineStr">
-        <is>
-          <t>이차전지</t>
-        </is>
-      </c>
-      <c r="B11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F11" s="28" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="inlineStr"/>
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>인공지능</t>
+        </is>
+      </c>
+      <c r="B11" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="36" t="n">
+        <v>12</v>
+      </c>
+      <c r="D11" s="36" t="n">
+        <v>12</v>
+      </c>
+      <c r="E11" s="36" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="F11" s="37" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="G11" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>이차전지</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
@@ -5212,17 +5200,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F12" s="28" t="inlineStr">
+      <c r="F12" s="29" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G12" s="28" t="inlineStr"/>
+      <c r="G12" s="29" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -5239,17 +5227,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F13" s="28" t="inlineStr">
+      <c r="F13" s="29" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G13" s="28" t="inlineStr"/>
+      <c r="G13" s="29" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5266,12 +5254,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F14" s="28" t="inlineStr">
+      <c r="F14" s="29" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G14" s="28" t="inlineStr"/>
+      <c r="G14" s="29" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
@@ -5293,12 +5281,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F15" s="28" t="inlineStr">
+      <c r="F15" s="29" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G15" s="28" t="inlineStr"/>
+      <c r="G15" s="29" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
@@ -5320,12 +5308,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F16" s="28" t="inlineStr">
+      <c r="F16" s="29" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G16" s="28" t="inlineStr"/>
+      <c r="G16" s="29" t="inlineStr"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
@@ -5347,12 +5335,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F17" s="28" t="inlineStr">
+      <c r="F17" s="29" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G17" s="28" t="inlineStr"/>
+      <c r="G17" s="29" t="inlineStr"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
@@ -5374,12 +5362,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F18" s="28" t="inlineStr">
+      <c r="F18" s="29" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G18" s="28" t="inlineStr"/>
+      <c r="G18" s="29" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
@@ -5401,12 +5389,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F19" s="28" t="inlineStr">
+      <c r="F19" s="29" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G19" s="28" t="inlineStr"/>
+      <c r="G19" s="29" t="inlineStr"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
@@ -5428,12 +5416,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F20" s="28" t="inlineStr">
+      <c r="F20" s="29" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G20" s="28" t="inlineStr"/>
+      <c r="G20" s="29" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
@@ -5455,12 +5443,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F21" s="28" t="inlineStr">
+      <c r="F21" s="29" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G21" s="28" t="inlineStr"/>
+      <c r="G21" s="29" t="inlineStr"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
@@ -5482,12 +5470,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F22" s="28" t="inlineStr">
+      <c r="F22" s="29" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G22" s="28" t="inlineStr"/>
+      <c r="G22" s="29" t="inlineStr"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
@@ -5509,12 +5497,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F23" s="28" t="inlineStr">
+      <c r="F23" s="29" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G23" s="28" t="inlineStr"/>
+      <c r="G23" s="29" t="inlineStr"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
@@ -5536,12 +5524,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F24" s="28" t="inlineStr">
+      <c r="F24" s="29" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G24" s="28" t="inlineStr"/>
+      <c r="G24" s="29" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
auto: 2026-08-03 07:18 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -261,11 +261,11 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-08-02 06:55</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-08-03 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-08-02) 상위: 반도체  점수 64.0점</t>
+          <t>⚡ 최신(2026-08-03) 상위: 반도체  점수 67.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-08-02) 상위: SK  점수 61.0점</t>
+          <t>⚡ 최신(2026-08-03) 상위: SK  점수 34.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-08-02) 상위: SK하이닉스  점수 44.0점</t>
+          <t>⚡ 최신(2026-08-03) 상위: SK하이닉스  점수 29.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -971,10 +971,10 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>61</v>
+        <v>34</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>61</v>
+        <v>34</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -990,7 +990,7 @@
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1014,10 +1014,10 @@
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1033,19 +1033,19 @@
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +57% / 중요공시 1건 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +62% / 중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1057,10 +1057,10 @@
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1076,19 +1076,19 @@
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 3건 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1096,14 +1096,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1111,15 +1111,15 @@
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I18" s="15" t="n">
-        <v/>
+      <c r="H18" s="18" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="I18" s="18" t="n">
+        <v>3.27</v>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K18" s="17" t="n">
@@ -1129,7 +1129,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1137,7 +1137,7 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K19" s="17" t="inlineStr">
@@ -1172,7 +1172,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1180,42 +1180,42 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F20" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G20" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I20" s="15" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H20" s="18" t="n">
+        <v>14.11</v>
+      </c>
+      <c r="I20" s="19" t="n">
+        <v>-16.47</v>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 5건 / 중요공시 3일 +67% / 중요공시 7일 +400% / Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K20" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>Google, 공시</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1223,14 +1223,14 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
@@ -1238,27 +1238,27 @@
       <c r="G21" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="18" t="n">
-        <v>29.92</v>
-      </c>
-      <c r="I21" s="19" t="n">
-        <v>-13.88</v>
+      <c r="H21" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I21" s="15" t="n">
+        <v/>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1266,30 +1266,30 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="F22" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G22" s="15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H22" s="18" t="n">
-        <v>14.11</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="I22" s="19" t="n">
-        <v>-16.47</v>
+        <v>-4.2</v>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>중요공시 5건 / 중요공시 3일 +150% / 중요공시 7일 +150% / 한국경제 헤드라인 언급</t>
+          <t>중요공시 4건 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="inlineStr">
@@ -1301,7 +1301,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1309,14 +1309,14 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F23" s="15" t="n">
         <v>0</v>
@@ -1324,25 +1324,27 @@
       <c r="G23" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="18" t="n">
-        <v>4.88</v>
-      </c>
-      <c r="I23" s="18" t="n">
-        <v>3.27</v>
+      <c r="H23" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I23" s="15" t="n">
+        <v/>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K23" s="17" t="n">
-        <v/>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K23" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1350,42 +1352,42 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>2</v>
       </c>
       <c r="G24" s="15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H24" s="18" t="n">
-        <v>7.44</v>
+        <v>26.08</v>
       </c>
       <c r="I24" s="19" t="n">
-        <v>-3.07</v>
+        <v>-14.38</v>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +200%</t>
         </is>
       </c>
       <c r="K24" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1393,14 +1395,14 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F25" s="15" t="n">
         <v>0</v>
@@ -1408,27 +1410,27 @@
       <c r="G25" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H25" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I25" s="15" t="n">
-        <v/>
+      <c r="H25" s="19" t="n">
+        <v>-1.74</v>
+      </c>
+      <c r="I25" s="18" t="n">
+        <v>5.12</v>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K25" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1436,42 +1438,42 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F26" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G26" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H26" s="18" t="n">
-        <v>8.51</v>
+        <v>10.54</v>
       </c>
       <c r="I26" s="19" t="n">
-        <v>-15</v>
+        <v>-3.24</v>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +50% / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K26" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -1479,7 +1481,7 @@
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>기업은행</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="D27" s="15" t="n">
@@ -1494,27 +1496,25 @@
       <c r="G27" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H27" s="18" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="I27" s="19" t="n">
-        <v>-3.28</v>
+      <c r="H27" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I27" s="15" t="n">
+        <v/>
       </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K27" s="17" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K27" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B28" s="15" t="n">
@@ -1522,7 +1522,7 @@
       </c>
       <c r="C28" s="16" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="D28" s="15" t="n">
@@ -1537,15 +1537,15 @@
       <c r="G28" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H28" s="18" t="n">
-        <v>10.54</v>
-      </c>
-      <c r="I28" s="19" t="n">
-        <v>-3.24</v>
+      <c r="H28" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I28" s="15" t="n">
+        <v/>
       </c>
       <c r="J28" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K28" s="17" t="n">
@@ -1553,50 +1553,50 @@
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="20" t="inlineStr">
-        <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="B29" s="20" t="n">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="n">
         <v>16</v>
       </c>
-      <c r="C29" s="21" t="inlineStr">
-        <is>
-          <t>카카오</t>
-        </is>
-      </c>
-      <c r="D29" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E29" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="F29" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="22" t="n">
-        <v>3.46</v>
-      </c>
-      <c r="I29" s="22" t="n">
-        <v>3.31</v>
-      </c>
-      <c r="J29" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K29" s="23" t="n">
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="E29" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="F29" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="19" t="n">
+        <v>-1.7</v>
+      </c>
+      <c r="I29" s="19" t="n">
+        <v>-4.07</v>
+      </c>
+      <c r="J29" s="17" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K29" s="17" t="n">
         <v/>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
@@ -1604,42 +1604,42 @@
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>야스</t>
         </is>
       </c>
       <c r="D30" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E30" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F30" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G30" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H30" s="22" t="n">
-        <v>26.08</v>
-      </c>
-      <c r="I30" s="24" t="n">
-        <v>-14.38</v>
-      </c>
-      <c r="J30" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 3건 / 중요공시 7일 +200%</t>
-        </is>
-      </c>
-      <c r="K30" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+        <v>8.359999999999999</v>
+      </c>
+      <c r="I30" s="23" t="n">
+        <v>-26.2</v>
+      </c>
+      <c r="J30" s="24" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +413% / 중요공시 2건 / 중요공시 3일 +100%</t>
+        </is>
+      </c>
+      <c r="K30" s="24" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1647,7 +1647,7 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
@@ -1662,27 +1662,27 @@
       <c r="G31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="22" t="n">
-        <v>9.529999999999999</v>
-      </c>
-      <c r="I31" s="24" t="n">
-        <v>-4.2</v>
-      </c>
-      <c r="J31" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 4건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K31" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="H31" s="23" t="n">
+        <v>-4</v>
+      </c>
+      <c r="I31" s="23" t="n">
+        <v>-10.25</v>
+      </c>
+      <c r="J31" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / Google 급상승 검색어 등장 (KR)</t>
+        </is>
+      </c>
+      <c r="K31" s="24" t="inlineStr">
+        <is>
+          <t>Google, 공시</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1690,42 +1690,42 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>GS건설</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F32" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G32" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H32" s="22" t="n">
-        <v>8.130000000000001</v>
-      </c>
-      <c r="I32" s="24" t="n">
-        <v>-7.44</v>
-      </c>
-      <c r="J32" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 3건 / 중요공시 7일 +200%</t>
-        </is>
-      </c>
-      <c r="K32" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+        <v>5.39</v>
+      </c>
+      <c r="I32" s="23" t="n">
+        <v>-22.48</v>
+      </c>
+      <c r="J32" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / Google 급상승 검색어 등장 (KR)</t>
+        </is>
+      </c>
+      <c r="K32" s="24" t="inlineStr">
+        <is>
+          <t>Google, 공시</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>스테이블코인</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
@@ -1748,25 +1748,27 @@
       <c r="G33" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H33" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I33" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J33" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K33" s="23" t="n">
-        <v/>
+      <c r="H33" s="22" t="n">
+        <v>15.79</v>
+      </c>
+      <c r="I33" s="23" t="n">
+        <v>-10.92</v>
+      </c>
+      <c r="J33" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / Google 급상승 검색어 등장 (KR)</t>
+        </is>
+      </c>
+      <c r="K33" s="24" t="inlineStr">
+        <is>
+          <t>Google, 공시</t>
+        </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1774,7 +1776,7 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>카카오뱅크</t>
+          <t>서희건설</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
@@ -1790,24 +1792,26 @@
         <v>0</v>
       </c>
       <c r="H34" s="22" t="n">
-        <v>1.38</v>
-      </c>
-      <c r="I34" s="22" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="J34" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K34" s="23" t="n">
-        <v/>
+        <v>2.51</v>
+      </c>
+      <c r="I34" s="23" t="n">
+        <v>-1.61</v>
+      </c>
+      <c r="J34" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / Google 급상승 검색어 등장 (KR)</t>
+        </is>
+      </c>
+      <c r="K34" s="24" t="inlineStr">
+        <is>
+          <t>Google, 공시</t>
+        </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1815,14 +1819,14 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>BNK금융지주</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F35" s="20" t="n">
         <v>0</v>
@@ -1830,27 +1834,25 @@
       <c r="G35" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H35" s="22" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="I35" s="24" t="n">
-        <v>-15.91</v>
-      </c>
-      <c r="J35" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +63% / 중요공시 6건</t>
-        </is>
-      </c>
-      <c r="K35" s="23" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
-        </is>
+      <c r="H35" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I35" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J35" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K35" s="24" t="n">
+        <v/>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1858,42 +1860,42 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>미래산업</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F36" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G36" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H36" s="22" t="n">
-        <v>18.43</v>
-      </c>
-      <c r="I36" s="24" t="n">
-        <v>-20.72</v>
-      </c>
-      <c r="J36" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 3건 / 중요공시 3일 +50%</t>
-        </is>
-      </c>
-      <c r="K36" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="H36" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I36" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J36" s="24" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K36" s="24" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1901,7 +1903,7 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>파두</t>
+          <t>BNK금융지주</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
@@ -1917,26 +1919,26 @@
         <v>0</v>
       </c>
       <c r="H37" s="22" t="n">
-        <v>29.92</v>
-      </c>
-      <c r="I37" s="24" t="n">
-        <v>-1.71</v>
-      </c>
-      <c r="J37" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K37" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+        <v>2.5</v>
+      </c>
+      <c r="I37" s="23" t="n">
+        <v>-15.91</v>
+      </c>
+      <c r="J37" s="24" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +67% / 중요공시 6건</t>
+        </is>
+      </c>
+      <c r="K37" s="24" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1944,42 +1946,42 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>KG스틸</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F38" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H38" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I38" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J38" s="23" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K38" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
+      <c r="H38" s="22" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="I38" s="22" t="n">
+        <v>5.43</v>
+      </c>
+      <c r="J38" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 3일 +50%</t>
+        </is>
+      </c>
+      <c r="K38" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1987,14 +1989,14 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>야스</t>
+          <t>일성건설</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F39" s="20" t="n">
         <v>0</v>
@@ -2003,26 +2005,26 @@
         <v>0</v>
       </c>
       <c r="H39" s="22" t="n">
-        <v>8.359999999999999</v>
-      </c>
-      <c r="I39" s="24" t="n">
-        <v>-26.2</v>
-      </c>
-      <c r="J39" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +392% / 중요공시 2건</t>
-        </is>
-      </c>
-      <c r="K39" s="23" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
+        <v>3.86</v>
+      </c>
+      <c r="I39" s="23" t="n">
+        <v>-0.74</v>
+      </c>
+      <c r="J39" s="24" t="inlineStr">
+        <is>
+          <t>Google 급상승 검색어 등장 (KR)</t>
+        </is>
+      </c>
+      <c r="K39" s="24" t="inlineStr">
+        <is>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2030,42 +2032,42 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>태영건설</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F40" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G40" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H40" s="22" t="n">
-        <v>19.56</v>
-      </c>
-      <c r="I40" s="22" t="n">
-        <v>2.78</v>
-      </c>
-      <c r="J40" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K40" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+        <v>0.87</v>
+      </c>
+      <c r="I40" s="23" t="n">
+        <v>-4.66</v>
+      </c>
+      <c r="J40" s="24" t="inlineStr">
+        <is>
+          <t>Google 급상승 검색어 등장 (KR)</t>
+        </is>
+      </c>
+      <c r="K40" s="24" t="inlineStr">
+        <is>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2073,42 +2075,42 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>지엔씨에너지</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E41" s="20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F41" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G41" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H41" s="22" t="n">
-        <v>23.03</v>
-      </c>
-      <c r="I41" s="24" t="n">
-        <v>-19.21</v>
-      </c>
-      <c r="J41" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K41" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+        <v>0</v>
+      </c>
+      <c r="H41" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I41" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J41" s="24" t="inlineStr">
+        <is>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K41" s="24" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2116,14 +2118,14 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>현대건설</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E42" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F42" s="20" t="n">
         <v>0</v>
@@ -2132,26 +2134,24 @@
         <v>0</v>
       </c>
       <c r="H42" s="22" t="n">
-        <v>15.79</v>
-      </c>
-      <c r="I42" s="24" t="n">
-        <v>-10.92</v>
-      </c>
-      <c r="J42" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K42" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+        <v>8.52</v>
+      </c>
+      <c r="I42" s="23" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="J42" s="24" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K42" s="24" t="n">
+        <v/>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2159,33 +2159,33 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>넥스트아이</t>
+          <t>삼성E&amp;A</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E43" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F43" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G43" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H43" s="22" t="n">
-        <v>10.96</v>
-      </c>
-      <c r="I43" s="22" t="n">
-        <v>1.28</v>
-      </c>
-      <c r="J43" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K43" s="23" t="inlineStr">
+        <v>6.83</v>
+      </c>
+      <c r="I43" s="23" t="n">
+        <v>-7.98</v>
+      </c>
+      <c r="J43" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K43" s="24" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
@@ -2194,7 +2194,7 @@
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2202,33 +2202,33 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>LG화학</t>
+          <t>삼성물산</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E44" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F44" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G44" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H44" s="22" t="n">
-        <v>5.09</v>
-      </c>
-      <c r="I44" s="24" t="n">
-        <v>-0.39</v>
-      </c>
-      <c r="J44" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K44" s="23" t="inlineStr">
+        <v>19.56</v>
+      </c>
+      <c r="I44" s="22" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="J44" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K44" s="24" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
@@ -2237,7 +2237,7 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2245,212 +2245,214 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>지엔씨에너지</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E45" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H45" s="22" t="n">
+        <v>23.03</v>
+      </c>
+      <c r="I45" s="23" t="n">
+        <v>-19.21</v>
+      </c>
+      <c r="J45" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K45" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B46" s="20" t="n">
+        <v>33</v>
+      </c>
+      <c r="C46" s="21" t="inlineStr">
+        <is>
+          <t>HL만도</t>
+        </is>
+      </c>
+      <c r="D46" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="F45" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G45" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H45" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I45" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J45" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K45" s="23" t="n">
-        <v/>
-      </c>
-    </row>
-    <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="25" t="inlineStr">
-        <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="B46" s="25" t="n">
-        <v>33</v>
-      </c>
-      <c r="C46" s="26" t="inlineStr">
-        <is>
-          <t>아이씨에이치</t>
-        </is>
-      </c>
-      <c r="D46" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E46" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F46" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G46" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" s="27" t="n">
-        <v>5.96</v>
-      </c>
-      <c r="I46" s="27" t="n">
-        <v>34.09</v>
-      </c>
-      <c r="J46" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +202%</t>
-        </is>
-      </c>
-      <c r="K46" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
+      <c r="E46" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F46" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="22" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="I46" s="22" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="J46" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K46" s="24" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="25" t="inlineStr">
-        <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="B47" s="25" t="n">
+      <c r="A47" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B47" s="20" t="n">
         <v>34</v>
       </c>
-      <c r="C47" s="26" t="inlineStr">
-        <is>
-          <t>동성제약</t>
-        </is>
-      </c>
-      <c r="D47" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E47" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F47" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" s="27" t="n">
+      <c r="C47" s="21" t="inlineStr">
+        <is>
+          <t>LG이노텍</t>
+        </is>
+      </c>
+      <c r="D47" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E47" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F47" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="22" t="n">
+        <v>21.23</v>
+      </c>
+      <c r="I47" s="23" t="n">
+        <v>-17.76</v>
+      </c>
+      <c r="J47" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K47" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B48" s="20" t="n">
+        <v>35</v>
+      </c>
+      <c r="C48" s="21" t="inlineStr">
+        <is>
+          <t>케이엠제약</t>
+        </is>
+      </c>
+      <c r="D48" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E48" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F48" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="22" t="n">
         <v>2.56</v>
       </c>
-      <c r="I47" s="29" t="n">
-        <v>-5.14</v>
-      </c>
-      <c r="J47" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +196%</t>
-        </is>
-      </c>
-      <c r="K47" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="25" t="inlineStr">
-        <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="B48" s="25" t="n">
-        <v>35</v>
-      </c>
-      <c r="C48" s="26" t="inlineStr">
-        <is>
-          <t>두산퓨얼셀</t>
-        </is>
-      </c>
-      <c r="D48" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E48" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F48" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="27" t="n">
-        <v>29.89</v>
-      </c>
-      <c r="I48" s="29" t="n">
-        <v>-42.64</v>
-      </c>
-      <c r="J48" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +193%</t>
-        </is>
-      </c>
-      <c r="K48" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
+      <c r="I48" s="22" t="n">
+        <v>24.57</v>
+      </c>
+      <c r="J48" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K48" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="25" t="inlineStr">
-        <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="B49" s="25" t="n">
+      <c r="A49" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B49" s="20" t="n">
         <v>36</v>
       </c>
-      <c r="C49" s="26" t="inlineStr">
-        <is>
-          <t>셀리드</t>
-        </is>
-      </c>
-      <c r="D49" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E49" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F49" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G49" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H49" s="27" t="n">
-        <v>1.13</v>
-      </c>
-      <c r="I49" s="27" t="n">
-        <v>62.26</v>
-      </c>
-      <c r="J49" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +191%</t>
-        </is>
-      </c>
-      <c r="K49" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
+      <c r="C49" s="21" t="inlineStr">
+        <is>
+          <t>LG화학</t>
+        </is>
+      </c>
+      <c r="D49" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E49" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F49" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="22" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="I49" s="23" t="n">
+        <v>-0.39</v>
+      </c>
+      <c r="J49" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K49" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -2458,7 +2460,7 @@
       </c>
       <c r="C50" s="26" t="inlineStr">
         <is>
-          <t>씨피시스템</t>
+          <t>아이씨에이치</t>
         </is>
       </c>
       <c r="D50" s="25" t="n">
@@ -2474,14 +2476,14 @@
         <v>0</v>
       </c>
       <c r="H50" s="27" t="n">
-        <v>8.869999999999999</v>
+        <v>5.96</v>
       </c>
       <c r="I50" s="27" t="n">
-        <v>23.48</v>
+        <v>34.09</v>
       </c>
       <c r="J50" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +138%</t>
+          <t>네이버 검색 당일 +217%</t>
         </is>
       </c>
       <c r="K50" s="28" t="inlineStr">
@@ -2493,7 +2495,7 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -2501,7 +2503,7 @@
       </c>
       <c r="C51" s="26" t="inlineStr">
         <is>
-          <t>일승</t>
+          <t>동성제약</t>
         </is>
       </c>
       <c r="D51" s="25" t="n">
@@ -2517,14 +2519,14 @@
         <v>0</v>
       </c>
       <c r="H51" s="27" t="n">
-        <v>8.83</v>
+        <v>2.56</v>
       </c>
       <c r="I51" s="29" t="n">
-        <v>-2.55</v>
+        <v>-5.14</v>
       </c>
       <c r="J51" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +103%</t>
+          <t>네이버 검색 당일 +210%</t>
         </is>
       </c>
       <c r="K51" s="28" t="inlineStr">
@@ -2536,7 +2538,7 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -2544,7 +2546,7 @@
       </c>
       <c r="C52" s="26" t="inlineStr">
         <is>
-          <t>세아메카닉스</t>
+          <t>두산퓨얼셀</t>
         </is>
       </c>
       <c r="D52" s="25" t="n">
@@ -2560,26 +2562,26 @@
         <v>0</v>
       </c>
       <c r="H52" s="27" t="n">
-        <v>6.48</v>
-      </c>
-      <c r="I52" s="27" t="n">
-        <v>17.76</v>
+        <v>29.89</v>
+      </c>
+      <c r="I52" s="29" t="n">
+        <v>-42.64</v>
       </c>
       <c r="J52" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +86% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +200%</t>
         </is>
       </c>
       <c r="K52" s="28" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2587,7 +2589,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>한화생명</t>
+          <t>셀리드</t>
         </is>
       </c>
       <c r="D53" s="25" t="n">
@@ -2603,24 +2605,26 @@
         <v>0</v>
       </c>
       <c r="H53" s="27" t="n">
-        <v>5.11</v>
-      </c>
-      <c r="I53" s="29" t="n">
-        <v>-3.7</v>
+        <v>1.13</v>
+      </c>
+      <c r="I53" s="27" t="n">
+        <v>62.26</v>
       </c>
       <c r="J53" s="28" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K53" s="28" t="n">
-        <v/>
+          <t>네이버 검색 당일 +200%</t>
+        </is>
+      </c>
+      <c r="K53" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2628,7 +2632,7 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>서한</t>
+          <t>씨피시스템</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -2644,26 +2648,26 @@
         <v>0</v>
       </c>
       <c r="H54" s="27" t="n">
-        <v>2.26</v>
-      </c>
-      <c r="I54" s="29" t="n">
-        <v>-6.69</v>
+        <v>8.869999999999999</v>
+      </c>
+      <c r="I54" s="27" t="n">
+        <v>23.48</v>
       </c>
       <c r="J54" s="28" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>네이버 검색 당일 +143%</t>
         </is>
       </c>
       <c r="K54" s="28" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2671,42 +2675,42 @@
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>GS건설</t>
+          <t>일승</t>
         </is>
       </c>
       <c r="D55" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E55" s="25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F55" s="25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G55" s="25" t="n">
         <v>0</v>
       </c>
       <c r="H55" s="27" t="n">
-        <v>5.39</v>
+        <v>8.83</v>
       </c>
       <c r="I55" s="29" t="n">
-        <v>-22.48</v>
+        <v>-2.55</v>
       </c>
       <c r="J55" s="28" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>네이버 검색 당일 +109%</t>
         </is>
       </c>
       <c r="K55" s="28" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2714,7 +2718,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>SK오션플랜트</t>
+          <t>세아메카닉스</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2730,26 +2734,26 @@
         <v>0</v>
       </c>
       <c r="H56" s="27" t="n">
-        <v>6.55</v>
-      </c>
-      <c r="I56" s="29" t="n">
-        <v>-31.77</v>
+        <v>6.48</v>
+      </c>
+      <c r="I56" s="27" t="n">
+        <v>17.76</v>
       </c>
       <c r="J56" s="28" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>네이버 검색 당일 +93% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K56" s="28" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2757,7 +2761,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>iM금융지주</t>
+          <t>조일알미늄</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2773,26 +2777,26 @@
         <v>0</v>
       </c>
       <c r="H57" s="27" t="n">
-        <v>2.67</v>
-      </c>
-      <c r="I57" s="29" t="n">
-        <v>-7.12</v>
+        <v>5.04</v>
+      </c>
+      <c r="I57" s="27" t="n">
+        <v>16.19</v>
       </c>
       <c r="J57" s="28" t="inlineStr">
         <is>
-          <t>중요공시 4건</t>
+          <t>네이버 검색 당일 +52% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K57" s="28" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2800,7 +2804,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>LG유플러스</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2815,27 +2819,25 @@
       <c r="G58" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="29" t="n">
-        <v>-3.78</v>
+      <c r="H58" s="27" t="n">
+        <v>3.46</v>
       </c>
       <c r="I58" s="27" t="n">
-        <v>0.27</v>
+        <v>3.31</v>
       </c>
       <c r="J58" s="28" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
-        </is>
-      </c>
-      <c r="K58" s="28" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K58" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2843,7 +2845,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>포스코인터내셔널</t>
+          <t>기업은행</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2859,14 +2861,14 @@
         <v>0</v>
       </c>
       <c r="H59" s="27" t="n">
-        <v>2.15</v>
+        <v>0.98</v>
       </c>
       <c r="I59" s="29" t="n">
-        <v>-7.28</v>
+        <v>-3.28</v>
       </c>
       <c r="J59" s="28" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>중요공시 1건 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K59" s="28" t="inlineStr">
@@ -2878,7 +2880,7 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2886,7 +2888,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>KG스틸</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2902,10 +2904,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="27" t="n">
-        <v>1.12</v>
-      </c>
-      <c r="I60" s="27" t="n">
-        <v>5.43</v>
+        <v>8.51</v>
+      </c>
+      <c r="I60" s="29" t="n">
+        <v>-15</v>
       </c>
       <c r="J60" s="28" t="inlineStr">
         <is>
@@ -2921,7 +2923,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2929,30 +2931,30 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>HD현대마린엔진</t>
+          <t>서한</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E61" s="25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F61" s="25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G61" s="25" t="n">
         <v>0</v>
       </c>
       <c r="H61" s="27" t="n">
-        <v>3.24</v>
+        <v>2.26</v>
       </c>
       <c r="I61" s="29" t="n">
-        <v>-26.85</v>
+        <v>-6.69</v>
       </c>
       <c r="J61" s="28" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>중요공시 3건</t>
         </is>
       </c>
       <c r="K61" s="28" t="inlineStr">
@@ -2964,7 +2966,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2972,7 +2974,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>서부T&amp;D</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2988,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="27" t="n">
-        <v>2.32</v>
+        <v>7.44</v>
       </c>
       <c r="I62" s="29" t="n">
-        <v>-3.19</v>
+        <v>-3.07</v>
       </c>
       <c r="J62" s="28" t="inlineStr">
         <is>
@@ -3007,7 +3009,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3015,7 +3017,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>SK오션플랜트</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3031,19 +3033,19 @@
         <v>0</v>
       </c>
       <c r="H63" s="27" t="n">
-        <v>10.74</v>
+        <v>6.55</v>
       </c>
       <c r="I63" s="29" t="n">
-        <v>-7.24</v>
+        <v>-31.77</v>
       </c>
       <c r="J63" s="28" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>중요공시 3건</t>
         </is>
       </c>
       <c r="K63" s="28" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
@@ -3140,22 +3142,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3171,22 +3173,22 @@
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>61</v>
+        <v>34</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>61</v>
+        <v>34</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H4" s="27" t="n">
@@ -3206,22 +3208,22 @@
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H5" s="27" t="n">
@@ -3234,73 +3236,77 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H6" s="27" t="n">
-        <v>26.81</v>
+        <v>4.88</v>
       </c>
       <c r="I6" s="27" t="n">
-        <v>5.21</v>
+        <v>3.27</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="H7" s="25" t="n"/>
-      <c r="I7" s="25" t="n"/>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="H7" s="27" t="n">
+        <v>26.81</v>
+      </c>
+      <c r="I7" s="27" t="n">
+        <v>5.21</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
@@ -3317,12 +3323,12 @@
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H8" s="25" t="n"/>
@@ -3331,244 +3337,244 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="H9" s="25" t="n"/>
-      <c r="I9" s="25" t="n"/>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="H9" s="27" t="n">
+        <v>14.11</v>
+      </c>
+      <c r="I9" s="29" t="n">
+        <v>-16.47</v>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="H10" s="27" t="n">
-        <v>29.92</v>
-      </c>
-      <c r="I10" s="29" t="n">
-        <v>-13.88</v>
-      </c>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="H10" s="25" t="n"/>
+      <c r="I10" s="25" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H11" s="27" t="n">
-        <v>4.88</v>
-      </c>
-      <c r="I11" s="27" t="n">
-        <v>3.27</v>
+        <v>9.529999999999999</v>
+      </c>
+      <c r="I11" s="29" t="n">
+        <v>-4.2</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="H12" s="27" t="n">
-        <v>14.11</v>
-      </c>
-      <c r="I12" s="29" t="n">
-        <v>-16.47</v>
-      </c>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="H12" s="25" t="n"/>
+      <c r="I12" s="25" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="H13" s="25" t="n"/>
-      <c r="I13" s="25" t="n"/>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="H13" s="27" t="n">
+        <v>26.08</v>
+      </c>
+      <c r="I13" s="29" t="n">
+        <v>-14.38</v>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="H14" s="27" t="n">
-        <v>7.44</v>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="H14" s="29" t="n">
+        <v>-1.7</v>
       </c>
       <c r="I14" s="29" t="n">
-        <v>-3.07</v>
+        <v>-4.07</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E15" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="H15" s="27" t="n">
-        <v>8.51</v>
-      </c>
-      <c r="I15" s="29" t="n">
-        <v>-15</v>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="H15" s="29" t="n">
+        <v>-1.74</v>
+      </c>
+      <c r="I15" s="27" t="n">
+        <v>5.12</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>기업은행</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -3585,25 +3591,21 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="H16" s="27" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="I16" s="29" t="n">
-        <v>-3.28</v>
-      </c>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="H16" s="25" t="n"/>
+      <c r="I16" s="25" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -3620,60 +3622,56 @@
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="H17" s="27" t="n">
-        <v>10.54</v>
-      </c>
-      <c r="I17" s="29" t="n">
-        <v>-3.24</v>
-      </c>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="H17" s="25" t="n"/>
+      <c r="I17" s="25" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E18" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H18" s="27" t="n">
-        <v>8.130000000000001</v>
+        <v>10.54</v>
       </c>
       <c r="I18" s="29" t="n">
-        <v>-7.44</v>
+        <v>-3.24</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -3690,25 +3688,21 @@
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="H19" s="27" t="n">
-        <v>9.529999999999999</v>
-      </c>
-      <c r="I19" s="29" t="n">
-        <v>-4.2</v>
-      </c>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="H19" s="25" t="n"/>
+      <c r="I19" s="25" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>GS건설</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
@@ -3725,25 +3719,25 @@
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H20" s="27" t="n">
-        <v>26.08</v>
+        <v>5.39</v>
       </c>
       <c r="I20" s="29" t="n">
-        <v>-14.38</v>
+        <v>-22.48</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>스테이블코인</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -3760,21 +3754,25 @@
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="H21" s="25" t="n"/>
-      <c r="I21" s="25" t="n"/>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="H21" s="29" t="n">
+        <v>-4</v>
+      </c>
+      <c r="I21" s="29" t="n">
+        <v>-10.25</v>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>서희건설</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -3791,25 +3789,25 @@
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H22" s="27" t="n">
-        <v>3.46</v>
-      </c>
-      <c r="I22" s="27" t="n">
-        <v>3.31</v>
+        <v>2.51</v>
+      </c>
+      <c r="I22" s="29" t="n">
+        <v>-1.61</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>카카오뱅크</t>
+          <t>야스</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3826,95 +3824,91 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H23" s="27" t="n">
-        <v>1.38</v>
-      </c>
-      <c r="I23" s="27" t="n">
-        <v>0.23</v>
+        <v>8.359999999999999</v>
+      </c>
+      <c r="I23" s="29" t="n">
+        <v>-26.2</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>BNK금융지주</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C24" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D24" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E24" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="H24" s="27" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="I24" s="29" t="n">
-        <v>-15.91</v>
-      </c>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="H24" s="25" t="n"/>
+      <c r="I24" s="25" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>미래산업</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C25" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D25" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E25" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H25" s="27" t="n">
-        <v>18.43</v>
+        <v>15.79</v>
       </c>
       <c r="I25" s="29" t="n">
-        <v>-20.72</v>
+        <v>-10.92</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>BNK금융지주</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
@@ -3931,21 +3925,25 @@
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="H26" s="25" t="n"/>
-      <c r="I26" s="25" t="n"/>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="H26" s="27" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I26" s="29" t="n">
+        <v>-15.91</v>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>파두</t>
+          <t>KG스틸</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
@@ -3962,165 +3960,161 @@
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H27" s="27" t="n">
-        <v>29.92</v>
-      </c>
-      <c r="I27" s="29" t="n">
-        <v>-1.71</v>
+        <v>1.12</v>
+      </c>
+      <c r="I27" s="27" t="n">
+        <v>5.43</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>LG화학</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C28" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D28" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E28" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H28" s="27" t="n">
-        <v>5.09</v>
+        <v>8.52</v>
       </c>
       <c r="I28" s="29" t="n">
-        <v>-0.39</v>
+        <v>-0.25</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>넥스트아이</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C29" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D29" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E29" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="H29" s="27" t="n">
-        <v>10.96</v>
-      </c>
-      <c r="I29" s="27" t="n">
-        <v>1.28</v>
-      </c>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="H29" s="25" t="n"/>
+      <c r="I29" s="25" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>일성건설</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C30" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D30" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E30" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H30" s="27" t="n">
-        <v>19.56</v>
-      </c>
-      <c r="I30" s="27" t="n">
-        <v>2.78</v>
+        <v>3.86</v>
+      </c>
+      <c r="I30" s="29" t="n">
+        <v>-0.74</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>야스</t>
+          <t>태영건설</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C31" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D31" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E31" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H31" s="27" t="n">
-        <v>8.359999999999999</v>
+        <v>0.87</v>
       </c>
       <c r="I31" s="29" t="n">
-        <v>-26.2</v>
+        <v>-4.66</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>HL만도</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -4137,21 +4131,25 @@
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="H32" s="25" t="n"/>
-      <c r="I32" s="25" t="n"/>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="H32" s="27" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="I32" s="27" t="n">
+        <v>0.22</v>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>지엔씨에너지</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4168,25 +4166,25 @@
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H33" s="27" t="n">
-        <v>23.03</v>
+        <v>21.23</v>
       </c>
       <c r="I33" s="29" t="n">
-        <v>-19.21</v>
+        <v>-17.76</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>현대건설</t>
+          <t>LG화학</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4203,159 +4201,159 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H34" s="27" t="n">
-        <v>15.79</v>
+        <v>5.09</v>
       </c>
       <c r="I34" s="29" t="n">
-        <v>-10.92</v>
+        <v>-0.39</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>GS건설</t>
+          <t>삼성E&amp;A</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D35" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E35" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H35" s="27" t="n">
-        <v>5.39</v>
+        <v>6.83</v>
       </c>
       <c r="I35" s="29" t="n">
-        <v>-22.48</v>
+        <v>-7.98</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>HD현대마린엔진</t>
+          <t>삼성물산</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C36" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D36" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E36" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H36" s="27" t="n">
-        <v>3.24</v>
-      </c>
-      <c r="I36" s="29" t="n">
-        <v>-26.85</v>
+        <v>19.56</v>
+      </c>
+      <c r="I36" s="27" t="n">
+        <v>2.78</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>KG스틸</t>
+          <t>지엔씨에너지</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C37" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D37" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E37" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H37" s="27" t="n">
-        <v>1.12</v>
-      </c>
-      <c r="I37" s="27" t="n">
-        <v>5.43</v>
+        <v>23.03</v>
+      </c>
+      <c r="I37" s="29" t="n">
+        <v>-19.21</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>LG유플러스</t>
+          <t>케이엠제약</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C38" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D38" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E38" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="H38" s="29" t="n">
-        <v>-3.78</v>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="H38" s="27" t="n">
+        <v>2.56</v>
       </c>
       <c r="I38" s="27" t="n">
-        <v>0.27</v>
+        <v>24.57</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
@@ -4378,12 +4376,12 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H39" s="27" t="n">
@@ -4396,7 +4394,7 @@
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>iM금융지주</t>
+          <t>기업은행</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4413,19 +4411,19 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H40" s="27" t="n">
-        <v>2.67</v>
+        <v>0.98</v>
       </c>
       <c r="I40" s="29" t="n">
-        <v>-7.12</v>
+        <v>-3.28</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
@@ -4448,12 +4446,12 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H41" s="27" t="n">
@@ -4483,12 +4481,12 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H42" s="27" t="n">
@@ -4501,7 +4499,7 @@
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>서한</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4518,25 +4516,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H43" s="27" t="n">
-        <v>10.74</v>
+        <v>2.26</v>
       </c>
       <c r="I43" s="29" t="n">
-        <v>-7.24</v>
+        <v>-6.69</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>서부T&amp;D</t>
+          <t>세아메카닉스</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4553,25 +4551,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H44" s="27" t="n">
-        <v>2.32</v>
-      </c>
-      <c r="I44" s="29" t="n">
-        <v>-3.19</v>
+        <v>6.48</v>
+      </c>
+      <c r="I44" s="27" t="n">
+        <v>17.76</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>서한</t>
+          <t>셀리드</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4588,25 +4586,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H45" s="27" t="n">
-        <v>2.26</v>
-      </c>
-      <c r="I45" s="29" t="n">
-        <v>-6.69</v>
+        <v>1.13</v>
+      </c>
+      <c r="I45" s="27" t="n">
+        <v>62.26</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>세아메카닉스</t>
+          <t>씨피시스템</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4623,25 +4621,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H46" s="27" t="n">
-        <v>6.48</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="I46" s="27" t="n">
-        <v>17.76</v>
+        <v>23.48</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>셀리드</t>
+          <t>아이씨에이치</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4658,25 +4656,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H47" s="27" t="n">
-        <v>1.13</v>
+        <v>5.96</v>
       </c>
       <c r="I47" s="27" t="n">
-        <v>62.26</v>
+        <v>34.09</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>씨피시스템</t>
+          <t>일승</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4693,25 +4691,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H48" s="27" t="n">
-        <v>8.869999999999999</v>
-      </c>
-      <c r="I48" s="27" t="n">
-        <v>23.48</v>
+        <v>8.83</v>
+      </c>
+      <c r="I48" s="29" t="n">
+        <v>-2.55</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>아이씨에이치</t>
+          <t>조일알미늄</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4728,25 +4726,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H49" s="27" t="n">
-        <v>5.96</v>
+        <v>5.04</v>
       </c>
       <c r="I49" s="27" t="n">
-        <v>34.09</v>
+        <v>16.19</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>일승</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4763,25 +4761,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H50" s="27" t="n">
-        <v>8.83</v>
-      </c>
-      <c r="I50" s="29" t="n">
-        <v>-2.55</v>
+        <v>3.46</v>
+      </c>
+      <c r="I50" s="27" t="n">
+        <v>3.31</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>포스코인터내셔널</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4798,25 +4796,25 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H51" s="27" t="n">
-        <v>2.15</v>
+        <v>8.51</v>
       </c>
       <c r="I51" s="29" t="n">
-        <v>-7.28</v>
+        <v>-15</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="26" t="inlineStr">
         <is>
-          <t>한화생명</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -4833,19 +4831,19 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H52" s="27" t="n">
-        <v>5.11</v>
+        <v>7.44</v>
       </c>
       <c r="I52" s="29" t="n">
-        <v>-3.7</v>
+        <v>-3.07</v>
       </c>
     </row>
   </sheetData>
@@ -4929,19 +4927,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4953,26 +4951,26 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="35" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B4" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4984,26 +4982,26 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="35" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B5" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5015,26 +5013,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5046,26 +5044,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5084,19 +5082,19 @@
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5108,92 +5106,100 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
+          <t>제약</t>
+        </is>
+      </c>
+      <c r="B9" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="36" t="n">
+        <v>14</v>
+      </c>
+      <c r="D9" s="36" t="n">
+        <v>14</v>
+      </c>
+      <c r="E9" s="36" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F9" s="37" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="G9" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
           <t>인공지능</t>
         </is>
       </c>
-      <c r="B9" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" s="36" t="n">
-        <v>12</v>
-      </c>
-      <c r="D9" s="36" t="n">
-        <v>12</v>
-      </c>
-      <c r="E9" s="36" t="inlineStr">
-        <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="F9" s="37" t="inlineStr">
-        <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="G9" s="37" t="inlineStr">
+      <c r="B10" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="36" t="n">
+        <v>11</v>
+      </c>
+      <c r="D10" s="36" t="n">
+        <v>11</v>
+      </c>
+      <c r="E10" s="36" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F10" s="37" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="G10" s="37" t="inlineStr">
         <is>
           <t>⚡ 관심</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="26" t="inlineStr">
-        <is>
-          <t>이차전지</t>
-        </is>
-      </c>
-      <c r="B10" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" s="28" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="inlineStr"/>
-    </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="26" t="inlineStr">
-        <is>
-          <t>바이오</t>
-        </is>
-      </c>
-      <c r="B11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F11" s="28" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="inlineStr"/>
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B11" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="36" t="n">
+        <v>6</v>
+      </c>
+      <c r="D11" s="36" t="n">
+        <v>6</v>
+      </c>
+      <c r="E11" s="36" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F11" s="37" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="G11" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>이차전지</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
@@ -5220,7 +5226,7 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -5247,7 +5253,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5274,7 +5280,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5301,7 +5307,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -5328,7 +5334,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>핀테크</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -5355,7 +5361,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -5382,7 +5388,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>핀테크</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -5409,7 +5415,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
@@ -5436,7 +5442,7 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -5463,7 +5469,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -5490,7 +5496,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>Tesla</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -5517,7 +5523,7 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Tesla</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-08-10 07:06 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -279,9 +279,6 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -289,6 +286,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-08-09 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-08-10 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-08-09) 상위: 반도체  점수 51.0점</t>
+          <t>⚡ 최신(2026-08-10) 상위: 반도체  점수 76.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-08-09) 상위: SK하이닉스  점수 31.0점</t>
+          <t>⚡ 최신(2026-08-10) 상위: SK하이닉스  점수 34.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-08-09) 상위: 네이버  점수 21.0점</t>
+          <t>⚡ 최신(2026-08-10) 상위: 로봇  점수 20.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>51</v>
+        <v>76</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>51</v>
+        <v>76</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,19 +947,19 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
+          <t>Google 급상승 검색어 등장 (KR) / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, Google</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -971,13 +971,13 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
+        <v>34</v>
+      </c>
+      <c r="E15" s="15" t="n">
         <v>31</v>
       </c>
-      <c r="E15" s="15" t="n">
-        <v>26</v>
-      </c>
       <c r="F15" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G15" s="15" t="n">
         <v>3</v>
@@ -990,7 +990,7 @@
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +200% / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 3건 / 중요공시 7일 +200% / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1010,14 +1010,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1033,17 +1033,19 @@
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K16" s="17" t="n">
-        <v/>
+          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K16" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1051,14 +1053,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1066,15 +1068,15 @@
       <c r="G17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I17" s="15" t="n">
-        <v/>
+      <c r="H17" s="19" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="I17" s="18" t="n">
+        <v>-12</v>
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
@@ -1086,7 +1088,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1094,14 +1096,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1109,15 +1111,15 @@
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="19" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="I18" s="18" t="n">
-        <v>-12</v>
+      <c r="H18" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I18" s="15" t="n">
+        <v/>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K18" s="17" t="inlineStr">
@@ -1129,7 +1131,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1137,14 +1139,14 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1160,19 +1162,17 @@
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K19" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K19" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1180,42 +1180,42 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="F20" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G20" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H20" s="19" t="n">
-        <v>14.96</v>
-      </c>
-      <c r="I20" s="19" t="n">
-        <v>49.68</v>
+        <v>0</v>
+      </c>
+      <c r="H20" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I20" s="15" t="n">
+        <v/>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +200%</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K20" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1223,40 +1223,42 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F21" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G21" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="18" t="n">
-        <v>-1.12</v>
+        <v>3</v>
+      </c>
+      <c r="H21" s="19" t="n">
+        <v>14.96</v>
       </c>
       <c r="I21" s="19" t="n">
-        <v>1.93</v>
+        <v>49.68</v>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K21" s="17" t="n">
-        <v/>
+          <t>네이버 검색 당일 +55% / 중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +200%</t>
+        </is>
+      </c>
+      <c r="K21" s="17" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1264,42 +1266,40 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>대양금속</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F22" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G22" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H22" s="19" t="n">
-        <v>2.48</v>
-      </c>
-      <c r="I22" s="19" t="n">
-        <v>17.96</v>
+        <v>0</v>
+      </c>
+      <c r="H22" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I22" s="15" t="n">
+        <v/>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +200%</t>
-        </is>
-      </c>
-      <c r="K22" s="17" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K22" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1307,14 +1307,14 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>테스</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F23" s="15" t="n">
         <v>0</v>
@@ -1322,15 +1322,15 @@
       <c r="G23" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I23" s="15" t="n">
-        <v/>
+      <c r="H23" s="18" t="n">
+        <v>-4.23</v>
+      </c>
+      <c r="I23" s="18" t="n">
+        <v>-4.15</v>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K23" s="17" t="inlineStr">
@@ -1342,7 +1342,7 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1350,42 +1350,42 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>빛과전자</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G24" s="15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H24" s="19" t="n">
-        <v>3.26</v>
+        <v>3.76</v>
       </c>
       <c r="I24" s="19" t="n">
-        <v>60.01</v>
+        <v>5.92</v>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +114% / 중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 4건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K24" s="17" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1393,14 +1393,14 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F25" s="15" t="n">
         <v>0</v>
@@ -1408,27 +1408,25 @@
       <c r="G25" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H25" s="19" t="n">
-        <v>4.18</v>
+      <c r="H25" s="18" t="n">
+        <v>-1.12</v>
       </c>
       <c r="I25" s="19" t="n">
-        <v>6.68</v>
+        <v>1.93</v>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K25" s="17" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K25" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1436,126 +1434,128 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>GS리테일</t>
+          <t>유티아이</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
         <v>7</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F26" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G26" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H26" s="19" t="n">
-        <v>7.18</v>
-      </c>
-      <c r="I26" s="19" t="n">
-        <v>14.55</v>
+        <v>13.2</v>
+      </c>
+      <c r="I26" s="18" t="n">
+        <v>-3.46</v>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +93% / 중요공시 5건 / 중요공시 3일 +400%</t>
         </is>
       </c>
       <c r="K26" s="17" t="inlineStr">
         <is>
+          <t>네이버, 공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B27" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="C27" s="21" t="inlineStr">
+        <is>
+          <t>금호건설</t>
+        </is>
+      </c>
+      <c r="D27" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E27" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F27" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H27" s="22" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="I27" s="22" t="n">
+        <v>7.24</v>
+      </c>
+      <c r="J27" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 7일 +200%</t>
+        </is>
+      </c>
+      <c r="K27" s="23" t="inlineStr">
+        <is>
           <t>공시</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="15" t="inlineStr">
-        <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="B27" s="15" t="n">
-        <v>14</v>
-      </c>
-      <c r="C27" s="16" t="inlineStr">
-        <is>
-          <t>제약</t>
-        </is>
-      </c>
-      <c r="D27" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E27" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F27" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I27" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J27" s="17" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K27" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="15" t="inlineStr">
-        <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="B28" s="15" t="n">
+      <c r="A28" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="C28" s="16" t="inlineStr">
-        <is>
-          <t>DB</t>
-        </is>
-      </c>
-      <c r="D28" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E28" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F28" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I28" s="19" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="J28" s="17" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K28" s="17" t="n">
-        <v/>
+      <c r="C28" s="21" t="inlineStr">
+        <is>
+          <t>HLB테라퓨틱스</t>
+        </is>
+      </c>
+      <c r="D28" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E28" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F28" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="22" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="I28" s="22" t="n">
+        <v>22.81</v>
+      </c>
+      <c r="J28" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 5건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K28" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B29" s="20" t="n">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>썸에이지</t>
         </is>
       </c>
       <c r="D29" s="20" t="n">
@@ -1578,15 +1578,15 @@
       <c r="G29" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="H29" s="22" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="I29" s="22" t="n">
-        <v>7.24</v>
+      <c r="H29" s="24" t="n">
+        <v>-2.69</v>
+      </c>
+      <c r="I29" s="24" t="n">
+        <v>-1.94</v>
       </c>
       <c r="J29" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 7일 +200%</t>
+          <t>중요공시 4건 / 중요공시 7일 +300%</t>
         </is>
       </c>
       <c r="K29" s="23" t="inlineStr">
@@ -1598,7 +1598,7 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
@@ -1606,30 +1606,30 @@
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>HLB테라퓨틱스</t>
+          <t>지엔씨에너지</t>
         </is>
       </c>
       <c r="D30" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E30" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F30" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G30" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H30" s="22" t="n">
-        <v>0.49</v>
+        <v>2.35</v>
       </c>
       <c r="I30" s="22" t="n">
-        <v>22.81</v>
+        <v>42.9</v>
       </c>
       <c r="J30" s="23" t="inlineStr">
         <is>
-          <t>중요공시 5건 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 3건 / 중요공시 7일 +50%</t>
         </is>
       </c>
       <c r="K30" s="23" t="inlineStr">
@@ -1641,7 +1641,7 @@
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>한울반도체</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
@@ -1664,27 +1664,27 @@
       <c r="G31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="22" t="n">
-        <v>3.99</v>
+      <c r="H31" s="24" t="n">
+        <v>-1.81</v>
       </c>
       <c r="I31" s="22" t="n">
-        <v>11.91</v>
+        <v>1.42</v>
       </c>
       <c r="J31" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 1건 / Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K31" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>Google, 공시</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1692,40 +1692,42 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>현대지에프홀딩스</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F32" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G32" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H32" s="24" t="n">
-        <v>-0.37</v>
+      <c r="H32" s="22" t="n">
+        <v>3.04</v>
       </c>
       <c r="I32" s="22" t="n">
-        <v>2.7</v>
+        <v>3.48</v>
       </c>
       <c r="J32" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K32" s="23" t="n">
-        <v/>
+          <t>중요공시 10건 / 중요공시 3일 +67%</t>
+        </is>
+      </c>
+      <c r="K32" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1733,40 +1735,42 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>티엘비</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F33" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G33" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H33" s="22" t="n">
-        <v>0.1</v>
+      <c r="H33" s="24" t="n">
+        <v>-6.18</v>
       </c>
       <c r="I33" s="22" t="n">
-        <v>11.12</v>
+        <v>6.44</v>
       </c>
       <c r="J33" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K33" s="23" t="n">
-        <v/>
+          <t>중요공시 4건 / 중요공시 3일 +300%</t>
+        </is>
+      </c>
+      <c r="K33" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1774,40 +1778,42 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>HMM</t>
+          <t>서진시스템</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F34" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G34" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="22" t="n">
-        <v>1.87</v>
+      <c r="H34" s="24" t="n">
+        <v>-3.94</v>
       </c>
       <c r="I34" s="22" t="n">
-        <v>4.06</v>
+        <v>3.33</v>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K34" s="23" t="n">
-        <v/>
+          <t>중요공시 3건 / 중요공시 3일 +200%</t>
+        </is>
+      </c>
+      <c r="K34" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1815,42 +1821,42 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>유티아이</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F35" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G35" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H35" s="22" t="n">
-        <v>13.2</v>
-      </c>
-      <c r="I35" s="24" t="n">
-        <v>-3.46</v>
+        <v>3.92</v>
+      </c>
+      <c r="I35" s="22" t="n">
+        <v>28.49</v>
       </c>
       <c r="J35" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +84% / 중요공시 5건</t>
+          <t>중요공시 3건 / 중요공시 3일 +50%</t>
         </is>
       </c>
       <c r="K35" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1858,7 +1864,7 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>대한광통신</t>
+          <t>제주반도체</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
@@ -1874,26 +1880,26 @@
         <v>0</v>
       </c>
       <c r="H36" s="22" t="n">
-        <v>3.52</v>
+        <v>1.48</v>
       </c>
       <c r="I36" s="22" t="n">
-        <v>34.35</v>
+        <v>15.82</v>
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +53% / 네이버뉴스 헤드라인 언급</t>
+          <t>Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K36" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1901,7 +1907,7 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>우리기술</t>
+          <t>SFA반도체</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
@@ -1917,26 +1923,26 @@
         <v>0</v>
       </c>
       <c r="H37" s="24" t="n">
-        <v>-0.36</v>
+        <v>-2.44</v>
       </c>
       <c r="I37" s="22" t="n">
-        <v>24.03</v>
+        <v>2.57</v>
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
+          <t>Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K37" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1944,42 +1950,42 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>현대지에프홀딩스</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F38" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H38" s="22" t="n">
-        <v>3.04</v>
-      </c>
-      <c r="I38" s="22" t="n">
-        <v>3.48</v>
+      <c r="H38" s="24" t="n">
+        <v>-4.09</v>
+      </c>
+      <c r="I38" s="24" t="n">
+        <v>-10.35</v>
       </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
-          <t>중요공시 10건 / 중요공시 3일 +233%</t>
+          <t>Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K38" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1987,42 +1993,42 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>티엘비</t>
+          <t>서울반도체</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F39" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G39" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H39" s="24" t="n">
-        <v>-6.18</v>
+        <v>-0.33</v>
       </c>
       <c r="I39" s="22" t="n">
-        <v>6.44</v>
+        <v>5.17</v>
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 중요공시 3일 +300%</t>
+          <t>Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K39" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2030,42 +2036,42 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>POSCO홀딩스</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F40" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G40" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H40" s="22" t="n">
-        <v>3.76</v>
-      </c>
-      <c r="I40" s="22" t="n">
-        <v>5.92</v>
+      <c r="H40" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I40" s="20" t="n">
+        <v/>
       </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 중요공시 3일 +100%</t>
+          <t>Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K40" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2073,42 +2079,42 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>서진시스템</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E41" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F41" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G41" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="24" t="n">
-        <v>-3.94</v>
+      <c r="H41" s="22" t="n">
+        <v>3.99</v>
       </c>
       <c r="I41" s="22" t="n">
-        <v>3.33</v>
+        <v>11.91</v>
       </c>
       <c r="J41" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200%</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K41" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2116,42 +2122,42 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>알테오젠</t>
+          <t>비큐AI</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E42" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F42" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G42" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H42" s="22" t="n">
-        <v>3.92</v>
+      <c r="H42" s="24" t="n">
+        <v>-11.88</v>
       </c>
       <c r="I42" s="22" t="n">
-        <v>28.49</v>
+        <v>93.48</v>
       </c>
       <c r="J42" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200%</t>
+          <t>네이버 검색 당일 +829% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K42" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2159,7 +2165,7 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>비큐AI</t>
+          <t>오이솔루션</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
@@ -2174,27 +2180,27 @@
       <c r="G43" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H43" s="24" t="n">
-        <v>-11.88</v>
+      <c r="H43" s="22" t="n">
+        <v>18.53</v>
       </c>
       <c r="I43" s="22" t="n">
-        <v>93.48</v>
+        <v>69.11</v>
       </c>
       <c r="J43" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +789% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +310% / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K43" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2202,7 +2208,7 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>오이솔루션</t>
+          <t>이스트에이드</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
@@ -2217,27 +2223,27 @@
       <c r="G44" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="22" t="n">
-        <v>18.53</v>
+      <c r="H44" s="20" t="n">
+        <v>0</v>
       </c>
       <c r="I44" s="22" t="n">
-        <v>69.11</v>
+        <v>65.42</v>
       </c>
       <c r="J44" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +281% / 매일경제 기사 언급</t>
+          <t>네이버 검색 당일 +219% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K44" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2245,7 +2251,7 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>이스트에이드</t>
+          <t>한국첨단소재</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
@@ -2260,15 +2266,15 @@
       <c r="G45" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H45" s="20" t="n">
-        <v>0</v>
+      <c r="H45" s="22" t="n">
+        <v>29.89</v>
       </c>
       <c r="I45" s="22" t="n">
-        <v>65.42</v>
+        <v>29.89</v>
       </c>
       <c r="J45" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +208% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +177% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K45" s="23" t="inlineStr">
@@ -2280,7 +2286,7 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
@@ -2288,7 +2294,7 @@
       </c>
       <c r="C46" s="21" t="inlineStr">
         <is>
-          <t>한국첨단소재</t>
+          <t>랩지노믹스</t>
         </is>
       </c>
       <c r="D46" s="20" t="n">
@@ -2304,14 +2310,14 @@
         <v>0</v>
       </c>
       <c r="H46" s="22" t="n">
-        <v>29.89</v>
+        <v>12.5</v>
       </c>
       <c r="I46" s="22" t="n">
-        <v>29.89</v>
+        <v>61.24</v>
       </c>
       <c r="J46" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +147% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +132% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K46" s="23" t="inlineStr">
@@ -2323,7 +2329,7 @@
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B47" s="20" t="n">
@@ -2331,7 +2337,7 @@
       </c>
       <c r="C47" s="21" t="inlineStr">
         <is>
-          <t>랩지노믹스</t>
+          <t>빛과전자</t>
         </is>
       </c>
       <c r="D47" s="20" t="n">
@@ -2347,14 +2353,14 @@
         <v>0</v>
       </c>
       <c r="H47" s="22" t="n">
-        <v>12.5</v>
+        <v>3.26</v>
       </c>
       <c r="I47" s="22" t="n">
-        <v>61.24</v>
+        <v>60.01</v>
       </c>
       <c r="J47" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +119% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +122% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K47" s="23" t="inlineStr">
@@ -2366,7 +2372,7 @@
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B48" s="20" t="n">
@@ -2409,7 +2415,7 @@
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B49" s="20" t="n">
@@ -2417,42 +2423,40 @@
       </c>
       <c r="C49" s="21" t="inlineStr">
         <is>
-          <t>SK디앤디</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="D49" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E49" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F49" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G49" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H49" s="24" t="n">
-        <v>-11.95</v>
+        <v>0</v>
+      </c>
+      <c r="H49" s="22" t="n">
+        <v>11.51</v>
       </c>
       <c r="I49" s="22" t="n">
-        <v>22.2</v>
+        <v>32.94</v>
       </c>
       <c r="J49" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K49" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K49" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B50" s="20" t="n">
@@ -2460,30 +2464,30 @@
       </c>
       <c r="C50" s="21" t="inlineStr">
         <is>
-          <t>아미코젠</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="D50" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E50" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F50" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G50" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H50" s="24" t="n">
-        <v>-1.82</v>
-      </c>
-      <c r="I50" s="24" t="n">
-        <v>-8.98</v>
+        <v>0</v>
+      </c>
+      <c r="H50" s="22" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="I50" s="22" t="n">
+        <v>6.68</v>
       </c>
       <c r="J50" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+          <t>중요공시 2건 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K50" s="23" t="inlineStr">
@@ -2495,7 +2499,7 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B51" s="20" t="n">
@@ -2503,7 +2507,7 @@
       </c>
       <c r="C51" s="21" t="inlineStr">
         <is>
-          <t>KG모빌리티</t>
+          <t>아미코젠</t>
         </is>
       </c>
       <c r="D51" s="20" t="n">
@@ -2519,10 +2523,10 @@
         <v>3</v>
       </c>
       <c r="H51" s="24" t="n">
-        <v>-0.17</v>
-      </c>
-      <c r="I51" s="22" t="n">
-        <v>1.76</v>
+        <v>-1.82</v>
+      </c>
+      <c r="I51" s="24" t="n">
+        <v>-8.98</v>
       </c>
       <c r="J51" s="23" t="inlineStr">
         <is>
@@ -2538,7 +2542,7 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B52" s="20" t="n">
@@ -2546,30 +2550,30 @@
       </c>
       <c r="C52" s="21" t="inlineStr">
         <is>
-          <t>엘앤에프</t>
+          <t>KG모빌리티</t>
         </is>
       </c>
       <c r="D52" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E52" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F52" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G52" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H52" s="22" t="n">
-        <v>13.03</v>
+        <v>3</v>
+      </c>
+      <c r="H52" s="24" t="n">
+        <v>-0.17</v>
       </c>
       <c r="I52" s="22" t="n">
-        <v>23.06</v>
+        <v>1.76</v>
       </c>
       <c r="J52" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K52" s="23" t="inlineStr">
@@ -2581,7 +2585,7 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B53" s="20" t="n">
@@ -2589,30 +2593,30 @@
       </c>
       <c r="C53" s="21" t="inlineStr">
         <is>
-          <t>기아</t>
+          <t>HJ중공업</t>
         </is>
       </c>
       <c r="D53" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E53" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F53" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G53" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H53" s="22" t="n">
-        <v>0.97</v>
+        <v>3</v>
+      </c>
+      <c r="H53" s="20" t="n">
+        <v>0</v>
       </c>
       <c r="I53" s="22" t="n">
-        <v>2.27</v>
+        <v>6.37</v>
       </c>
       <c r="J53" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K53" s="23" t="inlineStr">
@@ -2624,7 +2628,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B54" s="20" t="n">
@@ -2632,7 +2636,7 @@
       </c>
       <c r="C54" s="21" t="inlineStr">
         <is>
-          <t>서울전자통신</t>
+          <t>엘앤에프</t>
         </is>
       </c>
       <c r="D54" s="20" t="n">
@@ -2648,14 +2652,14 @@
         <v>0</v>
       </c>
       <c r="H54" s="22" t="n">
-        <v>12.83</v>
+        <v>13.03</v>
       </c>
       <c r="I54" s="22" t="n">
-        <v>31.66</v>
+        <v>23.06</v>
       </c>
       <c r="J54" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K54" s="23" t="inlineStr">
@@ -2667,7 +2671,7 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B55" s="20" t="n">
@@ -2675,7 +2679,7 @@
       </c>
       <c r="C55" s="21" t="inlineStr">
         <is>
-          <t>와이즈버즈</t>
+          <t>심텍</t>
         </is>
       </c>
       <c r="D55" s="20" t="n">
@@ -2691,10 +2695,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="22" t="n">
-        <v>4.85</v>
+        <v>3.77</v>
       </c>
       <c r="I55" s="22" t="n">
-        <v>33.59</v>
+        <v>32.69</v>
       </c>
       <c r="J55" s="23" t="inlineStr">
         <is>
@@ -2710,7 +2714,7 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B56" s="20" t="n">
@@ -2718,7 +2722,7 @@
       </c>
       <c r="C56" s="21" t="inlineStr">
         <is>
-          <t>신성이엔지</t>
+          <t>서울전자통신</t>
         </is>
       </c>
       <c r="D56" s="20" t="n">
@@ -2733,15 +2737,15 @@
       <c r="G56" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H56" s="24" t="n">
-        <v>-5.32</v>
+      <c r="H56" s="22" t="n">
+        <v>12.83</v>
       </c>
       <c r="I56" s="22" t="n">
-        <v>7.38</v>
+        <v>31.66</v>
       </c>
       <c r="J56" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K56" s="23" t="inlineStr">
@@ -2753,7 +2757,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B57" s="20" t="n">
@@ -2761,7 +2765,7 @@
       </c>
       <c r="C57" s="21" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>GS리테일</t>
         </is>
       </c>
       <c r="D57" s="20" t="n">
@@ -2776,25 +2780,27 @@
       <c r="G57" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H57" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I57" s="20" t="n">
-        <v/>
+      <c r="H57" s="22" t="n">
+        <v>7.18</v>
+      </c>
+      <c r="I57" s="22" t="n">
+        <v>14.55</v>
       </c>
       <c r="J57" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K57" s="23" t="n">
-        <v/>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K57" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B58" s="20" t="n">
@@ -2802,7 +2808,7 @@
       </c>
       <c r="C58" s="21" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D58" s="20" t="n">
@@ -2817,154 +2823,152 @@
       <c r="G58" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="22" t="n">
-        <v>7.49</v>
-      </c>
-      <c r="I58" s="22" t="n">
-        <v>15.62</v>
+      <c r="H58" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I58" s="20" t="n">
+        <v/>
       </c>
       <c r="J58" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K58" s="23" t="n">
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K58" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="18" customHeight="1">
+      <c r="A59" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B59" s="20" t="n">
+        <v>46</v>
+      </c>
+      <c r="C59" s="21" t="inlineStr">
+        <is>
+          <t>태양광</t>
+        </is>
+      </c>
+      <c r="D59" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E59" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F59" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" s="20" t="n">
         <v/>
       </c>
-    </row>
-    <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="25" t="inlineStr">
-        <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="B59" s="25" t="n">
-        <v>46</v>
-      </c>
-      <c r="C59" s="26" t="inlineStr">
-        <is>
-          <t>동화기업</t>
-        </is>
-      </c>
-      <c r="D59" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E59" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F59" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G59" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H59" s="27" t="n">
-        <v>30</v>
-      </c>
-      <c r="I59" s="27" t="n">
-        <v>44.19</v>
-      </c>
-      <c r="J59" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +236%</t>
-        </is>
-      </c>
-      <c r="K59" s="28" t="inlineStr">
+      <c r="I59" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J59" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K59" s="23" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="25" t="inlineStr">
-        <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="B60" s="25" t="n">
+      <c r="A60" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B60" s="20" t="n">
         <v>47</v>
       </c>
-      <c r="C60" s="26" t="inlineStr">
-        <is>
-          <t>삼기에너지솔루션즈</t>
-        </is>
-      </c>
-      <c r="D60" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E60" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F60" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G60" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H60" s="29" t="n">
-        <v>-1.91</v>
-      </c>
-      <c r="I60" s="27" t="n">
-        <v>39.11</v>
-      </c>
-      <c r="J60" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +234%</t>
-        </is>
-      </c>
-      <c r="K60" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+      <c r="C60" s="21" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="D60" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E60" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F60" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" s="22" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J60" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K60" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
-      <c r="A61" s="25" t="inlineStr">
-        <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="B61" s="25" t="n">
+      <c r="A61" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B61" s="20" t="n">
         <v>48</v>
       </c>
-      <c r="C61" s="26" t="inlineStr">
-        <is>
-          <t>신스틸</t>
-        </is>
-      </c>
-      <c r="D61" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E61" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F61" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G61" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H61" s="27" t="n">
-        <v>29.96</v>
-      </c>
-      <c r="I61" s="27" t="n">
-        <v>31.81</v>
-      </c>
-      <c r="J61" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +206%</t>
-        </is>
-      </c>
-      <c r="K61" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+      <c r="C61" s="21" t="inlineStr">
+        <is>
+          <t>HMM</t>
+        </is>
+      </c>
+      <c r="D61" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E61" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F61" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" s="22" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="I61" s="22" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="J61" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K61" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2972,7 +2976,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>상상인증권</t>
+          <t>동화기업</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2988,14 +2992,14 @@
         <v>0</v>
       </c>
       <c r="H62" s="27" t="n">
-        <v>29.91</v>
+        <v>30</v>
       </c>
       <c r="I62" s="27" t="n">
-        <v>85.08</v>
+        <v>44.19</v>
       </c>
       <c r="J62" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +193%</t>
+          <t>네이버 검색 당일 +279%</t>
         </is>
       </c>
       <c r="K62" s="28" t="inlineStr">
@@ -3007,7 +3011,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3015,7 +3019,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>광전자</t>
+          <t>신스틸</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3031,14 +3035,14 @@
         <v>0</v>
       </c>
       <c r="H63" s="27" t="n">
-        <v>15.02</v>
+        <v>29.96</v>
       </c>
       <c r="I63" s="27" t="n">
-        <v>50.48</v>
+        <v>31.81</v>
       </c>
       <c r="J63" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +104%</t>
+          <t>네이버 검색 당일 +274%</t>
         </is>
       </c>
       <c r="K63" s="28" t="inlineStr">
@@ -3077,54 +3081,54 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="30" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>🎯 종목별 신호 추적 - 연속 감지 및 누적 분석</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="31" t="inlineStr">
+      <c r="A2" s="30" t="inlineStr">
         <is>
           <t>종목/키워드</t>
         </is>
       </c>
-      <c r="B2" s="31" t="inlineStr">
+      <c r="B2" s="30" t="inlineStr">
         <is>
           <t>총감지횟수</t>
         </is>
       </c>
-      <c r="C2" s="31" t="inlineStr">
+      <c r="C2" s="30" t="inlineStr">
         <is>
           <t>최고점수</t>
         </is>
       </c>
-      <c r="D2" s="31" t="inlineStr">
+      <c r="D2" s="30" t="inlineStr">
         <is>
           <t>평균점수</t>
         </is>
       </c>
-      <c r="E2" s="31" t="inlineStr">
+      <c r="E2" s="30" t="inlineStr">
         <is>
           <t>연속감지일</t>
         </is>
       </c>
-      <c r="F2" s="31" t="inlineStr">
+      <c r="F2" s="30" t="inlineStr">
         <is>
           <t>최초감지일</t>
         </is>
       </c>
-      <c r="G2" s="31" t="inlineStr">
+      <c r="G2" s="30" t="inlineStr">
         <is>
           <t>최근감지일</t>
         </is>
       </c>
-      <c r="H2" s="31" t="inlineStr">
+      <c r="H2" s="30" t="inlineStr">
         <is>
           <t>평균주가당일(%)</t>
         </is>
       </c>
-      <c r="I2" s="31" t="inlineStr">
+      <c r="I2" s="30" t="inlineStr">
         <is>
           <t>평균주가7일(%)</t>
         </is>
@@ -3140,22 +3144,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>51</v>
+        <v>76</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>51</v>
-      </c>
-      <c r="E3" s="32" t="n">
+        <v>76</v>
+      </c>
+      <c r="E3" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3171,57 +3175,57 @@
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>31</v>
-      </c>
-      <c r="E4" s="32" t="n">
+        <v>34</v>
+      </c>
+      <c r="E4" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H4" s="29" t="n">
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H4" s="32" t="n">
         <v>-4.88</v>
       </c>
-      <c r="I4" s="29" t="n">
+      <c r="I4" s="32" t="n">
         <v>-17.23</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>21</v>
-      </c>
-      <c r="E5" s="32" t="n">
+        <v>20</v>
+      </c>
+      <c r="E5" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="H5" s="25" t="n"/>
@@ -3230,95 +3234,95 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>17</v>
-      </c>
-      <c r="E6" s="32" t="n">
+        <v>18</v>
+      </c>
+      <c r="E6" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H6" s="25" t="n"/>
-      <c r="I6" s="25" t="n"/>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H6" s="27" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="I6" s="32" t="n">
+        <v>-12</v>
+      </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>13</v>
-      </c>
-      <c r="E7" s="32" t="n">
+        <v>17</v>
+      </c>
+      <c r="E7" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H7" s="27" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="I7" s="29" t="n">
-        <v>-12</v>
-      </c>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H7" s="25" t="n"/>
+      <c r="I7" s="25" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>13</v>
-      </c>
-      <c r="E8" s="32" t="n">
+        <v>16</v>
+      </c>
+      <c r="E8" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="H8" s="25" t="n"/>
@@ -3327,213 +3331,209 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>9</v>
-      </c>
-      <c r="E9" s="32" t="n">
+        <v>14</v>
+      </c>
+      <c r="E9" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H9" s="27" t="n">
-        <v>14.96</v>
-      </c>
-      <c r="I9" s="27" t="n">
-        <v>49.68</v>
-      </c>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H9" s="25" t="n"/>
+      <c r="I9" s="25" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>9</v>
-      </c>
-      <c r="E10" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="E10" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H10" s="29" t="n">
-        <v>-1.12</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H10" s="27" t="n">
+        <v>14.96</v>
       </c>
       <c r="I10" s="27" t="n">
-        <v>1.93</v>
+        <v>49.68</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>대양금속</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>8</v>
-      </c>
-      <c r="E11" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="E11" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H11" s="27" t="n">
-        <v>2.48</v>
-      </c>
-      <c r="I11" s="27" t="n">
-        <v>17.96</v>
-      </c>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H11" s="25" t="n"/>
+      <c r="I11" s="25" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>테스</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>8</v>
-      </c>
-      <c r="E12" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="E12" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H12" s="25" t="n"/>
-      <c r="I12" s="25" t="n"/>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H12" s="32" t="n">
+        <v>-4.23</v>
+      </c>
+      <c r="I12" s="32" t="n">
+        <v>-4.15</v>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>7</v>
-      </c>
-      <c r="E13" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="E13" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H13" s="25" t="n">
-        <v>0</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H13" s="27" t="n">
+        <v>3.76</v>
       </c>
       <c r="I13" s="27" t="n">
-        <v>0.9</v>
+        <v>5.92</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>GS리테일</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>7</v>
-      </c>
-      <c r="E14" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="E14" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H14" s="27" t="n">
-        <v>7.18</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H14" s="32" t="n">
+        <v>-1.12</v>
       </c>
       <c r="I14" s="27" t="n">
-        <v>14.55</v>
+        <v>1.93</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>빛과전자</t>
+          <t>유티아이</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -3545,96 +3545,100 @@
       <c r="D15" s="25" t="n">
         <v>7</v>
       </c>
-      <c r="E15" s="32" t="n">
+      <c r="E15" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="H15" s="27" t="n">
-        <v>3.26</v>
-      </c>
-      <c r="I15" s="27" t="n">
-        <v>60.01</v>
+        <v>13.2</v>
+      </c>
+      <c r="I15" s="32" t="n">
+        <v>-3.46</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>HLB테라퓨틱스</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C16" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D16" s="25" t="n">
-        <v>7</v>
-      </c>
-      <c r="E16" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H16" s="25" t="n"/>
-      <c r="I16" s="25" t="n"/>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H16" s="27" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="I16" s="27" t="n">
+        <v>22.81</v>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>7</v>
-      </c>
-      <c r="E17" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="H17" s="27" t="n">
-        <v>4.18</v>
+        <v>1.14</v>
       </c>
       <c r="I17" s="27" t="n">
-        <v>6.68</v>
+        <v>7.24</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>썸에이지</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -3646,30 +3650,30 @@
       <c r="D18" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="E18" s="32" t="n">
+      <c r="E18" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H18" s="27" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I18" s="27" t="n">
-        <v>11.12</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H18" s="32" t="n">
+        <v>-2.69</v>
+      </c>
+      <c r="I18" s="32" t="n">
+        <v>-1.94</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>HLB테라퓨틱스</t>
+          <t>지엔씨에너지</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -3681,30 +3685,30 @@
       <c r="D19" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="E19" s="32" t="n">
+      <c r="E19" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="H19" s="27" t="n">
-        <v>0.49</v>
+        <v>2.35</v>
       </c>
       <c r="I19" s="27" t="n">
-        <v>22.81</v>
+        <v>42.9</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>HMM</t>
+          <t>한울반도체</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
@@ -3716,94 +3720,90 @@
       <c r="D20" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="E20" s="32" t="n">
+      <c r="E20" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H20" s="27" t="n">
-        <v>1.87</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H20" s="32" t="n">
+        <v>-1.81</v>
       </c>
       <c r="I20" s="27" t="n">
-        <v>4.06</v>
+        <v>1.42</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D21" s="25" t="n">
-        <v>6</v>
-      </c>
-      <c r="E21" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="E21" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H21" s="29" t="n">
-        <v>-0.37</v>
-      </c>
-      <c r="I21" s="27" t="n">
-        <v>2.7</v>
-      </c>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H21" s="25" t="n"/>
+      <c r="I21" s="25" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>SFA반도체</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D22" s="25" t="n">
-        <v>6</v>
-      </c>
-      <c r="E22" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="E22" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H22" s="27" t="n">
-        <v>1.14</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H22" s="32" t="n">
+        <v>-2.44</v>
       </c>
       <c r="I22" s="27" t="n">
-        <v>7.24</v>
+        <v>2.57</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
@@ -3816,22 +3816,22 @@
         <v>1</v>
       </c>
       <c r="C23" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D23" s="25" t="n">
-        <v>6</v>
-      </c>
-      <c r="E23" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="E23" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="H23" s="27" t="n">
@@ -3844,7 +3844,7 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>POSCO홀딩스</t>
+          <t>서울반도체</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3856,30 +3856,30 @@
       <c r="D24" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="E24" s="32" t="n">
+      <c r="E24" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H24" s="27" t="n">
-        <v>3.76</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H24" s="32" t="n">
+        <v>-0.33</v>
       </c>
       <c r="I24" s="27" t="n">
-        <v>5.92</v>
+        <v>5.17</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>대한광통신</t>
+          <t>서진시스템</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3891,30 +3891,30 @@
       <c r="D25" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="E25" s="32" t="n">
+      <c r="E25" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H25" s="27" t="n">
-        <v>3.52</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H25" s="32" t="n">
+        <v>-3.94</v>
       </c>
       <c r="I25" s="27" t="n">
-        <v>34.35</v>
+        <v>3.33</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>서진시스템</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
@@ -3926,30 +3926,30 @@
       <c r="D26" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="E26" s="32" t="n">
+      <c r="E26" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H26" s="29" t="n">
-        <v>-3.94</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H26" s="27" t="n">
+        <v>3.92</v>
       </c>
       <c r="I26" s="27" t="n">
-        <v>3.33</v>
+        <v>28.49</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>알테오젠</t>
+          <t>제주반도체</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
@@ -3961,30 +3961,30 @@
       <c r="D27" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="E27" s="32" t="n">
+      <c r="E27" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="H27" s="27" t="n">
-        <v>3.92</v>
+        <v>1.48</v>
       </c>
       <c r="I27" s="27" t="n">
-        <v>28.49</v>
+        <v>15.82</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>우리기술</t>
+          <t>티엘비</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
@@ -3996,30 +3996,30 @@
       <c r="D28" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="E28" s="32" t="n">
+      <c r="E28" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H28" s="29" t="n">
-        <v>-0.36</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H28" s="32" t="n">
+        <v>-6.18</v>
       </c>
       <c r="I28" s="27" t="n">
-        <v>24.03</v>
+        <v>6.44</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>유티아이</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
@@ -4031,30 +4031,30 @@
       <c r="D29" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="E29" s="32" t="n">
+      <c r="E29" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H29" s="27" t="n">
-        <v>13.2</v>
-      </c>
-      <c r="I29" s="29" t="n">
-        <v>-3.46</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H29" s="32" t="n">
+        <v>-4.09</v>
+      </c>
+      <c r="I29" s="32" t="n">
+        <v>-10.35</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>티엘비</t>
+          <t>현대지에프홀딩스</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -4066,65 +4066,65 @@
       <c r="D30" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="E30" s="32" t="n">
+      <c r="E30" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H30" s="29" t="n">
-        <v>-6.18</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H30" s="27" t="n">
+        <v>3.04</v>
       </c>
       <c r="I30" s="27" t="n">
-        <v>6.44</v>
+        <v>3.48</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>현대지에프홀딩스</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C31" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D31" s="25" t="n">
-        <v>5</v>
-      </c>
-      <c r="E31" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="E31" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H31" s="27" t="n">
-        <v>3.04</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H31" s="25" t="n">
+        <v>0</v>
       </c>
       <c r="I31" s="27" t="n">
-        <v>3.48</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>KG모빌리티</t>
+          <t>GS리테일</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -4136,30 +4136,30 @@
       <c r="D32" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="E32" s="32" t="n">
+      <c r="E32" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H32" s="29" t="n">
-        <v>-0.17</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H32" s="27" t="n">
+        <v>7.18</v>
       </c>
       <c r="I32" s="27" t="n">
-        <v>1.76</v>
+        <v>14.55</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>SK디앤디</t>
+          <t>HJ중공업</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4171,30 +4171,30 @@
       <c r="D33" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="E33" s="32" t="n">
+      <c r="E33" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H33" s="29" t="n">
-        <v>-11.95</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H33" s="25" t="n">
+        <v>0</v>
       </c>
       <c r="I33" s="27" t="n">
-        <v>22.2</v>
+        <v>6.37</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>기아</t>
+          <t>HMM</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4206,30 +4206,30 @@
       <c r="D34" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="E34" s="32" t="n">
+      <c r="E34" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="H34" s="27" t="n">
-        <v>0.97</v>
+        <v>1.87</v>
       </c>
       <c r="I34" s="27" t="n">
-        <v>2.27</v>
+        <v>4.06</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>KG모빌리티</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -4241,30 +4241,30 @@
       <c r="D35" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="E35" s="32" t="n">
+      <c r="E35" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H35" s="29" t="n">
-        <v>-2.73</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H35" s="32" t="n">
+        <v>-0.17</v>
       </c>
       <c r="I35" s="27" t="n">
-        <v>28.4</v>
+        <v>1.76</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>랩지노믹스</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
@@ -4276,30 +4276,30 @@
       <c r="D36" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="E36" s="32" t="n">
+      <c r="E36" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H36" s="27" t="n">
-        <v>12.5</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H36" s="32" t="n">
+        <v>-2.73</v>
       </c>
       <c r="I36" s="27" t="n">
-        <v>61.24</v>
+        <v>28.4</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>비큐AI</t>
+          <t>랩지노믹스</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
@@ -4311,30 +4311,30 @@
       <c r="D37" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="E37" s="32" t="n">
+      <c r="E37" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H37" s="29" t="n">
-        <v>-11.88</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H37" s="27" t="n">
+        <v>12.5</v>
       </c>
       <c r="I37" s="27" t="n">
-        <v>93.48</v>
+        <v>61.24</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>비큐AI</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4346,30 +4346,30 @@
       <c r="D38" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="E38" s="32" t="n">
+      <c r="E38" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H38" s="27" t="n">
-        <v>7.49</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H38" s="32" t="n">
+        <v>-11.88</v>
       </c>
       <c r="I38" s="27" t="n">
-        <v>15.62</v>
+        <v>93.48</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>서울전자통신</t>
+          <t>빛과전자</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4381,30 +4381,30 @@
       <c r="D39" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="E39" s="32" t="n">
+      <c r="E39" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="H39" s="27" t="n">
-        <v>12.83</v>
+        <v>3.26</v>
       </c>
       <c r="I39" s="27" t="n">
-        <v>31.66</v>
+        <v>60.01</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>신성이엔지</t>
+          <t>서울전자통신</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4416,30 +4416,30 @@
       <c r="D40" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="E40" s="32" t="n">
+      <c r="E40" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H40" s="29" t="n">
-        <v>-5.32</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H40" s="27" t="n">
+        <v>12.83</v>
       </c>
       <c r="I40" s="27" t="n">
-        <v>7.38</v>
+        <v>31.66</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>아미코젠</t>
+          <t>심텍</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4451,30 +4451,30 @@
       <c r="D41" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="E41" s="32" t="n">
+      <c r="E41" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H41" s="29" t="n">
-        <v>-1.82</v>
-      </c>
-      <c r="I41" s="29" t="n">
-        <v>-8.98</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H41" s="27" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="I41" s="27" t="n">
+        <v>32.69</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>엘앤에프</t>
+          <t>아미코젠</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4486,30 +4486,30 @@
       <c r="D42" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="E42" s="32" t="n">
+      <c r="E42" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H42" s="27" t="n">
-        <v>13.03</v>
-      </c>
-      <c r="I42" s="27" t="n">
-        <v>23.06</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H42" s="32" t="n">
+        <v>-1.82</v>
+      </c>
+      <c r="I42" s="32" t="n">
+        <v>-8.98</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>오이솔루션</t>
+          <t>엘앤에프</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4521,30 +4521,30 @@
       <c r="D43" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="E43" s="32" t="n">
+      <c r="E43" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="H43" s="27" t="n">
-        <v>18.53</v>
+        <v>13.03</v>
       </c>
       <c r="I43" s="27" t="n">
-        <v>69.11</v>
+        <v>23.06</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>와이즈버즈</t>
+          <t>오이솔루션</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4556,24 +4556,24 @@
       <c r="D44" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="E44" s="32" t="n">
+      <c r="E44" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="H44" s="27" t="n">
-        <v>4.85</v>
+        <v>18.53</v>
       </c>
       <c r="I44" s="27" t="n">
-        <v>33.59</v>
+        <v>69.11</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
@@ -4591,17 +4591,17 @@
       <c r="D45" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="E45" s="32" t="n">
+      <c r="E45" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="H45" s="25" t="n">
@@ -4614,7 +4614,7 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4626,17 +4626,17 @@
       <c r="D46" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="E46" s="32" t="n">
+      <c r="E46" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="H46" s="25" t="n"/>
@@ -4645,7 +4645,7 @@
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>한국첨단소재</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4657,135 +4657,131 @@
       <c r="D47" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="E47" s="32" t="n">
+      <c r="E47" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="H47" s="27" t="n">
-        <v>29.89</v>
+        <v>4.18</v>
       </c>
       <c r="I47" s="27" t="n">
-        <v>29.89</v>
+        <v>6.68</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>광전자</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C48" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D48" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E48" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="E48" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H48" s="27" t="n">
-        <v>15.02</v>
-      </c>
-      <c r="I48" s="27" t="n">
-        <v>50.48</v>
-      </c>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H48" s="25" t="n"/>
+      <c r="I48" s="25" t="n"/>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>동화기업</t>
+          <t>한국첨단소재</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C49" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D49" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E49" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="E49" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="H49" s="27" t="n">
-        <v>30</v>
+        <v>29.89</v>
       </c>
       <c r="I49" s="27" t="n">
-        <v>44.19</v>
+        <v>29.89</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>삼기에너지솔루션즈</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C50" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D50" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E50" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="E50" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H50" s="29" t="n">
-        <v>-1.91</v>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H50" s="27" t="n">
+        <v>11.51</v>
       </c>
       <c r="I50" s="27" t="n">
-        <v>39.11</v>
+        <v>32.94</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>상상인증권</t>
+          <t>동화기업</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4797,24 +4793,24 @@
       <c r="D51" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="E51" s="32" t="n">
+      <c r="E51" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="H51" s="27" t="n">
-        <v>29.91</v>
+        <v>30</v>
       </c>
       <c r="I51" s="27" t="n">
-        <v>85.08</v>
+        <v>44.19</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
@@ -4832,17 +4828,17 @@
       <c r="D52" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="E52" s="32" t="n">
+      <c r="E52" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="H52" s="27" t="n">
@@ -4933,19 +4929,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>51</v>
+        <v>76</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>51</v>
+        <v>76</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4964,19 +4960,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4988,26 +4984,26 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="35" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B5" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5026,19 +5022,19 @@
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5050,26 +5046,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5081,92 +5077,100 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
+          <t>조선</t>
+        </is>
+      </c>
+      <c r="B8" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="36" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" s="36" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" s="36" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="F8" s="37" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G8" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="35" t="inlineStr">
+        <is>
+          <t>제약</t>
+        </is>
+      </c>
+      <c r="B9" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" s="36" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="F9" s="37" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G9" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
           <t>인공지능</t>
         </is>
       </c>
-      <c r="B8" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" s="36" t="n">
-        <v>13</v>
-      </c>
-      <c r="D8" s="36" t="n">
-        <v>13</v>
-      </c>
-      <c r="E8" s="36" t="inlineStr">
-        <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="F8" s="37" t="inlineStr">
-        <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="G8" s="37" t="inlineStr">
+      <c r="B10" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="36" t="n">
+        <v>14</v>
+      </c>
+      <c r="D10" s="36" t="n">
+        <v>14</v>
+      </c>
+      <c r="E10" s="36" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="F10" s="37" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G10" s="37" t="inlineStr">
         <is>
           <t>⚡ 관심</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="26" t="inlineStr">
-        <is>
-          <t>이차전지</t>
-        </is>
-      </c>
-      <c r="B9" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F9" s="28" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="inlineStr"/>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="26" t="inlineStr">
-        <is>
-          <t>AI반도체</t>
-        </is>
-      </c>
-      <c r="B10" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" s="28" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>이차전지</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
@@ -5193,7 +5197,7 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
@@ -5220,7 +5224,7 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -5247,7 +5251,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5274,7 +5278,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5301,7 +5305,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -5328,7 +5332,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>핀테크</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -5355,7 +5359,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>핀테크</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -5382,7 +5386,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-08-11 07:02 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -258,13 +258,13 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-08-10 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-08-11 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-08-10) 상위: 반도체  점수 76.0점</t>
+          <t>⚡ 최신(2026-08-11) 상위: 반도체  점수 70.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-08-10) 상위: SK하이닉스  점수 34.0점</t>
+          <t>⚡ 최신(2026-08-11) 상위: 삼성전자  점수 32.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-08-10) 상위: 로봇  점수 20.0점</t>
+          <t>⚡ 최신(2026-08-11) 상위: SK하이닉스  점수 29.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,19 +947,19 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR) / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
         <is>
-          <t>네이버, Google</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -967,42 +967,40 @@
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G15" s="15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>-4.88</v>
+        <v>-0.43</v>
       </c>
       <c r="I15" s="18" t="n">
-        <v>-17.23</v>
+        <v>-3.97</v>
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 7일 +200% / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K15" s="17" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K15" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1010,42 +1008,42 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I16" s="15" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H16" s="18" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="I16" s="18" t="n">
+        <v>-9.380000000000001</v>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 3건 / 중요공시 7일 +200% / 매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1053,14 +1051,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1068,15 +1066,15 @@
       <c r="G17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="19" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="I17" s="18" t="n">
-        <v>-12</v>
+      <c r="H17" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I17" s="15" t="n">
+        <v/>
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
@@ -1088,7 +1086,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1096,14 +1094,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1119,7 +1117,7 @@
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K18" s="17" t="inlineStr">
@@ -1131,7 +1129,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1139,40 +1137,42 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
         <v>16</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F19" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G19" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I19" s="15" t="n">
-        <v/>
+      <c r="H19" s="19" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="I19" s="19" t="n">
+        <v>42.45</v>
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K19" s="17" t="n">
-        <v/>
+          <t>중요공시 3건 / 중요공시 3일 +50% / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K19" s="17" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1180,14 +1180,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>산일전기</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1195,27 +1195,27 @@
       <c r="G20" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I20" s="15" t="n">
-        <v/>
+      <c r="H20" s="19" t="n">
+        <v>16.85</v>
+      </c>
+      <c r="I20" s="19" t="n">
+        <v>26.24</v>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 2건 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K20" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1223,42 +1223,42 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>에코프로</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
         <v>10</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F21" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G21" s="15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H21" s="19" t="n">
-        <v>14.96</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="I21" s="19" t="n">
-        <v>49.68</v>
+        <v>20.8</v>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +55% / 중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +200%</t>
+          <t>중요공시 1건 / Google 급상승 검색어 등장 (KR) / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>Google, 공시</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1266,14 +1266,14 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="n">
@@ -1299,7 +1299,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>테스</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
@@ -1322,15 +1322,15 @@
       <c r="G23" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="18" t="n">
-        <v>-4.23</v>
-      </c>
-      <c r="I23" s="18" t="n">
-        <v>-4.15</v>
+      <c r="H23" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I23" s="15" t="n">
+        <v/>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K23" s="17" t="inlineStr">
@@ -1342,7 +1342,7 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1350,42 +1350,42 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>POSCO홀딩스</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
         <v>8</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G24" s="15" t="n">
         <v>3</v>
       </c>
       <c r="H24" s="19" t="n">
-        <v>3.76</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="I24" s="19" t="n">
-        <v>5.92</v>
+        <v>56.97</v>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+          <t>네이버 검색 당일 +61% / 중요공시 4건 / 중요공시 7일 +300%</t>
         </is>
       </c>
       <c r="K24" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1393,14 +1393,14 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>TSMC</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F25" s="15" t="n">
         <v>0</v>
@@ -1408,15 +1408,15 @@
       <c r="G25" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H25" s="18" t="n">
-        <v>-1.12</v>
-      </c>
-      <c r="I25" s="19" t="n">
-        <v>1.93</v>
+      <c r="H25" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I25" s="15" t="n">
+        <v/>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K25" s="17" t="n">
@@ -1424,52 +1424,52 @@
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="15" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="B26" s="15" t="n">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="n">
         <v>13</v>
       </c>
-      <c r="C26" s="16" t="inlineStr">
-        <is>
-          <t>유티아이</t>
-        </is>
-      </c>
-      <c r="D26" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E26" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="F26" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="G26" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="19" t="n">
-        <v>13.2</v>
-      </c>
-      <c r="I26" s="18" t="n">
-        <v>-3.46</v>
-      </c>
-      <c r="J26" s="17" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +93% / 중요공시 5건 / 중요공시 3일 +400%</t>
-        </is>
-      </c>
-      <c r="K26" s="17" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
+      <c r="C26" s="21" t="inlineStr">
+        <is>
+          <t>금호건설</t>
+        </is>
+      </c>
+      <c r="D26" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E26" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F26" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H26" s="22" t="n">
+        <v>-9.52</v>
+      </c>
+      <c r="I26" s="22" t="n">
+        <v>-1.56</v>
+      </c>
+      <c r="J26" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 7일 +200%</t>
+        </is>
+      </c>
+      <c r="K26" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B27" s="20" t="n">
@@ -1477,7 +1477,7 @@
       </c>
       <c r="C27" s="21" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>썸에이지</t>
         </is>
       </c>
       <c r="D27" s="20" t="n">
@@ -1493,14 +1493,14 @@
         <v>3</v>
       </c>
       <c r="H27" s="22" t="n">
-        <v>1.14</v>
+        <v>-12.06</v>
       </c>
       <c r="I27" s="22" t="n">
-        <v>7.24</v>
+        <v>-33.63</v>
       </c>
       <c r="J27" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 7일 +200%</t>
+          <t>중요공시 4건 / 중요공시 7일 +300%</t>
         </is>
       </c>
       <c r="K27" s="23" t="inlineStr">
@@ -1512,7 +1512,7 @@
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B28" s="20" t="n">
@@ -1520,30 +1520,30 @@
       </c>
       <c r="C28" s="21" t="inlineStr">
         <is>
-          <t>HLB테라퓨틱스</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="D28" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E28" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F28" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G28" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="22" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="I28" s="22" t="n">
-        <v>22.81</v>
+        <v>3</v>
+      </c>
+      <c r="H28" s="24" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="I28" s="24" t="n">
+        <v>10.71</v>
       </c>
       <c r="J28" s="23" t="inlineStr">
         <is>
-          <t>중요공시 5건 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 4건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K28" s="23" t="inlineStr">
@@ -1555,7 +1555,7 @@
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B29" s="20" t="n">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>썸에이지</t>
+          <t>LG씨엔에스</t>
         </is>
       </c>
       <c r="D29" s="20" t="n">
@@ -1579,14 +1579,14 @@
         <v>3</v>
       </c>
       <c r="H29" s="24" t="n">
-        <v>-2.69</v>
+        <v>1.38</v>
       </c>
       <c r="I29" s="24" t="n">
-        <v>-1.94</v>
+        <v>17.76</v>
       </c>
       <c r="J29" s="23" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 중요공시 7일 +300%</t>
+          <t>중요공시 3건 / 중요공시 7일 +200%</t>
         </is>
       </c>
       <c r="K29" s="23" t="inlineStr">
@@ -1598,7 +1598,7 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
@@ -1606,30 +1606,30 @@
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>지엔씨에너지</t>
+          <t>다보링크</t>
         </is>
       </c>
       <c r="D30" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E30" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F30" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G30" s="20" t="n">
         <v>3</v>
       </c>
       <c r="H30" s="22" t="n">
-        <v>2.35</v>
-      </c>
-      <c r="I30" s="22" t="n">
-        <v>42.9</v>
+        <v>-8.09</v>
+      </c>
+      <c r="I30" s="24" t="n">
+        <v>9.52</v>
       </c>
       <c r="J30" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 7일 +50%</t>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K30" s="23" t="inlineStr">
@@ -1641,7 +1641,7 @@
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1649,42 +1649,42 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>한울반도체</t>
+          <t>HJ중공업</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F31" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G31" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H31" s="24" t="n">
-        <v>-1.81</v>
-      </c>
-      <c r="I31" s="22" t="n">
-        <v>1.42</v>
+        <v>4.73</v>
+      </c>
+      <c r="I31" s="24" t="n">
+        <v>12.55</v>
       </c>
       <c r="J31" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / Google 급상승 검색어 등장 (KR)</t>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K31" s="23" t="inlineStr">
         <is>
-          <t>Google, 공시</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1692,42 +1692,40 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>현대지에프홀딩스</t>
+          <t>리노공업</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F32" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G32" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H32" s="22" t="n">
-        <v>3.04</v>
-      </c>
-      <c r="I32" s="22" t="n">
-        <v>3.48</v>
+      <c r="H32" s="24" t="n">
+        <v>7.61</v>
+      </c>
+      <c r="I32" s="24" t="n">
+        <v>15.15</v>
       </c>
       <c r="J32" s="23" t="inlineStr">
         <is>
-          <t>중요공시 10건 / 중요공시 3일 +67%</t>
-        </is>
-      </c>
-      <c r="K32" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K32" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1735,42 +1733,40 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>티엘비</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F33" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G33" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H33" s="24" t="n">
-        <v>-6.18</v>
-      </c>
-      <c r="I33" s="22" t="n">
-        <v>6.44</v>
+      <c r="H33" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I33" s="20" t="n">
+        <v/>
       </c>
       <c r="J33" s="23" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 중요공시 3일 +300%</t>
-        </is>
-      </c>
-      <c r="K33" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K33" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1778,42 +1774,42 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>서진시스템</t>
+          <t>유니켐</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F34" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G34" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="24" t="n">
-        <v>-3.94</v>
-      </c>
-      <c r="I34" s="22" t="n">
-        <v>3.33</v>
+      <c r="H34" s="22" t="n">
+        <v>-2.71</v>
+      </c>
+      <c r="I34" s="24" t="n">
+        <v>76.38</v>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200%</t>
+          <t>네이버 검색 당일 +76% / 중요공시 3건</t>
         </is>
       </c>
       <c r="K34" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1821,30 +1817,30 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>알테오젠</t>
+          <t>GS건설</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F35" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G35" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H35" s="22" t="n">
-        <v>3.92</v>
-      </c>
-      <c r="I35" s="22" t="n">
-        <v>28.49</v>
+      <c r="H35" s="24" t="n">
+        <v>10.27</v>
+      </c>
+      <c r="I35" s="24" t="n">
+        <v>43.92</v>
       </c>
       <c r="J35" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +50%</t>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K35" s="23" t="inlineStr">
@@ -1856,7 +1852,7 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1864,42 +1860,42 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>제주반도체</t>
+          <t>유니슨</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F36" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G36" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H36" s="22" t="n">
-        <v>1.48</v>
-      </c>
-      <c r="I36" s="22" t="n">
-        <v>15.82</v>
+        <v>3</v>
+      </c>
+      <c r="H36" s="24" t="n">
+        <v>8.93</v>
+      </c>
+      <c r="I36" s="24" t="n">
+        <v>38.7</v>
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K36" s="23" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1907,7 +1903,7 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>SFA반도체</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
@@ -1922,27 +1918,27 @@
       <c r="G37" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H37" s="24" t="n">
-        <v>-2.44</v>
-      </c>
-      <c r="I37" s="22" t="n">
-        <v>2.57</v>
+      <c r="H37" s="22" t="n">
+        <v>-0.88</v>
+      </c>
+      <c r="I37" s="24" t="n">
+        <v>6.32</v>
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
+          <t>중요공시 2건 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K37" s="23" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1950,42 +1946,42 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>한미반도체</t>
+          <t>현대지에프홀딩스</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F38" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H38" s="24" t="n">
-        <v>-4.09</v>
+      <c r="H38" s="22" t="n">
+        <v>-3.04</v>
       </c>
       <c r="I38" s="24" t="n">
-        <v>-10.35</v>
+        <v>0.34</v>
       </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
+          <t>중요공시 10건 / 중요공시 3일 +67%</t>
         </is>
       </c>
       <c r="K38" s="23" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1993,42 +1989,42 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>서울반도체</t>
+          <t>HLB테라퓨틱스</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F39" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G39" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H39" s="24" t="n">
-        <v>-0.33</v>
-      </c>
-      <c r="I39" s="22" t="n">
-        <v>5.17</v>
+        <v>12.04</v>
+      </c>
+      <c r="I39" s="24" t="n">
+        <v>31.79</v>
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
+          <t>중요공시 5건 / 중요공시 3일 +400%</t>
         </is>
       </c>
       <c r="K39" s="23" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2036,7 +2032,7 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
@@ -2051,27 +2047,25 @@
       <c r="G40" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H40" s="20" t="n">
+      <c r="H40" s="24" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="I40" s="24" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="J40" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K40" s="23" t="n">
         <v/>
-      </c>
-      <c r="I40" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J40" s="23" t="inlineStr">
-        <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
-        </is>
-      </c>
-      <c r="K40" s="23" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2079,7 +2073,7 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
@@ -2094,27 +2088,25 @@
       <c r="G41" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="22" t="n">
-        <v>3.99</v>
-      </c>
-      <c r="I41" s="22" t="n">
-        <v>11.91</v>
+      <c r="H41" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I41" s="20" t="n">
+        <v/>
       </c>
       <c r="J41" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K41" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K41" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2122,14 +2114,14 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>비큐AI</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E42" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F42" s="20" t="n">
         <v>0</v>
@@ -2137,27 +2129,25 @@
       <c r="G42" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H42" s="24" t="n">
-        <v>-11.88</v>
-      </c>
-      <c r="I42" s="22" t="n">
-        <v>93.48</v>
+      <c r="H42" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I42" s="20" t="n">
+        <v/>
       </c>
       <c r="J42" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +829% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K42" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K42" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2165,7 +2155,7 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>오이솔루션</t>
+          <t>비큐AI</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
@@ -2181,26 +2171,26 @@
         <v>0</v>
       </c>
       <c r="H43" s="22" t="n">
-        <v>18.53</v>
-      </c>
-      <c r="I43" s="22" t="n">
-        <v>69.11</v>
+        <v>-2.36</v>
+      </c>
+      <c r="I43" s="24" t="n">
+        <v>88.91</v>
       </c>
       <c r="J43" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +310% / 매일경제 기사 언급</t>
+          <t>네이버 검색 당일 +861% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K43" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2208,7 +2198,7 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>이스트에이드</t>
+          <t>윙입푸드</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
@@ -2223,15 +2213,15 @@
       <c r="G44" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I44" s="22" t="n">
-        <v>65.42</v>
+      <c r="H44" s="24" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="I44" s="24" t="n">
+        <v>94.79000000000001</v>
       </c>
       <c r="J44" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +219% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +554% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K44" s="23" t="inlineStr">
@@ -2243,7 +2233,7 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2267,14 +2257,14 @@
         <v>0</v>
       </c>
       <c r="H45" s="22" t="n">
-        <v>29.89</v>
-      </c>
-      <c r="I45" s="22" t="n">
-        <v>29.89</v>
+        <v>-0.17</v>
+      </c>
+      <c r="I45" s="24" t="n">
+        <v>29.68</v>
       </c>
       <c r="J45" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +177% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +207% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K45" s="23" t="inlineStr">
@@ -2286,7 +2276,7 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
@@ -2310,14 +2300,14 @@
         <v>0</v>
       </c>
       <c r="H46" s="22" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="I46" s="22" t="n">
-        <v>61.24</v>
+        <v>-6.69</v>
+      </c>
+      <c r="I46" s="24" t="n">
+        <v>42.39</v>
       </c>
       <c r="J46" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +132% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +143% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K46" s="23" t="inlineStr">
@@ -2329,7 +2319,7 @@
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B47" s="20" t="n">
@@ -2352,15 +2342,15 @@
       <c r="G47" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H47" s="22" t="n">
-        <v>3.26</v>
-      </c>
-      <c r="I47" s="22" t="n">
-        <v>60.01</v>
+      <c r="H47" s="24" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="I47" s="24" t="n">
+        <v>55.36</v>
       </c>
       <c r="J47" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +122% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +130% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K47" s="23" t="inlineStr">
@@ -2372,7 +2362,7 @@
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B48" s="20" t="n">
@@ -2380,7 +2370,7 @@
       </c>
       <c r="C48" s="21" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>LK삼양</t>
         </is>
       </c>
       <c r="D48" s="20" t="n">
@@ -2396,26 +2386,26 @@
         <v>0</v>
       </c>
       <c r="H48" s="24" t="n">
-        <v>-2.73</v>
-      </c>
-      <c r="I48" s="22" t="n">
-        <v>28.4</v>
+        <v>29.92</v>
+      </c>
+      <c r="I48" s="24" t="n">
+        <v>50.09</v>
       </c>
       <c r="J48" s="23" t="inlineStr">
         <is>
-          <t>중요공시 4건</t>
+          <t>네이버 검색 당일 +115% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K48" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B49" s="20" t="n">
@@ -2423,7 +2413,7 @@
       </c>
       <c r="C49" s="21" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>코칩</t>
         </is>
       </c>
       <c r="D49" s="20" t="n">
@@ -2438,25 +2428,27 @@
       <c r="G49" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="22" t="n">
-        <v>11.51</v>
-      </c>
-      <c r="I49" s="22" t="n">
-        <v>32.94</v>
+      <c r="H49" s="24" t="n">
+        <v>4.97</v>
+      </c>
+      <c r="I49" s="24" t="n">
+        <v>27.23</v>
       </c>
       <c r="J49" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K49" s="23" t="n">
-        <v/>
+          <t>네이버 검색 당일 +112% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K49" s="23" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B50" s="20" t="n">
@@ -2464,7 +2456,7 @@
       </c>
       <c r="C50" s="21" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>금강철강</t>
         </is>
       </c>
       <c r="D50" s="20" t="n">
@@ -2479,27 +2471,27 @@
       <c r="G50" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H50" s="22" t="n">
-        <v>4.18</v>
-      </c>
-      <c r="I50" s="22" t="n">
-        <v>6.68</v>
+      <c r="H50" s="24" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="I50" s="24" t="n">
+        <v>26.25</v>
       </c>
       <c r="J50" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 매일경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +106% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K50" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B51" s="20" t="n">
@@ -2507,30 +2499,30 @@
       </c>
       <c r="C51" s="21" t="inlineStr">
         <is>
-          <t>아미코젠</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="D51" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E51" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F51" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G51" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H51" s="24" t="n">
-        <v>-1.82</v>
+        <v>3.78</v>
       </c>
       <c r="I51" s="24" t="n">
-        <v>-8.98</v>
+        <v>28.05</v>
       </c>
       <c r="J51" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+          <t>중요공시 4건</t>
         </is>
       </c>
       <c r="K51" s="23" t="inlineStr">
@@ -2542,7 +2534,7 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B52" s="20" t="n">
@@ -2550,42 +2542,42 @@
       </c>
       <c r="C52" s="21" t="inlineStr">
         <is>
-          <t>KG모빌리티</t>
+          <t>대동</t>
         </is>
       </c>
       <c r="D52" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E52" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F52" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G52" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H52" s="24" t="n">
-        <v>-0.17</v>
-      </c>
-      <c r="I52" s="22" t="n">
-        <v>1.76</v>
+        <v>15.9</v>
+      </c>
+      <c r="I52" s="24" t="n">
+        <v>20.37</v>
       </c>
       <c r="J52" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K52" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B53" s="20" t="n">
@@ -2593,30 +2585,30 @@
       </c>
       <c r="C53" s="21" t="inlineStr">
         <is>
-          <t>HJ중공업</t>
+          <t>SK스퀘어</t>
         </is>
       </c>
       <c r="D53" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E53" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F53" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G53" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H53" s="20" t="n">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="H53" s="24" t="n">
+        <v>1.06</v>
       </c>
       <c r="I53" s="22" t="n">
-        <v>6.37</v>
+        <v>-7.41</v>
       </c>
       <c r="J53" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+          <t>중요공시 3건 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K53" s="23" t="inlineStr">
@@ -2628,7 +2620,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B54" s="20" t="n">
@@ -2636,30 +2628,30 @@
       </c>
       <c r="C54" s="21" t="inlineStr">
         <is>
-          <t>엘앤에프</t>
+          <t>아미코젠</t>
         </is>
       </c>
       <c r="D54" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E54" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F54" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G54" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H54" s="22" t="n">
-        <v>13.03</v>
+        <v>3</v>
+      </c>
+      <c r="H54" s="24" t="n">
+        <v>4</v>
       </c>
       <c r="I54" s="22" t="n">
-        <v>23.06</v>
+        <v>-6.5</v>
       </c>
       <c r="J54" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K54" s="23" t="inlineStr">
@@ -2671,7 +2663,7 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B55" s="20" t="n">
@@ -2679,30 +2671,30 @@
       </c>
       <c r="C55" s="21" t="inlineStr">
         <is>
-          <t>심텍</t>
+          <t>시선AI</t>
         </is>
       </c>
       <c r="D55" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E55" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F55" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G55" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H55" s="22" t="n">
-        <v>3.77</v>
-      </c>
-      <c r="I55" s="22" t="n">
-        <v>32.69</v>
+        <v>3</v>
+      </c>
+      <c r="H55" s="24" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="I55" s="24" t="n">
+        <v>5.76</v>
       </c>
       <c r="J55" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K55" s="23" t="inlineStr">
@@ -2714,7 +2706,7 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B56" s="20" t="n">
@@ -2722,30 +2714,30 @@
       </c>
       <c r="C56" s="21" t="inlineStr">
         <is>
-          <t>서울전자통신</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="D56" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E56" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F56" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G56" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H56" s="22" t="n">
-        <v>12.83</v>
-      </c>
-      <c r="I56" s="22" t="n">
-        <v>31.66</v>
+        <v>3</v>
+      </c>
+      <c r="H56" s="24" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="I56" s="24" t="n">
+        <v>15.69</v>
       </c>
       <c r="J56" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K56" s="23" t="inlineStr">
@@ -2757,7 +2749,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B57" s="20" t="n">
@@ -2765,7 +2757,7 @@
       </c>
       <c r="C57" s="21" t="inlineStr">
         <is>
-          <t>GS리테일</t>
+          <t>롯데케미칼</t>
         </is>
       </c>
       <c r="D57" s="20" t="n">
@@ -2781,10 +2773,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="22" t="n">
-        <v>7.18</v>
-      </c>
-      <c r="I57" s="22" t="n">
-        <v>14.55</v>
+        <v>-4.1</v>
+      </c>
+      <c r="I57" s="24" t="n">
+        <v>5.98</v>
       </c>
       <c r="J57" s="23" t="inlineStr">
         <is>
@@ -2800,7 +2792,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B58" s="20" t="n">
@@ -2808,7 +2800,7 @@
       </c>
       <c r="C58" s="21" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="D58" s="20" t="n">
@@ -2823,15 +2815,15 @@
       <c r="G58" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I58" s="20" t="n">
-        <v/>
+      <c r="H58" s="22" t="n">
+        <v>-1.62</v>
+      </c>
+      <c r="I58" s="24" t="n">
+        <v>15.01</v>
       </c>
       <c r="J58" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>한국경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K58" s="23" t="inlineStr">
@@ -2841,134 +2833,138 @@
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="20" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="B59" s="20" t="n">
+      <c r="A59" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B59" s="25" t="n">
         <v>46</v>
       </c>
-      <c r="C59" s="21" t="inlineStr">
-        <is>
-          <t>태양광</t>
-        </is>
-      </c>
-      <c r="D59" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E59" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F59" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G59" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H59" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I59" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J59" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K59" s="23" t="inlineStr">
+      <c r="C59" s="26" t="inlineStr">
+        <is>
+          <t>신스틸</t>
+        </is>
+      </c>
+      <c r="D59" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E59" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F59" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" s="27" t="n">
+        <v>7.24</v>
+      </c>
+      <c r="I59" s="27" t="n">
+        <v>38.01</v>
+      </c>
+      <c r="J59" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +329%</t>
+        </is>
+      </c>
+      <c r="K59" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="20" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="B60" s="20" t="n">
+      <c r="A60" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B60" s="25" t="n">
         <v>47</v>
       </c>
-      <c r="C60" s="21" t="inlineStr">
-        <is>
-          <t>DB</t>
-        </is>
-      </c>
-      <c r="D60" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E60" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F60" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G60" s="20" t="n">
-        <v>0</v>
-      </c>
